<commit_message>
Add July grocery expenses for CIUDAD.
Record Sol's kitchen siphon replacement, produce, and supermarket spending so the monthly ALMACEN total updates automatically.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -615,7 +615,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1370,7 +1369,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
@@ -2998,8 +2996,14 @@
         </is>
       </c>
       <c r="B106" s="17" t="n"/>
-      <c r="C106" s="14" t="n"/>
-      <c r="D106" s="27" t="n"/>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>Repuesto sifón cocina</t>
+        </is>
+      </c>
+      <c r="D106" s="27" t="n">
+        <v>20000</v>
+      </c>
       <c r="E106" s="28" t="n"/>
       <c r="F106" s="15">
         <f>IF(OR(D106&lt;&gt;"",E106&lt;&gt;""),IF(D106="",0,D106)+IF(E106="",0,E106),"")</f>
@@ -3013,8 +3017,14 @@
         </is>
       </c>
       <c r="B107" s="17" t="n"/>
-      <c r="C107" s="14" t="n"/>
-      <c r="D107" s="27" t="n"/>
+      <c r="C107" s="14" t="inlineStr">
+        <is>
+          <t>Verdulería</t>
+        </is>
+      </c>
+      <c r="D107" s="27" t="n">
+        <v>8400</v>
+      </c>
       <c r="E107" s="28" t="n"/>
       <c r="F107" s="15">
         <f>IF(OR(D107&lt;&gt;"",E107&lt;&gt;""),IF(D107="",0,D107)+IF(E107="",0,E107),"")</f>
@@ -3028,8 +3038,14 @@
         </is>
       </c>
       <c r="B108" s="17" t="n"/>
-      <c r="C108" s="14" t="n"/>
-      <c r="D108" s="27" t="n"/>
+      <c r="C108" s="14" t="inlineStr">
+        <is>
+          <t>Supermercado</t>
+        </is>
+      </c>
+      <c r="D108" s="27" t="n">
+        <v>70000</v>
+      </c>
       <c r="E108" s="28" t="n"/>
       <c r="F108" s="15">
         <f>IF(OR(D108&lt;&gt;"",E108&lt;&gt;""),IF(D108="",0,D108)+IF(E108="",0,E108),"")</f>

</xml_diff>

<commit_message>
Add more July grocery spending for CIUDAD Sol.
Include Coto supermarket and Día partido purchases so the ALMACEN SOL July total stays current.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3059,8 +3059,14 @@
         </is>
       </c>
       <c r="B109" s="17" t="n"/>
-      <c r="C109" s="14" t="n"/>
-      <c r="D109" s="27" t="n"/>
+      <c r="C109" s="14" t="inlineStr">
+        <is>
+          <t>Supermercado Coto</t>
+        </is>
+      </c>
+      <c r="D109" s="27" t="n">
+        <v>234000</v>
+      </c>
       <c r="E109" s="28" t="n"/>
       <c r="F109" s="15">
         <f>IF(OR(D109&lt;&gt;"",E109&lt;&gt;""),IF(D109="",0,D109)+IF(E109="",0,E109),"")</f>
@@ -3074,8 +3080,14 @@
         </is>
       </c>
       <c r="B110" s="17" t="n"/>
-      <c r="C110" s="14" t="n"/>
-      <c r="D110" s="27" t="n"/>
+      <c r="C110" s="14" t="inlineStr">
+        <is>
+          <t>Día partido</t>
+        </is>
+      </c>
+      <c r="D110" s="27" t="n">
+        <v>140000</v>
+      </c>
       <c r="E110" s="28" t="n"/>
       <c r="F110" s="15">
         <f>IF(OR(D110&lt;&gt;"",E110&lt;&gt;""),IF(D110="",0,D110)+IF(E110="",0,E110),"")</f>

</xml_diff>

<commit_message>
Add comments field to CIUDAD grocery details.
Allow contextual notes on each ALMACEN expense while preserving monthly totals and summary links.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1432,7 +1432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F212"/>
+  <dimension ref="A1:G212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1441,6 +1441,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1486,6 +1487,11 @@
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Total</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Comentario</t>
         </is>
       </c>
     </row>
@@ -1503,6 +1509,7 @@
         <f>IF(OR(D4&lt;&gt;"",E4&lt;&gt;""),IF(D4="",0,D4)+IF(E4="",0,E4),"")</f>
         <v/>
       </c>
+      <c r="G4" s="14" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -1518,6 +1525,7 @@
         <f>IF(OR(D5&lt;&gt;"",E5&lt;&gt;""),IF(D5="",0,D5)+IF(E5="",0,E5),"")</f>
         <v/>
       </c>
+      <c r="G5" s="14" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -1533,6 +1541,7 @@
         <f>IF(OR(D6&lt;&gt;"",E6&lt;&gt;""),IF(D6="",0,D6)+IF(E6="",0,E6),"")</f>
         <v/>
       </c>
+      <c r="G6" s="14" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
@@ -1548,6 +1557,7 @@
         <f>IF(OR(D7&lt;&gt;"",E7&lt;&gt;""),IF(D7="",0,D7)+IF(E7="",0,E7),"")</f>
         <v/>
       </c>
+      <c r="G7" s="14" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
@@ -1563,6 +1573,7 @@
         <f>IF(OR(D8&lt;&gt;"",E8&lt;&gt;""),IF(D8="",0,D8)+IF(E8="",0,E8),"")</f>
         <v/>
       </c>
+      <c r="G8" s="14" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
@@ -1578,6 +1589,7 @@
         <f>IF(OR(D9&lt;&gt;"",E9&lt;&gt;""),IF(D9="",0,D9)+IF(E9="",0,E9),"")</f>
         <v/>
       </c>
+      <c r="G9" s="14" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1593,6 +1605,7 @@
         <f>IF(OR(D10&lt;&gt;"",E10&lt;&gt;""),IF(D10="",0,D10)+IF(E10="",0,E10),"")</f>
         <v/>
       </c>
+      <c r="G10" s="14" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -1608,6 +1621,7 @@
         <f>IF(OR(D11&lt;&gt;"",E11&lt;&gt;""),IF(D11="",0,D11)+IF(E11="",0,E11),"")</f>
         <v/>
       </c>
+      <c r="G11" s="14" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1623,6 +1637,7 @@
         <f>IF(OR(D12&lt;&gt;"",E12&lt;&gt;""),IF(D12="",0,D12)+IF(E12="",0,E12),"")</f>
         <v/>
       </c>
+      <c r="G12" s="14" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
@@ -1638,6 +1653,7 @@
         <f>IF(OR(D13&lt;&gt;"",E13&lt;&gt;""),IF(D13="",0,D13)+IF(E13="",0,E13),"")</f>
         <v/>
       </c>
+      <c r="G13" s="14" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
@@ -1653,6 +1669,7 @@
         <f>IF(OR(D14&lt;&gt;"",E14&lt;&gt;""),IF(D14="",0,D14)+IF(E14="",0,E14),"")</f>
         <v/>
       </c>
+      <c r="G14" s="14" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
@@ -1668,6 +1685,7 @@
         <f>IF(OR(D15&lt;&gt;"",E15&lt;&gt;""),IF(D15="",0,D15)+IF(E15="",0,E15),"")</f>
         <v/>
       </c>
+      <c r="G15" s="14" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -1683,6 +1701,7 @@
         <f>IF(OR(D16&lt;&gt;"",E16&lt;&gt;""),IF(D16="",0,D16)+IF(E16="",0,E16),"")</f>
         <v/>
       </c>
+      <c r="G16" s="14" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
@@ -1698,6 +1717,7 @@
         <f>IF(OR(D17&lt;&gt;"",E17&lt;&gt;""),IF(D17="",0,D17)+IF(E17="",0,E17),"")</f>
         <v/>
       </c>
+      <c r="G17" s="14" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
@@ -1713,6 +1733,7 @@
         <f>IF(OR(D18&lt;&gt;"",E18&lt;&gt;""),IF(D18="",0,D18)+IF(E18="",0,E18),"")</f>
         <v/>
       </c>
+      <c r="G18" s="14" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -1738,7 +1759,9 @@
         <f>D19+E19</f>
         <v/>
       </c>
-    </row>
+      <c r="G19" s="14" t="n"/>
+    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
@@ -1753,6 +1776,7 @@
         <f>IF(OR(D21&lt;&gt;"",E21&lt;&gt;""),IF(D21="",0,D21)+IF(E21="",0,E21),"")</f>
         <v/>
       </c>
+      <c r="G21" s="14" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
@@ -1768,6 +1792,7 @@
         <f>IF(OR(D22&lt;&gt;"",E22&lt;&gt;""),IF(D22="",0,D22)+IF(E22="",0,E22),"")</f>
         <v/>
       </c>
+      <c r="G22" s="14" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
@@ -1783,6 +1808,7 @@
         <f>IF(OR(D23&lt;&gt;"",E23&lt;&gt;""),IF(D23="",0,D23)+IF(E23="",0,E23),"")</f>
         <v/>
       </c>
+      <c r="G23" s="14" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
@@ -1798,6 +1824,7 @@
         <f>IF(OR(D24&lt;&gt;"",E24&lt;&gt;""),IF(D24="",0,D24)+IF(E24="",0,E24),"")</f>
         <v/>
       </c>
+      <c r="G24" s="14" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
@@ -1813,6 +1840,7 @@
         <f>IF(OR(D25&lt;&gt;"",E25&lt;&gt;""),IF(D25="",0,D25)+IF(E25="",0,E25),"")</f>
         <v/>
       </c>
+      <c r="G25" s="14" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
@@ -1828,6 +1856,7 @@
         <f>IF(OR(D26&lt;&gt;"",E26&lt;&gt;""),IF(D26="",0,D26)+IF(E26="",0,E26),"")</f>
         <v/>
       </c>
+      <c r="G26" s="14" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
@@ -1843,6 +1872,7 @@
         <f>IF(OR(D27&lt;&gt;"",E27&lt;&gt;""),IF(D27="",0,D27)+IF(E27="",0,E27),"")</f>
         <v/>
       </c>
+      <c r="G27" s="14" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
@@ -1858,6 +1888,7 @@
         <f>IF(OR(D28&lt;&gt;"",E28&lt;&gt;""),IF(D28="",0,D28)+IF(E28="",0,E28),"")</f>
         <v/>
       </c>
+      <c r="G28" s="14" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
@@ -1873,6 +1904,7 @@
         <f>IF(OR(D29&lt;&gt;"",E29&lt;&gt;""),IF(D29="",0,D29)+IF(E29="",0,E29),"")</f>
         <v/>
       </c>
+      <c r="G29" s="14" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
@@ -1888,6 +1920,7 @@
         <f>IF(OR(D30&lt;&gt;"",E30&lt;&gt;""),IF(D30="",0,D30)+IF(E30="",0,E30),"")</f>
         <v/>
       </c>
+      <c r="G30" s="14" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
@@ -1903,6 +1936,7 @@
         <f>IF(OR(D31&lt;&gt;"",E31&lt;&gt;""),IF(D31="",0,D31)+IF(E31="",0,E31),"")</f>
         <v/>
       </c>
+      <c r="G31" s="14" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
@@ -1918,6 +1952,7 @@
         <f>IF(OR(D32&lt;&gt;"",E32&lt;&gt;""),IF(D32="",0,D32)+IF(E32="",0,E32),"")</f>
         <v/>
       </c>
+      <c r="G32" s="14" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
@@ -1933,6 +1968,7 @@
         <f>IF(OR(D33&lt;&gt;"",E33&lt;&gt;""),IF(D33="",0,D33)+IF(E33="",0,E33),"")</f>
         <v/>
       </c>
+      <c r="G33" s="14" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
@@ -1948,6 +1984,7 @@
         <f>IF(OR(D34&lt;&gt;"",E34&lt;&gt;""),IF(D34="",0,D34)+IF(E34="",0,E34),"")</f>
         <v/>
       </c>
+      <c r="G34" s="14" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
@@ -1963,6 +2000,7 @@
         <f>IF(OR(D35&lt;&gt;"",E35&lt;&gt;""),IF(D35="",0,D35)+IF(E35="",0,E35),"")</f>
         <v/>
       </c>
+      <c r="G35" s="14" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -1988,7 +2026,9 @@
         <f>D36+E36</f>
         <v/>
       </c>
-    </row>
+      <c r="G36" s="14" t="n"/>
+    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -2003,6 +2043,7 @@
         <f>IF(OR(D38&lt;&gt;"",E38&lt;&gt;""),IF(D38="",0,D38)+IF(E38="",0,E38),"")</f>
         <v/>
       </c>
+      <c r="G38" s="14" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
@@ -2018,6 +2059,7 @@
         <f>IF(OR(D39&lt;&gt;"",E39&lt;&gt;""),IF(D39="",0,D39)+IF(E39="",0,E39),"")</f>
         <v/>
       </c>
+      <c r="G39" s="14" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
@@ -2033,6 +2075,7 @@
         <f>IF(OR(D40&lt;&gt;"",E40&lt;&gt;""),IF(D40="",0,D40)+IF(E40="",0,E40),"")</f>
         <v/>
       </c>
+      <c r="G40" s="14" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
@@ -2048,6 +2091,7 @@
         <f>IF(OR(D41&lt;&gt;"",E41&lt;&gt;""),IF(D41="",0,D41)+IF(E41="",0,E41),"")</f>
         <v/>
       </c>
+      <c r="G41" s="14" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
@@ -2063,6 +2107,7 @@
         <f>IF(OR(D42&lt;&gt;"",E42&lt;&gt;""),IF(D42="",0,D42)+IF(E42="",0,E42),"")</f>
         <v/>
       </c>
+      <c r="G42" s="14" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
@@ -2078,6 +2123,7 @@
         <f>IF(OR(D43&lt;&gt;"",E43&lt;&gt;""),IF(D43="",0,D43)+IF(E43="",0,E43),"")</f>
         <v/>
       </c>
+      <c r="G43" s="14" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
@@ -2093,6 +2139,7 @@
         <f>IF(OR(D44&lt;&gt;"",E44&lt;&gt;""),IF(D44="",0,D44)+IF(E44="",0,E44),"")</f>
         <v/>
       </c>
+      <c r="G44" s="14" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
@@ -2108,6 +2155,7 @@
         <f>IF(OR(D45&lt;&gt;"",E45&lt;&gt;""),IF(D45="",0,D45)+IF(E45="",0,E45),"")</f>
         <v/>
       </c>
+      <c r="G45" s="14" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
@@ -2123,6 +2171,7 @@
         <f>IF(OR(D46&lt;&gt;"",E46&lt;&gt;""),IF(D46="",0,D46)+IF(E46="",0,E46),"")</f>
         <v/>
       </c>
+      <c r="G46" s="14" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
@@ -2138,6 +2187,7 @@
         <f>IF(OR(D47&lt;&gt;"",E47&lt;&gt;""),IF(D47="",0,D47)+IF(E47="",0,E47),"")</f>
         <v/>
       </c>
+      <c r="G47" s="14" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
@@ -2153,6 +2203,7 @@
         <f>IF(OR(D48&lt;&gt;"",E48&lt;&gt;""),IF(D48="",0,D48)+IF(E48="",0,E48),"")</f>
         <v/>
       </c>
+      <c r="G48" s="14" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
@@ -2168,6 +2219,7 @@
         <f>IF(OR(D49&lt;&gt;"",E49&lt;&gt;""),IF(D49="",0,D49)+IF(E49="",0,E49),"")</f>
         <v/>
       </c>
+      <c r="G49" s="14" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
@@ -2183,6 +2235,7 @@
         <f>IF(OR(D50&lt;&gt;"",E50&lt;&gt;""),IF(D50="",0,D50)+IF(E50="",0,E50),"")</f>
         <v/>
       </c>
+      <c r="G50" s="14" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
@@ -2198,6 +2251,7 @@
         <f>IF(OR(D51&lt;&gt;"",E51&lt;&gt;""),IF(D51="",0,D51)+IF(E51="",0,E51),"")</f>
         <v/>
       </c>
+      <c r="G51" s="14" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
@@ -2213,6 +2267,7 @@
         <f>IF(OR(D52&lt;&gt;"",E52&lt;&gt;""),IF(D52="",0,D52)+IF(E52="",0,E52),"")</f>
         <v/>
       </c>
+      <c r="G52" s="14" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -2238,7 +2293,9 @@
         <f>D53+E53</f>
         <v/>
       </c>
-    </row>
+      <c r="G53" s="14" t="n"/>
+    </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -2253,6 +2310,7 @@
         <f>IF(OR(D55&lt;&gt;"",E55&lt;&gt;""),IF(D55="",0,D55)+IF(E55="",0,E55),"")</f>
         <v/>
       </c>
+      <c r="G55" s="14" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
@@ -2268,6 +2326,7 @@
         <f>IF(OR(D56&lt;&gt;"",E56&lt;&gt;""),IF(D56="",0,D56)+IF(E56="",0,E56),"")</f>
         <v/>
       </c>
+      <c r="G56" s="14" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
@@ -2283,6 +2342,7 @@
         <f>IF(OR(D57&lt;&gt;"",E57&lt;&gt;""),IF(D57="",0,D57)+IF(E57="",0,E57),"")</f>
         <v/>
       </c>
+      <c r="G57" s="14" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
@@ -2298,6 +2358,7 @@
         <f>IF(OR(D58&lt;&gt;"",E58&lt;&gt;""),IF(D58="",0,D58)+IF(E58="",0,E58),"")</f>
         <v/>
       </c>
+      <c r="G58" s="14" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
@@ -2313,6 +2374,7 @@
         <f>IF(OR(D59&lt;&gt;"",E59&lt;&gt;""),IF(D59="",0,D59)+IF(E59="",0,E59),"")</f>
         <v/>
       </c>
+      <c r="G59" s="14" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
@@ -2328,6 +2390,7 @@
         <f>IF(OR(D60&lt;&gt;"",E60&lt;&gt;""),IF(D60="",0,D60)+IF(E60="",0,E60),"")</f>
         <v/>
       </c>
+      <c r="G60" s="14" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
@@ -2343,6 +2406,7 @@
         <f>IF(OR(D61&lt;&gt;"",E61&lt;&gt;""),IF(D61="",0,D61)+IF(E61="",0,E61),"")</f>
         <v/>
       </c>
+      <c r="G61" s="14" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
@@ -2358,6 +2422,7 @@
         <f>IF(OR(D62&lt;&gt;"",E62&lt;&gt;""),IF(D62="",0,D62)+IF(E62="",0,E62),"")</f>
         <v/>
       </c>
+      <c r="G62" s="14" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
@@ -2373,6 +2438,7 @@
         <f>IF(OR(D63&lt;&gt;"",E63&lt;&gt;""),IF(D63="",0,D63)+IF(E63="",0,E63),"")</f>
         <v/>
       </c>
+      <c r="G63" s="14" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
@@ -2388,6 +2454,7 @@
         <f>IF(OR(D64&lt;&gt;"",E64&lt;&gt;""),IF(D64="",0,D64)+IF(E64="",0,E64),"")</f>
         <v/>
       </c>
+      <c r="G64" s="14" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
@@ -2403,6 +2470,7 @@
         <f>IF(OR(D65&lt;&gt;"",E65&lt;&gt;""),IF(D65="",0,D65)+IF(E65="",0,E65),"")</f>
         <v/>
       </c>
+      <c r="G65" s="14" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
@@ -2418,6 +2486,7 @@
         <f>IF(OR(D66&lt;&gt;"",E66&lt;&gt;""),IF(D66="",0,D66)+IF(E66="",0,E66),"")</f>
         <v/>
       </c>
+      <c r="G66" s="14" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
@@ -2433,6 +2502,7 @@
         <f>IF(OR(D67&lt;&gt;"",E67&lt;&gt;""),IF(D67="",0,D67)+IF(E67="",0,E67),"")</f>
         <v/>
       </c>
+      <c r="G67" s="14" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
@@ -2448,6 +2518,7 @@
         <f>IF(OR(D68&lt;&gt;"",E68&lt;&gt;""),IF(D68="",0,D68)+IF(E68="",0,E68),"")</f>
         <v/>
       </c>
+      <c r="G68" s="14" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="14" t="inlineStr">
@@ -2463,6 +2534,7 @@
         <f>IF(OR(D69&lt;&gt;"",E69&lt;&gt;""),IF(D69="",0,D69)+IF(E69="",0,E69),"")</f>
         <v/>
       </c>
+      <c r="G69" s="14" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -2488,7 +2560,9 @@
         <f>D70+E70</f>
         <v/>
       </c>
-    </row>
+      <c r="G70" s="14" t="n"/>
+    </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
@@ -2503,6 +2577,7 @@
         <f>IF(OR(D72&lt;&gt;"",E72&lt;&gt;""),IF(D72="",0,D72)+IF(E72="",0,E72),"")</f>
         <v/>
       </c>
+      <c r="G72" s="14" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
@@ -2518,6 +2593,7 @@
         <f>IF(OR(D73&lt;&gt;"",E73&lt;&gt;""),IF(D73="",0,D73)+IF(E73="",0,E73),"")</f>
         <v/>
       </c>
+      <c r="G73" s="14" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="14" t="inlineStr">
@@ -2533,6 +2609,7 @@
         <f>IF(OR(D74&lt;&gt;"",E74&lt;&gt;""),IF(D74="",0,D74)+IF(E74="",0,E74),"")</f>
         <v/>
       </c>
+      <c r="G74" s="14" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="14" t="inlineStr">
@@ -2548,6 +2625,7 @@
         <f>IF(OR(D75&lt;&gt;"",E75&lt;&gt;""),IF(D75="",0,D75)+IF(E75="",0,E75),"")</f>
         <v/>
       </c>
+      <c r="G75" s="14" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="14" t="inlineStr">
@@ -2563,6 +2641,7 @@
         <f>IF(OR(D76&lt;&gt;"",E76&lt;&gt;""),IF(D76="",0,D76)+IF(E76="",0,E76),"")</f>
         <v/>
       </c>
+      <c r="G76" s="14" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="14" t="inlineStr">
@@ -2578,6 +2657,7 @@
         <f>IF(OR(D77&lt;&gt;"",E77&lt;&gt;""),IF(D77="",0,D77)+IF(E77="",0,E77),"")</f>
         <v/>
       </c>
+      <c r="G77" s="14" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
@@ -2593,6 +2673,7 @@
         <f>IF(OR(D78&lt;&gt;"",E78&lt;&gt;""),IF(D78="",0,D78)+IF(E78="",0,E78),"")</f>
         <v/>
       </c>
+      <c r="G78" s="14" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="14" t="inlineStr">
@@ -2608,6 +2689,7 @@
         <f>IF(OR(D79&lt;&gt;"",E79&lt;&gt;""),IF(D79="",0,D79)+IF(E79="",0,E79),"")</f>
         <v/>
       </c>
+      <c r="G79" s="14" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="14" t="inlineStr">
@@ -2623,6 +2705,7 @@
         <f>IF(OR(D80&lt;&gt;"",E80&lt;&gt;""),IF(D80="",0,D80)+IF(E80="",0,E80),"")</f>
         <v/>
       </c>
+      <c r="G80" s="14" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="14" t="inlineStr">
@@ -2638,6 +2721,7 @@
         <f>IF(OR(D81&lt;&gt;"",E81&lt;&gt;""),IF(D81="",0,D81)+IF(E81="",0,E81),"")</f>
         <v/>
       </c>
+      <c r="G81" s="14" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
@@ -2653,6 +2737,7 @@
         <f>IF(OR(D82&lt;&gt;"",E82&lt;&gt;""),IF(D82="",0,D82)+IF(E82="",0,E82),"")</f>
         <v/>
       </c>
+      <c r="G82" s="14" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="14" t="inlineStr">
@@ -2668,6 +2753,7 @@
         <f>IF(OR(D83&lt;&gt;"",E83&lt;&gt;""),IF(D83="",0,D83)+IF(E83="",0,E83),"")</f>
         <v/>
       </c>
+      <c r="G83" s="14" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
@@ -2683,6 +2769,7 @@
         <f>IF(OR(D84&lt;&gt;"",E84&lt;&gt;""),IF(D84="",0,D84)+IF(E84="",0,E84),"")</f>
         <v/>
       </c>
+      <c r="G84" s="14" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="14" t="inlineStr">
@@ -2698,6 +2785,7 @@
         <f>IF(OR(D85&lt;&gt;"",E85&lt;&gt;""),IF(D85="",0,D85)+IF(E85="",0,E85),"")</f>
         <v/>
       </c>
+      <c r="G85" s="14" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
@@ -2713,6 +2801,7 @@
         <f>IF(OR(D86&lt;&gt;"",E86&lt;&gt;""),IF(D86="",0,D86)+IF(E86="",0,E86),"")</f>
         <v/>
       </c>
+      <c r="G86" s="14" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -2738,7 +2827,9 @@
         <f>D87+E87</f>
         <v/>
       </c>
-    </row>
+      <c r="G87" s="14" t="n"/>
+    </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="14" t="inlineStr">
         <is>
@@ -2753,6 +2844,7 @@
         <f>IF(OR(D89&lt;&gt;"",E89&lt;&gt;""),IF(D89="",0,D89)+IF(E89="",0,E89),"")</f>
         <v/>
       </c>
+      <c r="G89" s="14" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
@@ -2768,6 +2860,7 @@
         <f>IF(OR(D90&lt;&gt;"",E90&lt;&gt;""),IF(D90="",0,D90)+IF(E90="",0,E90),"")</f>
         <v/>
       </c>
+      <c r="G90" s="14" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="14" t="inlineStr">
@@ -2783,6 +2876,7 @@
         <f>IF(OR(D91&lt;&gt;"",E91&lt;&gt;""),IF(D91="",0,D91)+IF(E91="",0,E91),"")</f>
         <v/>
       </c>
+      <c r="G91" s="14" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
@@ -2798,6 +2892,7 @@
         <f>IF(OR(D92&lt;&gt;"",E92&lt;&gt;""),IF(D92="",0,D92)+IF(E92="",0,E92),"")</f>
         <v/>
       </c>
+      <c r="G92" s="14" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
@@ -2813,6 +2908,7 @@
         <f>IF(OR(D93&lt;&gt;"",E93&lt;&gt;""),IF(D93="",0,D93)+IF(E93="",0,E93),"")</f>
         <v/>
       </c>
+      <c r="G93" s="14" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
@@ -2828,6 +2924,7 @@
         <f>IF(OR(D94&lt;&gt;"",E94&lt;&gt;""),IF(D94="",0,D94)+IF(E94="",0,E94),"")</f>
         <v/>
       </c>
+      <c r="G94" s="14" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="14" t="inlineStr">
@@ -2843,6 +2940,7 @@
         <f>IF(OR(D95&lt;&gt;"",E95&lt;&gt;""),IF(D95="",0,D95)+IF(E95="",0,E95),"")</f>
         <v/>
       </c>
+      <c r="G95" s="14" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
@@ -2858,6 +2956,7 @@
         <f>IF(OR(D96&lt;&gt;"",E96&lt;&gt;""),IF(D96="",0,D96)+IF(E96="",0,E96),"")</f>
         <v/>
       </c>
+      <c r="G96" s="14" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="14" t="inlineStr">
@@ -2873,6 +2972,7 @@
         <f>IF(OR(D97&lt;&gt;"",E97&lt;&gt;""),IF(D97="",0,D97)+IF(E97="",0,E97),"")</f>
         <v/>
       </c>
+      <c r="G97" s="14" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
@@ -2888,6 +2988,7 @@
         <f>IF(OR(D98&lt;&gt;"",E98&lt;&gt;""),IF(D98="",0,D98)+IF(E98="",0,E98),"")</f>
         <v/>
       </c>
+      <c r="G98" s="14" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="14" t="inlineStr">
@@ -2903,6 +3004,7 @@
         <f>IF(OR(D99&lt;&gt;"",E99&lt;&gt;""),IF(D99="",0,D99)+IF(E99="",0,E99),"")</f>
         <v/>
       </c>
+      <c r="G99" s="14" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
@@ -2918,6 +3020,7 @@
         <f>IF(OR(D100&lt;&gt;"",E100&lt;&gt;""),IF(D100="",0,D100)+IF(E100="",0,E100),"")</f>
         <v/>
       </c>
+      <c r="G100" s="14" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="14" t="inlineStr">
@@ -2933,6 +3036,7 @@
         <f>IF(OR(D101&lt;&gt;"",E101&lt;&gt;""),IF(D101="",0,D101)+IF(E101="",0,E101),"")</f>
         <v/>
       </c>
+      <c r="G101" s="14" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
@@ -2948,6 +3052,7 @@
         <f>IF(OR(D102&lt;&gt;"",E102&lt;&gt;""),IF(D102="",0,D102)+IF(E102="",0,E102),"")</f>
         <v/>
       </c>
+      <c r="G102" s="14" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="14" t="inlineStr">
@@ -2963,6 +3068,7 @@
         <f>IF(OR(D103&lt;&gt;"",E103&lt;&gt;""),IF(D103="",0,D103)+IF(E103="",0,E103),"")</f>
         <v/>
       </c>
+      <c r="G103" s="14" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
@@ -2988,7 +3094,9 @@
         <f>D104+E104</f>
         <v/>
       </c>
-    </row>
+      <c r="G104" s="14" t="n"/>
+    </row>
+    <row r="105"/>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
@@ -3009,6 +3117,7 @@
         <f>IF(OR(D106&lt;&gt;"",E106&lt;&gt;""),IF(D106="",0,D106)+IF(E106="",0,E106),"")</f>
         <v/>
       </c>
+      <c r="G106" s="14" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="14" t="inlineStr">
@@ -3030,6 +3139,7 @@
         <f>IF(OR(D107&lt;&gt;"",E107&lt;&gt;""),IF(D107="",0,D107)+IF(E107="",0,E107),"")</f>
         <v/>
       </c>
+      <c r="G107" s="14" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="14" t="inlineStr">
@@ -3051,6 +3161,7 @@
         <f>IF(OR(D108&lt;&gt;"",E108&lt;&gt;""),IF(D108="",0,D108)+IF(E108="",0,E108),"")</f>
         <v/>
       </c>
+      <c r="G108" s="14" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="14" t="inlineStr">
@@ -3072,6 +3183,7 @@
         <f>IF(OR(D109&lt;&gt;"",E109&lt;&gt;""),IF(D109="",0,D109)+IF(E109="",0,E109),"")</f>
         <v/>
       </c>
+      <c r="G109" s="14" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
@@ -3093,6 +3205,7 @@
         <f>IF(OR(D110&lt;&gt;"",E110&lt;&gt;""),IF(D110="",0,D110)+IF(E110="",0,E110),"")</f>
         <v/>
       </c>
+      <c r="G110" s="14" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="14" t="inlineStr">
@@ -3108,6 +3221,7 @@
         <f>IF(OR(D111&lt;&gt;"",E111&lt;&gt;""),IF(D111="",0,D111)+IF(E111="",0,E111),"")</f>
         <v/>
       </c>
+      <c r="G111" s="14" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
@@ -3123,6 +3237,7 @@
         <f>IF(OR(D112&lt;&gt;"",E112&lt;&gt;""),IF(D112="",0,D112)+IF(E112="",0,E112),"")</f>
         <v/>
       </c>
+      <c r="G112" s="14" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="14" t="inlineStr">
@@ -3138,6 +3253,7 @@
         <f>IF(OR(D113&lt;&gt;"",E113&lt;&gt;""),IF(D113="",0,D113)+IF(E113="",0,E113),"")</f>
         <v/>
       </c>
+      <c r="G113" s="14" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
@@ -3153,6 +3269,7 @@
         <f>IF(OR(D114&lt;&gt;"",E114&lt;&gt;""),IF(D114="",0,D114)+IF(E114="",0,E114),"")</f>
         <v/>
       </c>
+      <c r="G114" s="14" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="14" t="inlineStr">
@@ -3168,6 +3285,7 @@
         <f>IF(OR(D115&lt;&gt;"",E115&lt;&gt;""),IF(D115="",0,D115)+IF(E115="",0,E115),"")</f>
         <v/>
       </c>
+      <c r="G115" s="14" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
@@ -3183,6 +3301,7 @@
         <f>IF(OR(D116&lt;&gt;"",E116&lt;&gt;""),IF(D116="",0,D116)+IF(E116="",0,E116),"")</f>
         <v/>
       </c>
+      <c r="G116" s="14" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="14" t="inlineStr">
@@ -3198,6 +3317,7 @@
         <f>IF(OR(D117&lt;&gt;"",E117&lt;&gt;""),IF(D117="",0,D117)+IF(E117="",0,E117),"")</f>
         <v/>
       </c>
+      <c r="G117" s="14" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
@@ -3213,6 +3333,7 @@
         <f>IF(OR(D118&lt;&gt;"",E118&lt;&gt;""),IF(D118="",0,D118)+IF(E118="",0,E118),"")</f>
         <v/>
       </c>
+      <c r="G118" s="14" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="14" t="inlineStr">
@@ -3228,6 +3349,7 @@
         <f>IF(OR(D119&lt;&gt;"",E119&lt;&gt;""),IF(D119="",0,D119)+IF(E119="",0,E119),"")</f>
         <v/>
       </c>
+      <c r="G119" s="14" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
@@ -3243,6 +3365,7 @@
         <f>IF(OR(D120&lt;&gt;"",E120&lt;&gt;""),IF(D120="",0,D120)+IF(E120="",0,E120),"")</f>
         <v/>
       </c>
+      <c r="G120" s="14" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
@@ -3268,7 +3391,9 @@
         <f>D121+E121</f>
         <v/>
       </c>
-    </row>
+      <c r="G121" s="14" t="n"/>
+    </row>
+    <row r="122"/>
     <row r="123">
       <c r="A123" s="14" t="inlineStr">
         <is>
@@ -3283,6 +3408,7 @@
         <f>IF(OR(D123&lt;&gt;"",E123&lt;&gt;""),IF(D123="",0,D123)+IF(E123="",0,E123),"")</f>
         <v/>
       </c>
+      <c r="G123" s="14" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
@@ -3298,6 +3424,7 @@
         <f>IF(OR(D124&lt;&gt;"",E124&lt;&gt;""),IF(D124="",0,D124)+IF(E124="",0,E124),"")</f>
         <v/>
       </c>
+      <c r="G124" s="14" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="14" t="inlineStr">
@@ -3313,6 +3440,7 @@
         <f>IF(OR(D125&lt;&gt;"",E125&lt;&gt;""),IF(D125="",0,D125)+IF(E125="",0,E125),"")</f>
         <v/>
       </c>
+      <c r="G125" s="14" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="14" t="inlineStr">
@@ -3328,6 +3456,7 @@
         <f>IF(OR(D126&lt;&gt;"",E126&lt;&gt;""),IF(D126="",0,D126)+IF(E126="",0,E126),"")</f>
         <v/>
       </c>
+      <c r="G126" s="14" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="14" t="inlineStr">
@@ -3343,6 +3472,7 @@
         <f>IF(OR(D127&lt;&gt;"",E127&lt;&gt;""),IF(D127="",0,D127)+IF(E127="",0,E127),"")</f>
         <v/>
       </c>
+      <c r="G127" s="14" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="14" t="inlineStr">
@@ -3358,6 +3488,7 @@
         <f>IF(OR(D128&lt;&gt;"",E128&lt;&gt;""),IF(D128="",0,D128)+IF(E128="",0,E128),"")</f>
         <v/>
       </c>
+      <c r="G128" s="14" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="14" t="inlineStr">
@@ -3373,6 +3504,7 @@
         <f>IF(OR(D129&lt;&gt;"",E129&lt;&gt;""),IF(D129="",0,D129)+IF(E129="",0,E129),"")</f>
         <v/>
       </c>
+      <c r="G129" s="14" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
@@ -3388,6 +3520,7 @@
         <f>IF(OR(D130&lt;&gt;"",E130&lt;&gt;""),IF(D130="",0,D130)+IF(E130="",0,E130),"")</f>
         <v/>
       </c>
+      <c r="G130" s="14" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="14" t="inlineStr">
@@ -3403,6 +3536,7 @@
         <f>IF(OR(D131&lt;&gt;"",E131&lt;&gt;""),IF(D131="",0,D131)+IF(E131="",0,E131),"")</f>
         <v/>
       </c>
+      <c r="G131" s="14" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="14" t="inlineStr">
@@ -3418,6 +3552,7 @@
         <f>IF(OR(D132&lt;&gt;"",E132&lt;&gt;""),IF(D132="",0,D132)+IF(E132="",0,E132),"")</f>
         <v/>
       </c>
+      <c r="G132" s="14" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="14" t="inlineStr">
@@ -3433,6 +3568,7 @@
         <f>IF(OR(D133&lt;&gt;"",E133&lt;&gt;""),IF(D133="",0,D133)+IF(E133="",0,E133),"")</f>
         <v/>
       </c>
+      <c r="G133" s="14" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="14" t="inlineStr">
@@ -3448,6 +3584,7 @@
         <f>IF(OR(D134&lt;&gt;"",E134&lt;&gt;""),IF(D134="",0,D134)+IF(E134="",0,E134),"")</f>
         <v/>
       </c>
+      <c r="G134" s="14" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="14" t="inlineStr">
@@ -3463,6 +3600,7 @@
         <f>IF(OR(D135&lt;&gt;"",E135&lt;&gt;""),IF(D135="",0,D135)+IF(E135="",0,E135),"")</f>
         <v/>
       </c>
+      <c r="G135" s="14" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="14" t="inlineStr">
@@ -3478,6 +3616,7 @@
         <f>IF(OR(D136&lt;&gt;"",E136&lt;&gt;""),IF(D136="",0,D136)+IF(E136="",0,E136),"")</f>
         <v/>
       </c>
+      <c r="G136" s="14" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
@@ -3493,6 +3632,7 @@
         <f>IF(OR(D137&lt;&gt;"",E137&lt;&gt;""),IF(D137="",0,D137)+IF(E137="",0,E137),"")</f>
         <v/>
       </c>
+      <c r="G137" s="14" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
@@ -3518,7 +3658,9 @@
         <f>D138+E138</f>
         <v/>
       </c>
-    </row>
+      <c r="G138" s="14" t="n"/>
+    </row>
+    <row r="139"/>
     <row r="140">
       <c r="A140" s="14" t="inlineStr">
         <is>
@@ -3533,6 +3675,7 @@
         <f>IF(OR(D140&lt;&gt;"",E140&lt;&gt;""),IF(D140="",0,D140)+IF(E140="",0,E140),"")</f>
         <v/>
       </c>
+      <c r="G140" s="14" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="14" t="inlineStr">
@@ -3548,6 +3691,7 @@
         <f>IF(OR(D141&lt;&gt;"",E141&lt;&gt;""),IF(D141="",0,D141)+IF(E141="",0,E141),"")</f>
         <v/>
       </c>
+      <c r="G141" s="14" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="14" t="inlineStr">
@@ -3563,6 +3707,7 @@
         <f>IF(OR(D142&lt;&gt;"",E142&lt;&gt;""),IF(D142="",0,D142)+IF(E142="",0,E142),"")</f>
         <v/>
       </c>
+      <c r="G142" s="14" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="14" t="inlineStr">
@@ -3578,6 +3723,7 @@
         <f>IF(OR(D143&lt;&gt;"",E143&lt;&gt;""),IF(D143="",0,D143)+IF(E143="",0,E143),"")</f>
         <v/>
       </c>
+      <c r="G143" s="14" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="14" t="inlineStr">
@@ -3593,6 +3739,7 @@
         <f>IF(OR(D144&lt;&gt;"",E144&lt;&gt;""),IF(D144="",0,D144)+IF(E144="",0,E144),"")</f>
         <v/>
       </c>
+      <c r="G144" s="14" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="14" t="inlineStr">
@@ -3608,6 +3755,7 @@
         <f>IF(OR(D145&lt;&gt;"",E145&lt;&gt;""),IF(D145="",0,D145)+IF(E145="",0,E145),"")</f>
         <v/>
       </c>
+      <c r="G145" s="14" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="14" t="inlineStr">
@@ -3623,6 +3771,7 @@
         <f>IF(OR(D146&lt;&gt;"",E146&lt;&gt;""),IF(D146="",0,D146)+IF(E146="",0,E146),"")</f>
         <v/>
       </c>
+      <c r="G146" s="14" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="14" t="inlineStr">
@@ -3638,6 +3787,7 @@
         <f>IF(OR(D147&lt;&gt;"",E147&lt;&gt;""),IF(D147="",0,D147)+IF(E147="",0,E147),"")</f>
         <v/>
       </c>
+      <c r="G147" s="14" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="14" t="inlineStr">
@@ -3653,6 +3803,7 @@
         <f>IF(OR(D148&lt;&gt;"",E148&lt;&gt;""),IF(D148="",0,D148)+IF(E148="",0,E148),"")</f>
         <v/>
       </c>
+      <c r="G148" s="14" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="14" t="inlineStr">
@@ -3668,6 +3819,7 @@
         <f>IF(OR(D149&lt;&gt;"",E149&lt;&gt;""),IF(D149="",0,D149)+IF(E149="",0,E149),"")</f>
         <v/>
       </c>
+      <c r="G149" s="14" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="14" t="inlineStr">
@@ -3683,6 +3835,7 @@
         <f>IF(OR(D150&lt;&gt;"",E150&lt;&gt;""),IF(D150="",0,D150)+IF(E150="",0,E150),"")</f>
         <v/>
       </c>
+      <c r="G150" s="14" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="14" t="inlineStr">
@@ -3698,6 +3851,7 @@
         <f>IF(OR(D151&lt;&gt;"",E151&lt;&gt;""),IF(D151="",0,D151)+IF(E151="",0,E151),"")</f>
         <v/>
       </c>
+      <c r="G151" s="14" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="14" t="inlineStr">
@@ -3713,6 +3867,7 @@
         <f>IF(OR(D152&lt;&gt;"",E152&lt;&gt;""),IF(D152="",0,D152)+IF(E152="",0,E152),"")</f>
         <v/>
       </c>
+      <c r="G152" s="14" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="14" t="inlineStr">
@@ -3728,6 +3883,7 @@
         <f>IF(OR(D153&lt;&gt;"",E153&lt;&gt;""),IF(D153="",0,D153)+IF(E153="",0,E153),"")</f>
         <v/>
       </c>
+      <c r="G153" s="14" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="14" t="inlineStr">
@@ -3743,6 +3899,7 @@
         <f>IF(OR(D154&lt;&gt;"",E154&lt;&gt;""),IF(D154="",0,D154)+IF(E154="",0,E154),"")</f>
         <v/>
       </c>
+      <c r="G154" s="14" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="10" t="inlineStr">
@@ -3768,7 +3925,9 @@
         <f>D155+E155</f>
         <v/>
       </c>
-    </row>
+      <c r="G155" s="14" t="n"/>
+    </row>
+    <row r="156"/>
     <row r="157">
       <c r="A157" s="14" t="inlineStr">
         <is>
@@ -3783,6 +3942,7 @@
         <f>IF(OR(D157&lt;&gt;"",E157&lt;&gt;""),IF(D157="",0,D157)+IF(E157="",0,E157),"")</f>
         <v/>
       </c>
+      <c r="G157" s="14" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="14" t="inlineStr">
@@ -3798,6 +3958,7 @@
         <f>IF(OR(D158&lt;&gt;"",E158&lt;&gt;""),IF(D158="",0,D158)+IF(E158="",0,E158),"")</f>
         <v/>
       </c>
+      <c r="G158" s="14" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="14" t="inlineStr">
@@ -3813,6 +3974,7 @@
         <f>IF(OR(D159&lt;&gt;"",E159&lt;&gt;""),IF(D159="",0,D159)+IF(E159="",0,E159),"")</f>
         <v/>
       </c>
+      <c r="G159" s="14" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="14" t="inlineStr">
@@ -3828,6 +3990,7 @@
         <f>IF(OR(D160&lt;&gt;"",E160&lt;&gt;""),IF(D160="",0,D160)+IF(E160="",0,E160),"")</f>
         <v/>
       </c>
+      <c r="G160" s="14" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="14" t="inlineStr">
@@ -3843,6 +4006,7 @@
         <f>IF(OR(D161&lt;&gt;"",E161&lt;&gt;""),IF(D161="",0,D161)+IF(E161="",0,E161),"")</f>
         <v/>
       </c>
+      <c r="G161" s="14" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="14" t="inlineStr">
@@ -3858,6 +4022,7 @@
         <f>IF(OR(D162&lt;&gt;"",E162&lt;&gt;""),IF(D162="",0,D162)+IF(E162="",0,E162),"")</f>
         <v/>
       </c>
+      <c r="G162" s="14" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="14" t="inlineStr">
@@ -3873,6 +4038,7 @@
         <f>IF(OR(D163&lt;&gt;"",E163&lt;&gt;""),IF(D163="",0,D163)+IF(E163="",0,E163),"")</f>
         <v/>
       </c>
+      <c r="G163" s="14" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="14" t="inlineStr">
@@ -3888,6 +4054,7 @@
         <f>IF(OR(D164&lt;&gt;"",E164&lt;&gt;""),IF(D164="",0,D164)+IF(E164="",0,E164),"")</f>
         <v/>
       </c>
+      <c r="G164" s="14" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="14" t="inlineStr">
@@ -3903,6 +4070,7 @@
         <f>IF(OR(D165&lt;&gt;"",E165&lt;&gt;""),IF(D165="",0,D165)+IF(E165="",0,E165),"")</f>
         <v/>
       </c>
+      <c r="G165" s="14" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="14" t="inlineStr">
@@ -3918,6 +4086,7 @@
         <f>IF(OR(D166&lt;&gt;"",E166&lt;&gt;""),IF(D166="",0,D166)+IF(E166="",0,E166),"")</f>
         <v/>
       </c>
+      <c r="G166" s="14" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="14" t="inlineStr">
@@ -3933,6 +4102,7 @@
         <f>IF(OR(D167&lt;&gt;"",E167&lt;&gt;""),IF(D167="",0,D167)+IF(E167="",0,E167),"")</f>
         <v/>
       </c>
+      <c r="G167" s="14" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="14" t="inlineStr">
@@ -3948,6 +4118,7 @@
         <f>IF(OR(D168&lt;&gt;"",E168&lt;&gt;""),IF(D168="",0,D168)+IF(E168="",0,E168),"")</f>
         <v/>
       </c>
+      <c r="G168" s="14" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="14" t="inlineStr">
@@ -3963,6 +4134,7 @@
         <f>IF(OR(D169&lt;&gt;"",E169&lt;&gt;""),IF(D169="",0,D169)+IF(E169="",0,E169),"")</f>
         <v/>
       </c>
+      <c r="G169" s="14" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="14" t="inlineStr">
@@ -3978,6 +4150,7 @@
         <f>IF(OR(D170&lt;&gt;"",E170&lt;&gt;""),IF(D170="",0,D170)+IF(E170="",0,E170),"")</f>
         <v/>
       </c>
+      <c r="G170" s="14" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="14" t="inlineStr">
@@ -3993,6 +4166,7 @@
         <f>IF(OR(D171&lt;&gt;"",E171&lt;&gt;""),IF(D171="",0,D171)+IF(E171="",0,E171),"")</f>
         <v/>
       </c>
+      <c r="G171" s="14" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="10" t="inlineStr">
@@ -4018,7 +4192,9 @@
         <f>D172+E172</f>
         <v/>
       </c>
-    </row>
+      <c r="G172" s="14" t="n"/>
+    </row>
+    <row r="173"/>
     <row r="174">
       <c r="A174" s="14" t="inlineStr">
         <is>
@@ -4033,6 +4209,7 @@
         <f>IF(OR(D174&lt;&gt;"",E174&lt;&gt;""),IF(D174="",0,D174)+IF(E174="",0,E174),"")</f>
         <v/>
       </c>
+      <c r="G174" s="14" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="14" t="inlineStr">
@@ -4048,6 +4225,7 @@
         <f>IF(OR(D175&lt;&gt;"",E175&lt;&gt;""),IF(D175="",0,D175)+IF(E175="",0,E175),"")</f>
         <v/>
       </c>
+      <c r="G175" s="14" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="14" t="inlineStr">
@@ -4063,6 +4241,7 @@
         <f>IF(OR(D176&lt;&gt;"",E176&lt;&gt;""),IF(D176="",0,D176)+IF(E176="",0,E176),"")</f>
         <v/>
       </c>
+      <c r="G176" s="14" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="14" t="inlineStr">
@@ -4078,6 +4257,7 @@
         <f>IF(OR(D177&lt;&gt;"",E177&lt;&gt;""),IF(D177="",0,D177)+IF(E177="",0,E177),"")</f>
         <v/>
       </c>
+      <c r="G177" s="14" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
@@ -4093,6 +4273,7 @@
         <f>IF(OR(D178&lt;&gt;"",E178&lt;&gt;""),IF(D178="",0,D178)+IF(E178="",0,E178),"")</f>
         <v/>
       </c>
+      <c r="G178" s="14" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="14" t="inlineStr">
@@ -4108,6 +4289,7 @@
         <f>IF(OR(D179&lt;&gt;"",E179&lt;&gt;""),IF(D179="",0,D179)+IF(E179="",0,E179),"")</f>
         <v/>
       </c>
+      <c r="G179" s="14" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="14" t="inlineStr">
@@ -4123,6 +4305,7 @@
         <f>IF(OR(D180&lt;&gt;"",E180&lt;&gt;""),IF(D180="",0,D180)+IF(E180="",0,E180),"")</f>
         <v/>
       </c>
+      <c r="G180" s="14" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="14" t="inlineStr">
@@ -4138,6 +4321,7 @@
         <f>IF(OR(D181&lt;&gt;"",E181&lt;&gt;""),IF(D181="",0,D181)+IF(E181="",0,E181),"")</f>
         <v/>
       </c>
+      <c r="G181" s="14" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="14" t="inlineStr">
@@ -4153,6 +4337,7 @@
         <f>IF(OR(D182&lt;&gt;"",E182&lt;&gt;""),IF(D182="",0,D182)+IF(E182="",0,E182),"")</f>
         <v/>
       </c>
+      <c r="G182" s="14" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="14" t="inlineStr">
@@ -4168,6 +4353,7 @@
         <f>IF(OR(D183&lt;&gt;"",E183&lt;&gt;""),IF(D183="",0,D183)+IF(E183="",0,E183),"")</f>
         <v/>
       </c>
+      <c r="G183" s="14" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="14" t="inlineStr">
@@ -4183,6 +4369,7 @@
         <f>IF(OR(D184&lt;&gt;"",E184&lt;&gt;""),IF(D184="",0,D184)+IF(E184="",0,E184),"")</f>
         <v/>
       </c>
+      <c r="G184" s="14" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="14" t="inlineStr">
@@ -4198,6 +4385,7 @@
         <f>IF(OR(D185&lt;&gt;"",E185&lt;&gt;""),IF(D185="",0,D185)+IF(E185="",0,E185),"")</f>
         <v/>
       </c>
+      <c r="G185" s="14" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="14" t="inlineStr">
@@ -4213,6 +4401,7 @@
         <f>IF(OR(D186&lt;&gt;"",E186&lt;&gt;""),IF(D186="",0,D186)+IF(E186="",0,E186),"")</f>
         <v/>
       </c>
+      <c r="G186" s="14" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="14" t="inlineStr">
@@ -4228,6 +4417,7 @@
         <f>IF(OR(D187&lt;&gt;"",E187&lt;&gt;""),IF(D187="",0,D187)+IF(E187="",0,E187),"")</f>
         <v/>
       </c>
+      <c r="G187" s="14" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="14" t="inlineStr">
@@ -4243,6 +4433,7 @@
         <f>IF(OR(D188&lt;&gt;"",E188&lt;&gt;""),IF(D188="",0,D188)+IF(E188="",0,E188),"")</f>
         <v/>
       </c>
+      <c r="G188" s="14" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="10" t="inlineStr">
@@ -4268,7 +4459,9 @@
         <f>D189+E189</f>
         <v/>
       </c>
-    </row>
+      <c r="G189" s="14" t="n"/>
+    </row>
+    <row r="190"/>
     <row r="191">
       <c r="A191" s="14" t="inlineStr">
         <is>
@@ -4283,6 +4476,7 @@
         <f>IF(OR(D191&lt;&gt;"",E191&lt;&gt;""),IF(D191="",0,D191)+IF(E191="",0,E191),"")</f>
         <v/>
       </c>
+      <c r="G191" s="14" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="14" t="inlineStr">
@@ -4298,6 +4492,7 @@
         <f>IF(OR(D192&lt;&gt;"",E192&lt;&gt;""),IF(D192="",0,D192)+IF(E192="",0,E192),"")</f>
         <v/>
       </c>
+      <c r="G192" s="14" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="14" t="inlineStr">
@@ -4313,6 +4508,7 @@
         <f>IF(OR(D193&lt;&gt;"",E193&lt;&gt;""),IF(D193="",0,D193)+IF(E193="",0,E193),"")</f>
         <v/>
       </c>
+      <c r="G193" s="14" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="14" t="inlineStr">
@@ -4328,6 +4524,7 @@
         <f>IF(OR(D194&lt;&gt;"",E194&lt;&gt;""),IF(D194="",0,D194)+IF(E194="",0,E194),"")</f>
         <v/>
       </c>
+      <c r="G194" s="14" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="14" t="inlineStr">
@@ -4343,6 +4540,7 @@
         <f>IF(OR(D195&lt;&gt;"",E195&lt;&gt;""),IF(D195="",0,D195)+IF(E195="",0,E195),"")</f>
         <v/>
       </c>
+      <c r="G195" s="14" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="14" t="inlineStr">
@@ -4358,6 +4556,7 @@
         <f>IF(OR(D196&lt;&gt;"",E196&lt;&gt;""),IF(D196="",0,D196)+IF(E196="",0,E196),"")</f>
         <v/>
       </c>
+      <c r="G196" s="14" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="14" t="inlineStr">
@@ -4373,6 +4572,7 @@
         <f>IF(OR(D197&lt;&gt;"",E197&lt;&gt;""),IF(D197="",0,D197)+IF(E197="",0,E197),"")</f>
         <v/>
       </c>
+      <c r="G197" s="14" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="14" t="inlineStr">
@@ -4388,6 +4588,7 @@
         <f>IF(OR(D198&lt;&gt;"",E198&lt;&gt;""),IF(D198="",0,D198)+IF(E198="",0,E198),"")</f>
         <v/>
       </c>
+      <c r="G198" s="14" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="14" t="inlineStr">
@@ -4403,6 +4604,7 @@
         <f>IF(OR(D199&lt;&gt;"",E199&lt;&gt;""),IF(D199="",0,D199)+IF(E199="",0,E199),"")</f>
         <v/>
       </c>
+      <c r="G199" s="14" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="14" t="inlineStr">
@@ -4418,6 +4620,7 @@
         <f>IF(OR(D200&lt;&gt;"",E200&lt;&gt;""),IF(D200="",0,D200)+IF(E200="",0,E200),"")</f>
         <v/>
       </c>
+      <c r="G200" s="14" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="14" t="inlineStr">
@@ -4433,6 +4636,7 @@
         <f>IF(OR(D201&lt;&gt;"",E201&lt;&gt;""),IF(D201="",0,D201)+IF(E201="",0,E201),"")</f>
         <v/>
       </c>
+      <c r="G201" s="14" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="14" t="inlineStr">
@@ -4448,6 +4652,7 @@
         <f>IF(OR(D202&lt;&gt;"",E202&lt;&gt;""),IF(D202="",0,D202)+IF(E202="",0,E202),"")</f>
         <v/>
       </c>
+      <c r="G202" s="14" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="14" t="inlineStr">
@@ -4463,6 +4668,7 @@
         <f>IF(OR(D203&lt;&gt;"",E203&lt;&gt;""),IF(D203="",0,D203)+IF(E203="",0,E203),"")</f>
         <v/>
       </c>
+      <c r="G203" s="14" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="14" t="inlineStr">
@@ -4478,6 +4684,7 @@
         <f>IF(OR(D204&lt;&gt;"",E204&lt;&gt;""),IF(D204="",0,D204)+IF(E204="",0,E204),"")</f>
         <v/>
       </c>
+      <c r="G204" s="14" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="14" t="inlineStr">
@@ -4493,6 +4700,7 @@
         <f>IF(OR(D205&lt;&gt;"",E205&lt;&gt;""),IF(D205="",0,D205)+IF(E205="",0,E205),"")</f>
         <v/>
       </c>
+      <c r="G205" s="14" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="10" t="inlineStr">
@@ -4518,7 +4726,10 @@
         <f>D206+E206</f>
         <v/>
       </c>
-    </row>
+      <c r="G206" s="14" t="n"/>
+    </row>
+    <row r="207"/>
+    <row r="208"/>
     <row r="209">
       <c r="A209" s="11" t="inlineStr">
         <is>
@@ -4529,7 +4740,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>1) En cada mes, cargá Fecha + Detalle + Importe Sol y/o Importe Chris</t>
+          <t>1) En cada mes, cargá Fecha + Detalle + Importe Sol/Chris + Comentario (si corresponde)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Treat Cabify, Uber, and Didi as TRANSPORTE spending.
Reclassify Mercado Pago ride charges into a dedicated CIUDAD category instead of discarding them.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -615,6 +615,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1309,119 +1310,166 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>Cabify/Uber/Didi</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n">
+        <v>136132</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <v>122167</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v>38795</v>
+      </c>
+      <c r="J18" s="15" t="n">
+        <v>55446</v>
+      </c>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="15">
+        <f>SUM(D18:O18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="7">
-        <f>SUM(D5:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="7">
-        <f>SUM(E5:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="7">
-        <f>SUM(F5:F17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="7">
-        <f>SUM(G5:G17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="7">
-        <f>SUM(H5:H17)</f>
-        <v/>
-      </c>
-      <c r="I18" s="7">
-        <f>SUM(I5:I17)</f>
-        <v/>
-      </c>
-      <c r="J18" s="7">
-        <f>SUM(J5:J17)</f>
-        <v/>
-      </c>
-      <c r="K18" s="7">
-        <f>SUM(K5:K17)</f>
-        <v/>
-      </c>
-      <c r="L18" s="7">
-        <f>SUM(L5:L17)</f>
-        <v/>
-      </c>
-      <c r="M18" s="7">
-        <f>SUM(M5:M17)</f>
-        <v/>
-      </c>
-      <c r="N18" s="7">
-        <f>SUM(N5:N17)</f>
-        <v/>
-      </c>
-      <c r="O18" s="7">
-        <f>SUM(O5:O17)</f>
-        <v/>
-      </c>
-      <c r="P18" s="7">
-        <f>SUM(P5:P17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="7">
+        <f>SUM(D5:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="7">
+        <f>SUM(E5:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="7">
+        <f>SUM(F5:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="7">
+        <f>SUM(G5:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="7">
+        <f>SUM(H5:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="7">
+        <f>SUM(I5:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>SUM(J5:J18)</f>
+        <v/>
+      </c>
+      <c r="K19" s="7">
+        <f>SUM(K5:K18)</f>
+        <v/>
+      </c>
+      <c r="L19" s="7">
+        <f>SUM(L5:L18)</f>
+        <v/>
+      </c>
+      <c r="M19" s="7">
+        <f>SUM(M5:M18)</f>
+        <v/>
+      </c>
+      <c r="N19" s="7">
+        <f>SUM(N5:N18)</f>
+        <v/>
+      </c>
+      <c r="O19" s="7">
+        <f>SUM(O5:O18)</f>
+        <v/>
+      </c>
+      <c r="P19" s="7">
+        <f>SUM(P5:P18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
+        </is>
+      </c>
+    </row>
     <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A18:C18"/>

</xml_diff>

<commit_message>
Fix April grocery and transport updates for CIUDAD.
Persist the latest Mercado Pago almacén entries and refresh TRANSPORTE monthly totals after the interrupted save.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -615,7 +615,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1315,16 +1314,8 @@
           <t>SERVICIOS</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>Cabify/Uber/Didi</t>
-        </is>
-      </c>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="24" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="15" t="n"/>
       <c r="F18" s="15" t="n"/>
@@ -1351,125 +1342,167 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Cabify/Uber/Didi</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="n">
+        <v>146933</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>122167</v>
+      </c>
+      <c r="I19" s="26" t="n">
+        <v>38795</v>
+      </c>
+      <c r="J19" s="26" t="n">
+        <v>55446</v>
+      </c>
+      <c r="P19">
+        <f>SUM(D19:O19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="7">
-        <f>SUM(D5:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="7">
-        <f>SUM(E5:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="7">
-        <f>SUM(F5:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="7">
-        <f>SUM(G5:G18)</f>
-        <v/>
-      </c>
-      <c r="H19" s="7">
-        <f>SUM(H5:H18)</f>
-        <v/>
-      </c>
-      <c r="I19" s="7">
-        <f>SUM(I5:I18)</f>
-        <v/>
-      </c>
-      <c r="J19" s="7">
-        <f>SUM(J5:J18)</f>
-        <v/>
-      </c>
-      <c r="K19" s="7">
-        <f>SUM(K5:K18)</f>
-        <v/>
-      </c>
-      <c r="L19" s="7">
-        <f>SUM(L5:L18)</f>
-        <v/>
-      </c>
-      <c r="M19" s="7">
-        <f>SUM(M5:M18)</f>
-        <v/>
-      </c>
-      <c r="N19" s="7">
-        <f>SUM(N5:N18)</f>
-        <v/>
-      </c>
-      <c r="O19" s="7">
-        <f>SUM(O5:O18)</f>
-        <v/>
-      </c>
-      <c r="P19" s="7">
-        <f>SUM(P5:P18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="7">
+        <f>SUM(D5:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="7">
+        <f>SUM(E5:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="7">
+        <f>SUM(F5:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="7">
+        <f>SUM(G5:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="7">
+        <f>SUM(H5:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="7">
+        <f>SUM(I5:I19)</f>
+        <v/>
+      </c>
+      <c r="J20" s="7">
+        <f>SUM(J5:J19)</f>
+        <v/>
+      </c>
+      <c r="K20" s="7">
+        <f>SUM(K5:K19)</f>
+        <v/>
+      </c>
+      <c r="L20" s="7">
+        <f>SUM(L5:L19)</f>
+        <v/>
+      </c>
+      <c r="M20" s="7">
+        <f>SUM(M5:M19)</f>
+        <v/>
+      </c>
+      <c r="N20" s="7">
+        <f>SUM(N5:N19)</f>
+        <v/>
+      </c>
+      <c r="O20" s="7">
+        <f>SUM(O5:O19)</f>
+        <v/>
+      </c>
+      <c r="P20" s="7">
+        <f>SUM(P5:P19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A18:C18"/>
@@ -2213,6 +2246,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -2879,6 +2913,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -3545,6 +3580,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -3803,15 +3839,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B139" s="17" t="n"/>
-      <c r="C139" s="14" t="n"/>
-      <c r="D139" s="27" t="n"/>
+      <c r="B139" s="17" t="n">
+        <v>46122</v>
+      </c>
+      <c r="C139" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Propina</t>
+        </is>
+      </c>
+      <c r="D139" s="27" t="n">
+        <v>800</v>
+      </c>
       <c r="E139" s="28" t="n"/>
       <c r="F139" s="15">
         <f>IF(OR(D139&lt;&gt;"",E139&lt;&gt;""),IF(D139="",0,D139)+IF(E139="",0,E139),"")</f>
         <v/>
       </c>
-      <c r="G139" s="14" t="n"/>
+      <c r="G139" s="14" t="inlineStr">
+        <is>
+          <t>MP · delivery propina</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="14" t="inlineStr">
@@ -3819,15 +3867,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B140" s="17" t="n"/>
-      <c r="C140" s="14" t="n"/>
-      <c r="D140" s="27" t="n"/>
+      <c r="B140" s="17" t="n">
+        <v>46122</v>
+      </c>
+      <c r="C140" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa</t>
+        </is>
+      </c>
+      <c r="D140" s="27" t="n">
+        <v>2599</v>
+      </c>
       <c r="E140" s="28" t="n"/>
       <c r="F140" s="15">
         <f>IF(OR(D140&lt;&gt;"",E140&lt;&gt;""),IF(D140="",0,D140)+IF(E140="",0,E140),"")</f>
         <v/>
       </c>
-      <c r="G140" s="14" t="n"/>
+      <c r="G140" s="14" t="inlineStr">
+        <is>
+          <t>MP · delivery</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="14" t="inlineStr">
@@ -3835,15 +3895,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B141" s="17" t="n"/>
-      <c r="C141" s="14" t="n"/>
-      <c r="D141" s="27" t="n"/>
+      <c r="B141" s="17" t="n">
+        <v>46120</v>
+      </c>
+      <c r="C141" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering</t>
+        </is>
+      </c>
+      <c r="D141" s="27" t="n">
+        <v>17050</v>
+      </c>
       <c r="E141" s="28" t="n"/>
       <c r="F141" s="15">
         <f>IF(OR(D141&lt;&gt;"",E141&lt;&gt;""),IF(D141="",0,D141)+IF(E141="",0,E141),"")</f>
         <v/>
       </c>
-      <c r="G141" s="14" t="n"/>
+      <c r="G141" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="14" t="inlineStr">
@@ -3851,15 +3923,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B142" s="17" t="n"/>
-      <c r="C142" s="14" t="n"/>
-      <c r="D142" s="27" t="n"/>
+      <c r="B142" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="C142" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Dia</t>
+        </is>
+      </c>
+      <c r="D142" s="27" t="n">
+        <v>71961</v>
+      </c>
       <c r="E142" s="28" t="n"/>
       <c r="F142" s="15">
         <f>IF(OR(D142&lt;&gt;"",E142&lt;&gt;""),IF(D142="",0,D142)+IF(E142="",0,E142),"")</f>
         <v/>
       </c>
-      <c r="G142" s="14" t="n"/>
+      <c r="G142" s="14" t="inlineStr">
+        <is>
+          <t>MP · supermercado</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Clean up duplicate TRANSPORTE row in CIUDAD summary.
Remove the orphaned services row left from the interrupted transport update.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P40"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -615,6 +615,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1309,200 +1310,156 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>SERVICIOS</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="15" t="n">
-        <v>136132</v>
-      </c>
-      <c r="H18" s="15" t="n">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Cabify/Uber/Didi</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="n">
+        <v>146933</v>
+      </c>
+      <c r="H18" s="26" t="n">
         <v>122167</v>
       </c>
-      <c r="I18" s="15" t="n">
+      <c r="I18" s="26" t="n">
         <v>38795</v>
       </c>
-      <c r="J18" s="15" t="n">
+      <c r="J18" s="26" t="n">
         <v>55446</v>
       </c>
-      <c r="K18" s="15" t="n"/>
-      <c r="L18" s="15" t="n"/>
-      <c r="M18" s="15" t="n"/>
-      <c r="N18" s="15" t="n"/>
-      <c r="O18" s="15" t="n"/>
-      <c r="P18" s="15">
-        <f>SUM(D18:O18)</f>
+      <c r="P18">
+        <f>SUM(D19:O19)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SERVICIOS</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>Cabify/Uber/Didi</t>
-        </is>
-      </c>
-      <c r="G19" s="26" t="n">
-        <v>146933</v>
-      </c>
-      <c r="H19" s="26" t="n">
-        <v>122167</v>
-      </c>
-      <c r="I19" s="26" t="n">
-        <v>38795</v>
-      </c>
-      <c r="J19" s="26" t="n">
-        <v>55446</v>
-      </c>
-      <c r="P19">
-        <f>SUM(D19:O19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="23" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="7">
-        <f>SUM(D5:D19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="7">
-        <f>SUM(E5:E19)</f>
-        <v/>
-      </c>
-      <c r="F20" s="7">
-        <f>SUM(F5:F19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="7">
-        <f>SUM(G5:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="7">
-        <f>SUM(H5:H19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="7">
-        <f>SUM(I5:I19)</f>
-        <v/>
-      </c>
-      <c r="J20" s="7">
-        <f>SUM(J5:J19)</f>
-        <v/>
-      </c>
-      <c r="K20" s="7">
-        <f>SUM(K5:K19)</f>
-        <v/>
-      </c>
-      <c r="L20" s="7">
-        <f>SUM(L5:L19)</f>
-        <v/>
-      </c>
-      <c r="M20" s="7">
-        <f>SUM(M5:M19)</f>
-        <v/>
-      </c>
-      <c r="N20" s="7">
-        <f>SUM(N5:N19)</f>
-        <v/>
-      </c>
-      <c r="O20" s="7">
-        <f>SUM(O5:O19)</f>
-        <v/>
-      </c>
-      <c r="P20" s="7">
-        <f>SUM(P5:P19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21"/>
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="7">
+        <f>SUM(D5:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="7">
+        <f>SUM(E5:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="7">
+        <f>SUM(F5:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="7">
+        <f>SUM(G5:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="7">
+        <f>SUM(H5:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="7">
+        <f>SUM(I5:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>SUM(J5:J18)</f>
+        <v/>
+      </c>
+      <c r="K19" s="7">
+        <f>SUM(K5:K18)</f>
+        <v/>
+      </c>
+      <c r="L19" s="7">
+        <f>SUM(L5:L18)</f>
+        <v/>
+      </c>
+      <c r="M19" s="7">
+        <f>SUM(M5:M18)</f>
+        <v/>
+      </c>
+      <c r="N19" s="7">
+        <f>SUM(N5:N18)</f>
+        <v/>
+      </c>
+      <c r="O19" s="7">
+        <f>SUM(O5:O18)</f>
+        <v/>
+      </c>
+      <c r="P19" s="7">
+        <f>SUM(P5:P18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Notas</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A18:C18"/>
@@ -2246,7 +2203,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -2913,7 +2869,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -3580,7 +3535,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Persist April almacén and transport updates for CIUDAD.
Save grocery entries and refreshed TRANSPORTE totals after the interrupted workbook write.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -615,7 +615,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1315,16 +1314,6 @@
           <t>SERVICIOS</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Cabify/Uber/Didi</t>
-        </is>
-      </c>
       <c r="G18" s="26" t="n">
         <v>146933</v>
       </c>
@@ -1343,123 +1332,157 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Cabify/Uber/Didi</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="n">
+        <v>172424</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>122167</v>
+      </c>
+      <c r="I19" s="26" t="n">
+        <v>38795</v>
+      </c>
+      <c r="J19" s="26" t="n">
+        <v>55446</v>
+      </c>
+      <c r="P19">
+        <f>SUM(D19:O19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="7">
-        <f>SUM(D5:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="7">
-        <f>SUM(E5:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="7">
-        <f>SUM(F5:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="7">
-        <f>SUM(G5:G18)</f>
-        <v/>
-      </c>
-      <c r="H19" s="7">
-        <f>SUM(H5:H18)</f>
-        <v/>
-      </c>
-      <c r="I19" s="7">
-        <f>SUM(I5:I18)</f>
-        <v/>
-      </c>
-      <c r="J19" s="7">
-        <f>SUM(J5:J18)</f>
-        <v/>
-      </c>
-      <c r="K19" s="7">
-        <f>SUM(K5:K18)</f>
-        <v/>
-      </c>
-      <c r="L19" s="7">
-        <f>SUM(L5:L18)</f>
-        <v/>
-      </c>
-      <c r="M19" s="7">
-        <f>SUM(M5:M18)</f>
-        <v/>
-      </c>
-      <c r="N19" s="7">
-        <f>SUM(N5:N18)</f>
-        <v/>
-      </c>
-      <c r="O19" s="7">
-        <f>SUM(O5:O18)</f>
-        <v/>
-      </c>
-      <c r="P19" s="7">
-        <f>SUM(P5:P18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="7">
+        <f>SUM(D5:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="7">
+        <f>SUM(E5:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="7">
+        <f>SUM(F5:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="7">
+        <f>SUM(G5:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="7">
+        <f>SUM(H5:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="7">
+        <f>SUM(I5:I19)</f>
+        <v/>
+      </c>
+      <c r="J20" s="7">
+        <f>SUM(J5:J19)</f>
+        <v/>
+      </c>
+      <c r="K20" s="7">
+        <f>SUM(K5:K19)</f>
+        <v/>
+      </c>
+      <c r="L20" s="7">
+        <f>SUM(L5:L19)</f>
+        <v/>
+      </c>
+      <c r="M20" s="7">
+        <f>SUM(M5:M19)</f>
+        <v/>
+      </c>
+      <c r="N20" s="7">
+        <f>SUM(N5:N19)</f>
+        <v/>
+      </c>
+      <c r="O20" s="7">
+        <f>SUM(O5:O19)</f>
+        <v/>
+      </c>
+      <c r="P20" s="7">
+        <f>SUM(P5:P19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A18:C18"/>
@@ -2203,6 +2226,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -2869,6 +2893,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -3535,6 +3560,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -3905,15 +3931,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B143" s="17" t="n"/>
-      <c r="C143" s="14" t="n"/>
-      <c r="D143" s="27" t="n"/>
+      <c r="B143" s="17" t="n">
+        <v>46115</v>
+      </c>
+      <c r="C143" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Dia</t>
+        </is>
+      </c>
+      <c r="D143" s="27" t="n">
+        <v>27350</v>
+      </c>
       <c r="E143" s="28" t="n"/>
       <c r="F143" s="15">
         <f>IF(OR(D143&lt;&gt;"",E143&lt;&gt;""),IF(D143="",0,D143)+IF(E143="",0,E143),"")</f>
         <v/>
       </c>
-      <c r="G143" s="14" t="n"/>
+      <c r="G143" s="14" t="inlineStr">
+        <is>
+          <t>MP · supermercado</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="14" t="inlineStr">
@@ -3921,15 +3959,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B144" s="17" t="n"/>
-      <c r="C144" s="14" t="n"/>
-      <c r="D144" s="27" t="n"/>
+      <c r="B144" s="17" t="n">
+        <v>46115</v>
+      </c>
+      <c r="C144" s="14" t="inlineStr">
+        <is>
+          <t>Coto</t>
+        </is>
+      </c>
+      <c r="D144" s="27" t="n">
+        <v>149320</v>
+      </c>
       <c r="E144" s="28" t="n"/>
       <c r="F144" s="15">
         <f>IF(OR(D144&lt;&gt;"",E144&lt;&gt;""),IF(D144="",0,D144)+IF(E144="",0,E144),"")</f>
         <v/>
       </c>
-      <c r="G144" s="14" t="n"/>
+      <c r="G144" s="14" t="inlineStr">
+        <is>
+          <t>MP · supermercado</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="14" t="inlineStr">
@@ -3937,15 +3987,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B145" s="17" t="n"/>
-      <c r="C145" s="14" t="n"/>
-      <c r="D145" s="27" t="n"/>
+      <c r="B145" s="17" t="n">
+        <v>46114</v>
+      </c>
+      <c r="C145" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Propina</t>
+        </is>
+      </c>
+      <c r="D145" s="27" t="n">
+        <v>2000</v>
+      </c>
       <c r="E145" s="28" t="n"/>
       <c r="F145" s="15">
         <f>IF(OR(D145&lt;&gt;"",E145&lt;&gt;""),IF(D145="",0,D145)+IF(E145="",0,E145),"")</f>
         <v/>
       </c>
-      <c r="G145" s="14" t="n"/>
+      <c r="G145" s="14" t="inlineStr">
+        <is>
+          <t>MP · delivery propina</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="14" t="inlineStr">
@@ -3953,15 +4015,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B146" s="17" t="n"/>
-      <c r="C146" s="14" t="n"/>
-      <c r="D146" s="27" t="n"/>
+      <c r="B146" s="17" t="n">
+        <v>46114</v>
+      </c>
+      <c r="C146" s="14" t="inlineStr">
+        <is>
+          <t>Pedidosya Empanada</t>
+        </is>
+      </c>
+      <c r="D146" s="27" t="n">
+        <v>36519</v>
+      </c>
       <c r="E146" s="28" t="n"/>
       <c r="F146" s="15">
         <f>IF(OR(D146&lt;&gt;"",E146&lt;&gt;""),IF(D146="",0,D146)+IF(E146="",0,E146),"")</f>
         <v/>
       </c>
-      <c r="G146" s="14" t="n"/>
+      <c r="G146" s="14" t="inlineStr">
+        <is>
+          <t>MP · delivery</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Remove orphan CIUDAD summary row after transport insert.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1314,8 +1314,18 @@
           <t>SERVICIOS</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Cabify/Uber/Didi</t>
+        </is>
+      </c>
       <c r="G18" s="26" t="n">
-        <v>146933</v>
+        <v>172424</v>
       </c>
       <c r="H18" s="26" t="n">
         <v>122167</v>
@@ -1332,157 +1342,123 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SERVICIOS</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>Cabify/Uber/Didi</t>
-        </is>
-      </c>
-      <c r="G19" s="26" t="n">
-        <v>172424</v>
-      </c>
-      <c r="H19" s="26" t="n">
-        <v>122167</v>
-      </c>
-      <c r="I19" s="26" t="n">
-        <v>38795</v>
-      </c>
-      <c r="J19" s="26" t="n">
-        <v>55446</v>
-      </c>
-      <c r="P19">
-        <f>SUM(D19:O19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="23" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="7">
-        <f>SUM(D5:D19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="7">
-        <f>SUM(E5:E19)</f>
-        <v/>
-      </c>
-      <c r="F20" s="7">
-        <f>SUM(F5:F19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="7">
-        <f>SUM(G5:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="7">
-        <f>SUM(H5:H19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="7">
-        <f>SUM(I5:I19)</f>
-        <v/>
-      </c>
-      <c r="J20" s="7">
-        <f>SUM(J5:J19)</f>
-        <v/>
-      </c>
-      <c r="K20" s="7">
-        <f>SUM(K5:K19)</f>
-        <v/>
-      </c>
-      <c r="L20" s="7">
-        <f>SUM(L5:L19)</f>
-        <v/>
-      </c>
-      <c r="M20" s="7">
-        <f>SUM(M5:M19)</f>
-        <v/>
-      </c>
-      <c r="N20" s="7">
-        <f>SUM(N5:N19)</f>
-        <v/>
-      </c>
-      <c r="O20" s="7">
-        <f>SUM(O5:O19)</f>
-        <v/>
-      </c>
-      <c r="P20" s="7">
-        <f>SUM(P5:P19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21"/>
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="7">
+        <f>SUM(D5:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="7">
+        <f>SUM(E5:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="7">
+        <f>SUM(F5:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="7">
+        <f>SUM(G5:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="7">
+        <f>SUM(H5:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="7">
+        <f>SUM(I5:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>SUM(J5:J18)</f>
+        <v/>
+      </c>
+      <c r="K19" s="7">
+        <f>SUM(K5:K18)</f>
+        <v/>
+      </c>
+      <c r="L19" s="7">
+        <f>SUM(L5:L18)</f>
+        <v/>
+      </c>
+      <c r="M19" s="7">
+        <f>SUM(M5:M18)</f>
+        <v/>
+      </c>
+      <c r="N19" s="7">
+        <f>SUM(N5:N18)</f>
+        <v/>
+      </c>
+      <c r="O19" s="7">
+        <f>SUM(O5:O18)</f>
+        <v/>
+      </c>
+      <c r="P19" s="7">
+        <f>SUM(P5:P18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Notas</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A18:C18"/>
@@ -2226,7 +2202,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -2893,7 +2868,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -3560,7 +3534,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Classify YPF and Shell as CIUDAD almacén combustible.
Route fuel purchases into ALMACEN SOL detail instead of treating them as separate auto extras.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1314,16 +1314,6 @@
           <t>SERVICIOS</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Cabify/Uber/Didi</t>
-        </is>
-      </c>
       <c r="G18" s="26" t="n">
         <v>172424</v>
       </c>
@@ -1402,7 +1392,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
@@ -2202,6 +2191,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -2868,6 +2858,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -3534,6 +3525,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -4016,15 +4008,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B147" s="17" t="n"/>
-      <c r="C147" s="14" t="n"/>
-      <c r="D147" s="27" t="n"/>
+      <c r="B147" s="17" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C147" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D147" s="27" t="n">
+        <v>27579</v>
+      </c>
       <c r="E147" s="28" t="n"/>
       <c r="F147" s="15">
         <f>IF(OR(D147&lt;&gt;"",E147&lt;&gt;""),IF(D147="",0,D147)+IF(E147="",0,E147),"")</f>
         <v/>
       </c>
-      <c r="G147" s="14" t="n"/>
+      <c r="G147" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible · nafta · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="14" t="inlineStr">
@@ -4032,15 +4036,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B148" s="17" t="n"/>
-      <c r="C148" s="14" t="n"/>
-      <c r="D148" s="27" t="n"/>
+      <c r="B148" s="17" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C148" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D148" s="27" t="n">
+        <v>1307</v>
+      </c>
       <c r="E148" s="28" t="n"/>
       <c r="F148" s="15">
         <f>IF(OR(D148&lt;&gt;"",E148&lt;&gt;""),IF(D148="",0,D148)+IF(E148="",0,E148),"")</f>
         <v/>
       </c>
-      <c r="G148" s="14" t="n"/>
+      <c r="G148" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible · nafta · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="14" t="inlineStr">
@@ -4404,6 +4420,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -4718,15 +4735,27 @@
           <t>Mayo</t>
         </is>
       </c>
-      <c r="B183" s="17" t="n"/>
-      <c r="C183" s="14" t="n"/>
-      <c r="D183" s="27" t="n"/>
+      <c r="B183" s="17" t="n">
+        <v>46172</v>
+      </c>
+      <c r="C183" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D183" s="27" t="n">
+        <v>18314</v>
+      </c>
       <c r="E183" s="28" t="n"/>
       <c r="F183" s="15">
         <f>IF(OR(D183&lt;&gt;"",E183&lt;&gt;""),IF(D183="",0,D183)+IF(E183="",0,E183),"")</f>
         <v/>
       </c>
-      <c r="G183" s="14" t="n"/>
+      <c r="G183" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible · nafta · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="14" t="inlineStr">
@@ -4734,15 +4763,27 @@
           <t>Mayo</t>
         </is>
       </c>
-      <c r="B184" s="17" t="n"/>
-      <c r="C184" s="14" t="n"/>
-      <c r="D184" s="27" t="n"/>
+      <c r="B184" s="17" t="n">
+        <v>46172</v>
+      </c>
+      <c r="C184" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D184" s="27" t="n">
+        <v>1415</v>
+      </c>
       <c r="E184" s="28" t="n"/>
       <c r="F184" s="15">
         <f>IF(OR(D184&lt;&gt;"",E184&lt;&gt;""),IF(D184="",0,D184)+IF(E184="",0,E184),"")</f>
         <v/>
       </c>
-      <c r="G184" s="14" t="n"/>
+      <c r="G184" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible · nafta · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="14" t="inlineStr">
@@ -5202,6 +5243,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -5768,15 +5810,27 @@
           <t>Junio</t>
         </is>
       </c>
-      <c r="B234" s="17" t="n"/>
-      <c r="C234" s="14" t="n"/>
-      <c r="D234" s="27" t="n"/>
+      <c r="B234" s="17" t="n">
+        <v>46194</v>
+      </c>
+      <c r="C234" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D234" s="27" t="n">
+        <v>1648</v>
+      </c>
       <c r="E234" s="28" t="n"/>
       <c r="F234" s="15">
         <f>IF(OR(D234&lt;&gt;"",E234&lt;&gt;""),IF(D234="",0,D234)+IF(E234="",0,E234),"")</f>
         <v/>
       </c>
-      <c r="G234" s="14" t="n"/>
+      <c r="G234" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible · nafta · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="14" t="inlineStr">
@@ -6108,6 +6162,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -6912,6 +6967,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -7578,6 +7634,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -8244,6 +8301,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -8910,6 +8968,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -9576,6 +9635,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add late March Mercado Pago expenses for CIUDAD.
Load grocery and fuel charges into almacén, refresh transport totals, and keep unresolved merchants pending.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1314,6 +1314,19 @@
           <t>SERVICIOS</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TRANSPORTE</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Cabify/Uber/Didi</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="n">
+        <v>21609</v>
+      </c>
       <c r="G18" s="26" t="n">
         <v>172424</v>
       </c>
@@ -1392,6 +1405,7 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
@@ -1448,6 +1462,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A18:C18"/>
@@ -2865,15 +2880,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B88" s="17" t="n"/>
-      <c r="C88" s="14" t="n"/>
-      <c r="D88" s="27" t="n"/>
+      <c r="B88" s="17" t="n">
+        <v>46112</v>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D88" s="27" t="n">
+        <v>264</v>
+      </c>
       <c r="E88" s="28" t="n"/>
       <c r="F88" s="15">
         <f>IF(OR(D88&lt;&gt;"",E88&lt;&gt;""),IF(D88="",0,D88)+IF(E88="",0,E88),"")</f>
         <v/>
       </c>
-      <c r="G88" s="14" t="n"/>
+      <c r="G88" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="14" t="inlineStr">
@@ -2881,15 +2908,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B89" s="17" t="n"/>
-      <c r="C89" s="14" t="n"/>
-      <c r="D89" s="27" t="n"/>
+      <c r="B89" s="17" t="n">
+        <v>46112</v>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D89" s="27" t="n">
+        <v>1118</v>
+      </c>
       <c r="E89" s="28" t="n"/>
       <c r="F89" s="15">
         <f>IF(OR(D89&lt;&gt;"",E89&lt;&gt;""),IF(D89="",0,D89)+IF(E89="",0,E89),"")</f>
         <v/>
       </c>
-      <c r="G89" s="14" t="n"/>
+      <c r="G89" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
@@ -2897,15 +2936,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B90" s="17" t="n"/>
-      <c r="C90" s="14" t="n"/>
-      <c r="D90" s="27" t="n"/>
+      <c r="B90" s="17" t="n">
+        <v>46112</v>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D90" s="27" t="n">
+        <v>653</v>
+      </c>
       <c r="E90" s="28" t="n"/>
       <c r="F90" s="15">
         <f>IF(OR(D90&lt;&gt;"",E90&lt;&gt;""),IF(D90="",0,D90)+IF(E90="",0,E90),"")</f>
         <v/>
       </c>
-      <c r="G90" s="14" t="n"/>
+      <c r="G90" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="14" t="inlineStr">
@@ -2913,15 +2964,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B91" s="17" t="n"/>
-      <c r="C91" s="14" t="n"/>
-      <c r="D91" s="27" t="n"/>
+      <c r="B91" s="17" t="n">
+        <v>46112</v>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering</t>
+        </is>
+      </c>
+      <c r="D91" s="27" t="n">
+        <v>13500</v>
+      </c>
       <c r="E91" s="28" t="n"/>
       <c r="F91" s="15">
         <f>IF(OR(D91&lt;&gt;"",E91&lt;&gt;""),IF(D91="",0,D91)+IF(E91="",0,E91),"")</f>
         <v/>
       </c>
-      <c r="G91" s="14" t="n"/>
+      <c r="G91" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
@@ -2929,15 +2992,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B92" s="17" t="n"/>
-      <c r="C92" s="14" t="n"/>
-      <c r="D92" s="27" t="n"/>
+      <c r="B92" s="17" t="n">
+        <v>46111</v>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Generacion 20</t>
+        </is>
+      </c>
+      <c r="D92" s="27" t="n">
+        <v>88999</v>
+      </c>
       <c r="E92" s="28" t="n"/>
       <c r="F92" s="15">
         <f>IF(OR(D92&lt;&gt;"",E92&lt;&gt;""),IF(D92="",0,D92)+IF(E92="",0,E92),"")</f>
         <v/>
       </c>
-      <c r="G92" s="14" t="n"/>
+      <c r="G92" s="14" t="inlineStr">
+        <is>
+          <t>MP · combustible</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
@@ -2945,15 +3020,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B93" s="17" t="n"/>
-      <c r="C93" s="14" t="n"/>
-      <c r="D93" s="27" t="n"/>
+      <c r="B93" s="17" t="n">
+        <v>46104</v>
+      </c>
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Dia</t>
+        </is>
+      </c>
+      <c r="D93" s="27" t="n">
+        <v>47664</v>
+      </c>
       <c r="E93" s="28" t="n"/>
       <c r="F93" s="15">
         <f>IF(OR(D93&lt;&gt;"",E93&lt;&gt;""),IF(D93="",0,D93)+IF(E93="",0,E93),"")</f>
         <v/>
       </c>
-      <c r="G93" s="14" t="n"/>
+      <c r="G93" s="14" t="inlineStr">
+        <is>
+          <t>MP · supermercado</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
@@ -2961,15 +3048,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B94" s="17" t="n"/>
-      <c r="C94" s="14" t="n"/>
-      <c r="D94" s="27" t="n"/>
+      <c r="B94" s="17" t="n">
+        <v>46103</v>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>Open 25</t>
+        </is>
+      </c>
+      <c r="D94" s="27" t="n">
+        <v>50000</v>
+      </c>
       <c r="E94" s="28" t="n"/>
       <c r="F94" s="15">
         <f>IF(OR(D94&lt;&gt;"",E94&lt;&gt;""),IF(D94="",0,D94)+IF(E94="",0,E94),"")</f>
         <v/>
       </c>
-      <c r="G94" s="14" t="n"/>
+      <c r="G94" s="14" t="inlineStr">
+        <is>
+          <t>MP · tienda</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Restore TRANSPORTE row and load mid-March CIUDAD charges.
Re-add Cabify/Uber/Didi monthly totals and Burger King to Almacén Sol after a failed workbook save.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1319,13 +1319,13 @@
           <t>TRANSPORTE</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Cabify/Uber/Didi</t>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Cabify / Uber / Didi</t>
         </is>
       </c>
       <c r="F18" s="26" t="n">
-        <v>21609</v>
+        <v>70650</v>
       </c>
       <c r="G18" s="26" t="n">
         <v>172424</v>
@@ -1339,8 +1339,8 @@
       <c r="J18" s="26" t="n">
         <v>55446</v>
       </c>
-      <c r="P18">
-        <f>SUM(D19:O19)</f>
+      <c r="P18" s="26">
+        <f>SUM(D18:O18)</f>
         <v/>
       </c>
     </row>
@@ -1405,7 +1405,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
@@ -1462,11 +1461,7 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A18:C18"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3076,15 +3071,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B95" s="17" t="n"/>
-      <c r="C95" s="14" t="n"/>
-      <c r="D95" s="27" t="n"/>
+      <c r="B95" s="17" t="n">
+        <v>46101</v>
+      </c>
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>Burger King</t>
+        </is>
+      </c>
+      <c r="D95" s="27" t="n">
+        <v>22100</v>
+      </c>
       <c r="E95" s="28" t="n"/>
       <c r="F95" s="15">
         <f>IF(OR(D95&lt;&gt;"",E95&lt;&gt;""),IF(D95="",0,D95)+IF(E95="",0,E95),"")</f>
         <v/>
       </c>
-      <c r="G95" s="14" t="n"/>
+      <c r="G95" s="14" t="inlineStr">
+        <is>
+          <t>MP · comida</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
@@ -3624,7 +3631,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -4519,7 +4525,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -5342,7 +5347,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -6261,7 +6265,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7066,7 +7069,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -7733,7 +7735,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -8400,7 +8401,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9067,7 +9067,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -9734,7 +9733,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Link ALMACEN SOL/CHRIS monthly columns to each month total.
Enero was hard-coded to D44; point Febrero–Diciembre at their Almacen Detalle TOTAL rows.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1472,7 +1472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:G599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3631,6 +3631,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -4525,6 +4526,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -5347,6 +5349,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -6265,6 +6268,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7069,6 +7073,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -7735,6 +7740,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -8401,6 +8407,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9067,6 +9074,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -9733,6 +9741,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -10399,6 +10408,99 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Load March 11–16 Mercado Pago activity for CIUDAD.
Add almacén and transport charges, bump Susana cleaning for mid-March, and keep transfers pending.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -947,7 +947,7 @@
         <v>515550</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>524479</v>
+        <v>611047</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>501015</v>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="F18" s="26" t="n">
-        <v>70650</v>
+        <v>101110</v>
       </c>
       <c r="G18" s="26" t="n">
         <v>172424</v>
@@ -1472,7 +1472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G599"/>
+  <dimension ref="A1:G506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3099,15 +3099,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B96" s="17" t="n"/>
-      <c r="C96" s="14" t="n"/>
-      <c r="D96" s="27" t="n"/>
+      <c r="B96" s="17" t="n">
+        <v>46095</v>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>Galletotas</t>
+        </is>
+      </c>
+      <c r="D96" s="27" t="n">
+        <v>19500</v>
+      </c>
       <c r="E96" s="28" t="n"/>
       <c r="F96" s="15">
         <f>IF(OR(D96&lt;&gt;"",E96&lt;&gt;""),IF(D96="",0,D96)+IF(E96="",0,E96),"")</f>
         <v/>
       </c>
-      <c r="G96" s="14" t="n"/>
+      <c r="G96" s="14" t="inlineStr">
+        <is>
+          <t>MP · galletitas</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="14" t="inlineStr">
@@ -3115,15 +3127,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B97" s="17" t="n"/>
-      <c r="C97" s="14" t="n"/>
-      <c r="D97" s="27" t="n"/>
+      <c r="B97" s="17" t="n">
+        <v>46095</v>
+      </c>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>Oporto Almacen</t>
+        </is>
+      </c>
+      <c r="D97" s="27" t="n">
+        <v>51920</v>
+      </c>
       <c r="E97" s="28" t="n"/>
       <c r="F97" s="15">
         <f>IF(OR(D97&lt;&gt;"",E97&lt;&gt;""),IF(D97="",0,D97)+IF(E97="",0,E97),"")</f>
         <v/>
       </c>
-      <c r="G97" s="14" t="n"/>
+      <c r="G97" s="14" t="inlineStr">
+        <is>
+          <t>MP · almacén</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
@@ -3131,15 +3155,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B98" s="17" t="n"/>
-      <c r="C98" s="14" t="n"/>
-      <c r="D98" s="27" t="n"/>
+      <c r="B98" s="17" t="n">
+        <v>46093</v>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>Súper Pollo</t>
+        </is>
+      </c>
+      <c r="D98" s="27" t="n">
+        <v>33619</v>
+      </c>
       <c r="E98" s="28" t="n"/>
       <c r="F98" s="15">
         <f>IF(OR(D98&lt;&gt;"",E98&lt;&gt;""),IF(D98="",0,D98)+IF(E98="",0,E98),"")</f>
         <v/>
       </c>
-      <c r="G98" s="14" t="n"/>
+      <c r="G98" s="14" t="inlineStr">
+        <is>
+          <t>MP · pollo</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="14" t="inlineStr">
@@ -3147,15 +3183,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B99" s="17" t="n"/>
-      <c r="C99" s="14" t="n"/>
-      <c r="D99" s="27" t="n"/>
+      <c r="B99" s="17" t="n">
+        <v>46092</v>
+      </c>
+      <c r="C99" s="14" t="inlineStr">
+        <is>
+          <t>Bee Coffee</t>
+        </is>
+      </c>
+      <c r="D99" s="27" t="n">
+        <v>6100</v>
+      </c>
       <c r="E99" s="28" t="n"/>
       <c r="F99" s="15">
         <f>IF(OR(D99&lt;&gt;"",E99&lt;&gt;""),IF(D99="",0,D99)+IF(E99="",0,E99),"")</f>
         <v/>
       </c>
-      <c r="G99" s="14" t="n"/>
+      <c r="G99" s="14" t="inlineStr">
+        <is>
+          <t>MP · café</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
@@ -3631,7 +3679,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -4526,7 +4573,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -5349,7 +5395,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -6268,7 +6313,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7073,7 +7117,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -7740,7 +7783,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -8407,7 +8449,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9074,7 +9115,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -9741,7 +9781,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -10408,99 +10447,6 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Load early March Mercado Pago activity for CIUDAD.
Add almacén and transport, bump Susana cleaning, and keep AVA/own transfers out of CIUDAD totals.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -947,7 +947,7 @@
         <v>515550</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>611047</v>
+        <v>722888</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>501015</v>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="F18" s="26" t="n">
-        <v>101110</v>
+        <v>107090</v>
       </c>
       <c r="G18" s="26" t="n">
         <v>172424</v>
@@ -3211,15 +3211,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B100" s="17" t="n"/>
-      <c r="C100" s="14" t="n"/>
-      <c r="D100" s="27" t="n"/>
+      <c r="B100" s="17" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C100" s="14" t="inlineStr">
+        <is>
+          <t>Todo Tartas</t>
+        </is>
+      </c>
+      <c r="D100" s="27" t="n">
+        <v>11000</v>
+      </c>
       <c r="E100" s="28" t="n"/>
       <c r="F100" s="15">
         <f>IF(OR(D100&lt;&gt;"",E100&lt;&gt;""),IF(D100="",0,D100)+IF(E100="",0,E100),"")</f>
         <v/>
       </c>
-      <c r="G100" s="14" t="n"/>
+      <c r="G100" s="14" t="inlineStr">
+        <is>
+          <t>MP · tartas</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="14" t="inlineStr">
@@ -3227,15 +3239,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B101" s="17" t="n"/>
-      <c r="C101" s="14" t="n"/>
-      <c r="D101" s="27" t="n"/>
+      <c r="B101" s="17" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>Kiosko Duendes (propina)</t>
+        </is>
+      </c>
+      <c r="D101" s="27" t="n">
+        <v>1930</v>
+      </c>
       <c r="E101" s="28" t="n"/>
       <c r="F101" s="15">
         <f>IF(OR(D101&lt;&gt;"",E101&lt;&gt;""),IF(D101="",0,D101)+IF(E101="",0,E101),"")</f>
         <v/>
       </c>
-      <c r="G101" s="14" t="n"/>
+      <c r="G101" s="14" t="inlineStr">
+        <is>
+          <t>MP · propina</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
@@ -3243,15 +3267,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B102" s="17" t="n"/>
-      <c r="C102" s="14" t="n"/>
-      <c r="D102" s="27" t="n"/>
+      <c r="B102" s="17" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C102" s="14" t="inlineStr">
+        <is>
+          <t>El Patio De Los Duendes</t>
+        </is>
+      </c>
+      <c r="D102" s="27" t="n">
+        <v>17049</v>
+      </c>
       <c r="E102" s="28" t="n"/>
       <c r="F102" s="15">
         <f>IF(OR(D102&lt;&gt;"",E102&lt;&gt;""),IF(D102="",0,D102)+IF(E102="",0,E102),"")</f>
         <v/>
       </c>
-      <c r="G102" s="14" t="n"/>
+      <c r="G102" s="14" t="inlineStr">
+        <is>
+          <t>MP · comida</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="14" t="inlineStr">
@@ -3259,15 +3295,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B103" s="17" t="n"/>
-      <c r="C103" s="14" t="n"/>
-      <c r="D103" s="27" t="n"/>
+      <c r="B103" s="17" t="n">
+        <v>46087</v>
+      </c>
+      <c r="C103" s="14" t="inlineStr">
+        <is>
+          <t>Coto</t>
+        </is>
+      </c>
+      <c r="D103" s="27" t="n">
+        <v>114263</v>
+      </c>
       <c r="E103" s="28" t="n"/>
       <c r="F103" s="15">
         <f>IF(OR(D103&lt;&gt;"",E103&lt;&gt;""),IF(D103="",0,D103)+IF(E103="",0,E103),"")</f>
         <v/>
       </c>
-      <c r="G103" s="14" t="n"/>
+      <c r="G103" s="14" t="inlineStr">
+        <is>
+          <t>MP · super</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
@@ -3275,15 +3323,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B104" s="17" t="n"/>
-      <c r="C104" s="14" t="n"/>
-      <c r="D104" s="27" t="n"/>
+      <c r="B104" s="17" t="n">
+        <v>46086</v>
+      </c>
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>Huevos Point</t>
+        </is>
+      </c>
+      <c r="D104" s="27" t="n">
+        <v>14500</v>
+      </c>
       <c r="E104" s="28" t="n"/>
       <c r="F104" s="15">
         <f>IF(OR(D104&lt;&gt;"",E104&lt;&gt;""),IF(D104="",0,D104)+IF(E104="",0,E104),"")</f>
         <v/>
       </c>
-      <c r="G104" s="14" t="n"/>
+      <c r="G104" s="14" t="inlineStr">
+        <is>
+          <t>MP · huevos</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load late February and early March Mercado Pago for CIUDAD.
Add Shell fuel, Le Pain Quotidien, ABL, Susana cleaning, and February transport; exclude own transfers.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -909,7 +910,9 @@
       </c>
       <c r="D9" s="5" t="n"/>
       <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
+      <c r="F9" s="5" t="n">
+        <v>88141</v>
+      </c>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="5" t="n"/>
@@ -947,7 +950,7 @@
         <v>515550</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>722888</v>
+        <v>872390</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>501015</v>
@@ -1323,6 +1326,9 @@
         <is>
           <t>Cabify / Uber / Didi</t>
         </is>
+      </c>
+      <c r="E18" s="26" t="n">
+        <v>9950</v>
       </c>
       <c r="F18" s="26" t="n">
         <v>107090</v>
@@ -2201,22 +2207,33 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B46" s="17" t="n"/>
-      <c r="C46" s="14" t="n"/>
-      <c r="D46" s="27" t="n"/>
+      <c r="B46" s="17" t="n">
+        <v>46081</v>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D46" s="27" t="n">
+        <v>61</v>
+      </c>
       <c r="E46" s="28" t="n"/>
       <c r="F46" s="15">
         <f>IF(OR(D46&lt;&gt;"",E46&lt;&gt;""),IF(D46="",0,D46)+IF(E46="",0,E46),"")</f>
         <v/>
       </c>
-      <c r="G46" s="14" t="n"/>
+      <c r="G46" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
@@ -2224,15 +2241,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B47" s="17" t="n"/>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="27" t="n"/>
+      <c r="B47" s="17" t="n">
+        <v>46081</v>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D47" s="27" t="n">
+        <v>418</v>
+      </c>
       <c r="E47" s="28" t="n"/>
       <c r="F47" s="15">
         <f>IF(OR(D47&lt;&gt;"",E47&lt;&gt;""),IF(D47="",0,D47)+IF(E47="",0,E47),"")</f>
         <v/>
       </c>
-      <c r="G47" s="14" t="n"/>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
@@ -2240,15 +2269,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B48" s="17" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="27" t="n"/>
+      <c r="B48" s="17" t="n">
+        <v>46081</v>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D48" s="27" t="n">
+        <v>788</v>
+      </c>
       <c r="E48" s="28" t="n"/>
       <c r="F48" s="15">
         <f>IF(OR(D48&lt;&gt;"",E48&lt;&gt;""),IF(D48="",0,D48)+IF(E48="",0,E48),"")</f>
         <v/>
       </c>
-      <c r="G48" s="14" t="n"/>
+      <c r="G48" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
@@ -2256,15 +2297,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B49" s="17" t="n"/>
-      <c r="C49" s="14" t="n"/>
-      <c r="D49" s="27" t="n"/>
+      <c r="B49" s="17" t="n">
+        <v>46081</v>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D49" s="27" t="n">
+        <v>605</v>
+      </c>
       <c r="E49" s="28" t="n"/>
       <c r="F49" s="15">
         <f>IF(OR(D49&lt;&gt;"",E49&lt;&gt;""),IF(D49="",0,D49)+IF(E49="",0,E49),"")</f>
         <v/>
       </c>
-      <c r="G49" s="14" t="n"/>
+      <c r="G49" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
@@ -2868,7 +2921,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -3351,15 +3403,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B105" s="17" t="n"/>
-      <c r="C105" s="14" t="n"/>
-      <c r="D105" s="27" t="n"/>
+      <c r="B105" s="17" t="n">
+        <v>46084</v>
+      </c>
+      <c r="C105" s="14" t="inlineStr">
+        <is>
+          <t>Le Pain Quotidien</t>
+        </is>
+      </c>
+      <c r="D105" s="27" t="n">
+        <v>1344</v>
+      </c>
       <c r="E105" s="28" t="n"/>
       <c r="F105" s="15">
         <f>IF(OR(D105&lt;&gt;"",E105&lt;&gt;""),IF(D105="",0,D105)+IF(E105="",0,E105),"")</f>
         <v/>
       </c>
-      <c r="G105" s="14" t="n"/>
+      <c r="G105" s="14" t="inlineStr">
+        <is>
+          <t>MP · panadería</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
@@ -10518,7 +10582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12166,6 +12230,39 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="25" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Agip ABL GCBA</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="n">
+        <v>88141</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ceil desde $88.140,38</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Load mid-February Mercado Pago activity for CIUDAD.
Add almacén, transport, and Susana cleaning; keep pharmacy/clinic and transfers in catalog.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -947,7 +946,7 @@
         <v>650122</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>515550</v>
+        <v>727278</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>872390</v>
@@ -1328,7 +1327,7 @@
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>9950</v>
+        <v>30976</v>
       </c>
       <c r="F18" s="26" t="n">
         <v>107090</v>
@@ -2207,6 +2206,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -2325,15 +2325,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B50" s="17" t="n"/>
-      <c r="C50" s="14" t="n"/>
-      <c r="D50" s="27" t="n"/>
+      <c r="B50" s="17" t="n">
+        <v>46077</v>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering</t>
+        </is>
+      </c>
+      <c r="D50" s="27" t="n">
+        <v>13500</v>
+      </c>
       <c r="E50" s="28" t="n"/>
       <c r="F50" s="15">
         <f>IF(OR(D50&lt;&gt;"",E50&lt;&gt;""),IF(D50="",0,D50)+IF(E50="",0,E50),"")</f>
         <v/>
       </c>
-      <c r="G50" s="14" t="n"/>
+      <c r="G50" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
@@ -2341,15 +2353,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B51" s="17" t="n"/>
-      <c r="C51" s="14" t="n"/>
-      <c r="D51" s="27" t="n"/>
+      <c r="B51" s="17" t="n">
+        <v>46075</v>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>Havanna</t>
+        </is>
+      </c>
+      <c r="D51" s="27" t="n">
+        <v>9600</v>
+      </c>
       <c r="E51" s="28" t="n"/>
       <c r="F51" s="15">
         <f>IF(OR(D51&lt;&gt;"",E51&lt;&gt;""),IF(D51="",0,D51)+IF(E51="",0,E51),"")</f>
         <v/>
       </c>
-      <c r="G51" s="14" t="n"/>
+      <c r="G51" s="14" t="inlineStr">
+        <is>
+          <t>MP · Havanna</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
@@ -2357,15 +2381,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B52" s="17" t="n"/>
-      <c r="C52" s="14" t="n"/>
-      <c r="D52" s="27" t="n"/>
+      <c r="B52" s="17" t="n">
+        <v>46073</v>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Havanna (2)</t>
+        </is>
+      </c>
+      <c r="D52" s="27" t="n">
+        <v>9600</v>
+      </c>
       <c r="E52" s="28" t="n"/>
       <c r="F52" s="15">
         <f>IF(OR(D52&lt;&gt;"",E52&lt;&gt;""),IF(D52="",0,D52)+IF(E52="",0,E52),"")</f>
         <v/>
       </c>
-      <c r="G52" s="14" t="n"/>
+      <c r="G52" s="14" t="inlineStr">
+        <is>
+          <t>MP · Havanna</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
@@ -2373,15 +2409,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B53" s="17" t="n"/>
-      <c r="C53" s="14" t="n"/>
-      <c r="D53" s="27" t="n"/>
+      <c r="B53" s="17" t="n">
+        <v>46071</v>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Día</t>
+        </is>
+      </c>
+      <c r="D53" s="27" t="n">
+        <v>37335</v>
+      </c>
       <c r="E53" s="28" t="n"/>
       <c r="F53" s="15">
         <f>IF(OR(D53&lt;&gt;"",E53&lt;&gt;""),IF(D53="",0,D53)+IF(E53="",0,E53),"")</f>
         <v/>
       </c>
-      <c r="G53" s="14" t="n"/>
+      <c r="G53" s="14" t="inlineStr">
+        <is>
+          <t>MP · Día</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
@@ -2389,15 +2437,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B54" s="17" t="n"/>
-      <c r="C54" s="14" t="n"/>
-      <c r="D54" s="27" t="n"/>
+      <c r="B54" s="17" t="n">
+        <v>46071</v>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering</t>
+        </is>
+      </c>
+      <c r="D54" s="27" t="n">
+        <v>2703</v>
+      </c>
       <c r="E54" s="28" t="n"/>
       <c r="F54" s="15">
         <f>IF(OR(D54&lt;&gt;"",E54&lt;&gt;""),IF(D54="",0,D54)+IF(E54="",0,E54),"")</f>
         <v/>
       </c>
-      <c r="G54" s="14" t="n"/>
+      <c r="G54" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load early-mid February Mercado Pago activity for CIUDAD.
Add almacén, Cabify/Didi transport, ABL, and Sodastream; exclude refunds and own transfers.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -908,7 +909,9 @@
         </is>
       </c>
       <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
+      <c r="E9" s="5" t="n">
+        <v>83757</v>
+      </c>
       <c r="F9" s="5" t="n">
         <v>88141</v>
       </c>
@@ -1228,7 +1231,9 @@
         </is>
       </c>
       <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
+      <c r="E15" s="5" t="n">
+        <v>53037</v>
+      </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="n"/>
@@ -1327,7 +1332,7 @@
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>30976</v>
+        <v>66906</v>
       </c>
       <c r="F18" s="26" t="n">
         <v>107090</v>
@@ -2465,15 +2470,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B55" s="17" t="n"/>
-      <c r="C55" s="14" t="n"/>
-      <c r="D55" s="27" t="n"/>
+      <c r="B55" s="17" t="n">
+        <v>46067</v>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Día</t>
+        </is>
+      </c>
+      <c r="D55" s="27" t="n">
+        <v>5622</v>
+      </c>
       <c r="E55" s="28" t="n"/>
       <c r="F55" s="15">
         <f>IF(OR(D55&lt;&gt;"",E55&lt;&gt;""),IF(D55="",0,D55)+IF(E55="",0,E55),"")</f>
         <v/>
       </c>
-      <c r="G55" s="14" t="n"/>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>MP · Día</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
@@ -2481,15 +2498,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B56" s="17" t="n"/>
-      <c r="C56" s="14" t="n"/>
-      <c r="D56" s="27" t="n"/>
+      <c r="B56" s="17" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Feed</t>
+        </is>
+      </c>
+      <c r="D56" s="27" t="n">
+        <v>645</v>
+      </c>
       <c r="E56" s="28" t="n"/>
       <c r="F56" s="15">
         <f>IF(OR(D56&lt;&gt;"",E56&lt;&gt;""),IF(D56="",0,D56)+IF(E56="",0,E56),"")</f>
         <v/>
       </c>
-      <c r="G56" s="14" t="n"/>
+      <c r="G56" s="14" t="inlineStr">
+        <is>
+          <t>MP · comida</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
@@ -2497,15 +2526,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B57" s="17" t="n"/>
-      <c r="C57" s="14" t="n"/>
-      <c r="D57" s="27" t="n"/>
+      <c r="B57" s="17" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering</t>
+        </is>
+      </c>
+      <c r="D57" s="27" t="n">
+        <v>2940</v>
+      </c>
       <c r="E57" s="28" t="n"/>
       <c r="F57" s="15">
         <f>IF(OR(D57&lt;&gt;"",E57&lt;&gt;""),IF(D57="",0,D57)+IF(E57="",0,E57),"")</f>
         <v/>
       </c>
-      <c r="G57" s="14" t="n"/>
+      <c r="G57" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
@@ -2513,15 +2554,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B58" s="17" t="n"/>
-      <c r="C58" s="14" t="n"/>
-      <c r="D58" s="27" t="n"/>
+      <c r="B58" s="17" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (2)</t>
+        </is>
+      </c>
+      <c r="D58" s="27" t="n">
+        <v>1770</v>
+      </c>
       <c r="E58" s="28" t="n"/>
       <c r="F58" s="15">
         <f>IF(OR(D58&lt;&gt;"",E58&lt;&gt;""),IF(D58="",0,D58)+IF(E58="",0,E58),"")</f>
         <v/>
       </c>
-      <c r="G58" s="14" t="n"/>
+      <c r="G58" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
@@ -10642,7 +10695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12323,6 +12376,39 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="25" t="n">
+        <v>46066</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Agip ABL GCBA</t>
+        </is>
+      </c>
+      <c r="D53" s="26" t="n">
+        <v>83757</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ceil desde $83.756,62</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Load early February Mercado Pago activity for CIUDAD.
Add Carrefour/Open 25 almacén, Cabify/Didi transport, and Susana cleaning; exclude own USD and loan payments.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -949,7 +948,7 @@
         <v>650122</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>727278</v>
+        <v>853298</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>872390</v>
@@ -1332,7 +1331,7 @@
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>66906</v>
+        <v>93624</v>
       </c>
       <c r="F18" s="26" t="n">
         <v>107090</v>
@@ -2582,15 +2581,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B59" s="17" t="n"/>
-      <c r="C59" s="14" t="n"/>
-      <c r="D59" s="27" t="n"/>
+      <c r="B59" s="17" t="n">
+        <v>46061</v>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>Carrefour Ecommerce</t>
+        </is>
+      </c>
+      <c r="D59" s="27" t="n">
+        <v>21990</v>
+      </c>
       <c r="E59" s="28" t="n"/>
       <c r="F59" s="15">
         <f>IF(OR(D59&lt;&gt;"",E59&lt;&gt;""),IF(D59="",0,D59)+IF(E59="",0,E59),"")</f>
         <v/>
       </c>
-      <c r="G59" s="14" t="n"/>
+      <c r="G59" s="14" t="inlineStr">
+        <is>
+          <t>MP · Carrefour</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
@@ -2598,15 +2609,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B60" s="17" t="n"/>
-      <c r="C60" s="14" t="n"/>
-      <c r="D60" s="27" t="n"/>
+      <c r="B60" s="17" t="n">
+        <v>46060</v>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>Open 25</t>
+        </is>
+      </c>
+      <c r="D60" s="27" t="n">
+        <v>1170</v>
+      </c>
       <c r="E60" s="28" t="n"/>
       <c r="F60" s="15">
         <f>IF(OR(D60&lt;&gt;"",E60&lt;&gt;""),IF(D60="",0,D60)+IF(E60="",0,E60),"")</f>
         <v/>
       </c>
-      <c r="G60" s="14" t="n"/>
+      <c r="G60" s="14" t="inlineStr">
+        <is>
+          <t>MP · Open 25</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
@@ -2614,15 +2637,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B61" s="17" t="n"/>
-      <c r="C61" s="14" t="n"/>
-      <c r="D61" s="27" t="n"/>
+      <c r="B61" s="17" t="n">
+        <v>46059</v>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>Carrefour Ecommerce (2)</t>
+        </is>
+      </c>
+      <c r="D61" s="27" t="n">
+        <v>22768</v>
+      </c>
       <c r="E61" s="28" t="n"/>
       <c r="F61" s="15">
         <f>IF(OR(D61&lt;&gt;"",E61&lt;&gt;""),IF(D61="",0,D61)+IF(E61="",0,E61),"")</f>
         <v/>
       </c>
-      <c r="G61" s="14" t="n"/>
+      <c r="G61" s="14" t="inlineStr">
+        <is>
+          <t>MP · Carrefour</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
@@ -2630,15 +2665,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B62" s="17" t="n"/>
-      <c r="C62" s="14" t="n"/>
-      <c r="D62" s="27" t="n"/>
+      <c r="B62" s="17" t="n">
+        <v>46058</v>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Feed (5/2)</t>
+        </is>
+      </c>
+      <c r="D62" s="27" t="n">
+        <v>645</v>
+      </c>
       <c r="E62" s="28" t="n"/>
       <c r="F62" s="15">
         <f>IF(OR(D62&lt;&gt;"",E62&lt;&gt;""),IF(D62="",0,D62)+IF(E62="",0,E62),"")</f>
         <v/>
       </c>
-      <c r="G62" s="14" t="n"/>
+      <c r="G62" s="14" t="inlineStr">
+        <is>
+          <t>MP · comida</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
@@ -2646,15 +2693,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B63" s="17" t="n"/>
-      <c r="C63" s="14" t="n"/>
-      <c r="D63" s="27" t="n"/>
+      <c r="B63" s="17" t="n">
+        <v>46058</v>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (5/2)</t>
+        </is>
+      </c>
+      <c r="D63" s="27" t="n">
+        <v>2940</v>
+      </c>
       <c r="E63" s="28" t="n"/>
       <c r="F63" s="15">
         <f>IF(OR(D63&lt;&gt;"",E63&lt;&gt;""),IF(D63="",0,D63)+IF(E63="",0,E63),"")</f>
         <v/>
       </c>
-      <c r="G63" s="14" t="n"/>
+      <c r="G63" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load early February and late January Mercado Pago for CIUDAD.
Add PedidosYa/Feed almacén, Shell fuel, transport, and Susana cleaning; exclude own transfers.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -948,7 +948,7 @@
         <v>650122</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>853298</v>
+        <v>1020100</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>872390</v>
@@ -1330,8 +1330,11 @@
           <t>Cabify / Uber / Didi</t>
         </is>
       </c>
+      <c r="D18" s="26" t="n">
+        <v>12570</v>
+      </c>
       <c r="E18" s="26" t="n">
-        <v>93624</v>
+        <v>115793</v>
       </c>
       <c r="F18" s="26" t="n">
         <v>107090</v>
@@ -1550,15 +1553,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="27" t="n"/>
+      <c r="B4" s="17" t="n">
+        <v>46053</v>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="n">
+        <v>985</v>
+      </c>
       <c r="E4" s="28" t="n"/>
       <c r="F4" s="15">
         <f>IF(OR(D4&lt;&gt;"",E4&lt;&gt;""),IF(D4="",0,D4)+IF(E4="",0,E4),"")</f>
         <v/>
       </c>
-      <c r="G4" s="14" t="n"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -1566,15 +1581,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="27" t="n"/>
+      <c r="B5" s="17" t="n">
+        <v>46053</v>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell (2)</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>831</v>
+      </c>
       <c r="E5" s="28" t="n"/>
       <c r="F5" s="15">
         <f>IF(OR(D5&lt;&gt;"",E5&lt;&gt;""),IF(D5="",0,D5)+IF(E5="",0,E5),"")</f>
         <v/>
       </c>
-      <c r="G5" s="14" t="n"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -2721,15 +2748,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B64" s="17" t="n"/>
-      <c r="C64" s="14" t="n"/>
-      <c r="D64" s="27" t="n"/>
+      <c r="B64" s="17" t="n">
+        <v>46056</v>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>Feed (3/2)</t>
+        </is>
+      </c>
+      <c r="D64" s="27" t="n">
+        <v>645</v>
+      </c>
       <c r="E64" s="28" t="n"/>
       <c r="F64" s="15">
         <f>IF(OR(D64&lt;&gt;"",E64&lt;&gt;""),IF(D64="",0,D64)+IF(E64="",0,E64),"")</f>
         <v/>
       </c>
-      <c r="G64" s="14" t="n"/>
+      <c r="G64" s="14" t="inlineStr">
+        <is>
+          <t>MP · comida</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
@@ -2737,15 +2776,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B65" s="17" t="n"/>
-      <c r="C65" s="14" t="n"/>
-      <c r="D65" s="27" t="n"/>
+      <c r="B65" s="17" t="n">
+        <v>46056</v>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (3/2)</t>
+        </is>
+      </c>
+      <c r="D65" s="27" t="n">
+        <v>3585</v>
+      </c>
       <c r="E65" s="28" t="n"/>
       <c r="F65" s="15">
         <f>IF(OR(D65&lt;&gt;"",E65&lt;&gt;""),IF(D65="",0,D65)+IF(E65="",0,E65),"")</f>
         <v/>
       </c>
-      <c r="G65" s="14" t="n"/>
+      <c r="G65" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
@@ -2753,15 +2804,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B66" s="17" t="n"/>
-      <c r="C66" s="14" t="n"/>
-      <c r="D66" s="27" t="n"/>
+      <c r="B66" s="17" t="n">
+        <v>46054</v>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Propina</t>
+        </is>
+      </c>
+      <c r="D66" s="27" t="n">
+        <v>750</v>
+      </c>
       <c r="E66" s="28" t="n"/>
       <c r="F66" s="15">
         <f>IF(OR(D66&lt;&gt;"",E66&lt;&gt;""),IF(D66="",0,D66)+IF(E66="",0,E66),"")</f>
         <v/>
       </c>
-      <c r="G66" s="14" t="n"/>
+      <c r="G66" s="14" t="inlineStr">
+        <is>
+          <t>MP · propina</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
@@ -2769,15 +2832,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B67" s="17" t="n"/>
-      <c r="C67" s="14" t="n"/>
-      <c r="D67" s="27" t="n"/>
+      <c r="B67" s="17" t="n">
+        <v>46054</v>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa</t>
+        </is>
+      </c>
+      <c r="D67" s="27" t="n">
+        <v>1499</v>
+      </c>
       <c r="E67" s="28" t="n"/>
       <c r="F67" s="15">
         <f>IF(OR(D67&lt;&gt;"",E67&lt;&gt;""),IF(D67="",0,D67)+IF(E67="",0,E67),"")</f>
         <v/>
       </c>
-      <c r="G67" s="14" t="n"/>
+      <c r="G67" s="14" t="inlineStr">
+        <is>
+          <t>MP · PedidosYa</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
@@ -2785,15 +2860,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B68" s="17" t="n"/>
-      <c r="C68" s="14" t="n"/>
-      <c r="D68" s="27" t="n"/>
+      <c r="B68" s="17" t="n">
+        <v>46054</v>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Market</t>
+        </is>
+      </c>
+      <c r="D68" s="27" t="n">
+        <v>118132</v>
+      </c>
       <c r="E68" s="28" t="n"/>
       <c r="F68" s="15">
         <f>IF(OR(D68&lt;&gt;"",E68&lt;&gt;""),IF(D68="",0,D68)+IF(E68="",0,E68),"")</f>
         <v/>
       </c>
-      <c r="G68" s="14" t="n"/>
+      <c r="G68" s="14" t="inlineStr">
+        <is>
+          <t>MP · Market</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load late January Mercado Pago activity for CIUDAD.
Add almacén and Didi transport, bump Susana cleaning, and keep Mercado Libre transfers pending.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>650122</v>
+        <v>815717</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>1020100</v>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="D18" s="26" t="n">
-        <v>12570</v>
+        <v>27564</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>115793</v>
@@ -1609,15 +1609,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="27" t="n"/>
+      <c r="B6" s="17" t="n">
+        <v>46051</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Feed</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>2150</v>
+      </c>
       <c r="E6" s="28" t="n"/>
       <c r="F6" s="15">
         <f>IF(OR(D6&lt;&gt;"",E6&lt;&gt;""),IF(D6="",0,D6)+IF(E6="",0,E6),"")</f>
         <v/>
       </c>
-      <c r="G6" s="14" t="n"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>MP · comida</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
@@ -1625,15 +1637,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="27" t="n"/>
+      <c r="B7" s="17" t="n">
+        <v>46051</v>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>9800</v>
+      </c>
       <c r="E7" s="28" t="n"/>
       <c r="F7" s="15">
         <f>IF(OR(D7&lt;&gt;"",E7&lt;&gt;""),IF(D7="",0,D7)+IF(E7="",0,E7),"")</f>
         <v/>
       </c>
-      <c r="G7" s="14" t="n"/>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
@@ -1641,15 +1665,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="27" t="n"/>
+      <c r="B8" s="17" t="n">
+        <v>46049</v>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Propina</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>750</v>
+      </c>
       <c r="E8" s="28" t="n"/>
       <c r="F8" s="15">
         <f>IF(OR(D8&lt;&gt;"",E8&lt;&gt;""),IF(D8="",0,D8)+IF(E8="",0,E8),"")</f>
         <v/>
       </c>
-      <c r="G8" s="14" t="n"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>MP · propina</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
@@ -1657,15 +1693,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="27" t="n"/>
+      <c r="B9" s="17" t="n">
+        <v>46049</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Market</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>35404</v>
+      </c>
       <c r="E9" s="28" t="n"/>
       <c r="F9" s="15">
         <f>IF(OR(D9&lt;&gt;"",E9&lt;&gt;""),IF(D9="",0,D9)+IF(E9="",0,E9),"")</f>
         <v/>
       </c>
-      <c r="G9" s="14" t="n"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>MP · Market</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1673,15 +1721,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="27" t="n"/>
+      <c r="B10" s="17" t="n">
+        <v>46049</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (27/1)</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="n">
+        <v>19550</v>
+      </c>
       <c r="E10" s="28" t="n"/>
       <c r="F10" s="15">
         <f>IF(OR(D10&lt;&gt;"",E10&lt;&gt;""),IF(D10="",0,D10)+IF(E10="",0,E10),"")</f>
         <v/>
       </c>
-      <c r="G10" s="14" t="n"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -1689,15 +1749,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="27" t="n"/>
+      <c r="B11" s="17" t="n">
+        <v>46046</v>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Oporto Almacen</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>37767</v>
+      </c>
       <c r="E11" s="28" t="n"/>
       <c r="F11" s="15">
         <f>IF(OR(D11&lt;&gt;"",E11&lt;&gt;""),IF(D11="",0,D11)+IF(E11="",0,E11),"")</f>
         <v/>
       </c>
-      <c r="G11" s="14" t="n"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>MP · almacén</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1705,15 +1777,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="27" t="n"/>
+      <c r="B12" s="17" t="n">
+        <v>46046</v>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Bee Coffee</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="n">
+        <v>10500</v>
+      </c>
       <c r="E12" s="28" t="n"/>
       <c r="F12" s="15">
         <f>IF(OR(D12&lt;&gt;"",E12&lt;&gt;""),IF(D12="",0,D12)+IF(E12="",0,E12),"")</f>
         <v/>
       </c>
-      <c r="G12" s="14" t="n"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>MP · café</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
@@ -1721,15 +1805,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="27" t="n"/>
+      <c r="B13" s="17" t="n">
+        <v>46044</v>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Open 25</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>2100</v>
+      </c>
       <c r="E13" s="28" t="n"/>
       <c r="F13" s="15">
         <f>IF(OR(D13&lt;&gt;"",E13&lt;&gt;""),IF(D13="",0,D13)+IF(E13="",0,E13),"")</f>
         <v/>
       </c>
-      <c r="G13" s="14" t="n"/>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>MP · Open 25</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
@@ -1737,15 +1833,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="27" t="n"/>
+      <c r="B14" s="17" t="n">
+        <v>46044</v>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (22/1)</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="n">
+        <v>11950</v>
+      </c>
       <c r="E14" s="28" t="n"/>
       <c r="F14" s="15">
         <f>IF(OR(D14&lt;&gt;"",E14&lt;&gt;""),IF(D14="",0,D14)+IF(E14="",0,E14),"")</f>
         <v/>
       </c>
-      <c r="G14" s="14" t="n"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
@@ -2237,7 +2345,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Load mid-January Mercado Pago activity for CIUDAD.
Add Copetin/Carrefour almacén and Didi transport, bump Susana cleaning, and exclude own transfers and card statements.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>815717</v>
+        <v>980619</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>1020100</v>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="D18" s="26" t="n">
-        <v>27564</v>
+        <v>45800</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>115793</v>
@@ -1861,15 +1861,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="27" t="n"/>
+      <c r="B15" s="17" t="n">
+        <v>46042</v>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (20/1)</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>3585</v>
+      </c>
       <c r="E15" s="28" t="n"/>
       <c r="F15" s="15">
         <f>IF(OR(D15&lt;&gt;"",E15&lt;&gt;""),IF(D15="",0,D15)+IF(E15="",0,E15),"")</f>
         <v/>
       </c>
-      <c r="G15" s="14" t="n"/>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -1877,15 +1889,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="27" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46041</v>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (19/1)</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="n">
+        <v>3585</v>
+      </c>
       <c r="E16" s="28" t="n"/>
       <c r="F16" s="15">
         <f>IF(OR(D16&lt;&gt;"",E16&lt;&gt;""),IF(D16="",0,D16)+IF(E16="",0,E16),"")</f>
         <v/>
       </c>
-      <c r="G16" s="14" t="n"/>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
@@ -1893,15 +1917,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="27" t="n"/>
+      <c r="B17" s="17" t="n">
+        <v>46040</v>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Carrefour</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>4089</v>
+      </c>
       <c r="E17" s="28" t="n"/>
       <c r="F17" s="15">
         <f>IF(OR(D17&lt;&gt;"",E17&lt;&gt;""),IF(D17="",0,D17)+IF(E17="",0,E17),"")</f>
         <v/>
       </c>
-      <c r="G17" s="14" t="n"/>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>MP · Carrefour</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
@@ -1909,15 +1945,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="27" t="n"/>
+      <c r="B18" s="17" t="n">
+        <v>46035</v>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (13/1)</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="n">
+        <v>2940</v>
+      </c>
       <c r="E18" s="28" t="n"/>
       <c r="F18" s="15">
         <f>IF(OR(D18&lt;&gt;"",E18&lt;&gt;""),IF(D18="",0,D18)+IF(E18="",0,E18),"")</f>
         <v/>
       </c>
-      <c r="G18" s="14" t="n"/>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load early January Mercado Pago activity for CIUDAD.
Add Havanna and PedidosYa (net of partial refund), bump Susana cleaning, and exclude incomes and own transfers.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>980619</v>
+        <v>1146921</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>1020100</v>
@@ -1973,15 +1973,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="27" t="n"/>
+      <c r="B19" s="17" t="n">
+        <v>46033</v>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Havanna</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="n">
+        <v>22100</v>
+      </c>
       <c r="E19" s="28" t="n"/>
       <c r="F19" s="15">
         <f>IF(OR(D19&lt;&gt;"",E19&lt;&gt;""),IF(D19="",0,D19)+IF(E19="",0,E19),"")</f>
         <v/>
       </c>
-      <c r="G19" s="14" t="n"/>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>MP · Havanna</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
@@ -1989,15 +2001,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="27" t="n"/>
+      <c r="B20" s="17" t="n">
+        <v>46032</v>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Propina</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="n">
+        <v>1000</v>
+      </c>
       <c r="E20" s="28" t="n"/>
       <c r="F20" s="15">
         <f>IF(OR(D20&lt;&gt;"",E20&lt;&gt;""),IF(D20="",0,D20)+IF(E20="",0,E20),"")</f>
         <v/>
       </c>
-      <c r="G20" s="14" t="n"/>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>MP · propina</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
@@ -2005,15 +2029,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="27" t="n"/>
+      <c r="B21" s="17" t="n">
+        <v>46032</v>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa (neto)</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="n">
+        <v>51455</v>
+      </c>
       <c r="E21" s="28" t="n"/>
       <c r="F21" s="15">
         <f>IF(OR(D21&lt;&gt;"",E21&lt;&gt;""),IF(D21="",0,D21)+IF(E21="",0,E21),"")</f>
         <v/>
       </c>
-      <c r="G21" s="14" t="n"/>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>MP · neto tras devolución parcial</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
@@ -2021,15 +2057,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B22" s="17" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="27" t="n"/>
+      <c r="B22" s="17" t="n">
+        <v>46030</v>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>PedidosYa Propina (8/1)</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="n">
+        <v>750</v>
+      </c>
       <c r="E22" s="28" t="n"/>
       <c r="F22" s="15">
         <f>IF(OR(D22&lt;&gt;"",E22&lt;&gt;""),IF(D22="",0,D22)+IF(E22="",0,E22),"")</f>
         <v/>
       </c>
-      <c r="G22" s="14" t="n"/>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>MP · propina</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load early January Mercado Pago charges for CIUDAD.
Add almacén and Shell fuel, set January ABL from Agip, bump Susana cleaning, and keep large pending purchases out of totals.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -907,7 +908,9 @@
           <t>ABL</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n"/>
+      <c r="D9" s="5" t="n">
+        <v>12435</v>
+      </c>
       <c r="E9" s="5" t="n">
         <v>83757</v>
       </c>
@@ -945,7 +948,7 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>1146921</v>
+        <v>1300244</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>1020100</v>
@@ -2085,15 +2088,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="27" t="n"/>
+      <c r="B23" s="17" t="n">
+        <v>46030</v>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (8/1)</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="n">
+        <v>3585</v>
+      </c>
       <c r="E23" s="28" t="n"/>
       <c r="F23" s="15">
         <f>IF(OR(D23&lt;&gt;"",E23&lt;&gt;""),IF(D23="",0,D23)+IF(E23="",0,E23),"")</f>
         <v/>
       </c>
-      <c r="G23" s="14" t="n"/>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
@@ -2101,15 +2116,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="27" t="n"/>
+      <c r="B24" s="17" t="n">
+        <v>46028</v>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Copetin Catering (6/1)</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="n">
+        <v>645</v>
+      </c>
       <c r="E24" s="28" t="n"/>
       <c r="F24" s="15">
         <f>IF(OR(D24&lt;&gt;"",E24&lt;&gt;""),IF(D24="",0,D24)+IF(E24="",0,E24),"")</f>
         <v/>
       </c>
-      <c r="G24" s="14" t="n"/>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>MP · catering</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
@@ -2117,15 +2144,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B25" s="17" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="27" t="n"/>
+      <c r="B25" s="17" t="n">
+        <v>46027</v>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell (5/1)</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="n">
+        <v>197</v>
+      </c>
       <c r="E25" s="28" t="n"/>
       <c r="F25" s="15">
         <f>IF(OR(D25&lt;&gt;"",E25&lt;&gt;""),IF(D25="",0,D25)+IF(E25="",0,E25),"")</f>
         <v/>
       </c>
-      <c r="G25" s="14" t="n"/>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
@@ -2133,15 +2172,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B26" s="17" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="27" t="n"/>
+      <c r="B26" s="17" t="n">
+        <v>46027</v>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Combustible — Shell (5/1b)</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="n">
+        <v>46</v>
+      </c>
       <c r="E26" s="28" t="n"/>
       <c r="F26" s="15">
         <f>IF(OR(D26&lt;&gt;"",E26&lt;&gt;""),IF(D26="",0,D26)+IF(E26="",0,E26),"")</f>
         <v/>
       </c>
-      <c r="G26" s="14" t="n"/>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>MP · Shell</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
@@ -2149,15 +2200,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B27" s="17" t="n"/>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="27" t="n"/>
+      <c r="B27" s="17" t="n">
+        <v>46027</v>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Día Online</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="n">
+        <v>15092</v>
+      </c>
       <c r="E27" s="28" t="n"/>
       <c r="F27" s="15">
         <f>IF(OR(D27&lt;&gt;"",E27&lt;&gt;""),IF(D27="",0,D27)+IF(E27="",0,E27),"")</f>
         <v/>
       </c>
-      <c r="G27" s="14" t="n"/>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>MP · Día Online</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
@@ -2165,15 +2228,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B28" s="17" t="n"/>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="27" t="n"/>
+      <c r="B28" s="17" t="n">
+        <v>46025</v>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Día</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="n">
+        <v>3624</v>
+      </c>
       <c r="E28" s="28" t="n"/>
       <c r="F28" s="15">
         <f>IF(OR(D28&lt;&gt;"",E28&lt;&gt;""),IF(D28="",0,D28)+IF(E28="",0,E28),"")</f>
         <v/>
       </c>
-      <c r="G28" s="14" t="n"/>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>MP · Día</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
@@ -11044,7 +11119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12758,6 +12833,39 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="25" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Agip</t>
+        </is>
+      </c>
+      <c r="D54" s="26" t="n">
+        <v>12435</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>ceil desde $12.434,16 — confirmar si es ABL</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Load 2 Jan 2026 Mercado Pago almacén for CIUDAD.
Catalog December 2025 activity without writing it into the 2026 workbook months.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -2256,15 +2255,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B29" s="17" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="27" t="n"/>
+      <c r="B29" s="17" t="n">
+        <v>46024</v>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Día (2/1)</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="n">
+        <v>17603</v>
+      </c>
       <c r="E29" s="28" t="n"/>
       <c r="F29" s="15">
         <f>IF(OR(D29&lt;&gt;"",E29&lt;&gt;""),IF(D29="",0,D29)+IF(E29="",0,E29),"")</f>
         <v/>
       </c>
-      <c r="G29" s="14" t="n"/>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>MP · Día</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
@@ -2272,15 +2283,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B30" s="17" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="27" t="n"/>
+      <c r="B30" s="17" t="n">
+        <v>46024</v>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Carrefour (2/1)</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>8037</v>
+      </c>
       <c r="E30" s="28" t="n"/>
       <c r="F30" s="15">
         <f>IF(OR(D30&lt;&gt;"",E30&lt;&gt;""),IF(D30="",0,D30)+IF(E30="",0,E30),"")</f>
         <v/>
       </c>
-      <c r="G30" s="14" t="n"/>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>MP · Carrefour</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
@@ -2288,15 +2311,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B31" s="17" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="27" t="n"/>
+      <c r="B31" s="17" t="n">
+        <v>46024</v>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Supermercados Día (2/1b)</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="n">
+        <v>4005</v>
+      </c>
       <c r="E31" s="28" t="n"/>
       <c r="F31" s="15">
         <f>IF(OR(D31&lt;&gt;"",E31&lt;&gt;""),IF(D31="",0,D31)+IF(E31="",0,E31),"")</f>
         <v/>
       </c>
-      <c r="G31" s="14" t="n"/>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>MP · Día</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Tag PedidosYa lines as supermarket or food in comments.
Distinguish Market vs restaurant/empanada (and tips) in the catalog, Almacen Detalle, and CIUDAD rules.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1486,7 +1486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:G599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>MP · propina</t>
+          <t>PEDIDOS YA · SUPERMERCADO · propina</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>MP · Market</t>
+          <t>PEDIDOS YA · SUPERMERCADO</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>MP · propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>MP · neto tras devolución parcial</t>
+          <t>PEDIDOS YA · COMIDA · neto</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>MP · propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -2551,6 +2551,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3135,7 +3136,7 @@
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
-          <t>MP · propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3164,7 @@
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
-          <t>MP · PedidosYa</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3192,7 @@
       </c>
       <c r="G68" s="14" t="inlineStr">
         <is>
-          <t>MP · Market</t>
+          <t>PEDIDOS YA · SUPERMERCADO</t>
         </is>
       </c>
     </row>
@@ -3493,6 +3494,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4375,6 +4377,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -4651,7 +4654,7 @@
       </c>
       <c r="G139" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4682,7 @@
       </c>
       <c r="G140" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -4819,7 +4822,7 @@
       </c>
       <c r="G145" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -4847,7 +4850,7 @@
       </c>
       <c r="G146" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -5269,6 +5272,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -5377,7 +5381,7 @@
       </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -5405,7 +5409,7 @@
       </c>
       <c r="G176" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5493,7 @@
       </c>
       <c r="G179" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -5517,7 +5521,7 @@
       </c>
       <c r="G180" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -6091,6 +6095,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -6255,7 +6260,7 @@
       </c>
       <c r="G219" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -6283,7 +6288,7 @@
       </c>
       <c r="G220" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery neto parcial</t>
+          <t>PEDIDOS YA · COMIDA · neto</t>
         </is>
       </c>
     </row>
@@ -6367,7 +6372,7 @@
       </c>
       <c r="G223" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6428,7 @@
       </c>
       <c r="G225" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -6451,7 +6456,7 @@
       </c>
       <c r="G226" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6484,7 @@
       </c>
       <c r="G227" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -6507,7 +6512,7 @@
       </c>
       <c r="G228" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -7009,6 +7014,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7143,7 +7149,7 @@
       </c>
       <c r="G261" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -7311,7 +7317,7 @@
       </c>
       <c r="G267" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery propina</t>
+          <t>PEDIDOS YA · COMIDA · propina</t>
         </is>
       </c>
     </row>
@@ -7339,7 +7345,7 @@
       </c>
       <c r="G268" s="14" t="inlineStr">
         <is>
-          <t>MP · delivery</t>
+          <t>PEDIDOS YA · COMIDA</t>
         </is>
       </c>
     </row>
@@ -7813,6 +7819,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8479,6 +8486,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9145,6 +9153,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9811,6 +9820,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10477,6 +10487,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11143,6 +11154,99 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Keep Susana Carmen Ortiz only under LIMPIEZA CASA.
Restore monthly cleaning totals from Detalle (undo double-counting) and ban Susana from Almacén.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -938,7 +938,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>LIMPIEZA</t>
+          <t>LIMPIEZA CASA</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>1300244</v>
+        <v>650122</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1020100</v>
+        <v>515550</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>872390</v>
+        <v>524479</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>501015</v>
@@ -1486,7 +1486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G599"/>
+  <dimension ref="A1:G506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2551,7 +2551,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3494,7 +3493,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4377,7 +4375,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5272,7 +5269,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6095,7 +6091,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7014,7 +7009,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7819,7 +7813,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8486,7 +8479,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9153,7 +9145,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9820,7 +9811,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10487,7 +10477,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11154,99 +11143,6 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11258,7 +11154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11332,12 +11228,12 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Limpieza Susana</t>
+          <t>LIMPIEZA CASA</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Limpieza — Enero 2026</t>
+          <t>LIMPIEZA CASA — Enero 2026</t>
         </is>
       </c>
       <c r="D4" s="15" t="n">
@@ -11460,12 +11356,12 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Limpieza Susana</t>
+          <t>LIMPIEZA CASA</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>Limpieza — Febrero 2026</t>
+          <t>LIMPIEZA CASA — Febrero 2026</t>
         </is>
       </c>
       <c r="D8" s="15" t="n">
@@ -11600,12 +11496,12 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Limpieza Susana</t>
+          <t>LIMPIEZA CASA</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Limpieza — Marzo 2026</t>
+          <t>LIMPIEZA CASA — Marzo 2026</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
@@ -11812,12 +11708,12 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Limpieza Susana</t>
+          <t>LIMPIEZA CASA</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Limpieza — Abril 2026</t>
+          <t>LIMPIEZA CASA — Abril 2026</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
@@ -11985,12 +11881,12 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Limpieza Susana</t>
+          <t>LIMPIEZA CASA</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Limpieza — Mayo 2026</t>
+          <t>LIMPIEZA CASA — Mayo 2026</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
@@ -12125,12 +12021,12 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Limpieza Susana</t>
+          <t>LIMPIEZA CASA</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Limpieza — Junio 2026</t>
+          <t>LIMPIEZA CASA — Junio 2026</t>
         </is>
       </c>
       <c r="D27" s="15" t="n">
@@ -13005,6 +12901,151 @@
         </is>
       </c>
     </row>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Dinero Retirado sheet for Mercado Pago withdrawals.
Track cash-outs separately from CIUDAD expenses with a monthly summary that does not feed the 2026 total.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -10,6 +10,7 @@
     <sheet name="2026" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Almacen Detalle" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Detalle" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dinero Retirado" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle'!$A$3:$I$51</definedName>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,8 +68,19 @@
       <b val="1"/>
       <i val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -103,6 +115,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E3F2FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E3F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -176,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -215,6 +232,10 @@
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -580,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1472,6 +1493,13 @@
       <c r="A28" t="inlineStr">
         <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
@@ -11154,7 +11182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12901,153 +12929,1209 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F142"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132 — Dinero retirado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Retiros de Mercado Pago (concepto «Dinero retirado» / efectivo). No entra en el TOTAL de gastos de la hoja 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Resumen por mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Total retirado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>SUMIF($B$23:$B$142,A6,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>SUMIF($B$23:$B$142,A7,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>SUMIF($B$23:$B$142,A8,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>SUMIF($B$23:$B$142,A9,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
+        <f>SUMIF($B$23:$B$142,A10,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B11" s="15">
+        <f>SUMIF($B$23:$B$142,A11,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>SUMIF($B$23:$B$142,A12,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B13" s="15">
+        <f>SUMIF($B$23:$B$142,A13,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>SUMIF($B$23:$B$142,A14,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>SUMIF($B$23:$B$142,A15,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>SUMIF($B$23:$B$142,A16,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>SUMIF($B$23:$B$142,A17,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL AÑO</t>
+        </is>
+      </c>
+      <c r="B18" s="33">
+        <f>SUM(B6:B17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Medio / destino</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="n"/>
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="n"/>
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="14" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="14" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n"/>
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="14" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n"/>
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="14" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n"/>
+      <c r="B28" s="14" t="n"/>
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="14" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n"/>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n"/>
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="14" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n"/>
+      <c r="B32" s="14" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n"/>
+      <c r="B33" s="14" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n"/>
+      <c r="B34" s="14" t="n"/>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="14" t="n"/>
+      <c r="F34" s="14" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n"/>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="n"/>
+      <c r="B36" s="14" t="n"/>
+      <c r="C36" s="14" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="14" t="n"/>
+      <c r="F36" s="14" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="n"/>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="n"/>
+      <c r="B38" s="14" t="n"/>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n"/>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="14" t="n"/>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="14" t="n"/>
+      <c r="F40" s="14" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n"/>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="n"/>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="14" t="n"/>
+      <c r="F43" s="14" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="14" t="n"/>
+      <c r="C44" s="14" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="14" t="n"/>
+      <c r="F44" s="14" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="n"/>
+      <c r="B46" s="14" t="n"/>
+      <c r="C46" s="14" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="14" t="n"/>
+      <c r="F46" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="14" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="n"/>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="14" t="n"/>
+      <c r="F48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n"/>
+      <c r="B49" s="14" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="14" t="n"/>
+      <c r="F49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="n"/>
+      <c r="B50" s="14" t="n"/>
+      <c r="C50" s="14" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="14" t="n"/>
+      <c r="F50" s="14" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="14" t="n"/>
+      <c r="C51" s="14" t="n"/>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="14" t="n"/>
+      <c r="F51" s="14" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="n"/>
+      <c r="B52" s="14" t="n"/>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="14" t="n"/>
+      <c r="F52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="14" t="n"/>
+      <c r="F53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="14" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="14" t="n"/>
+      <c r="F54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="14" t="n"/>
+      <c r="F55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="n"/>
+      <c r="B56" s="14" t="n"/>
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="14" t="n"/>
+      <c r="F56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="n"/>
+      <c r="B57" s="14" t="n"/>
+      <c r="C57" s="14" t="n"/>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="14" t="n"/>
+      <c r="F57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="n"/>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="14" t="n"/>
+      <c r="F58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="n"/>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="15" t="n"/>
+      <c r="E59" s="14" t="n"/>
+      <c r="F59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="n"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="14" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="14" t="n"/>
+      <c r="F60" s="14" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="n"/>
+      <c r="B61" s="14" t="n"/>
+      <c r="C61" s="14" t="n"/>
+      <c r="D61" s="15" t="n"/>
+      <c r="E61" s="14" t="n"/>
+      <c r="F61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="n"/>
+      <c r="B62" s="14" t="n"/>
+      <c r="C62" s="14" t="n"/>
+      <c r="D62" s="15" t="n"/>
+      <c r="E62" s="14" t="n"/>
+      <c r="F62" s="14" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="n"/>
+      <c r="B63" s="14" t="n"/>
+      <c r="C63" s="14" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="14" t="n"/>
+      <c r="F63" s="14" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="n"/>
+      <c r="B64" s="14" t="n"/>
+      <c r="C64" s="14" t="n"/>
+      <c r="D64" s="15" t="n"/>
+      <c r="E64" s="14" t="n"/>
+      <c r="F64" s="14" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="n"/>
+      <c r="B65" s="14" t="n"/>
+      <c r="C65" s="14" t="n"/>
+      <c r="D65" s="15" t="n"/>
+      <c r="E65" s="14" t="n"/>
+      <c r="F65" s="14" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="n"/>
+      <c r="B66" s="14" t="n"/>
+      <c r="C66" s="14" t="n"/>
+      <c r="D66" s="15" t="n"/>
+      <c r="E66" s="14" t="n"/>
+      <c r="F66" s="14" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="n"/>
+      <c r="B67" s="14" t="n"/>
+      <c r="C67" s="14" t="n"/>
+      <c r="D67" s="15" t="n"/>
+      <c r="E67" s="14" t="n"/>
+      <c r="F67" s="14" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="n"/>
+      <c r="B68" s="14" t="n"/>
+      <c r="C68" s="14" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="14" t="n"/>
+      <c r="F68" s="14" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="n"/>
+      <c r="B69" s="14" t="n"/>
+      <c r="C69" s="14" t="n"/>
+      <c r="D69" s="15" t="n"/>
+      <c r="E69" s="14" t="n"/>
+      <c r="F69" s="14" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="n"/>
+      <c r="B70" s="14" t="n"/>
+      <c r="C70" s="14" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="14" t="n"/>
+      <c r="F70" s="14" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="n"/>
+      <c r="B71" s="14" t="n"/>
+      <c r="C71" s="14" t="n"/>
+      <c r="D71" s="15" t="n"/>
+      <c r="E71" s="14" t="n"/>
+      <c r="F71" s="14" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="n"/>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="15" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="n"/>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="14" t="n"/>
+      <c r="D73" s="15" t="n"/>
+      <c r="E73" s="14" t="n"/>
+      <c r="F73" s="14" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="n"/>
+      <c r="B74" s="14" t="n"/>
+      <c r="C74" s="14" t="n"/>
+      <c r="D74" s="15" t="n"/>
+      <c r="E74" s="14" t="n"/>
+      <c r="F74" s="14" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="17" t="n"/>
+      <c r="B75" s="14" t="n"/>
+      <c r="C75" s="14" t="n"/>
+      <c r="D75" s="15" t="n"/>
+      <c r="E75" s="14" t="n"/>
+      <c r="F75" s="14" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="n"/>
+      <c r="B76" s="14" t="n"/>
+      <c r="C76" s="14" t="n"/>
+      <c r="D76" s="15" t="n"/>
+      <c r="E76" s="14" t="n"/>
+      <c r="F76" s="14" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="n"/>
+      <c r="B77" s="14" t="n"/>
+      <c r="C77" s="14" t="n"/>
+      <c r="D77" s="15" t="n"/>
+      <c r="E77" s="14" t="n"/>
+      <c r="F77" s="14" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="n"/>
+      <c r="B78" s="14" t="n"/>
+      <c r="C78" s="14" t="n"/>
+      <c r="D78" s="15" t="n"/>
+      <c r="E78" s="14" t="n"/>
+      <c r="F78" s="14" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="n"/>
+      <c r="B79" s="14" t="n"/>
+      <c r="C79" s="14" t="n"/>
+      <c r="D79" s="15" t="n"/>
+      <c r="E79" s="14" t="n"/>
+      <c r="F79" s="14" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="n"/>
+      <c r="B80" s="14" t="n"/>
+      <c r="C80" s="14" t="n"/>
+      <c r="D80" s="15" t="n"/>
+      <c r="E80" s="14" t="n"/>
+      <c r="F80" s="14" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="n"/>
+      <c r="B81" s="14" t="n"/>
+      <c r="C81" s="14" t="n"/>
+      <c r="D81" s="15" t="n"/>
+      <c r="E81" s="14" t="n"/>
+      <c r="F81" s="14" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="n"/>
+      <c r="B82" s="14" t="n"/>
+      <c r="C82" s="14" t="n"/>
+      <c r="D82" s="15" t="n"/>
+      <c r="E82" s="14" t="n"/>
+      <c r="F82" s="14" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="n"/>
+      <c r="B83" s="14" t="n"/>
+      <c r="C83" s="14" t="n"/>
+      <c r="D83" s="15" t="n"/>
+      <c r="E83" s="14" t="n"/>
+      <c r="F83" s="14" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="n"/>
+      <c r="B84" s="14" t="n"/>
+      <c r="C84" s="14" t="n"/>
+      <c r="D84" s="15" t="n"/>
+      <c r="E84" s="14" t="n"/>
+      <c r="F84" s="14" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="n"/>
+      <c r="B85" s="14" t="n"/>
+      <c r="C85" s="14" t="n"/>
+      <c r="D85" s="15" t="n"/>
+      <c r="E85" s="14" t="n"/>
+      <c r="F85" s="14" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="n"/>
+      <c r="B86" s="14" t="n"/>
+      <c r="C86" s="14" t="n"/>
+      <c r="D86" s="15" t="n"/>
+      <c r="E86" s="14" t="n"/>
+      <c r="F86" s="14" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="n"/>
+      <c r="B87" s="14" t="n"/>
+      <c r="C87" s="14" t="n"/>
+      <c r="D87" s="15" t="n"/>
+      <c r="E87" s="14" t="n"/>
+      <c r="F87" s="14" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="n"/>
+      <c r="B88" s="14" t="n"/>
+      <c r="C88" s="14" t="n"/>
+      <c r="D88" s="15" t="n"/>
+      <c r="E88" s="14" t="n"/>
+      <c r="F88" s="14" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="17" t="n"/>
+      <c r="B89" s="14" t="n"/>
+      <c r="C89" s="14" t="n"/>
+      <c r="D89" s="15" t="n"/>
+      <c r="E89" s="14" t="n"/>
+      <c r="F89" s="14" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="n"/>
+      <c r="B90" s="14" t="n"/>
+      <c r="C90" s="14" t="n"/>
+      <c r="D90" s="15" t="n"/>
+      <c r="E90" s="14" t="n"/>
+      <c r="F90" s="14" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="n"/>
+      <c r="B91" s="14" t="n"/>
+      <c r="C91" s="14" t="n"/>
+      <c r="D91" s="15" t="n"/>
+      <c r="E91" s="14" t="n"/>
+      <c r="F91" s="14" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="n"/>
+      <c r="B92" s="14" t="n"/>
+      <c r="C92" s="14" t="n"/>
+      <c r="D92" s="15" t="n"/>
+      <c r="E92" s="14" t="n"/>
+      <c r="F92" s="14" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="n"/>
+      <c r="B93" s="14" t="n"/>
+      <c r="C93" s="14" t="n"/>
+      <c r="D93" s="15" t="n"/>
+      <c r="E93" s="14" t="n"/>
+      <c r="F93" s="14" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="n"/>
+      <c r="B94" s="14" t="n"/>
+      <c r="C94" s="14" t="n"/>
+      <c r="D94" s="15" t="n"/>
+      <c r="E94" s="14" t="n"/>
+      <c r="F94" s="14" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="n"/>
+      <c r="B95" s="14" t="n"/>
+      <c r="C95" s="14" t="n"/>
+      <c r="D95" s="15" t="n"/>
+      <c r="E95" s="14" t="n"/>
+      <c r="F95" s="14" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="n"/>
+      <c r="B96" s="14" t="n"/>
+      <c r="C96" s="14" t="n"/>
+      <c r="D96" s="15" t="n"/>
+      <c r="E96" s="14" t="n"/>
+      <c r="F96" s="14" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="n"/>
+      <c r="B97" s="14" t="n"/>
+      <c r="C97" s="14" t="n"/>
+      <c r="D97" s="15" t="n"/>
+      <c r="E97" s="14" t="n"/>
+      <c r="F97" s="14" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="n"/>
+      <c r="B98" s="14" t="n"/>
+      <c r="C98" s="14" t="n"/>
+      <c r="D98" s="15" t="n"/>
+      <c r="E98" s="14" t="n"/>
+      <c r="F98" s="14" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="17" t="n"/>
+      <c r="B99" s="14" t="n"/>
+      <c r="C99" s="14" t="n"/>
+      <c r="D99" s="15" t="n"/>
+      <c r="E99" s="14" t="n"/>
+      <c r="F99" s="14" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="17" t="n"/>
+      <c r="B100" s="14" t="n"/>
+      <c r="C100" s="14" t="n"/>
+      <c r="D100" s="15" t="n"/>
+      <c r="E100" s="14" t="n"/>
+      <c r="F100" s="14" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="17" t="n"/>
+      <c r="B101" s="14" t="n"/>
+      <c r="C101" s="14" t="n"/>
+      <c r="D101" s="15" t="n"/>
+      <c r="E101" s="14" t="n"/>
+      <c r="F101" s="14" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="17" t="n"/>
+      <c r="B102" s="14" t="n"/>
+      <c r="C102" s="14" t="n"/>
+      <c r="D102" s="15" t="n"/>
+      <c r="E102" s="14" t="n"/>
+      <c r="F102" s="14" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="17" t="n"/>
+      <c r="B103" s="14" t="n"/>
+      <c r="C103" s="14" t="n"/>
+      <c r="D103" s="15" t="n"/>
+      <c r="E103" s="14" t="n"/>
+      <c r="F103" s="14" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="17" t="n"/>
+      <c r="B104" s="14" t="n"/>
+      <c r="C104" s="14" t="n"/>
+      <c r="D104" s="15" t="n"/>
+      <c r="E104" s="14" t="n"/>
+      <c r="F104" s="14" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="17" t="n"/>
+      <c r="B105" s="14" t="n"/>
+      <c r="C105" s="14" t="n"/>
+      <c r="D105" s="15" t="n"/>
+      <c r="E105" s="14" t="n"/>
+      <c r="F105" s="14" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="n"/>
+      <c r="B106" s="14" t="n"/>
+      <c r="C106" s="14" t="n"/>
+      <c r="D106" s="15" t="n"/>
+      <c r="E106" s="14" t="n"/>
+      <c r="F106" s="14" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="n"/>
+      <c r="B107" s="14" t="n"/>
+      <c r="C107" s="14" t="n"/>
+      <c r="D107" s="15" t="n"/>
+      <c r="E107" s="14" t="n"/>
+      <c r="F107" s="14" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="17" t="n"/>
+      <c r="B108" s="14" t="n"/>
+      <c r="C108" s="14" t="n"/>
+      <c r="D108" s="15" t="n"/>
+      <c r="E108" s="14" t="n"/>
+      <c r="F108" s="14" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="17" t="n"/>
+      <c r="B109" s="14" t="n"/>
+      <c r="C109" s="14" t="n"/>
+      <c r="D109" s="15" t="n"/>
+      <c r="E109" s="14" t="n"/>
+      <c r="F109" s="14" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="17" t="n"/>
+      <c r="B110" s="14" t="n"/>
+      <c r="C110" s="14" t="n"/>
+      <c r="D110" s="15" t="n"/>
+      <c r="E110" s="14" t="n"/>
+      <c r="F110" s="14" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="17" t="n"/>
+      <c r="B111" s="14" t="n"/>
+      <c r="C111" s="14" t="n"/>
+      <c r="D111" s="15" t="n"/>
+      <c r="E111" s="14" t="n"/>
+      <c r="F111" s="14" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="17" t="n"/>
+      <c r="B112" s="14" t="n"/>
+      <c r="C112" s="14" t="n"/>
+      <c r="D112" s="15" t="n"/>
+      <c r="E112" s="14" t="n"/>
+      <c r="F112" s="14" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="17" t="n"/>
+      <c r="B113" s="14" t="n"/>
+      <c r="C113" s="14" t="n"/>
+      <c r="D113" s="15" t="n"/>
+      <c r="E113" s="14" t="n"/>
+      <c r="F113" s="14" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="n"/>
+      <c r="B114" s="14" t="n"/>
+      <c r="C114" s="14" t="n"/>
+      <c r="D114" s="15" t="n"/>
+      <c r="E114" s="14" t="n"/>
+      <c r="F114" s="14" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="17" t="n"/>
+      <c r="B115" s="14" t="n"/>
+      <c r="C115" s="14" t="n"/>
+      <c r="D115" s="15" t="n"/>
+      <c r="E115" s="14" t="n"/>
+      <c r="F115" s="14" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="17" t="n"/>
+      <c r="B116" s="14" t="n"/>
+      <c r="C116" s="14" t="n"/>
+      <c r="D116" s="15" t="n"/>
+      <c r="E116" s="14" t="n"/>
+      <c r="F116" s="14" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="n"/>
+      <c r="B117" s="14" t="n"/>
+      <c r="C117" s="14" t="n"/>
+      <c r="D117" s="15" t="n"/>
+      <c r="E117" s="14" t="n"/>
+      <c r="F117" s="14" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="17" t="n"/>
+      <c r="B118" s="14" t="n"/>
+      <c r="C118" s="14" t="n"/>
+      <c r="D118" s="15" t="n"/>
+      <c r="E118" s="14" t="n"/>
+      <c r="F118" s="14" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="17" t="n"/>
+      <c r="B119" s="14" t="n"/>
+      <c r="C119" s="14" t="n"/>
+      <c r="D119" s="15" t="n"/>
+      <c r="E119" s="14" t="n"/>
+      <c r="F119" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="17" t="n"/>
+      <c r="B120" s="14" t="n"/>
+      <c r="C120" s="14" t="n"/>
+      <c r="D120" s="15" t="n"/>
+      <c r="E120" s="14" t="n"/>
+      <c r="F120" s="14" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="17" t="n"/>
+      <c r="B121" s="14" t="n"/>
+      <c r="C121" s="14" t="n"/>
+      <c r="D121" s="15" t="n"/>
+      <c r="E121" s="14" t="n"/>
+      <c r="F121" s="14" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="17" t="n"/>
+      <c r="B122" s="14" t="n"/>
+      <c r="C122" s="14" t="n"/>
+      <c r="D122" s="15" t="n"/>
+      <c r="E122" s="14" t="n"/>
+      <c r="F122" s="14" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="n"/>
+      <c r="B123" s="14" t="n"/>
+      <c r="C123" s="14" t="n"/>
+      <c r="D123" s="15" t="n"/>
+      <c r="E123" s="14" t="n"/>
+      <c r="F123" s="14" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="n"/>
+      <c r="B124" s="14" t="n"/>
+      <c r="C124" s="14" t="n"/>
+      <c r="D124" s="15" t="n"/>
+      <c r="E124" s="14" t="n"/>
+      <c r="F124" s="14" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="n"/>
+      <c r="B125" s="14" t="n"/>
+      <c r="C125" s="14" t="n"/>
+      <c r="D125" s="15" t="n"/>
+      <c r="E125" s="14" t="n"/>
+      <c r="F125" s="14" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="n"/>
+      <c r="B126" s="14" t="n"/>
+      <c r="C126" s="14" t="n"/>
+      <c r="D126" s="15" t="n"/>
+      <c r="E126" s="14" t="n"/>
+      <c r="F126" s="14" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="n"/>
+      <c r="B127" s="14" t="n"/>
+      <c r="C127" s="14" t="n"/>
+      <c r="D127" s="15" t="n"/>
+      <c r="E127" s="14" t="n"/>
+      <c r="F127" s="14" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="17" t="n"/>
+      <c r="B128" s="14" t="n"/>
+      <c r="C128" s="14" t="n"/>
+      <c r="D128" s="15" t="n"/>
+      <c r="E128" s="14" t="n"/>
+      <c r="F128" s="14" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="17" t="n"/>
+      <c r="B129" s="14" t="n"/>
+      <c r="C129" s="14" t="n"/>
+      <c r="D129" s="15" t="n"/>
+      <c r="E129" s="14" t="n"/>
+      <c r="F129" s="14" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="17" t="n"/>
+      <c r="B130" s="14" t="n"/>
+      <c r="C130" s="14" t="n"/>
+      <c r="D130" s="15" t="n"/>
+      <c r="E130" s="14" t="n"/>
+      <c r="F130" s="14" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="17" t="n"/>
+      <c r="B131" s="14" t="n"/>
+      <c r="C131" s="14" t="n"/>
+      <c r="D131" s="15" t="n"/>
+      <c r="E131" s="14" t="n"/>
+      <c r="F131" s="14" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="17" t="n"/>
+      <c r="B132" s="14" t="n"/>
+      <c r="C132" s="14" t="n"/>
+      <c r="D132" s="15" t="n"/>
+      <c r="E132" s="14" t="n"/>
+      <c r="F132" s="14" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="n"/>
+      <c r="B133" s="14" t="n"/>
+      <c r="C133" s="14" t="n"/>
+      <c r="D133" s="15" t="n"/>
+      <c r="E133" s="14" t="n"/>
+      <c r="F133" s="14" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="17" t="n"/>
+      <c r="B134" s="14" t="n"/>
+      <c r="C134" s="14" t="n"/>
+      <c r="D134" s="15" t="n"/>
+      <c r="E134" s="14" t="n"/>
+      <c r="F134" s="14" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="17" t="n"/>
+      <c r="B135" s="14" t="n"/>
+      <c r="C135" s="14" t="n"/>
+      <c r="D135" s="15" t="n"/>
+      <c r="E135" s="14" t="n"/>
+      <c r="F135" s="14" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="17" t="n"/>
+      <c r="B136" s="14" t="n"/>
+      <c r="C136" s="14" t="n"/>
+      <c r="D136" s="15" t="n"/>
+      <c r="E136" s="14" t="n"/>
+      <c r="F136" s="14" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="17" t="n"/>
+      <c r="B137" s="14" t="n"/>
+      <c r="C137" s="14" t="n"/>
+      <c r="D137" s="15" t="n"/>
+      <c r="E137" s="14" t="n"/>
+      <c r="F137" s="14" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="17" t="n"/>
+      <c r="B138" s="14" t="n"/>
+      <c r="C138" s="14" t="n"/>
+      <c r="D138" s="15" t="n"/>
+      <c r="E138" s="14" t="n"/>
+      <c r="F138" s="14" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="17" t="n"/>
+      <c r="B139" s="14" t="n"/>
+      <c r="C139" s="14" t="n"/>
+      <c r="D139" s="15" t="n"/>
+      <c r="E139" s="14" t="n"/>
+      <c r="F139" s="14" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="n"/>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="15" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="n"/>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="14" t="n"/>
+      <c r="D141" s="15" t="n"/>
+      <c r="E141" s="14" t="n"/>
+      <c r="F141" s="14" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="n"/>
+      <c r="B142" s="14" t="n"/>
+      <c r="C142" s="14" t="n"/>
+      <c r="D142" s="15" t="n"/>
+      <c r="E142" s="14" t="n"/>
+      <c r="F142" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Route pharmacy spend to FARMACIA with store name in comments.
Add a FARMACIA row on the 2026 sheet and reclassify Farmacity, Maure, and Selma from Extras.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -21,8 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -601,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1380,126 +1381,170 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="n">
+        <v>146046</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <v>124100</v>
+      </c>
+      <c r="G19" s="26" t="n">
+        <v>191500</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>85034</v>
+      </c>
+      <c r="J19" s="26" t="n">
+        <v>218500</v>
+      </c>
+      <c r="P19" s="26">
+        <f>SUM(D19:O19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="7">
-        <f>SUM(D5:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="7">
-        <f>SUM(E5:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="7">
-        <f>SUM(F5:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="7">
-        <f>SUM(G5:G18)</f>
-        <v/>
-      </c>
-      <c r="H19" s="7">
-        <f>SUM(H5:H18)</f>
-        <v/>
-      </c>
-      <c r="I19" s="7">
-        <f>SUM(I5:I18)</f>
-        <v/>
-      </c>
-      <c r="J19" s="7">
-        <f>SUM(J5:J18)</f>
-        <v/>
-      </c>
-      <c r="K19" s="7">
-        <f>SUM(K5:K18)</f>
-        <v/>
-      </c>
-      <c r="L19" s="7">
-        <f>SUM(L5:L18)</f>
-        <v/>
-      </c>
-      <c r="M19" s="7">
-        <f>SUM(M5:M18)</f>
-        <v/>
-      </c>
-      <c r="N19" s="7">
-        <f>SUM(N5:N18)</f>
-        <v/>
-      </c>
-      <c r="O19" s="7">
-        <f>SUM(O5:O18)</f>
-        <v/>
-      </c>
-      <c r="P19" s="7">
-        <f>SUM(P5:P18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="7">
+        <f>SUM(D5:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="7">
+        <f>SUM(E5:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="7">
+        <f>SUM(F5:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="7">
+        <f>SUM(G5:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="7">
+        <f>SUM(H5:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="7">
+        <f>SUM(I5:I19)</f>
+        <v/>
+      </c>
+      <c r="J20" s="7">
+        <f>SUM(J5:J19)</f>
+        <v/>
+      </c>
+      <c r="K20" s="7">
+        <f>SUM(K5:K19)</f>
+        <v/>
+      </c>
+      <c r="L20" s="7">
+        <f>SUM(L5:L19)</f>
+        <v/>
+      </c>
+      <c r="M20" s="7">
+        <f>SUM(M5:M19)</f>
+        <v/>
+      </c>
+      <c r="N20" s="7">
+        <f>SUM(N5:N19)</f>
+        <v/>
+      </c>
+      <c r="O20" s="7">
+        <f>SUM(O5:O19)</f>
+        <v/>
+      </c>
+      <c r="P20" s="7">
+        <f>SUM(P5:P19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• Expensas abril/mayo 2026: PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
         <is>
           <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>• FARMACIA: Farmacity / Farmacia Selma / Farmacia Maure — nombre de farmacia en comentario</t>
         </is>
       </c>
     </row>
@@ -11182,7 +11227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12926,6 +12971,204 @@
       <c r="I54" t="inlineStr">
         <is>
           <t>Enero</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="D55" s="26" t="n">
+        <v>29546</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacia Selma</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="25" t="n">
+        <v>46032</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="D56" s="26" t="n">
+        <v>116500</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacia Maure</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="n">
+        <v>46073</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="D57" s="26" t="n">
+        <v>124100</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacia Maure</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="25" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="D58" s="26" t="n">
+        <v>191500</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacia Maure</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="25" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="D59" s="26" t="n">
+        <v>85034</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacity</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="25" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
+      <c r="D60" s="26" t="n">
+        <v>218500</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacia Maure</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Julio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classify Florencia Londero as Chocolates CHIAZZA food.
Move the July transfer from pending into Almacén Sol with a COMIDA comment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -21,9 +21,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1477,7 +1476,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -2624,6 +2622,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3566,6 +3565,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4448,6 +4448,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5342,6 +5343,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6164,6 +6166,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7082,6 +7085,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7450,15 +7454,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B270" s="17" t="n"/>
-      <c r="C270" s="14" t="n"/>
-      <c r="D270" s="27" t="n"/>
+      <c r="B270" s="17" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C270" s="14" t="inlineStr">
+        <is>
+          <t>Chocolates CHIAZZA (Florencia Londero)</t>
+        </is>
+      </c>
+      <c r="D270" s="27" t="n">
+        <v>8000</v>
+      </c>
       <c r="E270" s="28" t="n"/>
       <c r="F270" s="15">
         <f>IF(OR(D270&lt;&gt;"",E270&lt;&gt;""),IF(D270="",0,D270)+IF(E270="",0,E270),"")</f>
         <v/>
       </c>
-      <c r="G270" s="14" t="n"/>
+      <c r="G270" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Chocolates CHIAZZA</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Route Personal pago directo to OHIGGINS TV CABLE-INTERNET.
Keep those charges out of CIUDAD and load January–July Personal totals into the OHIGGINS workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1476,6 +1476,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1543,6 +1544,13 @@
       <c r="A31" s="30" t="inlineStr">
         <is>
           <t>• FARMACIA: Farmacity / Farmacia Selma / Farmacia Maure — nombre de farmacia en comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>• Personal (Pago directo): va a OHIGGINS → TV CABLE-INTERNET — no CIUDAD</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2630,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3565,7 +3572,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4448,7 +4454,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5343,7 +5348,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6166,7 +6170,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7085,7 +7088,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -11243,7 +11245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13188,6 +13190,145 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add a separate investment tracking sheet.
Track bonds, fixed-term deposits, redemptions, and returns without affecting CIUDAD expense totals.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -11,9 +11,11 @@
     <sheet name="Almacen Detalle" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Detalle" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Dinero Retirado" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Inversión" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle'!$A$3:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Inversión'!$A$23:$J$223</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -24,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,6 +80,11 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="9">
@@ -193,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -236,6 +243,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1554,6 +1565,39 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>• Inversión: hoja "Inversión" (bonos, plazos fijos y otros; no suma al TOTAL de gastos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11245,7 +11289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13190,145 +13234,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14534,4 +14439,2841 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J223"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132 — Inversión</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Bonos, plazos fijos, fondos y otros movimientos de inversión. No suma al TOTAL de gastos de la hoja 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Resumen por mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Invertido</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Rescatado</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Rendimiento</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>Neto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A6,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C6" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A6,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A6,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>C6+D6-B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A7,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C7" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A7,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A7,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>C7+D7-B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A8,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C8" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A8,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D8" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A8,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E8" s="15">
+        <f>C8+D8-B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A9,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C9" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A9,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D9" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A9,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
+        <f>C9+D9-B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A10,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C10" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A10,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D10" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A10,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>C10+D10-B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B11" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A11,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C11" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A11,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D11" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A11,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E11" s="15">
+        <f>C11+D11-B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A12,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C12" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A12,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D12" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A12,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E12" s="15">
+        <f>C12+D12-B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B13" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A13,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C13" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A13,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D13" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A13,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E13" s="15">
+        <f>C13+D13-B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A14,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C14" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A14,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D14" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A14,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E14" s="15">
+        <f>C14+D14-B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A15,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C15" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A15,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D15" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A15,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>C15+D15-B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A16,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A16,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A16,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>C16+D16-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A17,$D$24:$D$223,"Inversión")</f>
+        <v/>
+      </c>
+      <c r="C17" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A17,$D$24:$D$223,"Rescate")</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>SUMIFS($F$24:$F$223,$B$24:$B$223,A17,$D$24:$D$223,"Rendimiento")</f>
+        <v/>
+      </c>
+      <c r="E17" s="15">
+        <f>C17+D17-B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL AÑO</t>
+        </is>
+      </c>
+      <c r="B18" s="36">
+        <f>SUM(B6:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="36">
+        <f>SUM(C6:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="36">
+        <f>SUM(D6:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="36">
+        <f>SUM(E6:E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="34" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C23" s="34" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D23" s="34" t="inlineStr">
+        <is>
+          <t>Movimiento</t>
+        </is>
+      </c>
+      <c r="E23" s="34" t="inlineStr">
+        <is>
+          <t>Instrumento / concepto</t>
+        </is>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="G23" s="34" t="inlineStr">
+        <is>
+          <t>Entidad / medio</t>
+        </is>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>Vencimiento</t>
+        </is>
+      </c>
+      <c r="I23" s="34" t="inlineStr">
+        <is>
+          <t>Tasa / rendimiento</t>
+        </is>
+      </c>
+      <c r="J23" s="34" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="n"/>
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="14" t="n"/>
+      <c r="H24" s="17" t="n"/>
+      <c r="I24" s="37" t="n"/>
+      <c r="J24" s="14" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="14" t="n"/>
+      <c r="H25" s="17" t="n"/>
+      <c r="I25" s="37" t="n"/>
+      <c r="J25" s="14" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n"/>
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="14" t="n"/>
+      <c r="H26" s="17" t="n"/>
+      <c r="I26" s="37" t="n"/>
+      <c r="J26" s="14" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n"/>
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="n"/>
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="15" t="n"/>
+      <c r="G27" s="14" t="n"/>
+      <c r="H27" s="17" t="n"/>
+      <c r="I27" s="37" t="n"/>
+      <c r="J27" s="14" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n"/>
+      <c r="B28" s="14" t="n"/>
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="14" t="n"/>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="14" t="n"/>
+      <c r="H28" s="17" t="n"/>
+      <c r="I28" s="37" t="n"/>
+      <c r="J28" s="14" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n"/>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="15" t="n"/>
+      <c r="G29" s="14" t="n"/>
+      <c r="H29" s="17" t="n"/>
+      <c r="I29" s="37" t="n"/>
+      <c r="J29" s="14" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n"/>
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="15" t="n"/>
+      <c r="G30" s="14" t="n"/>
+      <c r="H30" s="17" t="n"/>
+      <c r="I30" s="37" t="n"/>
+      <c r="J30" s="14" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="17" t="n"/>
+      <c r="I31" s="37" t="n"/>
+      <c r="J31" s="14" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n"/>
+      <c r="B32" s="14" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="17" t="n"/>
+      <c r="I32" s="37" t="n"/>
+      <c r="J32" s="14" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n"/>
+      <c r="B33" s="14" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="17" t="n"/>
+      <c r="I33" s="37" t="n"/>
+      <c r="J33" s="14" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n"/>
+      <c r="B34" s="14" t="n"/>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="14" t="n"/>
+      <c r="E34" s="14" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="14" t="n"/>
+      <c r="H34" s="17" t="n"/>
+      <c r="I34" s="37" t="n"/>
+      <c r="J34" s="14" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n"/>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="15" t="n"/>
+      <c r="G35" s="14" t="n"/>
+      <c r="H35" s="17" t="n"/>
+      <c r="I35" s="37" t="n"/>
+      <c r="J35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="n"/>
+      <c r="B36" s="14" t="n"/>
+      <c r="C36" s="14" t="n"/>
+      <c r="D36" s="14" t="n"/>
+      <c r="E36" s="14" t="n"/>
+      <c r="F36" s="15" t="n"/>
+      <c r="G36" s="14" t="n"/>
+      <c r="H36" s="17" t="n"/>
+      <c r="I36" s="37" t="n"/>
+      <c r="J36" s="14" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="n"/>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="14" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="14" t="n"/>
+      <c r="H37" s="17" t="n"/>
+      <c r="I37" s="37" t="n"/>
+      <c r="J37" s="14" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="n"/>
+      <c r="B38" s="14" t="n"/>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="14" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="15" t="n"/>
+      <c r="G38" s="14" t="n"/>
+      <c r="H38" s="17" t="n"/>
+      <c r="I38" s="37" t="n"/>
+      <c r="J38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n"/>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="15" t="n"/>
+      <c r="G39" s="14" t="n"/>
+      <c r="H39" s="17" t="n"/>
+      <c r="I39" s="37" t="n"/>
+      <c r="J39" s="14" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="14" t="n"/>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="14" t="n"/>
+      <c r="E40" s="14" t="n"/>
+      <c r="F40" s="15" t="n"/>
+      <c r="G40" s="14" t="n"/>
+      <c r="H40" s="17" t="n"/>
+      <c r="I40" s="37" t="n"/>
+      <c r="J40" s="14" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n"/>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="14" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="15" t="n"/>
+      <c r="G41" s="14" t="n"/>
+      <c r="H41" s="17" t="n"/>
+      <c r="I41" s="37" t="n"/>
+      <c r="J41" s="14" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="n"/>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="14" t="n"/>
+      <c r="H42" s="17" t="n"/>
+      <c r="I42" s="37" t="n"/>
+      <c r="J42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="14" t="n"/>
+      <c r="E43" s="14" t="n"/>
+      <c r="F43" s="15" t="n"/>
+      <c r="G43" s="14" t="n"/>
+      <c r="H43" s="17" t="n"/>
+      <c r="I43" s="37" t="n"/>
+      <c r="J43" s="14" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="14" t="n"/>
+      <c r="C44" s="14" t="n"/>
+      <c r="D44" s="14" t="n"/>
+      <c r="E44" s="14" t="n"/>
+      <c r="F44" s="15" t="n"/>
+      <c r="G44" s="14" t="n"/>
+      <c r="H44" s="17" t="n"/>
+      <c r="I44" s="37" t="n"/>
+      <c r="J44" s="14" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="14" t="n"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="15" t="n"/>
+      <c r="G45" s="14" t="n"/>
+      <c r="H45" s="17" t="n"/>
+      <c r="I45" s="37" t="n"/>
+      <c r="J45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="n"/>
+      <c r="B46" s="14" t="n"/>
+      <c r="C46" s="14" t="n"/>
+      <c r="D46" s="14" t="n"/>
+      <c r="E46" s="14" t="n"/>
+      <c r="F46" s="15" t="n"/>
+      <c r="G46" s="14" t="n"/>
+      <c r="H46" s="17" t="n"/>
+      <c r="I46" s="37" t="n"/>
+      <c r="J46" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="14" t="n"/>
+      <c r="H47" s="17" t="n"/>
+      <c r="I47" s="37" t="n"/>
+      <c r="J47" s="14" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="n"/>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="14" t="n"/>
+      <c r="E48" s="14" t="n"/>
+      <c r="F48" s="15" t="n"/>
+      <c r="G48" s="14" t="n"/>
+      <c r="H48" s="17" t="n"/>
+      <c r="I48" s="37" t="n"/>
+      <c r="J48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n"/>
+      <c r="B49" s="14" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="14" t="n"/>
+      <c r="E49" s="14" t="n"/>
+      <c r="F49" s="15" t="n"/>
+      <c r="G49" s="14" t="n"/>
+      <c r="H49" s="17" t="n"/>
+      <c r="I49" s="37" t="n"/>
+      <c r="J49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="n"/>
+      <c r="B50" s="14" t="n"/>
+      <c r="C50" s="14" t="n"/>
+      <c r="D50" s="14" t="n"/>
+      <c r="E50" s="14" t="n"/>
+      <c r="F50" s="15" t="n"/>
+      <c r="G50" s="14" t="n"/>
+      <c r="H50" s="17" t="n"/>
+      <c r="I50" s="37" t="n"/>
+      <c r="J50" s="14" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="14" t="n"/>
+      <c r="C51" s="14" t="n"/>
+      <c r="D51" s="14" t="n"/>
+      <c r="E51" s="14" t="n"/>
+      <c r="F51" s="15" t="n"/>
+      <c r="G51" s="14" t="n"/>
+      <c r="H51" s="17" t="n"/>
+      <c r="I51" s="37" t="n"/>
+      <c r="J51" s="14" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="n"/>
+      <c r="B52" s="14" t="n"/>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="14" t="n"/>
+      <c r="E52" s="14" t="n"/>
+      <c r="F52" s="15" t="n"/>
+      <c r="G52" s="14" t="n"/>
+      <c r="H52" s="17" t="n"/>
+      <c r="I52" s="37" t="n"/>
+      <c r="J52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
+      <c r="E53" s="14" t="n"/>
+      <c r="F53" s="15" t="n"/>
+      <c r="G53" s="14" t="n"/>
+      <c r="H53" s="17" t="n"/>
+      <c r="I53" s="37" t="n"/>
+      <c r="J53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="14" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="14" t="n"/>
+      <c r="E54" s="14" t="n"/>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="14" t="n"/>
+      <c r="H54" s="17" t="n"/>
+      <c r="I54" s="37" t="n"/>
+      <c r="J54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="14" t="n"/>
+      <c r="E55" s="14" t="n"/>
+      <c r="F55" s="15" t="n"/>
+      <c r="G55" s="14" t="n"/>
+      <c r="H55" s="17" t="n"/>
+      <c r="I55" s="37" t="n"/>
+      <c r="J55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="n"/>
+      <c r="B56" s="14" t="n"/>
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="14" t="n"/>
+      <c r="E56" s="14" t="n"/>
+      <c r="F56" s="15" t="n"/>
+      <c r="G56" s="14" t="n"/>
+      <c r="H56" s="17" t="n"/>
+      <c r="I56" s="37" t="n"/>
+      <c r="J56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="n"/>
+      <c r="B57" s="14" t="n"/>
+      <c r="C57" s="14" t="n"/>
+      <c r="D57" s="14" t="n"/>
+      <c r="E57" s="14" t="n"/>
+      <c r="F57" s="15" t="n"/>
+      <c r="G57" s="14" t="n"/>
+      <c r="H57" s="17" t="n"/>
+      <c r="I57" s="37" t="n"/>
+      <c r="J57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="n"/>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="14" t="n"/>
+      <c r="E58" s="14" t="n"/>
+      <c r="F58" s="15" t="n"/>
+      <c r="G58" s="14" t="n"/>
+      <c r="H58" s="17" t="n"/>
+      <c r="I58" s="37" t="n"/>
+      <c r="J58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="n"/>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="14" t="n"/>
+      <c r="E59" s="14" t="n"/>
+      <c r="F59" s="15" t="n"/>
+      <c r="G59" s="14" t="n"/>
+      <c r="H59" s="17" t="n"/>
+      <c r="I59" s="37" t="n"/>
+      <c r="J59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="n"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="14" t="n"/>
+      <c r="D60" s="14" t="n"/>
+      <c r="E60" s="14" t="n"/>
+      <c r="F60" s="15" t="n"/>
+      <c r="G60" s="14" t="n"/>
+      <c r="H60" s="17" t="n"/>
+      <c r="I60" s="37" t="n"/>
+      <c r="J60" s="14" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="n"/>
+      <c r="B61" s="14" t="n"/>
+      <c r="C61" s="14" t="n"/>
+      <c r="D61" s="14" t="n"/>
+      <c r="E61" s="14" t="n"/>
+      <c r="F61" s="15" t="n"/>
+      <c r="G61" s="14" t="n"/>
+      <c r="H61" s="17" t="n"/>
+      <c r="I61" s="37" t="n"/>
+      <c r="J61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="n"/>
+      <c r="B62" s="14" t="n"/>
+      <c r="C62" s="14" t="n"/>
+      <c r="D62" s="14" t="n"/>
+      <c r="E62" s="14" t="n"/>
+      <c r="F62" s="15" t="n"/>
+      <c r="G62" s="14" t="n"/>
+      <c r="H62" s="17" t="n"/>
+      <c r="I62" s="37" t="n"/>
+      <c r="J62" s="14" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="n"/>
+      <c r="B63" s="14" t="n"/>
+      <c r="C63" s="14" t="n"/>
+      <c r="D63" s="14" t="n"/>
+      <c r="E63" s="14" t="n"/>
+      <c r="F63" s="15" t="n"/>
+      <c r="G63" s="14" t="n"/>
+      <c r="H63" s="17" t="n"/>
+      <c r="I63" s="37" t="n"/>
+      <c r="J63" s="14" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="n"/>
+      <c r="B64" s="14" t="n"/>
+      <c r="C64" s="14" t="n"/>
+      <c r="D64" s="14" t="n"/>
+      <c r="E64" s="14" t="n"/>
+      <c r="F64" s="15" t="n"/>
+      <c r="G64" s="14" t="n"/>
+      <c r="H64" s="17" t="n"/>
+      <c r="I64" s="37" t="n"/>
+      <c r="J64" s="14" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="n"/>
+      <c r="B65" s="14" t="n"/>
+      <c r="C65" s="14" t="n"/>
+      <c r="D65" s="14" t="n"/>
+      <c r="E65" s="14" t="n"/>
+      <c r="F65" s="15" t="n"/>
+      <c r="G65" s="14" t="n"/>
+      <c r="H65" s="17" t="n"/>
+      <c r="I65" s="37" t="n"/>
+      <c r="J65" s="14" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="n"/>
+      <c r="B66" s="14" t="n"/>
+      <c r="C66" s="14" t="n"/>
+      <c r="D66" s="14" t="n"/>
+      <c r="E66" s="14" t="n"/>
+      <c r="F66" s="15" t="n"/>
+      <c r="G66" s="14" t="n"/>
+      <c r="H66" s="17" t="n"/>
+      <c r="I66" s="37" t="n"/>
+      <c r="J66" s="14" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="n"/>
+      <c r="B67" s="14" t="n"/>
+      <c r="C67" s="14" t="n"/>
+      <c r="D67" s="14" t="n"/>
+      <c r="E67" s="14" t="n"/>
+      <c r="F67" s="15" t="n"/>
+      <c r="G67" s="14" t="n"/>
+      <c r="H67" s="17" t="n"/>
+      <c r="I67" s="37" t="n"/>
+      <c r="J67" s="14" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="n"/>
+      <c r="B68" s="14" t="n"/>
+      <c r="C68" s="14" t="n"/>
+      <c r="D68" s="14" t="n"/>
+      <c r="E68" s="14" t="n"/>
+      <c r="F68" s="15" t="n"/>
+      <c r="G68" s="14" t="n"/>
+      <c r="H68" s="17" t="n"/>
+      <c r="I68" s="37" t="n"/>
+      <c r="J68" s="14" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="n"/>
+      <c r="B69" s="14" t="n"/>
+      <c r="C69" s="14" t="n"/>
+      <c r="D69" s="14" t="n"/>
+      <c r="E69" s="14" t="n"/>
+      <c r="F69" s="15" t="n"/>
+      <c r="G69" s="14" t="n"/>
+      <c r="H69" s="17" t="n"/>
+      <c r="I69" s="37" t="n"/>
+      <c r="J69" s="14" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="n"/>
+      <c r="B70" s="14" t="n"/>
+      <c r="C70" s="14" t="n"/>
+      <c r="D70" s="14" t="n"/>
+      <c r="E70" s="14" t="n"/>
+      <c r="F70" s="15" t="n"/>
+      <c r="G70" s="14" t="n"/>
+      <c r="H70" s="17" t="n"/>
+      <c r="I70" s="37" t="n"/>
+      <c r="J70" s="14" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="n"/>
+      <c r="B71" s="14" t="n"/>
+      <c r="C71" s="14" t="n"/>
+      <c r="D71" s="14" t="n"/>
+      <c r="E71" s="14" t="n"/>
+      <c r="F71" s="15" t="n"/>
+      <c r="G71" s="14" t="n"/>
+      <c r="H71" s="17" t="n"/>
+      <c r="I71" s="37" t="n"/>
+      <c r="J71" s="14" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="n"/>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="15" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="17" t="n"/>
+      <c r="I72" s="37" t="n"/>
+      <c r="J72" s="14" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="n"/>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="14" t="n"/>
+      <c r="D73" s="14" t="n"/>
+      <c r="E73" s="14" t="n"/>
+      <c r="F73" s="15" t="n"/>
+      <c r="G73" s="14" t="n"/>
+      <c r="H73" s="17" t="n"/>
+      <c r="I73" s="37" t="n"/>
+      <c r="J73" s="14" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="n"/>
+      <c r="B74" s="14" t="n"/>
+      <c r="C74" s="14" t="n"/>
+      <c r="D74" s="14" t="n"/>
+      <c r="E74" s="14" t="n"/>
+      <c r="F74" s="15" t="n"/>
+      <c r="G74" s="14" t="n"/>
+      <c r="H74" s="17" t="n"/>
+      <c r="I74" s="37" t="n"/>
+      <c r="J74" s="14" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="17" t="n"/>
+      <c r="B75" s="14" t="n"/>
+      <c r="C75" s="14" t="n"/>
+      <c r="D75" s="14" t="n"/>
+      <c r="E75" s="14" t="n"/>
+      <c r="F75" s="15" t="n"/>
+      <c r="G75" s="14" t="n"/>
+      <c r="H75" s="17" t="n"/>
+      <c r="I75" s="37" t="n"/>
+      <c r="J75" s="14" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="n"/>
+      <c r="B76" s="14" t="n"/>
+      <c r="C76" s="14" t="n"/>
+      <c r="D76" s="14" t="n"/>
+      <c r="E76" s="14" t="n"/>
+      <c r="F76" s="15" t="n"/>
+      <c r="G76" s="14" t="n"/>
+      <c r="H76" s="17" t="n"/>
+      <c r="I76" s="37" t="n"/>
+      <c r="J76" s="14" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="n"/>
+      <c r="B77" s="14" t="n"/>
+      <c r="C77" s="14" t="n"/>
+      <c r="D77" s="14" t="n"/>
+      <c r="E77" s="14" t="n"/>
+      <c r="F77" s="15" t="n"/>
+      <c r="G77" s="14" t="n"/>
+      <c r="H77" s="17" t="n"/>
+      <c r="I77" s="37" t="n"/>
+      <c r="J77" s="14" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="n"/>
+      <c r="B78" s="14" t="n"/>
+      <c r="C78" s="14" t="n"/>
+      <c r="D78" s="14" t="n"/>
+      <c r="E78" s="14" t="n"/>
+      <c r="F78" s="15" t="n"/>
+      <c r="G78" s="14" t="n"/>
+      <c r="H78" s="17" t="n"/>
+      <c r="I78" s="37" t="n"/>
+      <c r="J78" s="14" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="n"/>
+      <c r="B79" s="14" t="n"/>
+      <c r="C79" s="14" t="n"/>
+      <c r="D79" s="14" t="n"/>
+      <c r="E79" s="14" t="n"/>
+      <c r="F79" s="15" t="n"/>
+      <c r="G79" s="14" t="n"/>
+      <c r="H79" s="17" t="n"/>
+      <c r="I79" s="37" t="n"/>
+      <c r="J79" s="14" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="n"/>
+      <c r="B80" s="14" t="n"/>
+      <c r="C80" s="14" t="n"/>
+      <c r="D80" s="14" t="n"/>
+      <c r="E80" s="14" t="n"/>
+      <c r="F80" s="15" t="n"/>
+      <c r="G80" s="14" t="n"/>
+      <c r="H80" s="17" t="n"/>
+      <c r="I80" s="37" t="n"/>
+      <c r="J80" s="14" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="n"/>
+      <c r="B81" s="14" t="n"/>
+      <c r="C81" s="14" t="n"/>
+      <c r="D81" s="14" t="n"/>
+      <c r="E81" s="14" t="n"/>
+      <c r="F81" s="15" t="n"/>
+      <c r="G81" s="14" t="n"/>
+      <c r="H81" s="17" t="n"/>
+      <c r="I81" s="37" t="n"/>
+      <c r="J81" s="14" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="n"/>
+      <c r="B82" s="14" t="n"/>
+      <c r="C82" s="14" t="n"/>
+      <c r="D82" s="14" t="n"/>
+      <c r="E82" s="14" t="n"/>
+      <c r="F82" s="15" t="n"/>
+      <c r="G82" s="14" t="n"/>
+      <c r="H82" s="17" t="n"/>
+      <c r="I82" s="37" t="n"/>
+      <c r="J82" s="14" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="n"/>
+      <c r="B83" s="14" t="n"/>
+      <c r="C83" s="14" t="n"/>
+      <c r="D83" s="14" t="n"/>
+      <c r="E83" s="14" t="n"/>
+      <c r="F83" s="15" t="n"/>
+      <c r="G83" s="14" t="n"/>
+      <c r="H83" s="17" t="n"/>
+      <c r="I83" s="37" t="n"/>
+      <c r="J83" s="14" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="n"/>
+      <c r="B84" s="14" t="n"/>
+      <c r="C84" s="14" t="n"/>
+      <c r="D84" s="14" t="n"/>
+      <c r="E84" s="14" t="n"/>
+      <c r="F84" s="15" t="n"/>
+      <c r="G84" s="14" t="n"/>
+      <c r="H84" s="17" t="n"/>
+      <c r="I84" s="37" t="n"/>
+      <c r="J84" s="14" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="n"/>
+      <c r="B85" s="14" t="n"/>
+      <c r="C85" s="14" t="n"/>
+      <c r="D85" s="14" t="n"/>
+      <c r="E85" s="14" t="n"/>
+      <c r="F85" s="15" t="n"/>
+      <c r="G85" s="14" t="n"/>
+      <c r="H85" s="17" t="n"/>
+      <c r="I85" s="37" t="n"/>
+      <c r="J85" s="14" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="n"/>
+      <c r="B86" s="14" t="n"/>
+      <c r="C86" s="14" t="n"/>
+      <c r="D86" s="14" t="n"/>
+      <c r="E86" s="14" t="n"/>
+      <c r="F86" s="15" t="n"/>
+      <c r="G86" s="14" t="n"/>
+      <c r="H86" s="17" t="n"/>
+      <c r="I86" s="37" t="n"/>
+      <c r="J86" s="14" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="n"/>
+      <c r="B87" s="14" t="n"/>
+      <c r="C87" s="14" t="n"/>
+      <c r="D87" s="14" t="n"/>
+      <c r="E87" s="14" t="n"/>
+      <c r="F87" s="15" t="n"/>
+      <c r="G87" s="14" t="n"/>
+      <c r="H87" s="17" t="n"/>
+      <c r="I87" s="37" t="n"/>
+      <c r="J87" s="14" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="n"/>
+      <c r="B88" s="14" t="n"/>
+      <c r="C88" s="14" t="n"/>
+      <c r="D88" s="14" t="n"/>
+      <c r="E88" s="14" t="n"/>
+      <c r="F88" s="15" t="n"/>
+      <c r="G88" s="14" t="n"/>
+      <c r="H88" s="17" t="n"/>
+      <c r="I88" s="37" t="n"/>
+      <c r="J88" s="14" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="17" t="n"/>
+      <c r="B89" s="14" t="n"/>
+      <c r="C89" s="14" t="n"/>
+      <c r="D89" s="14" t="n"/>
+      <c r="E89" s="14" t="n"/>
+      <c r="F89" s="15" t="n"/>
+      <c r="G89" s="14" t="n"/>
+      <c r="H89" s="17" t="n"/>
+      <c r="I89" s="37" t="n"/>
+      <c r="J89" s="14" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="n"/>
+      <c r="B90" s="14" t="n"/>
+      <c r="C90" s="14" t="n"/>
+      <c r="D90" s="14" t="n"/>
+      <c r="E90" s="14" t="n"/>
+      <c r="F90" s="15" t="n"/>
+      <c r="G90" s="14" t="n"/>
+      <c r="H90" s="17" t="n"/>
+      <c r="I90" s="37" t="n"/>
+      <c r="J90" s="14" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="n"/>
+      <c r="B91" s="14" t="n"/>
+      <c r="C91" s="14" t="n"/>
+      <c r="D91" s="14" t="n"/>
+      <c r="E91" s="14" t="n"/>
+      <c r="F91" s="15" t="n"/>
+      <c r="G91" s="14" t="n"/>
+      <c r="H91" s="17" t="n"/>
+      <c r="I91" s="37" t="n"/>
+      <c r="J91" s="14" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="n"/>
+      <c r="B92" s="14" t="n"/>
+      <c r="C92" s="14" t="n"/>
+      <c r="D92" s="14" t="n"/>
+      <c r="E92" s="14" t="n"/>
+      <c r="F92" s="15" t="n"/>
+      <c r="G92" s="14" t="n"/>
+      <c r="H92" s="17" t="n"/>
+      <c r="I92" s="37" t="n"/>
+      <c r="J92" s="14" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="n"/>
+      <c r="B93" s="14" t="n"/>
+      <c r="C93" s="14" t="n"/>
+      <c r="D93" s="14" t="n"/>
+      <c r="E93" s="14" t="n"/>
+      <c r="F93" s="15" t="n"/>
+      <c r="G93" s="14" t="n"/>
+      <c r="H93" s="17" t="n"/>
+      <c r="I93" s="37" t="n"/>
+      <c r="J93" s="14" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="n"/>
+      <c r="B94" s="14" t="n"/>
+      <c r="C94" s="14" t="n"/>
+      <c r="D94" s="14" t="n"/>
+      <c r="E94" s="14" t="n"/>
+      <c r="F94" s="15" t="n"/>
+      <c r="G94" s="14" t="n"/>
+      <c r="H94" s="17" t="n"/>
+      <c r="I94" s="37" t="n"/>
+      <c r="J94" s="14" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="n"/>
+      <c r="B95" s="14" t="n"/>
+      <c r="C95" s="14" t="n"/>
+      <c r="D95" s="14" t="n"/>
+      <c r="E95" s="14" t="n"/>
+      <c r="F95" s="15" t="n"/>
+      <c r="G95" s="14" t="n"/>
+      <c r="H95" s="17" t="n"/>
+      <c r="I95" s="37" t="n"/>
+      <c r="J95" s="14" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="n"/>
+      <c r="B96" s="14" t="n"/>
+      <c r="C96" s="14" t="n"/>
+      <c r="D96" s="14" t="n"/>
+      <c r="E96" s="14" t="n"/>
+      <c r="F96" s="15" t="n"/>
+      <c r="G96" s="14" t="n"/>
+      <c r="H96" s="17" t="n"/>
+      <c r="I96" s="37" t="n"/>
+      <c r="J96" s="14" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="n"/>
+      <c r="B97" s="14" t="n"/>
+      <c r="C97" s="14" t="n"/>
+      <c r="D97" s="14" t="n"/>
+      <c r="E97" s="14" t="n"/>
+      <c r="F97" s="15" t="n"/>
+      <c r="G97" s="14" t="n"/>
+      <c r="H97" s="17" t="n"/>
+      <c r="I97" s="37" t="n"/>
+      <c r="J97" s="14" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="n"/>
+      <c r="B98" s="14" t="n"/>
+      <c r="C98" s="14" t="n"/>
+      <c r="D98" s="14" t="n"/>
+      <c r="E98" s="14" t="n"/>
+      <c r="F98" s="15" t="n"/>
+      <c r="G98" s="14" t="n"/>
+      <c r="H98" s="17" t="n"/>
+      <c r="I98" s="37" t="n"/>
+      <c r="J98" s="14" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="17" t="n"/>
+      <c r="B99" s="14" t="n"/>
+      <c r="C99" s="14" t="n"/>
+      <c r="D99" s="14" t="n"/>
+      <c r="E99" s="14" t="n"/>
+      <c r="F99" s="15" t="n"/>
+      <c r="G99" s="14" t="n"/>
+      <c r="H99" s="17" t="n"/>
+      <c r="I99" s="37" t="n"/>
+      <c r="J99" s="14" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="17" t="n"/>
+      <c r="B100" s="14" t="n"/>
+      <c r="C100" s="14" t="n"/>
+      <c r="D100" s="14" t="n"/>
+      <c r="E100" s="14" t="n"/>
+      <c r="F100" s="15" t="n"/>
+      <c r="G100" s="14" t="n"/>
+      <c r="H100" s="17" t="n"/>
+      <c r="I100" s="37" t="n"/>
+      <c r="J100" s="14" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="17" t="n"/>
+      <c r="B101" s="14" t="n"/>
+      <c r="C101" s="14" t="n"/>
+      <c r="D101" s="14" t="n"/>
+      <c r="E101" s="14" t="n"/>
+      <c r="F101" s="15" t="n"/>
+      <c r="G101" s="14" t="n"/>
+      <c r="H101" s="17" t="n"/>
+      <c r="I101" s="37" t="n"/>
+      <c r="J101" s="14" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="17" t="n"/>
+      <c r="B102" s="14" t="n"/>
+      <c r="C102" s="14" t="n"/>
+      <c r="D102" s="14" t="n"/>
+      <c r="E102" s="14" t="n"/>
+      <c r="F102" s="15" t="n"/>
+      <c r="G102" s="14" t="n"/>
+      <c r="H102" s="17" t="n"/>
+      <c r="I102" s="37" t="n"/>
+      <c r="J102" s="14" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="17" t="n"/>
+      <c r="B103" s="14" t="n"/>
+      <c r="C103" s="14" t="n"/>
+      <c r="D103" s="14" t="n"/>
+      <c r="E103" s="14" t="n"/>
+      <c r="F103" s="15" t="n"/>
+      <c r="G103" s="14" t="n"/>
+      <c r="H103" s="17" t="n"/>
+      <c r="I103" s="37" t="n"/>
+      <c r="J103" s="14" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="17" t="n"/>
+      <c r="B104" s="14" t="n"/>
+      <c r="C104" s="14" t="n"/>
+      <c r="D104" s="14" t="n"/>
+      <c r="E104" s="14" t="n"/>
+      <c r="F104" s="15" t="n"/>
+      <c r="G104" s="14" t="n"/>
+      <c r="H104" s="17" t="n"/>
+      <c r="I104" s="37" t="n"/>
+      <c r="J104" s="14" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="17" t="n"/>
+      <c r="B105" s="14" t="n"/>
+      <c r="C105" s="14" t="n"/>
+      <c r="D105" s="14" t="n"/>
+      <c r="E105" s="14" t="n"/>
+      <c r="F105" s="15" t="n"/>
+      <c r="G105" s="14" t="n"/>
+      <c r="H105" s="17" t="n"/>
+      <c r="I105" s="37" t="n"/>
+      <c r="J105" s="14" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="n"/>
+      <c r="B106" s="14" t="n"/>
+      <c r="C106" s="14" t="n"/>
+      <c r="D106" s="14" t="n"/>
+      <c r="E106" s="14" t="n"/>
+      <c r="F106" s="15" t="n"/>
+      <c r="G106" s="14" t="n"/>
+      <c r="H106" s="17" t="n"/>
+      <c r="I106" s="37" t="n"/>
+      <c r="J106" s="14" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="n"/>
+      <c r="B107" s="14" t="n"/>
+      <c r="C107" s="14" t="n"/>
+      <c r="D107" s="14" t="n"/>
+      <c r="E107" s="14" t="n"/>
+      <c r="F107" s="15" t="n"/>
+      <c r="G107" s="14" t="n"/>
+      <c r="H107" s="17" t="n"/>
+      <c r="I107" s="37" t="n"/>
+      <c r="J107" s="14" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="17" t="n"/>
+      <c r="B108" s="14" t="n"/>
+      <c r="C108" s="14" t="n"/>
+      <c r="D108" s="14" t="n"/>
+      <c r="E108" s="14" t="n"/>
+      <c r="F108" s="15" t="n"/>
+      <c r="G108" s="14" t="n"/>
+      <c r="H108" s="17" t="n"/>
+      <c r="I108" s="37" t="n"/>
+      <c r="J108" s="14" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="17" t="n"/>
+      <c r="B109" s="14" t="n"/>
+      <c r="C109" s="14" t="n"/>
+      <c r="D109" s="14" t="n"/>
+      <c r="E109" s="14" t="n"/>
+      <c r="F109" s="15" t="n"/>
+      <c r="G109" s="14" t="n"/>
+      <c r="H109" s="17" t="n"/>
+      <c r="I109" s="37" t="n"/>
+      <c r="J109" s="14" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="17" t="n"/>
+      <c r="B110" s="14" t="n"/>
+      <c r="C110" s="14" t="n"/>
+      <c r="D110" s="14" t="n"/>
+      <c r="E110" s="14" t="n"/>
+      <c r="F110" s="15" t="n"/>
+      <c r="G110" s="14" t="n"/>
+      <c r="H110" s="17" t="n"/>
+      <c r="I110" s="37" t="n"/>
+      <c r="J110" s="14" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="17" t="n"/>
+      <c r="B111" s="14" t="n"/>
+      <c r="C111" s="14" t="n"/>
+      <c r="D111" s="14" t="n"/>
+      <c r="E111" s="14" t="n"/>
+      <c r="F111" s="15" t="n"/>
+      <c r="G111" s="14" t="n"/>
+      <c r="H111" s="17" t="n"/>
+      <c r="I111" s="37" t="n"/>
+      <c r="J111" s="14" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="17" t="n"/>
+      <c r="B112" s="14" t="n"/>
+      <c r="C112" s="14" t="n"/>
+      <c r="D112" s="14" t="n"/>
+      <c r="E112" s="14" t="n"/>
+      <c r="F112" s="15" t="n"/>
+      <c r="G112" s="14" t="n"/>
+      <c r="H112" s="17" t="n"/>
+      <c r="I112" s="37" t="n"/>
+      <c r="J112" s="14" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="17" t="n"/>
+      <c r="B113" s="14" t="n"/>
+      <c r="C113" s="14" t="n"/>
+      <c r="D113" s="14" t="n"/>
+      <c r="E113" s="14" t="n"/>
+      <c r="F113" s="15" t="n"/>
+      <c r="G113" s="14" t="n"/>
+      <c r="H113" s="17" t="n"/>
+      <c r="I113" s="37" t="n"/>
+      <c r="J113" s="14" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="n"/>
+      <c r="B114" s="14" t="n"/>
+      <c r="C114" s="14" t="n"/>
+      <c r="D114" s="14" t="n"/>
+      <c r="E114" s="14" t="n"/>
+      <c r="F114" s="15" t="n"/>
+      <c r="G114" s="14" t="n"/>
+      <c r="H114" s="17" t="n"/>
+      <c r="I114" s="37" t="n"/>
+      <c r="J114" s="14" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="17" t="n"/>
+      <c r="B115" s="14" t="n"/>
+      <c r="C115" s="14" t="n"/>
+      <c r="D115" s="14" t="n"/>
+      <c r="E115" s="14" t="n"/>
+      <c r="F115" s="15" t="n"/>
+      <c r="G115" s="14" t="n"/>
+      <c r="H115" s="17" t="n"/>
+      <c r="I115" s="37" t="n"/>
+      <c r="J115" s="14" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="17" t="n"/>
+      <c r="B116" s="14" t="n"/>
+      <c r="C116" s="14" t="n"/>
+      <c r="D116" s="14" t="n"/>
+      <c r="E116" s="14" t="n"/>
+      <c r="F116" s="15" t="n"/>
+      <c r="G116" s="14" t="n"/>
+      <c r="H116" s="17" t="n"/>
+      <c r="I116" s="37" t="n"/>
+      <c r="J116" s="14" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="n"/>
+      <c r="B117" s="14" t="n"/>
+      <c r="C117" s="14" t="n"/>
+      <c r="D117" s="14" t="n"/>
+      <c r="E117" s="14" t="n"/>
+      <c r="F117" s="15" t="n"/>
+      <c r="G117" s="14" t="n"/>
+      <c r="H117" s="17" t="n"/>
+      <c r="I117" s="37" t="n"/>
+      <c r="J117" s="14" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="17" t="n"/>
+      <c r="B118" s="14" t="n"/>
+      <c r="C118" s="14" t="n"/>
+      <c r="D118" s="14" t="n"/>
+      <c r="E118" s="14" t="n"/>
+      <c r="F118" s="15" t="n"/>
+      <c r="G118" s="14" t="n"/>
+      <c r="H118" s="17" t="n"/>
+      <c r="I118" s="37" t="n"/>
+      <c r="J118" s="14" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="17" t="n"/>
+      <c r="B119" s="14" t="n"/>
+      <c r="C119" s="14" t="n"/>
+      <c r="D119" s="14" t="n"/>
+      <c r="E119" s="14" t="n"/>
+      <c r="F119" s="15" t="n"/>
+      <c r="G119" s="14" t="n"/>
+      <c r="H119" s="17" t="n"/>
+      <c r="I119" s="37" t="n"/>
+      <c r="J119" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="17" t="n"/>
+      <c r="B120" s="14" t="n"/>
+      <c r="C120" s="14" t="n"/>
+      <c r="D120" s="14" t="n"/>
+      <c r="E120" s="14" t="n"/>
+      <c r="F120" s="15" t="n"/>
+      <c r="G120" s="14" t="n"/>
+      <c r="H120" s="17" t="n"/>
+      <c r="I120" s="37" t="n"/>
+      <c r="J120" s="14" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="17" t="n"/>
+      <c r="B121" s="14" t="n"/>
+      <c r="C121" s="14" t="n"/>
+      <c r="D121" s="14" t="n"/>
+      <c r="E121" s="14" t="n"/>
+      <c r="F121" s="15" t="n"/>
+      <c r="G121" s="14" t="n"/>
+      <c r="H121" s="17" t="n"/>
+      <c r="I121" s="37" t="n"/>
+      <c r="J121" s="14" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="17" t="n"/>
+      <c r="B122" s="14" t="n"/>
+      <c r="C122" s="14" t="n"/>
+      <c r="D122" s="14" t="n"/>
+      <c r="E122" s="14" t="n"/>
+      <c r="F122" s="15" t="n"/>
+      <c r="G122" s="14" t="n"/>
+      <c r="H122" s="17" t="n"/>
+      <c r="I122" s="37" t="n"/>
+      <c r="J122" s="14" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="n"/>
+      <c r="B123" s="14" t="n"/>
+      <c r="C123" s="14" t="n"/>
+      <c r="D123" s="14" t="n"/>
+      <c r="E123" s="14" t="n"/>
+      <c r="F123" s="15" t="n"/>
+      <c r="G123" s="14" t="n"/>
+      <c r="H123" s="17" t="n"/>
+      <c r="I123" s="37" t="n"/>
+      <c r="J123" s="14" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="n"/>
+      <c r="B124" s="14" t="n"/>
+      <c r="C124" s="14" t="n"/>
+      <c r="D124" s="14" t="n"/>
+      <c r="E124" s="14" t="n"/>
+      <c r="F124" s="15" t="n"/>
+      <c r="G124" s="14" t="n"/>
+      <c r="H124" s="17" t="n"/>
+      <c r="I124" s="37" t="n"/>
+      <c r="J124" s="14" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="n"/>
+      <c r="B125" s="14" t="n"/>
+      <c r="C125" s="14" t="n"/>
+      <c r="D125" s="14" t="n"/>
+      <c r="E125" s="14" t="n"/>
+      <c r="F125" s="15" t="n"/>
+      <c r="G125" s="14" t="n"/>
+      <c r="H125" s="17" t="n"/>
+      <c r="I125" s="37" t="n"/>
+      <c r="J125" s="14" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="n"/>
+      <c r="B126" s="14" t="n"/>
+      <c r="C126" s="14" t="n"/>
+      <c r="D126" s="14" t="n"/>
+      <c r="E126" s="14" t="n"/>
+      <c r="F126" s="15" t="n"/>
+      <c r="G126" s="14" t="n"/>
+      <c r="H126" s="17" t="n"/>
+      <c r="I126" s="37" t="n"/>
+      <c r="J126" s="14" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="n"/>
+      <c r="B127" s="14" t="n"/>
+      <c r="C127" s="14" t="n"/>
+      <c r="D127" s="14" t="n"/>
+      <c r="E127" s="14" t="n"/>
+      <c r="F127" s="15" t="n"/>
+      <c r="G127" s="14" t="n"/>
+      <c r="H127" s="17" t="n"/>
+      <c r="I127" s="37" t="n"/>
+      <c r="J127" s="14" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="17" t="n"/>
+      <c r="B128" s="14" t="n"/>
+      <c r="C128" s="14" t="n"/>
+      <c r="D128" s="14" t="n"/>
+      <c r="E128" s="14" t="n"/>
+      <c r="F128" s="15" t="n"/>
+      <c r="G128" s="14" t="n"/>
+      <c r="H128" s="17" t="n"/>
+      <c r="I128" s="37" t="n"/>
+      <c r="J128" s="14" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="17" t="n"/>
+      <c r="B129" s="14" t="n"/>
+      <c r="C129" s="14" t="n"/>
+      <c r="D129" s="14" t="n"/>
+      <c r="E129" s="14" t="n"/>
+      <c r="F129" s="15" t="n"/>
+      <c r="G129" s="14" t="n"/>
+      <c r="H129" s="17" t="n"/>
+      <c r="I129" s="37" t="n"/>
+      <c r="J129" s="14" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="17" t="n"/>
+      <c r="B130" s="14" t="n"/>
+      <c r="C130" s="14" t="n"/>
+      <c r="D130" s="14" t="n"/>
+      <c r="E130" s="14" t="n"/>
+      <c r="F130" s="15" t="n"/>
+      <c r="G130" s="14" t="n"/>
+      <c r="H130" s="17" t="n"/>
+      <c r="I130" s="37" t="n"/>
+      <c r="J130" s="14" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="17" t="n"/>
+      <c r="B131" s="14" t="n"/>
+      <c r="C131" s="14" t="n"/>
+      <c r="D131" s="14" t="n"/>
+      <c r="E131" s="14" t="n"/>
+      <c r="F131" s="15" t="n"/>
+      <c r="G131" s="14" t="n"/>
+      <c r="H131" s="17" t="n"/>
+      <c r="I131" s="37" t="n"/>
+      <c r="J131" s="14" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="17" t="n"/>
+      <c r="B132" s="14" t="n"/>
+      <c r="C132" s="14" t="n"/>
+      <c r="D132" s="14" t="n"/>
+      <c r="E132" s="14" t="n"/>
+      <c r="F132" s="15" t="n"/>
+      <c r="G132" s="14" t="n"/>
+      <c r="H132" s="17" t="n"/>
+      <c r="I132" s="37" t="n"/>
+      <c r="J132" s="14" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="n"/>
+      <c r="B133" s="14" t="n"/>
+      <c r="C133" s="14" t="n"/>
+      <c r="D133" s="14" t="n"/>
+      <c r="E133" s="14" t="n"/>
+      <c r="F133" s="15" t="n"/>
+      <c r="G133" s="14" t="n"/>
+      <c r="H133" s="17" t="n"/>
+      <c r="I133" s="37" t="n"/>
+      <c r="J133" s="14" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="17" t="n"/>
+      <c r="B134" s="14" t="n"/>
+      <c r="C134" s="14" t="n"/>
+      <c r="D134" s="14" t="n"/>
+      <c r="E134" s="14" t="n"/>
+      <c r="F134" s="15" t="n"/>
+      <c r="G134" s="14" t="n"/>
+      <c r="H134" s="17" t="n"/>
+      <c r="I134" s="37" t="n"/>
+      <c r="J134" s="14" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="17" t="n"/>
+      <c r="B135" s="14" t="n"/>
+      <c r="C135" s="14" t="n"/>
+      <c r="D135" s="14" t="n"/>
+      <c r="E135" s="14" t="n"/>
+      <c r="F135" s="15" t="n"/>
+      <c r="G135" s="14" t="n"/>
+      <c r="H135" s="17" t="n"/>
+      <c r="I135" s="37" t="n"/>
+      <c r="J135" s="14" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="17" t="n"/>
+      <c r="B136" s="14" t="n"/>
+      <c r="C136" s="14" t="n"/>
+      <c r="D136" s="14" t="n"/>
+      <c r="E136" s="14" t="n"/>
+      <c r="F136" s="15" t="n"/>
+      <c r="G136" s="14" t="n"/>
+      <c r="H136" s="17" t="n"/>
+      <c r="I136" s="37" t="n"/>
+      <c r="J136" s="14" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="17" t="n"/>
+      <c r="B137" s="14" t="n"/>
+      <c r="C137" s="14" t="n"/>
+      <c r="D137" s="14" t="n"/>
+      <c r="E137" s="14" t="n"/>
+      <c r="F137" s="15" t="n"/>
+      <c r="G137" s="14" t="n"/>
+      <c r="H137" s="17" t="n"/>
+      <c r="I137" s="37" t="n"/>
+      <c r="J137" s="14" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="17" t="n"/>
+      <c r="B138" s="14" t="n"/>
+      <c r="C138" s="14" t="n"/>
+      <c r="D138" s="14" t="n"/>
+      <c r="E138" s="14" t="n"/>
+      <c r="F138" s="15" t="n"/>
+      <c r="G138" s="14" t="n"/>
+      <c r="H138" s="17" t="n"/>
+      <c r="I138" s="37" t="n"/>
+      <c r="J138" s="14" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="17" t="n"/>
+      <c r="B139" s="14" t="n"/>
+      <c r="C139" s="14" t="n"/>
+      <c r="D139" s="14" t="n"/>
+      <c r="E139" s="14" t="n"/>
+      <c r="F139" s="15" t="n"/>
+      <c r="G139" s="14" t="n"/>
+      <c r="H139" s="17" t="n"/>
+      <c r="I139" s="37" t="n"/>
+      <c r="J139" s="14" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="n"/>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="14" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="15" t="n"/>
+      <c r="G140" s="14" t="n"/>
+      <c r="H140" s="17" t="n"/>
+      <c r="I140" s="37" t="n"/>
+      <c r="J140" s="14" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="n"/>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="14" t="n"/>
+      <c r="D141" s="14" t="n"/>
+      <c r="E141" s="14" t="n"/>
+      <c r="F141" s="15" t="n"/>
+      <c r="G141" s="14" t="n"/>
+      <c r="H141" s="17" t="n"/>
+      <c r="I141" s="37" t="n"/>
+      <c r="J141" s="14" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="n"/>
+      <c r="B142" s="14" t="n"/>
+      <c r="C142" s="14" t="n"/>
+      <c r="D142" s="14" t="n"/>
+      <c r="E142" s="14" t="n"/>
+      <c r="F142" s="15" t="n"/>
+      <c r="G142" s="14" t="n"/>
+      <c r="H142" s="17" t="n"/>
+      <c r="I142" s="37" t="n"/>
+      <c r="J142" s="14" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="17" t="n"/>
+      <c r="B143" s="14" t="n"/>
+      <c r="C143" s="14" t="n"/>
+      <c r="D143" s="14" t="n"/>
+      <c r="E143" s="14" t="n"/>
+      <c r="F143" s="15" t="n"/>
+      <c r="G143" s="14" t="n"/>
+      <c r="H143" s="17" t="n"/>
+      <c r="I143" s="37" t="n"/>
+      <c r="J143" s="14" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="17" t="n"/>
+      <c r="B144" s="14" t="n"/>
+      <c r="C144" s="14" t="n"/>
+      <c r="D144" s="14" t="n"/>
+      <c r="E144" s="14" t="n"/>
+      <c r="F144" s="15" t="n"/>
+      <c r="G144" s="14" t="n"/>
+      <c r="H144" s="17" t="n"/>
+      <c r="I144" s="37" t="n"/>
+      <c r="J144" s="14" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="17" t="n"/>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="15" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="17" t="n"/>
+      <c r="I145" s="37" t="n"/>
+      <c r="J145" s="14" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="17" t="n"/>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="14" t="n"/>
+      <c r="D146" s="14" t="n"/>
+      <c r="E146" s="14" t="n"/>
+      <c r="F146" s="15" t="n"/>
+      <c r="G146" s="14" t="n"/>
+      <c r="H146" s="17" t="n"/>
+      <c r="I146" s="37" t="n"/>
+      <c r="J146" s="14" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="17" t="n"/>
+      <c r="B147" s="14" t="n"/>
+      <c r="C147" s="14" t="n"/>
+      <c r="D147" s="14" t="n"/>
+      <c r="E147" s="14" t="n"/>
+      <c r="F147" s="15" t="n"/>
+      <c r="G147" s="14" t="n"/>
+      <c r="H147" s="17" t="n"/>
+      <c r="I147" s="37" t="n"/>
+      <c r="J147" s="14" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="17" t="n"/>
+      <c r="B148" s="14" t="n"/>
+      <c r="C148" s="14" t="n"/>
+      <c r="D148" s="14" t="n"/>
+      <c r="E148" s="14" t="n"/>
+      <c r="F148" s="15" t="n"/>
+      <c r="G148" s="14" t="n"/>
+      <c r="H148" s="17" t="n"/>
+      <c r="I148" s="37" t="n"/>
+      <c r="J148" s="14" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="17" t="n"/>
+      <c r="B149" s="14" t="n"/>
+      <c r="C149" s="14" t="n"/>
+      <c r="D149" s="14" t="n"/>
+      <c r="E149" s="14" t="n"/>
+      <c r="F149" s="15" t="n"/>
+      <c r="G149" s="14" t="n"/>
+      <c r="H149" s="17" t="n"/>
+      <c r="I149" s="37" t="n"/>
+      <c r="J149" s="14" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="17" t="n"/>
+      <c r="B150" s="14" t="n"/>
+      <c r="C150" s="14" t="n"/>
+      <c r="D150" s="14" t="n"/>
+      <c r="E150" s="14" t="n"/>
+      <c r="F150" s="15" t="n"/>
+      <c r="G150" s="14" t="n"/>
+      <c r="H150" s="17" t="n"/>
+      <c r="I150" s="37" t="n"/>
+      <c r="J150" s="14" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="17" t="n"/>
+      <c r="B151" s="14" t="n"/>
+      <c r="C151" s="14" t="n"/>
+      <c r="D151" s="14" t="n"/>
+      <c r="E151" s="14" t="n"/>
+      <c r="F151" s="15" t="n"/>
+      <c r="G151" s="14" t="n"/>
+      <c r="H151" s="17" t="n"/>
+      <c r="I151" s="37" t="n"/>
+      <c r="J151" s="14" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="17" t="n"/>
+      <c r="B152" s="14" t="n"/>
+      <c r="C152" s="14" t="n"/>
+      <c r="D152" s="14" t="n"/>
+      <c r="E152" s="14" t="n"/>
+      <c r="F152" s="15" t="n"/>
+      <c r="G152" s="14" t="n"/>
+      <c r="H152" s="17" t="n"/>
+      <c r="I152" s="37" t="n"/>
+      <c r="J152" s="14" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="17" t="n"/>
+      <c r="B153" s="14" t="n"/>
+      <c r="C153" s="14" t="n"/>
+      <c r="D153" s="14" t="n"/>
+      <c r="E153" s="14" t="n"/>
+      <c r="F153" s="15" t="n"/>
+      <c r="G153" s="14" t="n"/>
+      <c r="H153" s="17" t="n"/>
+      <c r="I153" s="37" t="n"/>
+      <c r="J153" s="14" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="17" t="n"/>
+      <c r="B154" s="14" t="n"/>
+      <c r="C154" s="14" t="n"/>
+      <c r="D154" s="14" t="n"/>
+      <c r="E154" s="14" t="n"/>
+      <c r="F154" s="15" t="n"/>
+      <c r="G154" s="14" t="n"/>
+      <c r="H154" s="17" t="n"/>
+      <c r="I154" s="37" t="n"/>
+      <c r="J154" s="14" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="17" t="n"/>
+      <c r="B155" s="14" t="n"/>
+      <c r="C155" s="14" t="n"/>
+      <c r="D155" s="14" t="n"/>
+      <c r="E155" s="14" t="n"/>
+      <c r="F155" s="15" t="n"/>
+      <c r="G155" s="14" t="n"/>
+      <c r="H155" s="17" t="n"/>
+      <c r="I155" s="37" t="n"/>
+      <c r="J155" s="14" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="17" t="n"/>
+      <c r="B156" s="14" t="n"/>
+      <c r="C156" s="14" t="n"/>
+      <c r="D156" s="14" t="n"/>
+      <c r="E156" s="14" t="n"/>
+      <c r="F156" s="15" t="n"/>
+      <c r="G156" s="14" t="n"/>
+      <c r="H156" s="17" t="n"/>
+      <c r="I156" s="37" t="n"/>
+      <c r="J156" s="14" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="17" t="n"/>
+      <c r="B157" s="14" t="n"/>
+      <c r="C157" s="14" t="n"/>
+      <c r="D157" s="14" t="n"/>
+      <c r="E157" s="14" t="n"/>
+      <c r="F157" s="15" t="n"/>
+      <c r="G157" s="14" t="n"/>
+      <c r="H157" s="17" t="n"/>
+      <c r="I157" s="37" t="n"/>
+      <c r="J157" s="14" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="17" t="n"/>
+      <c r="B158" s="14" t="n"/>
+      <c r="C158" s="14" t="n"/>
+      <c r="D158" s="14" t="n"/>
+      <c r="E158" s="14" t="n"/>
+      <c r="F158" s="15" t="n"/>
+      <c r="G158" s="14" t="n"/>
+      <c r="H158" s="17" t="n"/>
+      <c r="I158" s="37" t="n"/>
+      <c r="J158" s="14" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="17" t="n"/>
+      <c r="B159" s="14" t="n"/>
+      <c r="C159" s="14" t="n"/>
+      <c r="D159" s="14" t="n"/>
+      <c r="E159" s="14" t="n"/>
+      <c r="F159" s="15" t="n"/>
+      <c r="G159" s="14" t="n"/>
+      <c r="H159" s="17" t="n"/>
+      <c r="I159" s="37" t="n"/>
+      <c r="J159" s="14" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="17" t="n"/>
+      <c r="B160" s="14" t="n"/>
+      <c r="C160" s="14" t="n"/>
+      <c r="D160" s="14" t="n"/>
+      <c r="E160" s="14" t="n"/>
+      <c r="F160" s="15" t="n"/>
+      <c r="G160" s="14" t="n"/>
+      <c r="H160" s="17" t="n"/>
+      <c r="I160" s="37" t="n"/>
+      <c r="J160" s="14" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="17" t="n"/>
+      <c r="B161" s="14" t="n"/>
+      <c r="C161" s="14" t="n"/>
+      <c r="D161" s="14" t="n"/>
+      <c r="E161" s="14" t="n"/>
+      <c r="F161" s="15" t="n"/>
+      <c r="G161" s="14" t="n"/>
+      <c r="H161" s="17" t="n"/>
+      <c r="I161" s="37" t="n"/>
+      <c r="J161" s="14" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="17" t="n"/>
+      <c r="B162" s="14" t="n"/>
+      <c r="C162" s="14" t="n"/>
+      <c r="D162" s="14" t="n"/>
+      <c r="E162" s="14" t="n"/>
+      <c r="F162" s="15" t="n"/>
+      <c r="G162" s="14" t="n"/>
+      <c r="H162" s="17" t="n"/>
+      <c r="I162" s="37" t="n"/>
+      <c r="J162" s="14" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="17" t="n"/>
+      <c r="B163" s="14" t="n"/>
+      <c r="C163" s="14" t="n"/>
+      <c r="D163" s="14" t="n"/>
+      <c r="E163" s="14" t="n"/>
+      <c r="F163" s="15" t="n"/>
+      <c r="G163" s="14" t="n"/>
+      <c r="H163" s="17" t="n"/>
+      <c r="I163" s="37" t="n"/>
+      <c r="J163" s="14" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="17" t="n"/>
+      <c r="B164" s="14" t="n"/>
+      <c r="C164" s="14" t="n"/>
+      <c r="D164" s="14" t="n"/>
+      <c r="E164" s="14" t="n"/>
+      <c r="F164" s="15" t="n"/>
+      <c r="G164" s="14" t="n"/>
+      <c r="H164" s="17" t="n"/>
+      <c r="I164" s="37" t="n"/>
+      <c r="J164" s="14" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="17" t="n"/>
+      <c r="B165" s="14" t="n"/>
+      <c r="C165" s="14" t="n"/>
+      <c r="D165" s="14" t="n"/>
+      <c r="E165" s="14" t="n"/>
+      <c r="F165" s="15" t="n"/>
+      <c r="G165" s="14" t="n"/>
+      <c r="H165" s="17" t="n"/>
+      <c r="I165" s="37" t="n"/>
+      <c r="J165" s="14" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="17" t="n"/>
+      <c r="B166" s="14" t="n"/>
+      <c r="C166" s="14" t="n"/>
+      <c r="D166" s="14" t="n"/>
+      <c r="E166" s="14" t="n"/>
+      <c r="F166" s="15" t="n"/>
+      <c r="G166" s="14" t="n"/>
+      <c r="H166" s="17" t="n"/>
+      <c r="I166" s="37" t="n"/>
+      <c r="J166" s="14" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="17" t="n"/>
+      <c r="B167" s="14" t="n"/>
+      <c r="C167" s="14" t="n"/>
+      <c r="D167" s="14" t="n"/>
+      <c r="E167" s="14" t="n"/>
+      <c r="F167" s="15" t="n"/>
+      <c r="G167" s="14" t="n"/>
+      <c r="H167" s="17" t="n"/>
+      <c r="I167" s="37" t="n"/>
+      <c r="J167" s="14" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="17" t="n"/>
+      <c r="B168" s="14" t="n"/>
+      <c r="C168" s="14" t="n"/>
+      <c r="D168" s="14" t="n"/>
+      <c r="E168" s="14" t="n"/>
+      <c r="F168" s="15" t="n"/>
+      <c r="G168" s="14" t="n"/>
+      <c r="H168" s="17" t="n"/>
+      <c r="I168" s="37" t="n"/>
+      <c r="J168" s="14" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="17" t="n"/>
+      <c r="B169" s="14" t="n"/>
+      <c r="C169" s="14" t="n"/>
+      <c r="D169" s="14" t="n"/>
+      <c r="E169" s="14" t="n"/>
+      <c r="F169" s="15" t="n"/>
+      <c r="G169" s="14" t="n"/>
+      <c r="H169" s="17" t="n"/>
+      <c r="I169" s="37" t="n"/>
+      <c r="J169" s="14" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="17" t="n"/>
+      <c r="B170" s="14" t="n"/>
+      <c r="C170" s="14" t="n"/>
+      <c r="D170" s="14" t="n"/>
+      <c r="E170" s="14" t="n"/>
+      <c r="F170" s="15" t="n"/>
+      <c r="G170" s="14" t="n"/>
+      <c r="H170" s="17" t="n"/>
+      <c r="I170" s="37" t="n"/>
+      <c r="J170" s="14" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="17" t="n"/>
+      <c r="B171" s="14" t="n"/>
+      <c r="C171" s="14" t="n"/>
+      <c r="D171" s="14" t="n"/>
+      <c r="E171" s="14" t="n"/>
+      <c r="F171" s="15" t="n"/>
+      <c r="G171" s="14" t="n"/>
+      <c r="H171" s="17" t="n"/>
+      <c r="I171" s="37" t="n"/>
+      <c r="J171" s="14" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="17" t="n"/>
+      <c r="B172" s="14" t="n"/>
+      <c r="C172" s="14" t="n"/>
+      <c r="D172" s="14" t="n"/>
+      <c r="E172" s="14" t="n"/>
+      <c r="F172" s="15" t="n"/>
+      <c r="G172" s="14" t="n"/>
+      <c r="H172" s="17" t="n"/>
+      <c r="I172" s="37" t="n"/>
+      <c r="J172" s="14" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="17" t="n"/>
+      <c r="B173" s="14" t="n"/>
+      <c r="C173" s="14" t="n"/>
+      <c r="D173" s="14" t="n"/>
+      <c r="E173" s="14" t="n"/>
+      <c r="F173" s="15" t="n"/>
+      <c r="G173" s="14" t="n"/>
+      <c r="H173" s="17" t="n"/>
+      <c r="I173" s="37" t="n"/>
+      <c r="J173" s="14" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="17" t="n"/>
+      <c r="B174" s="14" t="n"/>
+      <c r="C174" s="14" t="n"/>
+      <c r="D174" s="14" t="n"/>
+      <c r="E174" s="14" t="n"/>
+      <c r="F174" s="15" t="n"/>
+      <c r="G174" s="14" t="n"/>
+      <c r="H174" s="17" t="n"/>
+      <c r="I174" s="37" t="n"/>
+      <c r="J174" s="14" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="17" t="n"/>
+      <c r="B175" s="14" t="n"/>
+      <c r="C175" s="14" t="n"/>
+      <c r="D175" s="14" t="n"/>
+      <c r="E175" s="14" t="n"/>
+      <c r="F175" s="15" t="n"/>
+      <c r="G175" s="14" t="n"/>
+      <c r="H175" s="17" t="n"/>
+      <c r="I175" s="37" t="n"/>
+      <c r="J175" s="14" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="17" t="n"/>
+      <c r="B176" s="14" t="n"/>
+      <c r="C176" s="14" t="n"/>
+      <c r="D176" s="14" t="n"/>
+      <c r="E176" s="14" t="n"/>
+      <c r="F176" s="15" t="n"/>
+      <c r="G176" s="14" t="n"/>
+      <c r="H176" s="17" t="n"/>
+      <c r="I176" s="37" t="n"/>
+      <c r="J176" s="14" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="17" t="n"/>
+      <c r="B177" s="14" t="n"/>
+      <c r="C177" s="14" t="n"/>
+      <c r="D177" s="14" t="n"/>
+      <c r="E177" s="14" t="n"/>
+      <c r="F177" s="15" t="n"/>
+      <c r="G177" s="14" t="n"/>
+      <c r="H177" s="17" t="n"/>
+      <c r="I177" s="37" t="n"/>
+      <c r="J177" s="14" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="17" t="n"/>
+      <c r="B178" s="14" t="n"/>
+      <c r="C178" s="14" t="n"/>
+      <c r="D178" s="14" t="n"/>
+      <c r="E178" s="14" t="n"/>
+      <c r="F178" s="15" t="n"/>
+      <c r="G178" s="14" t="n"/>
+      <c r="H178" s="17" t="n"/>
+      <c r="I178" s="37" t="n"/>
+      <c r="J178" s="14" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="17" t="n"/>
+      <c r="B179" s="14" t="n"/>
+      <c r="C179" s="14" t="n"/>
+      <c r="D179" s="14" t="n"/>
+      <c r="E179" s="14" t="n"/>
+      <c r="F179" s="15" t="n"/>
+      <c r="G179" s="14" t="n"/>
+      <c r="H179" s="17" t="n"/>
+      <c r="I179" s="37" t="n"/>
+      <c r="J179" s="14" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="17" t="n"/>
+      <c r="B180" s="14" t="n"/>
+      <c r="C180" s="14" t="n"/>
+      <c r="D180" s="14" t="n"/>
+      <c r="E180" s="14" t="n"/>
+      <c r="F180" s="15" t="n"/>
+      <c r="G180" s="14" t="n"/>
+      <c r="H180" s="17" t="n"/>
+      <c r="I180" s="37" t="n"/>
+      <c r="J180" s="14" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="17" t="n"/>
+      <c r="B181" s="14" t="n"/>
+      <c r="C181" s="14" t="n"/>
+      <c r="D181" s="14" t="n"/>
+      <c r="E181" s="14" t="n"/>
+      <c r="F181" s="15" t="n"/>
+      <c r="G181" s="14" t="n"/>
+      <c r="H181" s="17" t="n"/>
+      <c r="I181" s="37" t="n"/>
+      <c r="J181" s="14" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="17" t="n"/>
+      <c r="B182" s="14" t="n"/>
+      <c r="C182" s="14" t="n"/>
+      <c r="D182" s="14" t="n"/>
+      <c r="E182" s="14" t="n"/>
+      <c r="F182" s="15" t="n"/>
+      <c r="G182" s="14" t="n"/>
+      <c r="H182" s="17" t="n"/>
+      <c r="I182" s="37" t="n"/>
+      <c r="J182" s="14" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="17" t="n"/>
+      <c r="B183" s="14" t="n"/>
+      <c r="C183" s="14" t="n"/>
+      <c r="D183" s="14" t="n"/>
+      <c r="E183" s="14" t="n"/>
+      <c r="F183" s="15" t="n"/>
+      <c r="G183" s="14" t="n"/>
+      <c r="H183" s="17" t="n"/>
+      <c r="I183" s="37" t="n"/>
+      <c r="J183" s="14" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="17" t="n"/>
+      <c r="B184" s="14" t="n"/>
+      <c r="C184" s="14" t="n"/>
+      <c r="D184" s="14" t="n"/>
+      <c r="E184" s="14" t="n"/>
+      <c r="F184" s="15" t="n"/>
+      <c r="G184" s="14" t="n"/>
+      <c r="H184" s="17" t="n"/>
+      <c r="I184" s="37" t="n"/>
+      <c r="J184" s="14" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="17" t="n"/>
+      <c r="B185" s="14" t="n"/>
+      <c r="C185" s="14" t="n"/>
+      <c r="D185" s="14" t="n"/>
+      <c r="E185" s="14" t="n"/>
+      <c r="F185" s="15" t="n"/>
+      <c r="G185" s="14" t="n"/>
+      <c r="H185" s="17" t="n"/>
+      <c r="I185" s="37" t="n"/>
+      <c r="J185" s="14" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="17" t="n"/>
+      <c r="B186" s="14" t="n"/>
+      <c r="C186" s="14" t="n"/>
+      <c r="D186" s="14" t="n"/>
+      <c r="E186" s="14" t="n"/>
+      <c r="F186" s="15" t="n"/>
+      <c r="G186" s="14" t="n"/>
+      <c r="H186" s="17" t="n"/>
+      <c r="I186" s="37" t="n"/>
+      <c r="J186" s="14" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="17" t="n"/>
+      <c r="B187" s="14" t="n"/>
+      <c r="C187" s="14" t="n"/>
+      <c r="D187" s="14" t="n"/>
+      <c r="E187" s="14" t="n"/>
+      <c r="F187" s="15" t="n"/>
+      <c r="G187" s="14" t="n"/>
+      <c r="H187" s="17" t="n"/>
+      <c r="I187" s="37" t="n"/>
+      <c r="J187" s="14" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="17" t="n"/>
+      <c r="B188" s="14" t="n"/>
+      <c r="C188" s="14" t="n"/>
+      <c r="D188" s="14" t="n"/>
+      <c r="E188" s="14" t="n"/>
+      <c r="F188" s="15" t="n"/>
+      <c r="G188" s="14" t="n"/>
+      <c r="H188" s="17" t="n"/>
+      <c r="I188" s="37" t="n"/>
+      <c r="J188" s="14" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="17" t="n"/>
+      <c r="B189" s="14" t="n"/>
+      <c r="C189" s="14" t="n"/>
+      <c r="D189" s="14" t="n"/>
+      <c r="E189" s="14" t="n"/>
+      <c r="F189" s="15" t="n"/>
+      <c r="G189" s="14" t="n"/>
+      <c r="H189" s="17" t="n"/>
+      <c r="I189" s="37" t="n"/>
+      <c r="J189" s="14" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="17" t="n"/>
+      <c r="B190" s="14" t="n"/>
+      <c r="C190" s="14" t="n"/>
+      <c r="D190" s="14" t="n"/>
+      <c r="E190" s="14" t="n"/>
+      <c r="F190" s="15" t="n"/>
+      <c r="G190" s="14" t="n"/>
+      <c r="H190" s="17" t="n"/>
+      <c r="I190" s="37" t="n"/>
+      <c r="J190" s="14" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="17" t="n"/>
+      <c r="B191" s="14" t="n"/>
+      <c r="C191" s="14" t="n"/>
+      <c r="D191" s="14" t="n"/>
+      <c r="E191" s="14" t="n"/>
+      <c r="F191" s="15" t="n"/>
+      <c r="G191" s="14" t="n"/>
+      <c r="H191" s="17" t="n"/>
+      <c r="I191" s="37" t="n"/>
+      <c r="J191" s="14" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="17" t="n"/>
+      <c r="B192" s="14" t="n"/>
+      <c r="C192" s="14" t="n"/>
+      <c r="D192" s="14" t="n"/>
+      <c r="E192" s="14" t="n"/>
+      <c r="F192" s="15" t="n"/>
+      <c r="G192" s="14" t="n"/>
+      <c r="H192" s="17" t="n"/>
+      <c r="I192" s="37" t="n"/>
+      <c r="J192" s="14" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="17" t="n"/>
+      <c r="B193" s="14" t="n"/>
+      <c r="C193" s="14" t="n"/>
+      <c r="D193" s="14" t="n"/>
+      <c r="E193" s="14" t="n"/>
+      <c r="F193" s="15" t="n"/>
+      <c r="G193" s="14" t="n"/>
+      <c r="H193" s="17" t="n"/>
+      <c r="I193" s="37" t="n"/>
+      <c r="J193" s="14" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="17" t="n"/>
+      <c r="B194" s="14" t="n"/>
+      <c r="C194" s="14" t="n"/>
+      <c r="D194" s="14" t="n"/>
+      <c r="E194" s="14" t="n"/>
+      <c r="F194" s="15" t="n"/>
+      <c r="G194" s="14" t="n"/>
+      <c r="H194" s="17" t="n"/>
+      <c r="I194" s="37" t="n"/>
+      <c r="J194" s="14" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="17" t="n"/>
+      <c r="B195" s="14" t="n"/>
+      <c r="C195" s="14" t="n"/>
+      <c r="D195" s="14" t="n"/>
+      <c r="E195" s="14" t="n"/>
+      <c r="F195" s="15" t="n"/>
+      <c r="G195" s="14" t="n"/>
+      <c r="H195" s="17" t="n"/>
+      <c r="I195" s="37" t="n"/>
+      <c r="J195" s="14" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="17" t="n"/>
+      <c r="B196" s="14" t="n"/>
+      <c r="C196" s="14" t="n"/>
+      <c r="D196" s="14" t="n"/>
+      <c r="E196" s="14" t="n"/>
+      <c r="F196" s="15" t="n"/>
+      <c r="G196" s="14" t="n"/>
+      <c r="H196" s="17" t="n"/>
+      <c r="I196" s="37" t="n"/>
+      <c r="J196" s="14" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="17" t="n"/>
+      <c r="B197" s="14" t="n"/>
+      <c r="C197" s="14" t="n"/>
+      <c r="D197" s="14" t="n"/>
+      <c r="E197" s="14" t="n"/>
+      <c r="F197" s="15" t="n"/>
+      <c r="G197" s="14" t="n"/>
+      <c r="H197" s="17" t="n"/>
+      <c r="I197" s="37" t="n"/>
+      <c r="J197" s="14" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="17" t="n"/>
+      <c r="B198" s="14" t="n"/>
+      <c r="C198" s="14" t="n"/>
+      <c r="D198" s="14" t="n"/>
+      <c r="E198" s="14" t="n"/>
+      <c r="F198" s="15" t="n"/>
+      <c r="G198" s="14" t="n"/>
+      <c r="H198" s="17" t="n"/>
+      <c r="I198" s="37" t="n"/>
+      <c r="J198" s="14" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="17" t="n"/>
+      <c r="B199" s="14" t="n"/>
+      <c r="C199" s="14" t="n"/>
+      <c r="D199" s="14" t="n"/>
+      <c r="E199" s="14" t="n"/>
+      <c r="F199" s="15" t="n"/>
+      <c r="G199" s="14" t="n"/>
+      <c r="H199" s="17" t="n"/>
+      <c r="I199" s="37" t="n"/>
+      <c r="J199" s="14" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="17" t="n"/>
+      <c r="B200" s="14" t="n"/>
+      <c r="C200" s="14" t="n"/>
+      <c r="D200" s="14" t="n"/>
+      <c r="E200" s="14" t="n"/>
+      <c r="F200" s="15" t="n"/>
+      <c r="G200" s="14" t="n"/>
+      <c r="H200" s="17" t="n"/>
+      <c r="I200" s="37" t="n"/>
+      <c r="J200" s="14" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="17" t="n"/>
+      <c r="B201" s="14" t="n"/>
+      <c r="C201" s="14" t="n"/>
+      <c r="D201" s="14" t="n"/>
+      <c r="E201" s="14" t="n"/>
+      <c r="F201" s="15" t="n"/>
+      <c r="G201" s="14" t="n"/>
+      <c r="H201" s="17" t="n"/>
+      <c r="I201" s="37" t="n"/>
+      <c r="J201" s="14" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="17" t="n"/>
+      <c r="B202" s="14" t="n"/>
+      <c r="C202" s="14" t="n"/>
+      <c r="D202" s="14" t="n"/>
+      <c r="E202" s="14" t="n"/>
+      <c r="F202" s="15" t="n"/>
+      <c r="G202" s="14" t="n"/>
+      <c r="H202" s="17" t="n"/>
+      <c r="I202" s="37" t="n"/>
+      <c r="J202" s="14" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="17" t="n"/>
+      <c r="B203" s="14" t="n"/>
+      <c r="C203" s="14" t="n"/>
+      <c r="D203" s="14" t="n"/>
+      <c r="E203" s="14" t="n"/>
+      <c r="F203" s="15" t="n"/>
+      <c r="G203" s="14" t="n"/>
+      <c r="H203" s="17" t="n"/>
+      <c r="I203" s="37" t="n"/>
+      <c r="J203" s="14" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="17" t="n"/>
+      <c r="B204" s="14" t="n"/>
+      <c r="C204" s="14" t="n"/>
+      <c r="D204" s="14" t="n"/>
+      <c r="E204" s="14" t="n"/>
+      <c r="F204" s="15" t="n"/>
+      <c r="G204" s="14" t="n"/>
+      <c r="H204" s="17" t="n"/>
+      <c r="I204" s="37" t="n"/>
+      <c r="J204" s="14" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="17" t="n"/>
+      <c r="B205" s="14" t="n"/>
+      <c r="C205" s="14" t="n"/>
+      <c r="D205" s="14" t="n"/>
+      <c r="E205" s="14" t="n"/>
+      <c r="F205" s="15" t="n"/>
+      <c r="G205" s="14" t="n"/>
+      <c r="H205" s="17" t="n"/>
+      <c r="I205" s="37" t="n"/>
+      <c r="J205" s="14" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="17" t="n"/>
+      <c r="B206" s="14" t="n"/>
+      <c r="C206" s="14" t="n"/>
+      <c r="D206" s="14" t="n"/>
+      <c r="E206" s="14" t="n"/>
+      <c r="F206" s="15" t="n"/>
+      <c r="G206" s="14" t="n"/>
+      <c r="H206" s="17" t="n"/>
+      <c r="I206" s="37" t="n"/>
+      <c r="J206" s="14" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="17" t="n"/>
+      <c r="B207" s="14" t="n"/>
+      <c r="C207" s="14" t="n"/>
+      <c r="D207" s="14" t="n"/>
+      <c r="E207" s="14" t="n"/>
+      <c r="F207" s="15" t="n"/>
+      <c r="G207" s="14" t="n"/>
+      <c r="H207" s="17" t="n"/>
+      <c r="I207" s="37" t="n"/>
+      <c r="J207" s="14" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="17" t="n"/>
+      <c r="B208" s="14" t="n"/>
+      <c r="C208" s="14" t="n"/>
+      <c r="D208" s="14" t="n"/>
+      <c r="E208" s="14" t="n"/>
+      <c r="F208" s="15" t="n"/>
+      <c r="G208" s="14" t="n"/>
+      <c r="H208" s="17" t="n"/>
+      <c r="I208" s="37" t="n"/>
+      <c r="J208" s="14" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="17" t="n"/>
+      <c r="B209" s="14" t="n"/>
+      <c r="C209" s="14" t="n"/>
+      <c r="D209" s="14" t="n"/>
+      <c r="E209" s="14" t="n"/>
+      <c r="F209" s="15" t="n"/>
+      <c r="G209" s="14" t="n"/>
+      <c r="H209" s="17" t="n"/>
+      <c r="I209" s="37" t="n"/>
+      <c r="J209" s="14" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="17" t="n"/>
+      <c r="B210" s="14" t="n"/>
+      <c r="C210" s="14" t="n"/>
+      <c r="D210" s="14" t="n"/>
+      <c r="E210" s="14" t="n"/>
+      <c r="F210" s="15" t="n"/>
+      <c r="G210" s="14" t="n"/>
+      <c r="H210" s="17" t="n"/>
+      <c r="I210" s="37" t="n"/>
+      <c r="J210" s="14" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="17" t="n"/>
+      <c r="B211" s="14" t="n"/>
+      <c r="C211" s="14" t="n"/>
+      <c r="D211" s="14" t="n"/>
+      <c r="E211" s="14" t="n"/>
+      <c r="F211" s="15" t="n"/>
+      <c r="G211" s="14" t="n"/>
+      <c r="H211" s="17" t="n"/>
+      <c r="I211" s="37" t="n"/>
+      <c r="J211" s="14" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="17" t="n"/>
+      <c r="B212" s="14" t="n"/>
+      <c r="C212" s="14" t="n"/>
+      <c r="D212" s="14" t="n"/>
+      <c r="E212" s="14" t="n"/>
+      <c r="F212" s="15" t="n"/>
+      <c r="G212" s="14" t="n"/>
+      <c r="H212" s="17" t="n"/>
+      <c r="I212" s="37" t="n"/>
+      <c r="J212" s="14" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="17" t="n"/>
+      <c r="B213" s="14" t="n"/>
+      <c r="C213" s="14" t="n"/>
+      <c r="D213" s="14" t="n"/>
+      <c r="E213" s="14" t="n"/>
+      <c r="F213" s="15" t="n"/>
+      <c r="G213" s="14" t="n"/>
+      <c r="H213" s="17" t="n"/>
+      <c r="I213" s="37" t="n"/>
+      <c r="J213" s="14" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="17" t="n"/>
+      <c r="B214" s="14" t="n"/>
+      <c r="C214" s="14" t="n"/>
+      <c r="D214" s="14" t="n"/>
+      <c r="E214" s="14" t="n"/>
+      <c r="F214" s="15" t="n"/>
+      <c r="G214" s="14" t="n"/>
+      <c r="H214" s="17" t="n"/>
+      <c r="I214" s="37" t="n"/>
+      <c r="J214" s="14" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="17" t="n"/>
+      <c r="B215" s="14" t="n"/>
+      <c r="C215" s="14" t="n"/>
+      <c r="D215" s="14" t="n"/>
+      <c r="E215" s="14" t="n"/>
+      <c r="F215" s="15" t="n"/>
+      <c r="G215" s="14" t="n"/>
+      <c r="H215" s="17" t="n"/>
+      <c r="I215" s="37" t="n"/>
+      <c r="J215" s="14" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="17" t="n"/>
+      <c r="B216" s="14" t="n"/>
+      <c r="C216" s="14" t="n"/>
+      <c r="D216" s="14" t="n"/>
+      <c r="E216" s="14" t="n"/>
+      <c r="F216" s="15" t="n"/>
+      <c r="G216" s="14" t="n"/>
+      <c r="H216" s="17" t="n"/>
+      <c r="I216" s="37" t="n"/>
+      <c r="J216" s="14" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="17" t="n"/>
+      <c r="B217" s="14" t="n"/>
+      <c r="C217" s="14" t="n"/>
+      <c r="D217" s="14" t="n"/>
+      <c r="E217" s="14" t="n"/>
+      <c r="F217" s="15" t="n"/>
+      <c r="G217" s="14" t="n"/>
+      <c r="H217" s="17" t="n"/>
+      <c r="I217" s="37" t="n"/>
+      <c r="J217" s="14" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="17" t="n"/>
+      <c r="B218" s="14" t="n"/>
+      <c r="C218" s="14" t="n"/>
+      <c r="D218" s="14" t="n"/>
+      <c r="E218" s="14" t="n"/>
+      <c r="F218" s="15" t="n"/>
+      <c r="G218" s="14" t="n"/>
+      <c r="H218" s="17" t="n"/>
+      <c r="I218" s="37" t="n"/>
+      <c r="J218" s="14" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="17" t="n"/>
+      <c r="B219" s="14" t="n"/>
+      <c r="C219" s="14" t="n"/>
+      <c r="D219" s="14" t="n"/>
+      <c r="E219" s="14" t="n"/>
+      <c r="F219" s="15" t="n"/>
+      <c r="G219" s="14" t="n"/>
+      <c r="H219" s="17" t="n"/>
+      <c r="I219" s="37" t="n"/>
+      <c r="J219" s="14" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="17" t="n"/>
+      <c r="B220" s="14" t="n"/>
+      <c r="C220" s="14" t="n"/>
+      <c r="D220" s="14" t="n"/>
+      <c r="E220" s="14" t="n"/>
+      <c r="F220" s="15" t="n"/>
+      <c r="G220" s="14" t="n"/>
+      <c r="H220" s="17" t="n"/>
+      <c r="I220" s="37" t="n"/>
+      <c r="J220" s="14" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="17" t="n"/>
+      <c r="B221" s="14" t="n"/>
+      <c r="C221" s="14" t="n"/>
+      <c r="D221" s="14" t="n"/>
+      <c r="E221" s="14" t="n"/>
+      <c r="F221" s="15" t="n"/>
+      <c r="G221" s="14" t="n"/>
+      <c r="H221" s="17" t="n"/>
+      <c r="I221" s="37" t="n"/>
+      <c r="J221" s="14" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="17" t="n"/>
+      <c r="B222" s="14" t="n"/>
+      <c r="C222" s="14" t="n"/>
+      <c r="D222" s="14" t="n"/>
+      <c r="E222" s="14" t="n"/>
+      <c r="F222" s="15" t="n"/>
+      <c r="G222" s="14" t="n"/>
+      <c r="H222" s="17" t="n"/>
+      <c r="I222" s="37" t="n"/>
+      <c r="J222" s="14" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="17" t="n"/>
+      <c r="B223" s="14" t="n"/>
+      <c r="C223" s="14" t="n"/>
+      <c r="D223" s="14" t="n"/>
+      <c r="E223" s="14" t="n"/>
+      <c r="F223" s="15" t="n"/>
+      <c r="G223" s="14" t="n"/>
+      <c r="H223" s="17" t="n"/>
+      <c r="I223" s="37" t="n"/>
+      <c r="J223" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A23:J223"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Classify Noelia Caballero transfers as verdulería food.
Always map those Mercado Pago transfers to Almacén Sol with COMIDA · VERDULERÍA.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1487,7 +1487,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1572,32 +1571,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2462,15 +2435,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B32" s="17" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="27" t="n"/>
+      <c r="B32" s="17" t="n">
+        <v>46026</v>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Verdulería (Noelia Caballero)</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="n">
+        <v>8180</v>
+      </c>
       <c r="E32" s="28" t="n"/>
       <c r="F32" s="15">
         <f>IF(OR(D32&lt;&gt;"",E32&lt;&gt;""),IF(D32="",0,D32)+IF(E32="",0,E32),"")</f>
         <v/>
       </c>
-      <c r="G32" s="14" t="n"/>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
@@ -2674,6 +2659,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3616,6 +3602,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4498,6 +4485,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5392,6 +5380,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6214,6 +6203,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7132,6 +7122,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7528,15 +7519,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B271" s="17" t="n"/>
-      <c r="C271" s="14" t="n"/>
-      <c r="D271" s="27" t="n"/>
+      <c r="B271" s="17" t="n">
+        <v>46217</v>
+      </c>
+      <c r="C271" s="14" t="inlineStr">
+        <is>
+          <t>Verdulería (Noelia Caballero)</t>
+        </is>
+      </c>
+      <c r="D271" s="27" t="n">
+        <v>8977</v>
+      </c>
       <c r="E271" s="28" t="n"/>
       <c r="F271" s="15">
         <f>IF(OR(D271&lt;&gt;"",E271&lt;&gt;""),IF(D271="",0,D271)+IF(E271="",0,E271),"")</f>
         <v/>
       </c>
-      <c r="G271" s="14" t="n"/>
+      <c r="G271" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Add Ingresos sheet for Mercado Pago money-in movements.
Track received transfers separately from CIUDAD expenses and load known income entries from the catalog.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Detalle" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Dinero Retirado" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Inversión" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Ingresos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle'!$A$3:$I$51</definedName>
@@ -26,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +86,10 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="9">
@@ -200,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -247,6 +252,8 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="12" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -612,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1487,6 +1494,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1571,6 +1579,38 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>• Ingresos de dinero: hoja "Ingresos" (transferencias recibidas; no suma al total de gastos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2659,7 +2699,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3602,7 +3641,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4485,7 +4523,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5380,7 +5417,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6203,7 +6239,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7122,7 +7157,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -17279,4 +17313,1445 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F142"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132 — Ingresos de dinero</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Ingresos / transferencias recibidas (Mercado Pago «Ingreso de dinero»). No entra en el total de gastos de la hoja 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Resumen por mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Total ingresos</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>SUMIF($B$23:$B$142,A6,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>SUMIF($B$23:$B$142,A7,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>SUMIF($B$23:$B$142,A8,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>SUMIF($B$23:$B$142,A9,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
+        <f>SUMIF($B$23:$B$142,A10,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B11" s="15">
+        <f>SUMIF($B$23:$B$142,A11,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>SUMIF($B$23:$B$142,A12,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B13" s="15">
+        <f>SUMIF($B$23:$B$142,A13,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>SUMIF($B$23:$B$142,A14,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>SUMIF($B$23:$B$142,A15,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>SUMIF($B$23:$B$142,A16,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>SUMIF($B$23:$B$142,A17,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL AÑO</t>
+        </is>
+      </c>
+      <c r="B18" s="39">
+        <f>SUM(B6:B17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C22" s="34" t="inlineStr">
+        <is>
+          <t>Concepto / origen</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="E22" s="34" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Maria Soledad Martinez</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Florencia Ivana Risi</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Gabriela Reggio</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Antonela Beatriz Guidobono</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Maria Lujan Paz</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>ingresos varios</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>117000</v>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>recibidas 39k x3 · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>ingresos varios</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>35070</v>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>recibidas ~34k x6 · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Tamara Ginesin</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>recibida · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Ana Magariños</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>recibida · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>4699990</v>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>reintegro ML · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Carlos Farinella</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>110000</v>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>recibida · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Carlos Farinella</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Ingreso de dinero</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>recibida · hoja Ingresos (no gasto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n"/>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="n"/>
+      <c r="B36" s="14" t="n"/>
+      <c r="C36" s="14" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="14" t="n"/>
+      <c r="F36" s="14" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="n"/>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="n"/>
+      <c r="B38" s="14" t="n"/>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n"/>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="14" t="n"/>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="14" t="n"/>
+      <c r="F40" s="14" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n"/>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="n"/>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="14" t="n"/>
+      <c r="F43" s="14" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="14" t="n"/>
+      <c r="C44" s="14" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="14" t="n"/>
+      <c r="F44" s="14" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="n"/>
+      <c r="B46" s="14" t="n"/>
+      <c r="C46" s="14" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="14" t="n"/>
+      <c r="F46" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="14" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="n"/>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="14" t="n"/>
+      <c r="F48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n"/>
+      <c r="B49" s="14" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="14" t="n"/>
+      <c r="F49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="n"/>
+      <c r="B50" s="14" t="n"/>
+      <c r="C50" s="14" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="14" t="n"/>
+      <c r="F50" s="14" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="14" t="n"/>
+      <c r="C51" s="14" t="n"/>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="14" t="n"/>
+      <c r="F51" s="14" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="n"/>
+      <c r="B52" s="14" t="n"/>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="14" t="n"/>
+      <c r="F52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="14" t="n"/>
+      <c r="F53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="14" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="14" t="n"/>
+      <c r="F54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="14" t="n"/>
+      <c r="F55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="n"/>
+      <c r="B56" s="14" t="n"/>
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="14" t="n"/>
+      <c r="F56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="n"/>
+      <c r="B57" s="14" t="n"/>
+      <c r="C57" s="14" t="n"/>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="14" t="n"/>
+      <c r="F57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="n"/>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="14" t="n"/>
+      <c r="F58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="n"/>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="15" t="n"/>
+      <c r="E59" s="14" t="n"/>
+      <c r="F59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="n"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="14" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="14" t="n"/>
+      <c r="F60" s="14" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="n"/>
+      <c r="B61" s="14" t="n"/>
+      <c r="C61" s="14" t="n"/>
+      <c r="D61" s="15" t="n"/>
+      <c r="E61" s="14" t="n"/>
+      <c r="F61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="n"/>
+      <c r="B62" s="14" t="n"/>
+      <c r="C62" s="14" t="n"/>
+      <c r="D62" s="15" t="n"/>
+      <c r="E62" s="14" t="n"/>
+      <c r="F62" s="14" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="n"/>
+      <c r="B63" s="14" t="n"/>
+      <c r="C63" s="14" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="14" t="n"/>
+      <c r="F63" s="14" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="n"/>
+      <c r="B64" s="14" t="n"/>
+      <c r="C64" s="14" t="n"/>
+      <c r="D64" s="15" t="n"/>
+      <c r="E64" s="14" t="n"/>
+      <c r="F64" s="14" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="n"/>
+      <c r="B65" s="14" t="n"/>
+      <c r="C65" s="14" t="n"/>
+      <c r="D65" s="15" t="n"/>
+      <c r="E65" s="14" t="n"/>
+      <c r="F65" s="14" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="n"/>
+      <c r="B66" s="14" t="n"/>
+      <c r="C66" s="14" t="n"/>
+      <c r="D66" s="15" t="n"/>
+      <c r="E66" s="14" t="n"/>
+      <c r="F66" s="14" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="n"/>
+      <c r="B67" s="14" t="n"/>
+      <c r="C67" s="14" t="n"/>
+      <c r="D67" s="15" t="n"/>
+      <c r="E67" s="14" t="n"/>
+      <c r="F67" s="14" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="n"/>
+      <c r="B68" s="14" t="n"/>
+      <c r="C68" s="14" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="14" t="n"/>
+      <c r="F68" s="14" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="n"/>
+      <c r="B69" s="14" t="n"/>
+      <c r="C69" s="14" t="n"/>
+      <c r="D69" s="15" t="n"/>
+      <c r="E69" s="14" t="n"/>
+      <c r="F69" s="14" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="n"/>
+      <c r="B70" s="14" t="n"/>
+      <c r="C70" s="14" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="14" t="n"/>
+      <c r="F70" s="14" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="n"/>
+      <c r="B71" s="14" t="n"/>
+      <c r="C71" s="14" t="n"/>
+      <c r="D71" s="15" t="n"/>
+      <c r="E71" s="14" t="n"/>
+      <c r="F71" s="14" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="n"/>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="15" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="n"/>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="14" t="n"/>
+      <c r="D73" s="15" t="n"/>
+      <c r="E73" s="14" t="n"/>
+      <c r="F73" s="14" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="n"/>
+      <c r="B74" s="14" t="n"/>
+      <c r="C74" s="14" t="n"/>
+      <c r="D74" s="15" t="n"/>
+      <c r="E74" s="14" t="n"/>
+      <c r="F74" s="14" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="17" t="n"/>
+      <c r="B75" s="14" t="n"/>
+      <c r="C75" s="14" t="n"/>
+      <c r="D75" s="15" t="n"/>
+      <c r="E75" s="14" t="n"/>
+      <c r="F75" s="14" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="n"/>
+      <c r="B76" s="14" t="n"/>
+      <c r="C76" s="14" t="n"/>
+      <c r="D76" s="15" t="n"/>
+      <c r="E76" s="14" t="n"/>
+      <c r="F76" s="14" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="n"/>
+      <c r="B77" s="14" t="n"/>
+      <c r="C77" s="14" t="n"/>
+      <c r="D77" s="15" t="n"/>
+      <c r="E77" s="14" t="n"/>
+      <c r="F77" s="14" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="n"/>
+      <c r="B78" s="14" t="n"/>
+      <c r="C78" s="14" t="n"/>
+      <c r="D78" s="15" t="n"/>
+      <c r="E78" s="14" t="n"/>
+      <c r="F78" s="14" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="n"/>
+      <c r="B79" s="14" t="n"/>
+      <c r="C79" s="14" t="n"/>
+      <c r="D79" s="15" t="n"/>
+      <c r="E79" s="14" t="n"/>
+      <c r="F79" s="14" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="n"/>
+      <c r="B80" s="14" t="n"/>
+      <c r="C80" s="14" t="n"/>
+      <c r="D80" s="15" t="n"/>
+      <c r="E80" s="14" t="n"/>
+      <c r="F80" s="14" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="n"/>
+      <c r="B81" s="14" t="n"/>
+      <c r="C81" s="14" t="n"/>
+      <c r="D81" s="15" t="n"/>
+      <c r="E81" s="14" t="n"/>
+      <c r="F81" s="14" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="n"/>
+      <c r="B82" s="14" t="n"/>
+      <c r="C82" s="14" t="n"/>
+      <c r="D82" s="15" t="n"/>
+      <c r="E82" s="14" t="n"/>
+      <c r="F82" s="14" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="n"/>
+      <c r="B83" s="14" t="n"/>
+      <c r="C83" s="14" t="n"/>
+      <c r="D83" s="15" t="n"/>
+      <c r="E83" s="14" t="n"/>
+      <c r="F83" s="14" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="n"/>
+      <c r="B84" s="14" t="n"/>
+      <c r="C84" s="14" t="n"/>
+      <c r="D84" s="15" t="n"/>
+      <c r="E84" s="14" t="n"/>
+      <c r="F84" s="14" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="n"/>
+      <c r="B85" s="14" t="n"/>
+      <c r="C85" s="14" t="n"/>
+      <c r="D85" s="15" t="n"/>
+      <c r="E85" s="14" t="n"/>
+      <c r="F85" s="14" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="n"/>
+      <c r="B86" s="14" t="n"/>
+      <c r="C86" s="14" t="n"/>
+      <c r="D86" s="15" t="n"/>
+      <c r="E86" s="14" t="n"/>
+      <c r="F86" s="14" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="n"/>
+      <c r="B87" s="14" t="n"/>
+      <c r="C87" s="14" t="n"/>
+      <c r="D87" s="15" t="n"/>
+      <c r="E87" s="14" t="n"/>
+      <c r="F87" s="14" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="n"/>
+      <c r="B88" s="14" t="n"/>
+      <c r="C88" s="14" t="n"/>
+      <c r="D88" s="15" t="n"/>
+      <c r="E88" s="14" t="n"/>
+      <c r="F88" s="14" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="17" t="n"/>
+      <c r="B89" s="14" t="n"/>
+      <c r="C89" s="14" t="n"/>
+      <c r="D89" s="15" t="n"/>
+      <c r="E89" s="14" t="n"/>
+      <c r="F89" s="14" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="n"/>
+      <c r="B90" s="14" t="n"/>
+      <c r="C90" s="14" t="n"/>
+      <c r="D90" s="15" t="n"/>
+      <c r="E90" s="14" t="n"/>
+      <c r="F90" s="14" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="n"/>
+      <c r="B91" s="14" t="n"/>
+      <c r="C91" s="14" t="n"/>
+      <c r="D91" s="15" t="n"/>
+      <c r="E91" s="14" t="n"/>
+      <c r="F91" s="14" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="n"/>
+      <c r="B92" s="14" t="n"/>
+      <c r="C92" s="14" t="n"/>
+      <c r="D92" s="15" t="n"/>
+      <c r="E92" s="14" t="n"/>
+      <c r="F92" s="14" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="n"/>
+      <c r="B93" s="14" t="n"/>
+      <c r="C93" s="14" t="n"/>
+      <c r="D93" s="15" t="n"/>
+      <c r="E93" s="14" t="n"/>
+      <c r="F93" s="14" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="n"/>
+      <c r="B94" s="14" t="n"/>
+      <c r="C94" s="14" t="n"/>
+      <c r="D94" s="15" t="n"/>
+      <c r="E94" s="14" t="n"/>
+      <c r="F94" s="14" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="n"/>
+      <c r="B95" s="14" t="n"/>
+      <c r="C95" s="14" t="n"/>
+      <c r="D95" s="15" t="n"/>
+      <c r="E95" s="14" t="n"/>
+      <c r="F95" s="14" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="n"/>
+      <c r="B96" s="14" t="n"/>
+      <c r="C96" s="14" t="n"/>
+      <c r="D96" s="15" t="n"/>
+      <c r="E96" s="14" t="n"/>
+      <c r="F96" s="14" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="n"/>
+      <c r="B97" s="14" t="n"/>
+      <c r="C97" s="14" t="n"/>
+      <c r="D97" s="15" t="n"/>
+      <c r="E97" s="14" t="n"/>
+      <c r="F97" s="14" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="n"/>
+      <c r="B98" s="14" t="n"/>
+      <c r="C98" s="14" t="n"/>
+      <c r="D98" s="15" t="n"/>
+      <c r="E98" s="14" t="n"/>
+      <c r="F98" s="14" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="17" t="n"/>
+      <c r="B99" s="14" t="n"/>
+      <c r="C99" s="14" t="n"/>
+      <c r="D99" s="15" t="n"/>
+      <c r="E99" s="14" t="n"/>
+      <c r="F99" s="14" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="17" t="n"/>
+      <c r="B100" s="14" t="n"/>
+      <c r="C100" s="14" t="n"/>
+      <c r="D100" s="15" t="n"/>
+      <c r="E100" s="14" t="n"/>
+      <c r="F100" s="14" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="17" t="n"/>
+      <c r="B101" s="14" t="n"/>
+      <c r="C101" s="14" t="n"/>
+      <c r="D101" s="15" t="n"/>
+      <c r="E101" s="14" t="n"/>
+      <c r="F101" s="14" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="17" t="n"/>
+      <c r="B102" s="14" t="n"/>
+      <c r="C102" s="14" t="n"/>
+      <c r="D102" s="15" t="n"/>
+      <c r="E102" s="14" t="n"/>
+      <c r="F102" s="14" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="17" t="n"/>
+      <c r="B103" s="14" t="n"/>
+      <c r="C103" s="14" t="n"/>
+      <c r="D103" s="15" t="n"/>
+      <c r="E103" s="14" t="n"/>
+      <c r="F103" s="14" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="17" t="n"/>
+      <c r="B104" s="14" t="n"/>
+      <c r="C104" s="14" t="n"/>
+      <c r="D104" s="15" t="n"/>
+      <c r="E104" s="14" t="n"/>
+      <c r="F104" s="14" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="17" t="n"/>
+      <c r="B105" s="14" t="n"/>
+      <c r="C105" s="14" t="n"/>
+      <c r="D105" s="15" t="n"/>
+      <c r="E105" s="14" t="n"/>
+      <c r="F105" s="14" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="n"/>
+      <c r="B106" s="14" t="n"/>
+      <c r="C106" s="14" t="n"/>
+      <c r="D106" s="15" t="n"/>
+      <c r="E106" s="14" t="n"/>
+      <c r="F106" s="14" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="n"/>
+      <c r="B107" s="14" t="n"/>
+      <c r="C107" s="14" t="n"/>
+      <c r="D107" s="15" t="n"/>
+      <c r="E107" s="14" t="n"/>
+      <c r="F107" s="14" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="17" t="n"/>
+      <c r="B108" s="14" t="n"/>
+      <c r="C108" s="14" t="n"/>
+      <c r="D108" s="15" t="n"/>
+      <c r="E108" s="14" t="n"/>
+      <c r="F108" s="14" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="17" t="n"/>
+      <c r="B109" s="14" t="n"/>
+      <c r="C109" s="14" t="n"/>
+      <c r="D109" s="15" t="n"/>
+      <c r="E109" s="14" t="n"/>
+      <c r="F109" s="14" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="17" t="n"/>
+      <c r="B110" s="14" t="n"/>
+      <c r="C110" s="14" t="n"/>
+      <c r="D110" s="15" t="n"/>
+      <c r="E110" s="14" t="n"/>
+      <c r="F110" s="14" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="17" t="n"/>
+      <c r="B111" s="14" t="n"/>
+      <c r="C111" s="14" t="n"/>
+      <c r="D111" s="15" t="n"/>
+      <c r="E111" s="14" t="n"/>
+      <c r="F111" s="14" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="17" t="n"/>
+      <c r="B112" s="14" t="n"/>
+      <c r="C112" s="14" t="n"/>
+      <c r="D112" s="15" t="n"/>
+      <c r="E112" s="14" t="n"/>
+      <c r="F112" s="14" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="17" t="n"/>
+      <c r="B113" s="14" t="n"/>
+      <c r="C113" s="14" t="n"/>
+      <c r="D113" s="15" t="n"/>
+      <c r="E113" s="14" t="n"/>
+      <c r="F113" s="14" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="n"/>
+      <c r="B114" s="14" t="n"/>
+      <c r="C114" s="14" t="n"/>
+      <c r="D114" s="15" t="n"/>
+      <c r="E114" s="14" t="n"/>
+      <c r="F114" s="14" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="17" t="n"/>
+      <c r="B115" s="14" t="n"/>
+      <c r="C115" s="14" t="n"/>
+      <c r="D115" s="15" t="n"/>
+      <c r="E115" s="14" t="n"/>
+      <c r="F115" s="14" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="17" t="n"/>
+      <c r="B116" s="14" t="n"/>
+      <c r="C116" s="14" t="n"/>
+      <c r="D116" s="15" t="n"/>
+      <c r="E116" s="14" t="n"/>
+      <c r="F116" s="14" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="n"/>
+      <c r="B117" s="14" t="n"/>
+      <c r="C117" s="14" t="n"/>
+      <c r="D117" s="15" t="n"/>
+      <c r="E117" s="14" t="n"/>
+      <c r="F117" s="14" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="17" t="n"/>
+      <c r="B118" s="14" t="n"/>
+      <c r="C118" s="14" t="n"/>
+      <c r="D118" s="15" t="n"/>
+      <c r="E118" s="14" t="n"/>
+      <c r="F118" s="14" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="17" t="n"/>
+      <c r="B119" s="14" t="n"/>
+      <c r="C119" s="14" t="n"/>
+      <c r="D119" s="15" t="n"/>
+      <c r="E119" s="14" t="n"/>
+      <c r="F119" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="17" t="n"/>
+      <c r="B120" s="14" t="n"/>
+      <c r="C120" s="14" t="n"/>
+      <c r="D120" s="15" t="n"/>
+      <c r="E120" s="14" t="n"/>
+      <c r="F120" s="14" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="17" t="n"/>
+      <c r="B121" s="14" t="n"/>
+      <c r="C121" s="14" t="n"/>
+      <c r="D121" s="15" t="n"/>
+      <c r="E121" s="14" t="n"/>
+      <c r="F121" s="14" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="17" t="n"/>
+      <c r="B122" s="14" t="n"/>
+      <c r="C122" s="14" t="n"/>
+      <c r="D122" s="15" t="n"/>
+      <c r="E122" s="14" t="n"/>
+      <c r="F122" s="14" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="n"/>
+      <c r="B123" s="14" t="n"/>
+      <c r="C123" s="14" t="n"/>
+      <c r="D123" s="15" t="n"/>
+      <c r="E123" s="14" t="n"/>
+      <c r="F123" s="14" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="n"/>
+      <c r="B124" s="14" t="n"/>
+      <c r="C124" s="14" t="n"/>
+      <c r="D124" s="15" t="n"/>
+      <c r="E124" s="14" t="n"/>
+      <c r="F124" s="14" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="n"/>
+      <c r="B125" s="14" t="n"/>
+      <c r="C125" s="14" t="n"/>
+      <c r="D125" s="15" t="n"/>
+      <c r="E125" s="14" t="n"/>
+      <c r="F125" s="14" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="n"/>
+      <c r="B126" s="14" t="n"/>
+      <c r="C126" s="14" t="n"/>
+      <c r="D126" s="15" t="n"/>
+      <c r="E126" s="14" t="n"/>
+      <c r="F126" s="14" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="n"/>
+      <c r="B127" s="14" t="n"/>
+      <c r="C127" s="14" t="n"/>
+      <c r="D127" s="15" t="n"/>
+      <c r="E127" s="14" t="n"/>
+      <c r="F127" s="14" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="17" t="n"/>
+      <c r="B128" s="14" t="n"/>
+      <c r="C128" s="14" t="n"/>
+      <c r="D128" s="15" t="n"/>
+      <c r="E128" s="14" t="n"/>
+      <c r="F128" s="14" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="17" t="n"/>
+      <c r="B129" s="14" t="n"/>
+      <c r="C129" s="14" t="n"/>
+      <c r="D129" s="15" t="n"/>
+      <c r="E129" s="14" t="n"/>
+      <c r="F129" s="14" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="17" t="n"/>
+      <c r="B130" s="14" t="n"/>
+      <c r="C130" s="14" t="n"/>
+      <c r="D130" s="15" t="n"/>
+      <c r="E130" s="14" t="n"/>
+      <c r="F130" s="14" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="17" t="n"/>
+      <c r="B131" s="14" t="n"/>
+      <c r="C131" s="14" t="n"/>
+      <c r="D131" s="15" t="n"/>
+      <c r="E131" s="14" t="n"/>
+      <c r="F131" s="14" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="17" t="n"/>
+      <c r="B132" s="14" t="n"/>
+      <c r="C132" s="14" t="n"/>
+      <c r="D132" s="15" t="n"/>
+      <c r="E132" s="14" t="n"/>
+      <c r="F132" s="14" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="n"/>
+      <c r="B133" s="14" t="n"/>
+      <c r="C133" s="14" t="n"/>
+      <c r="D133" s="15" t="n"/>
+      <c r="E133" s="14" t="n"/>
+      <c r="F133" s="14" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="17" t="n"/>
+      <c r="B134" s="14" t="n"/>
+      <c r="C134" s="14" t="n"/>
+      <c r="D134" s="15" t="n"/>
+      <c r="E134" s="14" t="n"/>
+      <c r="F134" s="14" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="17" t="n"/>
+      <c r="B135" s="14" t="n"/>
+      <c r="C135" s="14" t="n"/>
+      <c r="D135" s="15" t="n"/>
+      <c r="E135" s="14" t="n"/>
+      <c r="F135" s="14" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="17" t="n"/>
+      <c r="B136" s="14" t="n"/>
+      <c r="C136" s="14" t="n"/>
+      <c r="D136" s="15" t="n"/>
+      <c r="E136" s="14" t="n"/>
+      <c r="F136" s="14" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="17" t="n"/>
+      <c r="B137" s="14" t="n"/>
+      <c r="C137" s="14" t="n"/>
+      <c r="D137" s="15" t="n"/>
+      <c r="E137" s="14" t="n"/>
+      <c r="F137" s="14" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="17" t="n"/>
+      <c r="B138" s="14" t="n"/>
+      <c r="C138" s="14" t="n"/>
+      <c r="D138" s="15" t="n"/>
+      <c r="E138" s="14" t="n"/>
+      <c r="F138" s="14" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="17" t="n"/>
+      <c r="B139" s="14" t="n"/>
+      <c r="C139" s="14" t="n"/>
+      <c r="D139" s="15" t="n"/>
+      <c r="E139" s="14" t="n"/>
+      <c r="F139" s="14" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="n"/>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="15" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="n"/>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="14" t="n"/>
+      <c r="D141" s="15" t="n"/>
+      <c r="E141" s="14" t="n"/>
+      <c r="F141" s="14" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="n"/>
+      <c r="B142" s="14" t="n"/>
+      <c r="C142" s="14" t="n"/>
+      <c r="D142" s="15" t="n"/>
+      <c r="E142" s="14" t="n"/>
+      <c r="F142" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Classify Nemuri Sushi purchases as COMIDA · SUSHI.
Move the July charge into Almacén Sol and keep that mapping for future Mercado Pago activity.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1494,7 +1494,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1586,31 +1585,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2699,6 +2673,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3641,6 +3616,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4523,6 +4499,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5417,6 +5394,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6239,6 +6217,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7157,6 +7136,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7581,15 +7561,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B272" s="17" t="n"/>
-      <c r="C272" s="14" t="n"/>
-      <c r="D272" s="27" t="n"/>
+      <c r="B272" s="17" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C272" s="14" t="inlineStr">
+        <is>
+          <t>Nemuri Sushi</t>
+        </is>
+      </c>
+      <c r="D272" s="27" t="n">
+        <v>195360</v>
+      </c>
       <c r="E272" s="28" t="n"/>
       <c r="F272" s="15">
         <f>IF(OR(D272&lt;&gt;"",E272&lt;&gt;""),IF(D272="",0,D272)+IF(E272="",0,E272),"")</f>
         <v/>
       </c>
-      <c r="G272" s="14" t="n"/>
+      <c r="G272" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · SUSHI</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Tag Coto, Carrefour, and Día as SUPERMERCADO in comments.
Keep those supermarket charges in Almacén Sol with a consistent SUPERMERCADO brand label.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1596,7 +1596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:G599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>MP · Carrefour</t>
+          <t>SUPERMERCADO · Carrefour</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>MP · Día Online</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>MP · Día</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>MP · Día</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>MP · Carrefour</t>
+          <t>SUPERMERCADO · Carrefour</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>MP · Día</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
-          <t>MP · Día</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
-          <t>MP · Día</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>MP · Carrefour</t>
+          <t>SUPERMERCADO · Carrefour</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
-          <t>MP · Carrefour</t>
+          <t>SUPERMERCADO · Carrefour</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="G93" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="G103" s="14" t="inlineStr">
         <is>
-          <t>MP · super</t>
+          <t>SUPERMERCADO · Coto</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="G142" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -4888,7 +4888,7 @@
       </c>
       <c r="G143" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Día</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="G144" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Coto</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="G172" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Carrefour</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="G181" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Coto</t>
         </is>
       </c>
     </row>
@@ -6718,7 +6718,7 @@
       </c>
       <c r="G231" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Carrefour</t>
         </is>
       </c>
     </row>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="G232" s="14" t="inlineStr">
         <is>
-          <t>MP · supermercado</t>
+          <t>SUPERMERCADO · Coto</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,11 @@
         <f>IF(OR(D259&lt;&gt;"",E259&lt;&gt;""),IF(D259="",0,D259)+IF(E259="",0,E259),"")</f>
         <v/>
       </c>
-      <c r="G259" s="14" t="n"/>
+      <c r="G259" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Coto</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="14" t="inlineStr">
@@ -7245,7 +7249,11 @@
         <f>IF(OR(D260&lt;&gt;"",E260&lt;&gt;""),IF(D260="",0,D260)+IF(E260="",0,E260),"")</f>
         <v/>
       </c>
-      <c r="G260" s="14" t="n"/>
+      <c r="G260" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO · Día</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="14" t="inlineStr">
@@ -7977,6 +7985,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8643,6 +8652,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9309,6 +9319,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9975,6 +9986,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10641,6 +10653,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11307,6 +11320,99 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Transferencias recibidas sheet for incoming transfers.
Replace the Ingresos sheet with a dedicated tracker for Mercado Pago Transferencia recibida movements.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Detalle" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Dinero Retirado" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Inversión" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Ingresos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Transferencias recibidas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle'!$A$3:$I$51</definedName>
@@ -1494,6 +1494,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1581,7 +1582,7 @@
     <row r="34">
       <c r="A34" s="30" t="inlineStr">
         <is>
-          <t>• Ingresos de dinero: hoja "Ingresos" (transferencias recibidas; no suma al total de gastos)</t>
+          <t>• Transferencias recibidas: hoja "Transferencias recibidas" (no suma al total de gastos)</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G599"/>
+  <dimension ref="A1:G506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2673,7 +2674,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3616,7 +3616,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4499,7 +4498,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5394,7 +5392,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6217,7 +6214,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7136,7 +7132,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7985,7 +7980,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8652,7 +8646,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9319,7 +9312,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9986,7 +9978,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10653,7 +10644,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11320,99 +11310,6 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17419,28 +17316,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CIUDAD 1132 — Ingresos de dinero</t>
+          <t>CIUDAD 1132 — Transferencias recibidas</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Ingresos / transferencias recibidas (Mercado Pago «Ingreso de dinero»). No entra en el total de gastos de la hoja 2026.</t>
+          <t>Movimientos Mercado Pago «Transferencia recibida». No entra en el total de gastos de la hoja 2026.</t>
         </is>
       </c>
     </row>
@@ -17459,7 +17356,7 @@
       </c>
       <c r="B5" s="34" t="inlineStr">
         <is>
-          <t>Total ingresos</t>
+          <t>Total recibido</t>
         </is>
       </c>
     </row>
@@ -17470,7 +17367,7 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>SUMIF($B$23:$B$142,A6,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A6,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17481,7 +17378,7 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>SUMIF($B$23:$B$142,A7,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A7,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17492,7 +17389,7 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>SUMIF($B$23:$B$142,A8,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A8,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17503,7 +17400,7 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>SUMIF($B$23:$B$142,A9,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A9,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17514,7 +17411,7 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>SUMIF($B$23:$B$142,A10,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A10,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17525,7 +17422,7 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>SUMIF($B$23:$B$142,A11,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A11,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17536,7 +17433,7 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>SUMIF($B$23:$B$142,A12,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A12,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17547,7 +17444,7 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>SUMIF($B$23:$B$142,A13,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A13,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17558,7 +17455,7 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>SUMIF($B$23:$B$142,A14,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A14,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17569,7 +17466,7 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>SUMIF($B$23:$B$142,A15,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A15,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17580,7 +17477,7 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUMIF($B$23:$B$142,A16,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A16,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17591,7 +17488,7 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>SUMIF($B$23:$B$142,A17,$D$23:$D$142)</f>
+        <f>SUMIF($B$23:$B$172,A17,$D$23:$D$172)</f>
         <v/>
       </c>
     </row>
@@ -17626,7 +17523,7 @@
       </c>
       <c r="C22" s="34" t="inlineStr">
         <is>
-          <t>Concepto / origen</t>
+          <t>Origen / concepto</t>
         </is>
       </c>
       <c r="D22" s="34" t="inlineStr">
@@ -17656,7 +17553,7 @@
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Maria Soledad Martinez</t>
+          <t>Florencia Ivana Risi</t>
         </is>
       </c>
       <c r="D23" s="15" t="n">
@@ -17664,12 +17561,12 @@
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+          <t>ingreso recibido · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17684,7 +17581,7 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Florencia Ivana Risi</t>
+          <t>Gabriela Reggio</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
@@ -17692,12 +17589,12 @@
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+          <t>ingreso recibido · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17712,7 +17609,7 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>Gabriela Reggio</t>
+          <t>Maria Soledad Martinez</t>
         </is>
       </c>
       <c r="D25" s="15" t="n">
@@ -17720,12 +17617,12 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+          <t>ingreso recibido · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17748,12 +17645,12 @@
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+          <t>ingreso recibido · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17776,12 +17673,12 @@
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>ingreso recibido · hoja Ingresos (no gasto)</t>
+          <t>ingreso recibido · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17804,12 +17701,12 @@
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>recibidas 39k x3 · hoja Ingresos (no gasto)</t>
+          <t>recibidas 39k x3 · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17832,12 +17729,12 @@
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>recibidas ~34k x6 · hoja Ingresos (no gasto)</t>
+          <t>recibidas ~34k x6 · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17860,12 +17757,12 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
-          <t>recibida · hoja Ingresos (no gasto)</t>
+          <t>recibida · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17888,12 +17785,12 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>recibida · hoja Ingresos (no gasto)</t>
+          <t>recibida · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17916,12 +17813,12 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
-          <t>reintegro ML · hoja Ingresos (no gasto)</t>
+          <t>reintegro ML · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17944,12 +17841,12 @@
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>recibida · hoja Ingresos (no gasto)</t>
+          <t>recibida · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -17972,12 +17869,12 @@
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Ingreso de dinero</t>
+          <t>Mercado Pago — Transferencia recibida</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>recibida · hoja Ingresos (no gasto)</t>
+          <t>recibida · hoja Transferencias recibidas (no gasto)</t>
         </is>
       </c>
     </row>
@@ -18844,6 +18741,246 @@
       <c r="D142" s="15" t="n"/>
       <c r="E142" s="14" t="n"/>
       <c r="F142" s="14" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="17" t="n"/>
+      <c r="B143" s="14" t="n"/>
+      <c r="C143" s="14" t="n"/>
+      <c r="D143" s="15" t="n"/>
+      <c r="E143" s="14" t="n"/>
+      <c r="F143" s="14" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="17" t="n"/>
+      <c r="B144" s="14" t="n"/>
+      <c r="C144" s="14" t="n"/>
+      <c r="D144" s="15" t="n"/>
+      <c r="E144" s="14" t="n"/>
+      <c r="F144" s="14" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="17" t="n"/>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="15" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="17" t="n"/>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="14" t="n"/>
+      <c r="D146" s="15" t="n"/>
+      <c r="E146" s="14" t="n"/>
+      <c r="F146" s="14" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="17" t="n"/>
+      <c r="B147" s="14" t="n"/>
+      <c r="C147" s="14" t="n"/>
+      <c r="D147" s="15" t="n"/>
+      <c r="E147" s="14" t="n"/>
+      <c r="F147" s="14" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="17" t="n"/>
+      <c r="B148" s="14" t="n"/>
+      <c r="C148" s="14" t="n"/>
+      <c r="D148" s="15" t="n"/>
+      <c r="E148" s="14" t="n"/>
+      <c r="F148" s="14" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="17" t="n"/>
+      <c r="B149" s="14" t="n"/>
+      <c r="C149" s="14" t="n"/>
+      <c r="D149" s="15" t="n"/>
+      <c r="E149" s="14" t="n"/>
+      <c r="F149" s="14" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="17" t="n"/>
+      <c r="B150" s="14" t="n"/>
+      <c r="C150" s="14" t="n"/>
+      <c r="D150" s="15" t="n"/>
+      <c r="E150" s="14" t="n"/>
+      <c r="F150" s="14" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="17" t="n"/>
+      <c r="B151" s="14" t="n"/>
+      <c r="C151" s="14" t="n"/>
+      <c r="D151" s="15" t="n"/>
+      <c r="E151" s="14" t="n"/>
+      <c r="F151" s="14" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="17" t="n"/>
+      <c r="B152" s="14" t="n"/>
+      <c r="C152" s="14" t="n"/>
+      <c r="D152" s="15" t="n"/>
+      <c r="E152" s="14" t="n"/>
+      <c r="F152" s="14" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="17" t="n"/>
+      <c r="B153" s="14" t="n"/>
+      <c r="C153" s="14" t="n"/>
+      <c r="D153" s="15" t="n"/>
+      <c r="E153" s="14" t="n"/>
+      <c r="F153" s="14" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="17" t="n"/>
+      <c r="B154" s="14" t="n"/>
+      <c r="C154" s="14" t="n"/>
+      <c r="D154" s="15" t="n"/>
+      <c r="E154" s="14" t="n"/>
+      <c r="F154" s="14" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="17" t="n"/>
+      <c r="B155" s="14" t="n"/>
+      <c r="C155" s="14" t="n"/>
+      <c r="D155" s="15" t="n"/>
+      <c r="E155" s="14" t="n"/>
+      <c r="F155" s="14" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="17" t="n"/>
+      <c r="B156" s="14" t="n"/>
+      <c r="C156" s="14" t="n"/>
+      <c r="D156" s="15" t="n"/>
+      <c r="E156" s="14" t="n"/>
+      <c r="F156" s="14" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="17" t="n"/>
+      <c r="B157" s="14" t="n"/>
+      <c r="C157" s="14" t="n"/>
+      <c r="D157" s="15" t="n"/>
+      <c r="E157" s="14" t="n"/>
+      <c r="F157" s="14" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="17" t="n"/>
+      <c r="B158" s="14" t="n"/>
+      <c r="C158" s="14" t="n"/>
+      <c r="D158" s="15" t="n"/>
+      <c r="E158" s="14" t="n"/>
+      <c r="F158" s="14" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="17" t="n"/>
+      <c r="B159" s="14" t="n"/>
+      <c r="C159" s="14" t="n"/>
+      <c r="D159" s="15" t="n"/>
+      <c r="E159" s="14" t="n"/>
+      <c r="F159" s="14" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="17" t="n"/>
+      <c r="B160" s="14" t="n"/>
+      <c r="C160" s="14" t="n"/>
+      <c r="D160" s="15" t="n"/>
+      <c r="E160" s="14" t="n"/>
+      <c r="F160" s="14" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="17" t="n"/>
+      <c r="B161" s="14" t="n"/>
+      <c r="C161" s="14" t="n"/>
+      <c r="D161" s="15" t="n"/>
+      <c r="E161" s="14" t="n"/>
+      <c r="F161" s="14" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="17" t="n"/>
+      <c r="B162" s="14" t="n"/>
+      <c r="C162" s="14" t="n"/>
+      <c r="D162" s="15" t="n"/>
+      <c r="E162" s="14" t="n"/>
+      <c r="F162" s="14" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="17" t="n"/>
+      <c r="B163" s="14" t="n"/>
+      <c r="C163" s="14" t="n"/>
+      <c r="D163" s="15" t="n"/>
+      <c r="E163" s="14" t="n"/>
+      <c r="F163" s="14" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="17" t="n"/>
+      <c r="B164" s="14" t="n"/>
+      <c r="C164" s="14" t="n"/>
+      <c r="D164" s="15" t="n"/>
+      <c r="E164" s="14" t="n"/>
+      <c r="F164" s="14" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="17" t="n"/>
+      <c r="B165" s="14" t="n"/>
+      <c r="C165" s="14" t="n"/>
+      <c r="D165" s="15" t="n"/>
+      <c r="E165" s="14" t="n"/>
+      <c r="F165" s="14" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="17" t="n"/>
+      <c r="B166" s="14" t="n"/>
+      <c r="C166" s="14" t="n"/>
+      <c r="D166" s="15" t="n"/>
+      <c r="E166" s="14" t="n"/>
+      <c r="F166" s="14" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="17" t="n"/>
+      <c r="B167" s="14" t="n"/>
+      <c r="C167" s="14" t="n"/>
+      <c r="D167" s="15" t="n"/>
+      <c r="E167" s="14" t="n"/>
+      <c r="F167" s="14" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="17" t="n"/>
+      <c r="B168" s="14" t="n"/>
+      <c r="C168" s="14" t="n"/>
+      <c r="D168" s="15" t="n"/>
+      <c r="E168" s="14" t="n"/>
+      <c r="F168" s="14" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="17" t="n"/>
+      <c r="B169" s="14" t="n"/>
+      <c r="C169" s="14" t="n"/>
+      <c r="D169" s="15" t="n"/>
+      <c r="E169" s="14" t="n"/>
+      <c r="F169" s="14" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="17" t="n"/>
+      <c r="B170" s="14" t="n"/>
+      <c r="C170" s="14" t="n"/>
+      <c r="D170" s="15" t="n"/>
+      <c r="E170" s="14" t="n"/>
+      <c r="F170" s="14" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="17" t="n"/>
+      <c r="B171" s="14" t="n"/>
+      <c r="C171" s="14" t="n"/>
+      <c r="D171" s="15" t="n"/>
+      <c r="E171" s="14" t="n"/>
+      <c r="F171" s="14" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="17" t="n"/>
+      <c r="B172" s="14" t="n"/>
+      <c r="C172" s="14" t="n"/>
+      <c r="D172" s="15" t="n"/>
+      <c r="E172" s="14" t="n"/>
+      <c r="F172" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Classify Valenti SA purchases as COMIDA with venue name.
Always map Valenti to Almacén Sol food with a COMIDA · VALENTI SA comment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1494,7 +1494,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -2674,6 +2673,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3616,6 +3616,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4498,6 +4499,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5392,6 +5394,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6214,6 +6217,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7132,6 +7136,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7330,7 +7335,7 @@
       </c>
       <c r="G263" s="14" t="inlineStr">
         <is>
-          <t>MP · Valenti</t>
+          <t>COMIDA · VALENTI SA</t>
         </is>
       </c>
     </row>
@@ -7358,7 +7363,7 @@
       </c>
       <c r="G264" s="14" t="inlineStr">
         <is>
-          <t>MP · Valenti</t>
+          <t>COMIDA · VALENTI SA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Expensas Consorcios sheet for consortium expense payments.
Route Consorcio De Propiet and related transfers as Pago de Expensas by property, never to Almacén Sol.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Dinero Retirado" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Inversión" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Transferencias recibidas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Expensas Consorcios" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle'!$A$3:$I$51</definedName>
@@ -619,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1494,6 +1495,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1585,6 +1587,37 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>• Expensas consorcios: hoja "Expensas Consorcios" (Consorcio De Propiet = CIUDAD; no ALMACEN SOL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1596,7 +1629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:G599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7985,6 +8018,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8651,6 +8685,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9317,6 +9352,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9983,6 +10019,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10649,6 +10686,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11315,6 +11353,99 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18994,4 +19125,1730 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G148"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132 — Expensas Consorcios (Pago de Expensas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Transferencias a consorcios. Indica la propiedad. Consorcio De Propietarios = CIUDAD (ya refleja hoja 2026 EXPENSAS). No va a ALMACEN SOL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Resumen por propiedad</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Propiedad</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>SUMIF($D$29:$D$148,A6,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>BONORINO</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>SUMIF($D$29:$D$148,A7,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>SUMIF($D$29:$D$148,A8,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>SUMIF($D$29:$D$148,A9,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>Resumen por mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>SUMIF($B$29:$B$148,A12,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B13" s="15">
+        <f>SUMIF($B$29:$B$148,A13,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>SUMIF($B$29:$B$148,A14,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>SUMIF($B$29:$B$148,A15,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>SUMIF($B$29:$B$148,A16,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>SUMIF($B$29:$B$148,A17,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>SUMIF($B$29:$B$148,A18,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B19" s="15">
+        <f>SUMIF($B$29:$B$148,A19,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B20" s="15">
+        <f>SUMIF($B$29:$B$148,A20,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B21" s="15">
+        <f>SUMIF($B$29:$B$148,A21,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B22" s="15">
+        <f>SUMIF($B$29:$B$148,A22,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B23" s="15">
+        <f>SUMIF($B$29:$B$148,A23,$E$29:$E$148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL AÑO</t>
+        </is>
+      </c>
+      <c r="B24" s="39">
+        <f>SUM(B12:B23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="34" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B28" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C28" s="34" t="inlineStr">
+        <is>
+          <t>Consorcio</t>
+        </is>
+      </c>
+      <c r="D28" s="34" t="inlineStr">
+        <is>
+          <t>Propiedad</t>
+        </is>
+      </c>
+      <c r="E28" s="34" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G28" s="34" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>35260</v>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>238240</v>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Copropi</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>376564</v>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · ¿propiedad? (Consorcio De Copropi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Copropi</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>395551</v>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · ¿propiedad? (Consorcio De Copropi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>218800</v>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Copropi</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>402934</v>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · ¿propiedad? (Consorcio De Copropi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>218800</v>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>BONORINO</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>200340</v>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · BONORINO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>BONORINO</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>219145</v>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G37" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · BONORINO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Copropi</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>666347</v>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · ¿propiedad? (Consorcio De Copropi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="n">
+        <v>246150</v>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>BONORINO</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>209393</v>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · BONORINO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Copropi</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>829490</v>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · ¿propiedad? (Consorcio De Copropi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Consorcio De Propiet</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>273500</v>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia enviada</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>Pago de Expensas · CIUDAD 1132</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="14" t="n"/>
+      <c r="E43" s="15" t="n"/>
+      <c r="F43" s="14" t="n"/>
+      <c r="G43" s="14" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="14" t="n"/>
+      <c r="C44" s="14" t="n"/>
+      <c r="D44" s="14" t="n"/>
+      <c r="E44" s="15" t="n"/>
+      <c r="F44" s="14" t="n"/>
+      <c r="G44" s="14" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="14" t="n"/>
+      <c r="E45" s="15" t="n"/>
+      <c r="F45" s="14" t="n"/>
+      <c r="G45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="n"/>
+      <c r="B46" s="14" t="n"/>
+      <c r="C46" s="14" t="n"/>
+      <c r="D46" s="14" t="n"/>
+      <c r="E46" s="15" t="n"/>
+      <c r="F46" s="14" t="n"/>
+      <c r="G46" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="14" t="n"/>
+      <c r="G47" s="14" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="n"/>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="14" t="n"/>
+      <c r="E48" s="15" t="n"/>
+      <c r="F48" s="14" t="n"/>
+      <c r="G48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n"/>
+      <c r="B49" s="14" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="14" t="n"/>
+      <c r="E49" s="15" t="n"/>
+      <c r="F49" s="14" t="n"/>
+      <c r="G49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="n"/>
+      <c r="B50" s="14" t="n"/>
+      <c r="C50" s="14" t="n"/>
+      <c r="D50" s="14" t="n"/>
+      <c r="E50" s="15" t="n"/>
+      <c r="F50" s="14" t="n"/>
+      <c r="G50" s="14" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="14" t="n"/>
+      <c r="C51" s="14" t="n"/>
+      <c r="D51" s="14" t="n"/>
+      <c r="E51" s="15" t="n"/>
+      <c r="F51" s="14" t="n"/>
+      <c r="G51" s="14" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="n"/>
+      <c r="B52" s="14" t="n"/>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="14" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="14" t="n"/>
+      <c r="G52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
+      <c r="E53" s="15" t="n"/>
+      <c r="F53" s="14" t="n"/>
+      <c r="G53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="14" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="14" t="n"/>
+      <c r="E54" s="15" t="n"/>
+      <c r="F54" s="14" t="n"/>
+      <c r="G54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="14" t="n"/>
+      <c r="E55" s="15" t="n"/>
+      <c r="F55" s="14" t="n"/>
+      <c r="G55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="n"/>
+      <c r="B56" s="14" t="n"/>
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="14" t="n"/>
+      <c r="E56" s="15" t="n"/>
+      <c r="F56" s="14" t="n"/>
+      <c r="G56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="n"/>
+      <c r="B57" s="14" t="n"/>
+      <c r="C57" s="14" t="n"/>
+      <c r="D57" s="14" t="n"/>
+      <c r="E57" s="15" t="n"/>
+      <c r="F57" s="14" t="n"/>
+      <c r="G57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="n"/>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="14" t="n"/>
+      <c r="E58" s="15" t="n"/>
+      <c r="F58" s="14" t="n"/>
+      <c r="G58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="n"/>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="14" t="n"/>
+      <c r="E59" s="15" t="n"/>
+      <c r="F59" s="14" t="n"/>
+      <c r="G59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="n"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="14" t="n"/>
+      <c r="D60" s="14" t="n"/>
+      <c r="E60" s="15" t="n"/>
+      <c r="F60" s="14" t="n"/>
+      <c r="G60" s="14" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="n"/>
+      <c r="B61" s="14" t="n"/>
+      <c r="C61" s="14" t="n"/>
+      <c r="D61" s="14" t="n"/>
+      <c r="E61" s="15" t="n"/>
+      <c r="F61" s="14" t="n"/>
+      <c r="G61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="n"/>
+      <c r="B62" s="14" t="n"/>
+      <c r="C62" s="14" t="n"/>
+      <c r="D62" s="14" t="n"/>
+      <c r="E62" s="15" t="n"/>
+      <c r="F62" s="14" t="n"/>
+      <c r="G62" s="14" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="n"/>
+      <c r="B63" s="14" t="n"/>
+      <c r="C63" s="14" t="n"/>
+      <c r="D63" s="14" t="n"/>
+      <c r="E63" s="15" t="n"/>
+      <c r="F63" s="14" t="n"/>
+      <c r="G63" s="14" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="n"/>
+      <c r="B64" s="14" t="n"/>
+      <c r="C64" s="14" t="n"/>
+      <c r="D64" s="14" t="n"/>
+      <c r="E64" s="15" t="n"/>
+      <c r="F64" s="14" t="n"/>
+      <c r="G64" s="14" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="n"/>
+      <c r="B65" s="14" t="n"/>
+      <c r="C65" s="14" t="n"/>
+      <c r="D65" s="14" t="n"/>
+      <c r="E65" s="15" t="n"/>
+      <c r="F65" s="14" t="n"/>
+      <c r="G65" s="14" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="n"/>
+      <c r="B66" s="14" t="n"/>
+      <c r="C66" s="14" t="n"/>
+      <c r="D66" s="14" t="n"/>
+      <c r="E66" s="15" t="n"/>
+      <c r="F66" s="14" t="n"/>
+      <c r="G66" s="14" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="n"/>
+      <c r="B67" s="14" t="n"/>
+      <c r="C67" s="14" t="n"/>
+      <c r="D67" s="14" t="n"/>
+      <c r="E67" s="15" t="n"/>
+      <c r="F67" s="14" t="n"/>
+      <c r="G67" s="14" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="n"/>
+      <c r="B68" s="14" t="n"/>
+      <c r="C68" s="14" t="n"/>
+      <c r="D68" s="14" t="n"/>
+      <c r="E68" s="15" t="n"/>
+      <c r="F68" s="14" t="n"/>
+      <c r="G68" s="14" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="n"/>
+      <c r="B69" s="14" t="n"/>
+      <c r="C69" s="14" t="n"/>
+      <c r="D69" s="14" t="n"/>
+      <c r="E69" s="15" t="n"/>
+      <c r="F69" s="14" t="n"/>
+      <c r="G69" s="14" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="n"/>
+      <c r="B70" s="14" t="n"/>
+      <c r="C70" s="14" t="n"/>
+      <c r="D70" s="14" t="n"/>
+      <c r="E70" s="15" t="n"/>
+      <c r="F70" s="14" t="n"/>
+      <c r="G70" s="14" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="n"/>
+      <c r="B71" s="14" t="n"/>
+      <c r="C71" s="14" t="n"/>
+      <c r="D71" s="14" t="n"/>
+      <c r="E71" s="15" t="n"/>
+      <c r="F71" s="14" t="n"/>
+      <c r="G71" s="14" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="n"/>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="15" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="n"/>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="14" t="n"/>
+      <c r="D73" s="14" t="n"/>
+      <c r="E73" s="15" t="n"/>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="14" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="n"/>
+      <c r="B74" s="14" t="n"/>
+      <c r="C74" s="14" t="n"/>
+      <c r="D74" s="14" t="n"/>
+      <c r="E74" s="15" t="n"/>
+      <c r="F74" s="14" t="n"/>
+      <c r="G74" s="14" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="17" t="n"/>
+      <c r="B75" s="14" t="n"/>
+      <c r="C75" s="14" t="n"/>
+      <c r="D75" s="14" t="n"/>
+      <c r="E75" s="15" t="n"/>
+      <c r="F75" s="14" t="n"/>
+      <c r="G75" s="14" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="n"/>
+      <c r="B76" s="14" t="n"/>
+      <c r="C76" s="14" t="n"/>
+      <c r="D76" s="14" t="n"/>
+      <c r="E76" s="15" t="n"/>
+      <c r="F76" s="14" t="n"/>
+      <c r="G76" s="14" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="n"/>
+      <c r="B77" s="14" t="n"/>
+      <c r="C77" s="14" t="n"/>
+      <c r="D77" s="14" t="n"/>
+      <c r="E77" s="15" t="n"/>
+      <c r="F77" s="14" t="n"/>
+      <c r="G77" s="14" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="n"/>
+      <c r="B78" s="14" t="n"/>
+      <c r="C78" s="14" t="n"/>
+      <c r="D78" s="14" t="n"/>
+      <c r="E78" s="15" t="n"/>
+      <c r="F78" s="14" t="n"/>
+      <c r="G78" s="14" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="n"/>
+      <c r="B79" s="14" t="n"/>
+      <c r="C79" s="14" t="n"/>
+      <c r="D79" s="14" t="n"/>
+      <c r="E79" s="15" t="n"/>
+      <c r="F79" s="14" t="n"/>
+      <c r="G79" s="14" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="n"/>
+      <c r="B80" s="14" t="n"/>
+      <c r="C80" s="14" t="n"/>
+      <c r="D80" s="14" t="n"/>
+      <c r="E80" s="15" t="n"/>
+      <c r="F80" s="14" t="n"/>
+      <c r="G80" s="14" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="n"/>
+      <c r="B81" s="14" t="n"/>
+      <c r="C81" s="14" t="n"/>
+      <c r="D81" s="14" t="n"/>
+      <c r="E81" s="15" t="n"/>
+      <c r="F81" s="14" t="n"/>
+      <c r="G81" s="14" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="n"/>
+      <c r="B82" s="14" t="n"/>
+      <c r="C82" s="14" t="n"/>
+      <c r="D82" s="14" t="n"/>
+      <c r="E82" s="15" t="n"/>
+      <c r="F82" s="14" t="n"/>
+      <c r="G82" s="14" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="n"/>
+      <c r="B83" s="14" t="n"/>
+      <c r="C83" s="14" t="n"/>
+      <c r="D83" s="14" t="n"/>
+      <c r="E83" s="15" t="n"/>
+      <c r="F83" s="14" t="n"/>
+      <c r="G83" s="14" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="n"/>
+      <c r="B84" s="14" t="n"/>
+      <c r="C84" s="14" t="n"/>
+      <c r="D84" s="14" t="n"/>
+      <c r="E84" s="15" t="n"/>
+      <c r="F84" s="14" t="n"/>
+      <c r="G84" s="14" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="n"/>
+      <c r="B85" s="14" t="n"/>
+      <c r="C85" s="14" t="n"/>
+      <c r="D85" s="14" t="n"/>
+      <c r="E85" s="15" t="n"/>
+      <c r="F85" s="14" t="n"/>
+      <c r="G85" s="14" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="n"/>
+      <c r="B86" s="14" t="n"/>
+      <c r="C86" s="14" t="n"/>
+      <c r="D86" s="14" t="n"/>
+      <c r="E86" s="15" t="n"/>
+      <c r="F86" s="14" t="n"/>
+      <c r="G86" s="14" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="n"/>
+      <c r="B87" s="14" t="n"/>
+      <c r="C87" s="14" t="n"/>
+      <c r="D87" s="14" t="n"/>
+      <c r="E87" s="15" t="n"/>
+      <c r="F87" s="14" t="n"/>
+      <c r="G87" s="14" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="n"/>
+      <c r="B88" s="14" t="n"/>
+      <c r="C88" s="14" t="n"/>
+      <c r="D88" s="14" t="n"/>
+      <c r="E88" s="15" t="n"/>
+      <c r="F88" s="14" t="n"/>
+      <c r="G88" s="14" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="17" t="n"/>
+      <c r="B89" s="14" t="n"/>
+      <c r="C89" s="14" t="n"/>
+      <c r="D89" s="14" t="n"/>
+      <c r="E89" s="15" t="n"/>
+      <c r="F89" s="14" t="n"/>
+      <c r="G89" s="14" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="n"/>
+      <c r="B90" s="14" t="n"/>
+      <c r="C90" s="14" t="n"/>
+      <c r="D90" s="14" t="n"/>
+      <c r="E90" s="15" t="n"/>
+      <c r="F90" s="14" t="n"/>
+      <c r="G90" s="14" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="n"/>
+      <c r="B91" s="14" t="n"/>
+      <c r="C91" s="14" t="n"/>
+      <c r="D91" s="14" t="n"/>
+      <c r="E91" s="15" t="n"/>
+      <c r="F91" s="14" t="n"/>
+      <c r="G91" s="14" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="n"/>
+      <c r="B92" s="14" t="n"/>
+      <c r="C92" s="14" t="n"/>
+      <c r="D92" s="14" t="n"/>
+      <c r="E92" s="15" t="n"/>
+      <c r="F92" s="14" t="n"/>
+      <c r="G92" s="14" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="n"/>
+      <c r="B93" s="14" t="n"/>
+      <c r="C93" s="14" t="n"/>
+      <c r="D93" s="14" t="n"/>
+      <c r="E93" s="15" t="n"/>
+      <c r="F93" s="14" t="n"/>
+      <c r="G93" s="14" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="n"/>
+      <c r="B94" s="14" t="n"/>
+      <c r="C94" s="14" t="n"/>
+      <c r="D94" s="14" t="n"/>
+      <c r="E94" s="15" t="n"/>
+      <c r="F94" s="14" t="n"/>
+      <c r="G94" s="14" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="n"/>
+      <c r="B95" s="14" t="n"/>
+      <c r="C95" s="14" t="n"/>
+      <c r="D95" s="14" t="n"/>
+      <c r="E95" s="15" t="n"/>
+      <c r="F95" s="14" t="n"/>
+      <c r="G95" s="14" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="n"/>
+      <c r="B96" s="14" t="n"/>
+      <c r="C96" s="14" t="n"/>
+      <c r="D96" s="14" t="n"/>
+      <c r="E96" s="15" t="n"/>
+      <c r="F96" s="14" t="n"/>
+      <c r="G96" s="14" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="n"/>
+      <c r="B97" s="14" t="n"/>
+      <c r="C97" s="14" t="n"/>
+      <c r="D97" s="14" t="n"/>
+      <c r="E97" s="15" t="n"/>
+      <c r="F97" s="14" t="n"/>
+      <c r="G97" s="14" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="n"/>
+      <c r="B98" s="14" t="n"/>
+      <c r="C98" s="14" t="n"/>
+      <c r="D98" s="14" t="n"/>
+      <c r="E98" s="15" t="n"/>
+      <c r="F98" s="14" t="n"/>
+      <c r="G98" s="14" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="17" t="n"/>
+      <c r="B99" s="14" t="n"/>
+      <c r="C99" s="14" t="n"/>
+      <c r="D99" s="14" t="n"/>
+      <c r="E99" s="15" t="n"/>
+      <c r="F99" s="14" t="n"/>
+      <c r="G99" s="14" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="17" t="n"/>
+      <c r="B100" s="14" t="n"/>
+      <c r="C100" s="14" t="n"/>
+      <c r="D100" s="14" t="n"/>
+      <c r="E100" s="15" t="n"/>
+      <c r="F100" s="14" t="n"/>
+      <c r="G100" s="14" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="17" t="n"/>
+      <c r="B101" s="14" t="n"/>
+      <c r="C101" s="14" t="n"/>
+      <c r="D101" s="14" t="n"/>
+      <c r="E101" s="15" t="n"/>
+      <c r="F101" s="14" t="n"/>
+      <c r="G101" s="14" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="17" t="n"/>
+      <c r="B102" s="14" t="n"/>
+      <c r="C102" s="14" t="n"/>
+      <c r="D102" s="14" t="n"/>
+      <c r="E102" s="15" t="n"/>
+      <c r="F102" s="14" t="n"/>
+      <c r="G102" s="14" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="17" t="n"/>
+      <c r="B103" s="14" t="n"/>
+      <c r="C103" s="14" t="n"/>
+      <c r="D103" s="14" t="n"/>
+      <c r="E103" s="15" t="n"/>
+      <c r="F103" s="14" t="n"/>
+      <c r="G103" s="14" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="17" t="n"/>
+      <c r="B104" s="14" t="n"/>
+      <c r="C104" s="14" t="n"/>
+      <c r="D104" s="14" t="n"/>
+      <c r="E104" s="15" t="n"/>
+      <c r="F104" s="14" t="n"/>
+      <c r="G104" s="14" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="17" t="n"/>
+      <c r="B105" s="14" t="n"/>
+      <c r="C105" s="14" t="n"/>
+      <c r="D105" s="14" t="n"/>
+      <c r="E105" s="15" t="n"/>
+      <c r="F105" s="14" t="n"/>
+      <c r="G105" s="14" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="n"/>
+      <c r="B106" s="14" t="n"/>
+      <c r="C106" s="14" t="n"/>
+      <c r="D106" s="14" t="n"/>
+      <c r="E106" s="15" t="n"/>
+      <c r="F106" s="14" t="n"/>
+      <c r="G106" s="14" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="n"/>
+      <c r="B107" s="14" t="n"/>
+      <c r="C107" s="14" t="n"/>
+      <c r="D107" s="14" t="n"/>
+      <c r="E107" s="15" t="n"/>
+      <c r="F107" s="14" t="n"/>
+      <c r="G107" s="14" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="17" t="n"/>
+      <c r="B108" s="14" t="n"/>
+      <c r="C108" s="14" t="n"/>
+      <c r="D108" s="14" t="n"/>
+      <c r="E108" s="15" t="n"/>
+      <c r="F108" s="14" t="n"/>
+      <c r="G108" s="14" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="17" t="n"/>
+      <c r="B109" s="14" t="n"/>
+      <c r="C109" s="14" t="n"/>
+      <c r="D109" s="14" t="n"/>
+      <c r="E109" s="15" t="n"/>
+      <c r="F109" s="14" t="n"/>
+      <c r="G109" s="14" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="17" t="n"/>
+      <c r="B110" s="14" t="n"/>
+      <c r="C110" s="14" t="n"/>
+      <c r="D110" s="14" t="n"/>
+      <c r="E110" s="15" t="n"/>
+      <c r="F110" s="14" t="n"/>
+      <c r="G110" s="14" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="17" t="n"/>
+      <c r="B111" s="14" t="n"/>
+      <c r="C111" s="14" t="n"/>
+      <c r="D111" s="14" t="n"/>
+      <c r="E111" s="15" t="n"/>
+      <c r="F111" s="14" t="n"/>
+      <c r="G111" s="14" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="17" t="n"/>
+      <c r="B112" s="14" t="n"/>
+      <c r="C112" s="14" t="n"/>
+      <c r="D112" s="14" t="n"/>
+      <c r="E112" s="15" t="n"/>
+      <c r="F112" s="14" t="n"/>
+      <c r="G112" s="14" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="17" t="n"/>
+      <c r="B113" s="14" t="n"/>
+      <c r="C113" s="14" t="n"/>
+      <c r="D113" s="14" t="n"/>
+      <c r="E113" s="15" t="n"/>
+      <c r="F113" s="14" t="n"/>
+      <c r="G113" s="14" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="n"/>
+      <c r="B114" s="14" t="n"/>
+      <c r="C114" s="14" t="n"/>
+      <c r="D114" s="14" t="n"/>
+      <c r="E114" s="15" t="n"/>
+      <c r="F114" s="14" t="n"/>
+      <c r="G114" s="14" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="17" t="n"/>
+      <c r="B115" s="14" t="n"/>
+      <c r="C115" s="14" t="n"/>
+      <c r="D115" s="14" t="n"/>
+      <c r="E115" s="15" t="n"/>
+      <c r="F115" s="14" t="n"/>
+      <c r="G115" s="14" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="17" t="n"/>
+      <c r="B116" s="14" t="n"/>
+      <c r="C116" s="14" t="n"/>
+      <c r="D116" s="14" t="n"/>
+      <c r="E116" s="15" t="n"/>
+      <c r="F116" s="14" t="n"/>
+      <c r="G116" s="14" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="n"/>
+      <c r="B117" s="14" t="n"/>
+      <c r="C117" s="14" t="n"/>
+      <c r="D117" s="14" t="n"/>
+      <c r="E117" s="15" t="n"/>
+      <c r="F117" s="14" t="n"/>
+      <c r="G117" s="14" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="17" t="n"/>
+      <c r="B118" s="14" t="n"/>
+      <c r="C118" s="14" t="n"/>
+      <c r="D118" s="14" t="n"/>
+      <c r="E118" s="15" t="n"/>
+      <c r="F118" s="14" t="n"/>
+      <c r="G118" s="14" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="17" t="n"/>
+      <c r="B119" s="14" t="n"/>
+      <c r="C119" s="14" t="n"/>
+      <c r="D119" s="14" t="n"/>
+      <c r="E119" s="15" t="n"/>
+      <c r="F119" s="14" t="n"/>
+      <c r="G119" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="17" t="n"/>
+      <c r="B120" s="14" t="n"/>
+      <c r="C120" s="14" t="n"/>
+      <c r="D120" s="14" t="n"/>
+      <c r="E120" s="15" t="n"/>
+      <c r="F120" s="14" t="n"/>
+      <c r="G120" s="14" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="17" t="n"/>
+      <c r="B121" s="14" t="n"/>
+      <c r="C121" s="14" t="n"/>
+      <c r="D121" s="14" t="n"/>
+      <c r="E121" s="15" t="n"/>
+      <c r="F121" s="14" t="n"/>
+      <c r="G121" s="14" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="17" t="n"/>
+      <c r="B122" s="14" t="n"/>
+      <c r="C122" s="14" t="n"/>
+      <c r="D122" s="14" t="n"/>
+      <c r="E122" s="15" t="n"/>
+      <c r="F122" s="14" t="n"/>
+      <c r="G122" s="14" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="n"/>
+      <c r="B123" s="14" t="n"/>
+      <c r="C123" s="14" t="n"/>
+      <c r="D123" s="14" t="n"/>
+      <c r="E123" s="15" t="n"/>
+      <c r="F123" s="14" t="n"/>
+      <c r="G123" s="14" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="n"/>
+      <c r="B124" s="14" t="n"/>
+      <c r="C124" s="14" t="n"/>
+      <c r="D124" s="14" t="n"/>
+      <c r="E124" s="15" t="n"/>
+      <c r="F124" s="14" t="n"/>
+      <c r="G124" s="14" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="n"/>
+      <c r="B125" s="14" t="n"/>
+      <c r="C125" s="14" t="n"/>
+      <c r="D125" s="14" t="n"/>
+      <c r="E125" s="15" t="n"/>
+      <c r="F125" s="14" t="n"/>
+      <c r="G125" s="14" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="n"/>
+      <c r="B126" s="14" t="n"/>
+      <c r="C126" s="14" t="n"/>
+      <c r="D126" s="14" t="n"/>
+      <c r="E126" s="15" t="n"/>
+      <c r="F126" s="14" t="n"/>
+      <c r="G126" s="14" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="n"/>
+      <c r="B127" s="14" t="n"/>
+      <c r="C127" s="14" t="n"/>
+      <c r="D127" s="14" t="n"/>
+      <c r="E127" s="15" t="n"/>
+      <c r="F127" s="14" t="n"/>
+      <c r="G127" s="14" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="17" t="n"/>
+      <c r="B128" s="14" t="n"/>
+      <c r="C128" s="14" t="n"/>
+      <c r="D128" s="14" t="n"/>
+      <c r="E128" s="15" t="n"/>
+      <c r="F128" s="14" t="n"/>
+      <c r="G128" s="14" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="17" t="n"/>
+      <c r="B129" s="14" t="n"/>
+      <c r="C129" s="14" t="n"/>
+      <c r="D129" s="14" t="n"/>
+      <c r="E129" s="15" t="n"/>
+      <c r="F129" s="14" t="n"/>
+      <c r="G129" s="14" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="17" t="n"/>
+      <c r="B130" s="14" t="n"/>
+      <c r="C130" s="14" t="n"/>
+      <c r="D130" s="14" t="n"/>
+      <c r="E130" s="15" t="n"/>
+      <c r="F130" s="14" t="n"/>
+      <c r="G130" s="14" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="17" t="n"/>
+      <c r="B131" s="14" t="n"/>
+      <c r="C131" s="14" t="n"/>
+      <c r="D131" s="14" t="n"/>
+      <c r="E131" s="15" t="n"/>
+      <c r="F131" s="14" t="n"/>
+      <c r="G131" s="14" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="17" t="n"/>
+      <c r="B132" s="14" t="n"/>
+      <c r="C132" s="14" t="n"/>
+      <c r="D132" s="14" t="n"/>
+      <c r="E132" s="15" t="n"/>
+      <c r="F132" s="14" t="n"/>
+      <c r="G132" s="14" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="n"/>
+      <c r="B133" s="14" t="n"/>
+      <c r="C133" s="14" t="n"/>
+      <c r="D133" s="14" t="n"/>
+      <c r="E133" s="15" t="n"/>
+      <c r="F133" s="14" t="n"/>
+      <c r="G133" s="14" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="17" t="n"/>
+      <c r="B134" s="14" t="n"/>
+      <c r="C134" s="14" t="n"/>
+      <c r="D134" s="14" t="n"/>
+      <c r="E134" s="15" t="n"/>
+      <c r="F134" s="14" t="n"/>
+      <c r="G134" s="14" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="17" t="n"/>
+      <c r="B135" s="14" t="n"/>
+      <c r="C135" s="14" t="n"/>
+      <c r="D135" s="14" t="n"/>
+      <c r="E135" s="15" t="n"/>
+      <c r="F135" s="14" t="n"/>
+      <c r="G135" s="14" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="17" t="n"/>
+      <c r="B136" s="14" t="n"/>
+      <c r="C136" s="14" t="n"/>
+      <c r="D136" s="14" t="n"/>
+      <c r="E136" s="15" t="n"/>
+      <c r="F136" s="14" t="n"/>
+      <c r="G136" s="14" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="17" t="n"/>
+      <c r="B137" s="14" t="n"/>
+      <c r="C137" s="14" t="n"/>
+      <c r="D137" s="14" t="n"/>
+      <c r="E137" s="15" t="n"/>
+      <c r="F137" s="14" t="n"/>
+      <c r="G137" s="14" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="17" t="n"/>
+      <c r="B138" s="14" t="n"/>
+      <c r="C138" s="14" t="n"/>
+      <c r="D138" s="14" t="n"/>
+      <c r="E138" s="15" t="n"/>
+      <c r="F138" s="14" t="n"/>
+      <c r="G138" s="14" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="17" t="n"/>
+      <c r="B139" s="14" t="n"/>
+      <c r="C139" s="14" t="n"/>
+      <c r="D139" s="14" t="n"/>
+      <c r="E139" s="15" t="n"/>
+      <c r="F139" s="14" t="n"/>
+      <c r="G139" s="14" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="n"/>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="14" t="n"/>
+      <c r="E140" s="15" t="n"/>
+      <c r="F140" s="14" t="n"/>
+      <c r="G140" s="14" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="n"/>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="14" t="n"/>
+      <c r="D141" s="14" t="n"/>
+      <c r="E141" s="15" t="n"/>
+      <c r="F141" s="14" t="n"/>
+      <c r="G141" s="14" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="n"/>
+      <c r="B142" s="14" t="n"/>
+      <c r="C142" s="14" t="n"/>
+      <c r="D142" s="14" t="n"/>
+      <c r="E142" s="15" t="n"/>
+      <c r="F142" s="14" t="n"/>
+      <c r="G142" s="14" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="17" t="n"/>
+      <c r="B143" s="14" t="n"/>
+      <c r="C143" s="14" t="n"/>
+      <c r="D143" s="14" t="n"/>
+      <c r="E143" s="15" t="n"/>
+      <c r="F143" s="14" t="n"/>
+      <c r="G143" s="14" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="17" t="n"/>
+      <c r="B144" s="14" t="n"/>
+      <c r="C144" s="14" t="n"/>
+      <c r="D144" s="14" t="n"/>
+      <c r="E144" s="15" t="n"/>
+      <c r="F144" s="14" t="n"/>
+      <c r="G144" s="14" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="17" t="n"/>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="15" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="17" t="n"/>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="14" t="n"/>
+      <c r="D146" s="14" t="n"/>
+      <c r="E146" s="15" t="n"/>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="14" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="17" t="n"/>
+      <c r="B147" s="14" t="n"/>
+      <c r="C147" s="14" t="n"/>
+      <c r="D147" s="14" t="n"/>
+      <c r="E147" s="15" t="n"/>
+      <c r="F147" s="14" t="n"/>
+      <c r="G147" s="14" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="17" t="n"/>
+      <c r="B148" s="14" t="n"/>
+      <c r="C148" s="14" t="n"/>
+      <c r="D148" s="14" t="n"/>
+      <c r="E148" s="15" t="n"/>
+      <c r="F148" s="14" t="n"/>
+      <c r="G148" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Identify CIUDAD consortium expenses by Patagonia bank details.
Treat Banco Patagonia CBU/CUIL matches as CIUDAD expensas even when the consortium name varies.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1495,7 +1495,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1594,30 +1593,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1629,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G599"/>
+  <dimension ref="A1:G506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2706,7 +2681,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3649,7 +3623,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4532,7 +4505,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5427,7 +5399,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6250,7 +6221,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7169,7 +7139,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -8018,7 +7987,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8685,7 +8653,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9352,7 +9319,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -10019,7 +9985,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10686,7 +10651,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11353,99 +11317,6 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19133,7 +19004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G148"/>
+  <dimension ref="A1:G159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19155,7 +19026,7 @@
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Transferencias a consorcios. Indica la propiedad. Consorcio De Propietarios = CIUDAD (ya refleja hoja 2026 EXPENSAS). No va a ALMACEN SOL.</t>
+          <t>Transferencias a consorcios. CIUDAD = Consorcio De Propietarios o destino Banco Patagonia CBU 0340116900116010765007 / CUIL 30714962473. No va a ALMACEN SOL.</t>
         </is>
       </c>
     </row>
@@ -19165,6 +19036,11 @@
           <t>Resumen por propiedad</t>
         </is>
       </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>ID bancario CIUDAD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
@@ -19177,6 +19053,16 @@
           <t>Total</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Entidad</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Banco Patagonia</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -19188,6 +19074,16 @@
         <f>SUMIF($D$29:$D$148,A6,$E$29:$E$148)</f>
         <v/>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0340116900116010765007</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
@@ -19198,6 +19094,16 @@
       <c r="B7" s="15">
         <f>SUMIF($D$29:$D$148,A7,$E$29:$E$148)</f>
         <v/>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CUIL</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>30714962473</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -19457,7 +19363,7 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · CIUDAD 1132</t>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473</t>
         </is>
       </c>
     </row>
@@ -19490,7 +19396,7 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · CIUDAD 1132</t>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473</t>
         </is>
       </c>
     </row>
@@ -19589,7 +19495,7 @@
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · CIUDAD 1132</t>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473</t>
         </is>
       </c>
     </row>
@@ -19655,7 +19561,7 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · CIUDAD 1132</t>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473</t>
         </is>
       </c>
     </row>
@@ -19787,7 +19693,7 @@
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · CIUDAD 1132</t>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473</t>
         </is>
       </c>
     </row>
@@ -19886,7 +19792,7 @@
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
-          <t>Pago de Expensas · CIUDAD 1132</t>
+          <t>Pago de Expensas · CIUDAD 1132 · Patagonia CBU 0340116900116010765007 / CUIL 30714962473</t>
         </is>
       </c>
     </row>
@@ -20844,6 +20750,17 @@
       <c r="F148" s="14" t="n"/>
       <c r="G148" s="14" t="n"/>
     </row>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
Remove Pandora Jewelry purchases from CIUDAD tracking.
Drop those Mercado Pago buys from the catalog and keep them excluded going forward.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -655,6 +655,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1495,6 +1496,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1604,7 +1606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:N506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2681,6 +2683,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3623,6 +3626,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4505,6 +4509,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5399,6 +5404,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6221,6 +6227,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7139,6 +7146,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7987,6 +7995,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8653,6 +8662,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9319,6 +9329,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9985,6 +9996,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10651,6 +10663,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11328,7 +11341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:N60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11349,6 +11362,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -13310,6 +13324,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -13472,6 +13487,8 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
@@ -14515,6 +14532,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -14848,6 +14866,8 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
@@ -14855,6 +14875,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="34" t="inlineStr">
         <is>
@@ -17348,6 +17369,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -17510,6 +17532,8 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
@@ -19004,7 +19028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G159"/>
+  <dimension ref="A1:G148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19030,6 +19054,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -19290,6 +19315,8 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
         <is>
@@ -20750,17 +20777,6 @@
       <c r="F148" s="14" t="n"/>
       <c r="G148" s="14" t="n"/>
     </row>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
Classify Havanna purchases as COMIDA.
Keep Havanna in Almacén Sol with a consistent COMIDA · HAVANNA comment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -655,7 +655,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1496,7 +1495,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1606,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N506"/>
+  <dimension ref="A1:G599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2113,7 +2111,7 @@
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>MP · Havanna</t>
+          <t>COMIDA · HAVANNA</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2846,7 @@
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
-          <t>MP · Havanna</t>
+          <t>COMIDA · HAVANNA</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2874,7 @@
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
-          <t>MP · Havanna</t>
+          <t>COMIDA · HAVANNA</t>
         </is>
       </c>
     </row>
@@ -11330,6 +11328,99 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11341,7 +11432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11362,7 +11453,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -13324,7 +13414,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -13487,8 +13576,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
@@ -14532,7 +14619,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -14866,8 +14952,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
@@ -14875,7 +14959,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="34" t="inlineStr">
         <is>
@@ -17369,7 +17452,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -17532,8 +17614,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
@@ -19054,7 +19134,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -19315,8 +19394,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Classify Compraenkalbb as Kalbby food under COMIDA · RAMON.
Move pending Compraenkalbb charges into Almacén Sol with the Kalbby/Ramón venue label.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1604,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G599"/>
+  <dimension ref="A1:G506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2485,15 +2485,27 @@
           <t>Enero</t>
         </is>
       </c>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="27" t="n"/>
+      <c r="B33" s="17" t="n">
+        <v>46032</v>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Kalbby / Ramón</t>
+        </is>
+      </c>
+      <c r="D33" s="27" t="n">
+        <v>77748</v>
+      </c>
       <c r="E33" s="28" t="n"/>
       <c r="F33" s="15">
         <f>IF(OR(D33&lt;&gt;"",E33&lt;&gt;""),IF(D33="",0,D33)+IF(E33="",0,E33),"")</f>
         <v/>
       </c>
-      <c r="G33" s="14" t="n"/>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · RAMON</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
@@ -3332,15 +3344,27 @@
           <t>Febrero</t>
         </is>
       </c>
-      <c r="B69" s="17" t="n"/>
-      <c r="C69" s="14" t="n"/>
-      <c r="D69" s="27" t="n"/>
+      <c r="B69" s="17" t="n">
+        <v>46065</v>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>Kalbby / Ramón</t>
+        </is>
+      </c>
+      <c r="D69" s="27" t="n">
+        <v>30336</v>
+      </c>
       <c r="E69" s="28" t="n"/>
       <c r="F69" s="15">
         <f>IF(OR(D69&lt;&gt;"",E69&lt;&gt;""),IF(D69="",0,D69)+IF(E69="",0,E69),"")</f>
         <v/>
       </c>
-      <c r="G69" s="14" t="n"/>
+      <c r="G69" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · RAMON</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="14" t="inlineStr">
@@ -4135,15 +4159,27 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B106" s="17" t="n"/>
-      <c r="C106" s="14" t="n"/>
-      <c r="D106" s="27" t="n"/>
+      <c r="B106" s="17" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>Kalbby / Ramón</t>
+        </is>
+      </c>
+      <c r="D106" s="27" t="n">
+        <v>56250</v>
+      </c>
       <c r="E106" s="28" t="n"/>
       <c r="F106" s="15">
         <f>IF(OR(D106&lt;&gt;"",E106&lt;&gt;""),IF(D106="",0,D106)+IF(E106="",0,E106),"")</f>
         <v/>
       </c>
-      <c r="G106" s="14" t="n"/>
+      <c r="G106" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · RAMON</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="14" t="inlineStr">
@@ -5046,15 +5082,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B149" s="17" t="n"/>
-      <c r="C149" s="14" t="n"/>
-      <c r="D149" s="27" t="n"/>
+      <c r="B149" s="17" t="n">
+        <v>46114</v>
+      </c>
+      <c r="C149" s="14" t="inlineStr">
+        <is>
+          <t>Kalbby / Ramón</t>
+        </is>
+      </c>
+      <c r="D149" s="27" t="n">
+        <v>82746</v>
+      </c>
       <c r="E149" s="28" t="n"/>
       <c r="F149" s="15">
         <f>IF(OR(D149&lt;&gt;"",E149&lt;&gt;""),IF(D149="",0,D149)+IF(E149="",0,E149),"")</f>
         <v/>
       </c>
-      <c r="G149" s="14" t="n"/>
+      <c r="G149" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · RAMON</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="14" t="inlineStr">
@@ -5062,15 +5110,27 @@
           <t>Abril</t>
         </is>
       </c>
-      <c r="B150" s="17" t="n"/>
-      <c r="C150" s="14" t="n"/>
-      <c r="D150" s="27" t="n"/>
+      <c r="B150" s="17" t="n">
+        <v>46141</v>
+      </c>
+      <c r="C150" s="14" t="inlineStr">
+        <is>
+          <t>Kalbby / Ramón</t>
+        </is>
+      </c>
+      <c r="D150" s="27" t="n">
+        <v>86747</v>
+      </c>
       <c r="E150" s="28" t="n"/>
       <c r="F150" s="15">
         <f>IF(OR(D150&lt;&gt;"",E150&lt;&gt;""),IF(D150="",0,D150)+IF(E150="",0,E150),"")</f>
         <v/>
       </c>
-      <c r="G150" s="14" t="n"/>
+      <c r="G150" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · RAMON</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="14" t="inlineStr">
@@ -5402,7 +5462,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6225,7 +6284,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7144,7 +7202,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7993,7 +8050,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8660,7 +8716,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9327,7 +9382,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9994,7 +10048,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10661,7 +10714,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11328,99 +11380,6 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Súper Pollo 24000 to Almacén Sol (July).
Record cash/store chicken purchase in Almacen Detalle Importe Sol so ALMACEN SOL July total updates.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1604,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G599"/>
+  <dimension ref="A1:G506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2681,7 +2681,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3624,7 +3623,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4507,7 +4505,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5402,7 +5399,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6225,7 +6221,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -7144,7 +7139,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7605,15 +7599,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B273" s="17" t="n"/>
-      <c r="C273" s="14" t="n"/>
-      <c r="D273" s="27" t="n"/>
+      <c r="B273" s="17" t="n">
+        <v>46221</v>
+      </c>
+      <c r="C273" s="14" t="inlineStr">
+        <is>
+          <t>Súper Pollo</t>
+        </is>
+      </c>
+      <c r="D273" s="27" t="n">
+        <v>24000</v>
+      </c>
       <c r="E273" s="28" t="n"/>
       <c r="F273" s="15">
         <f>IF(OR(D273&lt;&gt;"",E273&lt;&gt;""),IF(D273="",0,D273)+IF(E273="",0,E273),"")</f>
         <v/>
       </c>
-      <c r="G273" s="14" t="n"/>
+      <c r="G273" s="14" t="inlineStr">
+        <is>
+          <t>MP · pollo</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="14" t="inlineStr">
@@ -7993,7 +7999,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8660,7 +8665,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9327,7 +9331,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9994,7 +9997,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10661,7 +10663,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11328,99 +11329,6 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Move Tuenti charges to a personal Sol expense sheet.
Keep Tuenti out of the CIUDAD expense total and track it on Gasto Personal Sol.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Inversión" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Transferencias recibidas" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Expensas Consorcios" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gasto Personal Sol" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle'!$A$3:$I$51</definedName>
@@ -620,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1495,6 +1496,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1593,6 +1595,36 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>• Tuenti: hoja "Gasto Personal Sol" (no suma al total de gastos CIUDAD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2693,7 +2725,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3648,7 +3679,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4543,7 +4573,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -20820,4 +20849,1485 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F142"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CIUDAD 1132 — Gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Gastos personales de Sol (ej. Tuenti). No suma al total de gastos de la hoja 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Resumen por mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>SUMIF($B$23:$B$142,A6,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>SUMIF($B$23:$B$142,A7,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>SUMIF($B$23:$B$142,A8,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>SUMIF($B$23:$B$142,A9,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
+        <f>SUMIF($B$23:$B$142,A10,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B11" s="15">
+        <f>SUMIF($B$23:$B$142,A11,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>SUMIF($B$23:$B$142,A12,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B13" s="15">
+        <f>SUMIF($B$23:$B$142,A13,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>SUMIF($B$23:$B$142,A14,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>SUMIF($B$23:$B$142,A15,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>SUMIF($B$23:$B$142,A16,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>SUMIF($B$23:$B$142,A17,$D$23:$D$142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL AÑO</t>
+        </is>
+      </c>
+      <c r="B18" s="39">
+        <f>SUM(B6:B17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C22" s="34" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="E22" s="34" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>14700</v>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="n">
+        <v>46061</v>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>14700</v>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>46087</v>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>16000</v>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>16650</v>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>16650</v>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>16650</v>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>17400</v>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Tuenti</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>Celular Tuenti — gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="n"/>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="n"/>
+      <c r="B38" s="14" t="n"/>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n"/>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="14" t="n"/>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="14" t="n"/>
+      <c r="F40" s="14" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n"/>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="n"/>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="14" t="n"/>
+      <c r="F43" s="14" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="14" t="n"/>
+      <c r="C44" s="14" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="14" t="n"/>
+      <c r="F44" s="14" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="n"/>
+      <c r="B46" s="14" t="n"/>
+      <c r="C46" s="14" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="14" t="n"/>
+      <c r="F46" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="14" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="14" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="n"/>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="14" t="n"/>
+      <c r="F48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n"/>
+      <c r="B49" s="14" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="14" t="n"/>
+      <c r="F49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="n"/>
+      <c r="B50" s="14" t="n"/>
+      <c r="C50" s="14" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="14" t="n"/>
+      <c r="F50" s="14" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="14" t="n"/>
+      <c r="C51" s="14" t="n"/>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="14" t="n"/>
+      <c r="F51" s="14" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="n"/>
+      <c r="B52" s="14" t="n"/>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="14" t="n"/>
+      <c r="F52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="14" t="n"/>
+      <c r="F53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="14" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="14" t="n"/>
+      <c r="F54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="14" t="n"/>
+      <c r="F55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="n"/>
+      <c r="B56" s="14" t="n"/>
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="14" t="n"/>
+      <c r="F56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="n"/>
+      <c r="B57" s="14" t="n"/>
+      <c r="C57" s="14" t="n"/>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="14" t="n"/>
+      <c r="F57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="n"/>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="14" t="n"/>
+      <c r="F58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="n"/>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="15" t="n"/>
+      <c r="E59" s="14" t="n"/>
+      <c r="F59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="n"/>
+      <c r="B60" s="14" t="n"/>
+      <c r="C60" s="14" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="14" t="n"/>
+      <c r="F60" s="14" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="n"/>
+      <c r="B61" s="14" t="n"/>
+      <c r="C61" s="14" t="n"/>
+      <c r="D61" s="15" t="n"/>
+      <c r="E61" s="14" t="n"/>
+      <c r="F61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="n"/>
+      <c r="B62" s="14" t="n"/>
+      <c r="C62" s="14" t="n"/>
+      <c r="D62" s="15" t="n"/>
+      <c r="E62" s="14" t="n"/>
+      <c r="F62" s="14" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="n"/>
+      <c r="B63" s="14" t="n"/>
+      <c r="C63" s="14" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="14" t="n"/>
+      <c r="F63" s="14" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="n"/>
+      <c r="B64" s="14" t="n"/>
+      <c r="C64" s="14" t="n"/>
+      <c r="D64" s="15" t="n"/>
+      <c r="E64" s="14" t="n"/>
+      <c r="F64" s="14" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="n"/>
+      <c r="B65" s="14" t="n"/>
+      <c r="C65" s="14" t="n"/>
+      <c r="D65" s="15" t="n"/>
+      <c r="E65" s="14" t="n"/>
+      <c r="F65" s="14" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="n"/>
+      <c r="B66" s="14" t="n"/>
+      <c r="C66" s="14" t="n"/>
+      <c r="D66" s="15" t="n"/>
+      <c r="E66" s="14" t="n"/>
+      <c r="F66" s="14" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="n"/>
+      <c r="B67" s="14" t="n"/>
+      <c r="C67" s="14" t="n"/>
+      <c r="D67" s="15" t="n"/>
+      <c r="E67" s="14" t="n"/>
+      <c r="F67" s="14" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="n"/>
+      <c r="B68" s="14" t="n"/>
+      <c r="C68" s="14" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="14" t="n"/>
+      <c r="F68" s="14" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="n"/>
+      <c r="B69" s="14" t="n"/>
+      <c r="C69" s="14" t="n"/>
+      <c r="D69" s="15" t="n"/>
+      <c r="E69" s="14" t="n"/>
+      <c r="F69" s="14" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="n"/>
+      <c r="B70" s="14" t="n"/>
+      <c r="C70" s="14" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="14" t="n"/>
+      <c r="F70" s="14" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="n"/>
+      <c r="B71" s="14" t="n"/>
+      <c r="C71" s="14" t="n"/>
+      <c r="D71" s="15" t="n"/>
+      <c r="E71" s="14" t="n"/>
+      <c r="F71" s="14" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="n"/>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="15" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="n"/>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="14" t="n"/>
+      <c r="D73" s="15" t="n"/>
+      <c r="E73" s="14" t="n"/>
+      <c r="F73" s="14" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="n"/>
+      <c r="B74" s="14" t="n"/>
+      <c r="C74" s="14" t="n"/>
+      <c r="D74" s="15" t="n"/>
+      <c r="E74" s="14" t="n"/>
+      <c r="F74" s="14" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="17" t="n"/>
+      <c r="B75" s="14" t="n"/>
+      <c r="C75" s="14" t="n"/>
+      <c r="D75" s="15" t="n"/>
+      <c r="E75" s="14" t="n"/>
+      <c r="F75" s="14" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="n"/>
+      <c r="B76" s="14" t="n"/>
+      <c r="C76" s="14" t="n"/>
+      <c r="D76" s="15" t="n"/>
+      <c r="E76" s="14" t="n"/>
+      <c r="F76" s="14" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="n"/>
+      <c r="B77" s="14" t="n"/>
+      <c r="C77" s="14" t="n"/>
+      <c r="D77" s="15" t="n"/>
+      <c r="E77" s="14" t="n"/>
+      <c r="F77" s="14" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="n"/>
+      <c r="B78" s="14" t="n"/>
+      <c r="C78" s="14" t="n"/>
+      <c r="D78" s="15" t="n"/>
+      <c r="E78" s="14" t="n"/>
+      <c r="F78" s="14" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="n"/>
+      <c r="B79" s="14" t="n"/>
+      <c r="C79" s="14" t="n"/>
+      <c r="D79" s="15" t="n"/>
+      <c r="E79" s="14" t="n"/>
+      <c r="F79" s="14" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="n"/>
+      <c r="B80" s="14" t="n"/>
+      <c r="C80" s="14" t="n"/>
+      <c r="D80" s="15" t="n"/>
+      <c r="E80" s="14" t="n"/>
+      <c r="F80" s="14" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="n"/>
+      <c r="B81" s="14" t="n"/>
+      <c r="C81" s="14" t="n"/>
+      <c r="D81" s="15" t="n"/>
+      <c r="E81" s="14" t="n"/>
+      <c r="F81" s="14" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="n"/>
+      <c r="B82" s="14" t="n"/>
+      <c r="C82" s="14" t="n"/>
+      <c r="D82" s="15" t="n"/>
+      <c r="E82" s="14" t="n"/>
+      <c r="F82" s="14" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="n"/>
+      <c r="B83" s="14" t="n"/>
+      <c r="C83" s="14" t="n"/>
+      <c r="D83" s="15" t="n"/>
+      <c r="E83" s="14" t="n"/>
+      <c r="F83" s="14" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="n"/>
+      <c r="B84" s="14" t="n"/>
+      <c r="C84" s="14" t="n"/>
+      <c r="D84" s="15" t="n"/>
+      <c r="E84" s="14" t="n"/>
+      <c r="F84" s="14" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="n"/>
+      <c r="B85" s="14" t="n"/>
+      <c r="C85" s="14" t="n"/>
+      <c r="D85" s="15" t="n"/>
+      <c r="E85" s="14" t="n"/>
+      <c r="F85" s="14" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="n"/>
+      <c r="B86" s="14" t="n"/>
+      <c r="C86" s="14" t="n"/>
+      <c r="D86" s="15" t="n"/>
+      <c r="E86" s="14" t="n"/>
+      <c r="F86" s="14" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="n"/>
+      <c r="B87" s="14" t="n"/>
+      <c r="C87" s="14" t="n"/>
+      <c r="D87" s="15" t="n"/>
+      <c r="E87" s="14" t="n"/>
+      <c r="F87" s="14" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="n"/>
+      <c r="B88" s="14" t="n"/>
+      <c r="C88" s="14" t="n"/>
+      <c r="D88" s="15" t="n"/>
+      <c r="E88" s="14" t="n"/>
+      <c r="F88" s="14" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="17" t="n"/>
+      <c r="B89" s="14" t="n"/>
+      <c r="C89" s="14" t="n"/>
+      <c r="D89" s="15" t="n"/>
+      <c r="E89" s="14" t="n"/>
+      <c r="F89" s="14" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="n"/>
+      <c r="B90" s="14" t="n"/>
+      <c r="C90" s="14" t="n"/>
+      <c r="D90" s="15" t="n"/>
+      <c r="E90" s="14" t="n"/>
+      <c r="F90" s="14" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="n"/>
+      <c r="B91" s="14" t="n"/>
+      <c r="C91" s="14" t="n"/>
+      <c r="D91" s="15" t="n"/>
+      <c r="E91" s="14" t="n"/>
+      <c r="F91" s="14" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="n"/>
+      <c r="B92" s="14" t="n"/>
+      <c r="C92" s="14" t="n"/>
+      <c r="D92" s="15" t="n"/>
+      <c r="E92" s="14" t="n"/>
+      <c r="F92" s="14" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="n"/>
+      <c r="B93" s="14" t="n"/>
+      <c r="C93" s="14" t="n"/>
+      <c r="D93" s="15" t="n"/>
+      <c r="E93" s="14" t="n"/>
+      <c r="F93" s="14" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="n"/>
+      <c r="B94" s="14" t="n"/>
+      <c r="C94" s="14" t="n"/>
+      <c r="D94" s="15" t="n"/>
+      <c r="E94" s="14" t="n"/>
+      <c r="F94" s="14" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="n"/>
+      <c r="B95" s="14" t="n"/>
+      <c r="C95" s="14" t="n"/>
+      <c r="D95" s="15" t="n"/>
+      <c r="E95" s="14" t="n"/>
+      <c r="F95" s="14" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="n"/>
+      <c r="B96" s="14" t="n"/>
+      <c r="C96" s="14" t="n"/>
+      <c r="D96" s="15" t="n"/>
+      <c r="E96" s="14" t="n"/>
+      <c r="F96" s="14" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="n"/>
+      <c r="B97" s="14" t="n"/>
+      <c r="C97" s="14" t="n"/>
+      <c r="D97" s="15" t="n"/>
+      <c r="E97" s="14" t="n"/>
+      <c r="F97" s="14" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="n"/>
+      <c r="B98" s="14" t="n"/>
+      <c r="C98" s="14" t="n"/>
+      <c r="D98" s="15" t="n"/>
+      <c r="E98" s="14" t="n"/>
+      <c r="F98" s="14" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="17" t="n"/>
+      <c r="B99" s="14" t="n"/>
+      <c r="C99" s="14" t="n"/>
+      <c r="D99" s="15" t="n"/>
+      <c r="E99" s="14" t="n"/>
+      <c r="F99" s="14" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="17" t="n"/>
+      <c r="B100" s="14" t="n"/>
+      <c r="C100" s="14" t="n"/>
+      <c r="D100" s="15" t="n"/>
+      <c r="E100" s="14" t="n"/>
+      <c r="F100" s="14" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="17" t="n"/>
+      <c r="B101" s="14" t="n"/>
+      <c r="C101" s="14" t="n"/>
+      <c r="D101" s="15" t="n"/>
+      <c r="E101" s="14" t="n"/>
+      <c r="F101" s="14" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="17" t="n"/>
+      <c r="B102" s="14" t="n"/>
+      <c r="C102" s="14" t="n"/>
+      <c r="D102" s="15" t="n"/>
+      <c r="E102" s="14" t="n"/>
+      <c r="F102" s="14" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="17" t="n"/>
+      <c r="B103" s="14" t="n"/>
+      <c r="C103" s="14" t="n"/>
+      <c r="D103" s="15" t="n"/>
+      <c r="E103" s="14" t="n"/>
+      <c r="F103" s="14" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="17" t="n"/>
+      <c r="B104" s="14" t="n"/>
+      <c r="C104" s="14" t="n"/>
+      <c r="D104" s="15" t="n"/>
+      <c r="E104" s="14" t="n"/>
+      <c r="F104" s="14" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="17" t="n"/>
+      <c r="B105" s="14" t="n"/>
+      <c r="C105" s="14" t="n"/>
+      <c r="D105" s="15" t="n"/>
+      <c r="E105" s="14" t="n"/>
+      <c r="F105" s="14" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="n"/>
+      <c r="B106" s="14" t="n"/>
+      <c r="C106" s="14" t="n"/>
+      <c r="D106" s="15" t="n"/>
+      <c r="E106" s="14" t="n"/>
+      <c r="F106" s="14" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="n"/>
+      <c r="B107" s="14" t="n"/>
+      <c r="C107" s="14" t="n"/>
+      <c r="D107" s="15" t="n"/>
+      <c r="E107" s="14" t="n"/>
+      <c r="F107" s="14" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="17" t="n"/>
+      <c r="B108" s="14" t="n"/>
+      <c r="C108" s="14" t="n"/>
+      <c r="D108" s="15" t="n"/>
+      <c r="E108" s="14" t="n"/>
+      <c r="F108" s="14" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="17" t="n"/>
+      <c r="B109" s="14" t="n"/>
+      <c r="C109" s="14" t="n"/>
+      <c r="D109" s="15" t="n"/>
+      <c r="E109" s="14" t="n"/>
+      <c r="F109" s="14" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="17" t="n"/>
+      <c r="B110" s="14" t="n"/>
+      <c r="C110" s="14" t="n"/>
+      <c r="D110" s="15" t="n"/>
+      <c r="E110" s="14" t="n"/>
+      <c r="F110" s="14" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="17" t="n"/>
+      <c r="B111" s="14" t="n"/>
+      <c r="C111" s="14" t="n"/>
+      <c r="D111" s="15" t="n"/>
+      <c r="E111" s="14" t="n"/>
+      <c r="F111" s="14" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="17" t="n"/>
+      <c r="B112" s="14" t="n"/>
+      <c r="C112" s="14" t="n"/>
+      <c r="D112" s="15" t="n"/>
+      <c r="E112" s="14" t="n"/>
+      <c r="F112" s="14" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="17" t="n"/>
+      <c r="B113" s="14" t="n"/>
+      <c r="C113" s="14" t="n"/>
+      <c r="D113" s="15" t="n"/>
+      <c r="E113" s="14" t="n"/>
+      <c r="F113" s="14" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="n"/>
+      <c r="B114" s="14" t="n"/>
+      <c r="C114" s="14" t="n"/>
+      <c r="D114" s="15" t="n"/>
+      <c r="E114" s="14" t="n"/>
+      <c r="F114" s="14" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="17" t="n"/>
+      <c r="B115" s="14" t="n"/>
+      <c r="C115" s="14" t="n"/>
+      <c r="D115" s="15" t="n"/>
+      <c r="E115" s="14" t="n"/>
+      <c r="F115" s="14" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="17" t="n"/>
+      <c r="B116" s="14" t="n"/>
+      <c r="C116" s="14" t="n"/>
+      <c r="D116" s="15" t="n"/>
+      <c r="E116" s="14" t="n"/>
+      <c r="F116" s="14" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="n"/>
+      <c r="B117" s="14" t="n"/>
+      <c r="C117" s="14" t="n"/>
+      <c r="D117" s="15" t="n"/>
+      <c r="E117" s="14" t="n"/>
+      <c r="F117" s="14" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="17" t="n"/>
+      <c r="B118" s="14" t="n"/>
+      <c r="C118" s="14" t="n"/>
+      <c r="D118" s="15" t="n"/>
+      <c r="E118" s="14" t="n"/>
+      <c r="F118" s="14" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="17" t="n"/>
+      <c r="B119" s="14" t="n"/>
+      <c r="C119" s="14" t="n"/>
+      <c r="D119" s="15" t="n"/>
+      <c r="E119" s="14" t="n"/>
+      <c r="F119" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="17" t="n"/>
+      <c r="B120" s="14" t="n"/>
+      <c r="C120" s="14" t="n"/>
+      <c r="D120" s="15" t="n"/>
+      <c r="E120" s="14" t="n"/>
+      <c r="F120" s="14" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="17" t="n"/>
+      <c r="B121" s="14" t="n"/>
+      <c r="C121" s="14" t="n"/>
+      <c r="D121" s="15" t="n"/>
+      <c r="E121" s="14" t="n"/>
+      <c r="F121" s="14" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="17" t="n"/>
+      <c r="B122" s="14" t="n"/>
+      <c r="C122" s="14" t="n"/>
+      <c r="D122" s="15" t="n"/>
+      <c r="E122" s="14" t="n"/>
+      <c r="F122" s="14" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="n"/>
+      <c r="B123" s="14" t="n"/>
+      <c r="C123" s="14" t="n"/>
+      <c r="D123" s="15" t="n"/>
+      <c r="E123" s="14" t="n"/>
+      <c r="F123" s="14" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="n"/>
+      <c r="B124" s="14" t="n"/>
+      <c r="C124" s="14" t="n"/>
+      <c r="D124" s="15" t="n"/>
+      <c r="E124" s="14" t="n"/>
+      <c r="F124" s="14" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="n"/>
+      <c r="B125" s="14" t="n"/>
+      <c r="C125" s="14" t="n"/>
+      <c r="D125" s="15" t="n"/>
+      <c r="E125" s="14" t="n"/>
+      <c r="F125" s="14" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="n"/>
+      <c r="B126" s="14" t="n"/>
+      <c r="C126" s="14" t="n"/>
+      <c r="D126" s="15" t="n"/>
+      <c r="E126" s="14" t="n"/>
+      <c r="F126" s="14" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="n"/>
+      <c r="B127" s="14" t="n"/>
+      <c r="C127" s="14" t="n"/>
+      <c r="D127" s="15" t="n"/>
+      <c r="E127" s="14" t="n"/>
+      <c r="F127" s="14" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="17" t="n"/>
+      <c r="B128" s="14" t="n"/>
+      <c r="C128" s="14" t="n"/>
+      <c r="D128" s="15" t="n"/>
+      <c r="E128" s="14" t="n"/>
+      <c r="F128" s="14" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="17" t="n"/>
+      <c r="B129" s="14" t="n"/>
+      <c r="C129" s="14" t="n"/>
+      <c r="D129" s="15" t="n"/>
+      <c r="E129" s="14" t="n"/>
+      <c r="F129" s="14" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="17" t="n"/>
+      <c r="B130" s="14" t="n"/>
+      <c r="C130" s="14" t="n"/>
+      <c r="D130" s="15" t="n"/>
+      <c r="E130" s="14" t="n"/>
+      <c r="F130" s="14" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="17" t="n"/>
+      <c r="B131" s="14" t="n"/>
+      <c r="C131" s="14" t="n"/>
+      <c r="D131" s="15" t="n"/>
+      <c r="E131" s="14" t="n"/>
+      <c r="F131" s="14" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="17" t="n"/>
+      <c r="B132" s="14" t="n"/>
+      <c r="C132" s="14" t="n"/>
+      <c r="D132" s="15" t="n"/>
+      <c r="E132" s="14" t="n"/>
+      <c r="F132" s="14" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="n"/>
+      <c r="B133" s="14" t="n"/>
+      <c r="C133" s="14" t="n"/>
+      <c r="D133" s="15" t="n"/>
+      <c r="E133" s="14" t="n"/>
+      <c r="F133" s="14" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="17" t="n"/>
+      <c r="B134" s="14" t="n"/>
+      <c r="C134" s="14" t="n"/>
+      <c r="D134" s="15" t="n"/>
+      <c r="E134" s="14" t="n"/>
+      <c r="F134" s="14" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="17" t="n"/>
+      <c r="B135" s="14" t="n"/>
+      <c r="C135" s="14" t="n"/>
+      <c r="D135" s="15" t="n"/>
+      <c r="E135" s="14" t="n"/>
+      <c r="F135" s="14" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="17" t="n"/>
+      <c r="B136" s="14" t="n"/>
+      <c r="C136" s="14" t="n"/>
+      <c r="D136" s="15" t="n"/>
+      <c r="E136" s="14" t="n"/>
+      <c r="F136" s="14" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="17" t="n"/>
+      <c r="B137" s="14" t="n"/>
+      <c r="C137" s="14" t="n"/>
+      <c r="D137" s="15" t="n"/>
+      <c r="E137" s="14" t="n"/>
+      <c r="F137" s="14" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="17" t="n"/>
+      <c r="B138" s="14" t="n"/>
+      <c r="C138" s="14" t="n"/>
+      <c r="D138" s="15" t="n"/>
+      <c r="E138" s="14" t="n"/>
+      <c r="F138" s="14" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="17" t="n"/>
+      <c r="B139" s="14" t="n"/>
+      <c r="C139" s="14" t="n"/>
+      <c r="D139" s="15" t="n"/>
+      <c r="E139" s="14" t="n"/>
+      <c r="F139" s="14" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="n"/>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="15" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="n"/>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="14" t="n"/>
+      <c r="D141" s="15" t="n"/>
+      <c r="E141" s="14" t="n"/>
+      <c r="F141" s="14" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="n"/>
+      <c r="B142" s="14" t="n"/>
+      <c r="C142" s="14" t="n"/>
+      <c r="D142" s="15" t="n"/>
+      <c r="E142" s="14" t="n"/>
+      <c r="F142" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Move Promarine purchases to personal Sol expenses.
Route Promarine Erisea out of pending and onto the Gasto Personal Sol sheet.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -621,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1496,7 +1496,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1602,29 +1601,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20857,7 +20833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21476,12 +21452,32 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="n"/>
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="14" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="14" t="n"/>
-      <c r="F37" s="14" t="n"/>
+      <c r="A37" s="17" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Promarine Erisea</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>350000</v>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Mastercard crédito</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>Compra — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="n"/>
@@ -22323,6 +22319,63 @@
       <c r="E142" s="14" t="n"/>
       <c r="F142" s="14" t="n"/>
     </row>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Classify July pollo entry as COMIDA · POLLO.
Keep amount 24000 on Almacén Sol with today's date (2026-07-18).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -7604,7 +7604,7 @@
       </c>
       <c r="C273" s="14" t="inlineStr">
         <is>
-          <t>Súper Pollo</t>
+          <t>Pollo</t>
         </is>
       </c>
       <c r="D273" s="27" t="n">
@@ -7617,7 +7617,7 @@
       </c>
       <c r="G273" s="14" t="inlineStr">
         <is>
-          <t>MP · pollo</t>
+          <t>COMIDA · POLLO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove Copetin Catering from Almacén Sol.
Clear Copetin lines from the detail sheet and keep those charges out of supermarket totals.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1612,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:G599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1760,32 +1760,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="n">
-        <v>46051</v>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D7" s="27" t="n">
-        <v>9800</v>
-      </c>
+      <c r="A7" s="14" t="n"/>
+      <c r="B7" s="17" t="n"/>
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="27" t="n"/>
       <c r="E7" s="28" t="n"/>
-      <c r="F7" s="15">
-        <f>IF(OR(D7&lt;&gt;"",E7&lt;&gt;""),IF(D7="",0,D7)+IF(E7="",0,E7),"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="14" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
@@ -1844,32 +1825,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="n">
-        <v>46049</v>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (27/1)</t>
-        </is>
-      </c>
-      <c r="D10" s="27" t="n">
-        <v>19550</v>
-      </c>
+      <c r="A10" s="14" t="n"/>
+      <c r="B10" s="17" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="27" t="n"/>
       <c r="E10" s="28" t="n"/>
-      <c r="F10" s="15">
-        <f>IF(OR(D10&lt;&gt;"",E10&lt;&gt;""),IF(D10="",0,D10)+IF(E10="",0,E10),"")</f>
-        <v/>
-      </c>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="14" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -1956,88 +1918,31 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B14" s="17" t="n">
-        <v>46044</v>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (22/1)</t>
-        </is>
-      </c>
-      <c r="D14" s="27" t="n">
-        <v>11950</v>
-      </c>
+      <c r="A14" s="14" t="n"/>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="27" t="n"/>
       <c r="E14" s="28" t="n"/>
-      <c r="F14" s="15">
-        <f>IF(OR(D14&lt;&gt;"",E14&lt;&gt;""),IF(D14="",0,D14)+IF(E14="",0,E14),"")</f>
-        <v/>
-      </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="n">
-        <v>46042</v>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (20/1)</t>
-        </is>
-      </c>
-      <c r="D15" s="27" t="n">
-        <v>3585</v>
-      </c>
+      <c r="A15" s="14" t="n"/>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="27" t="n"/>
       <c r="E15" s="28" t="n"/>
-      <c r="F15" s="15">
-        <f>IF(OR(D15&lt;&gt;"",E15&lt;&gt;""),IF(D15="",0,D15)+IF(E15="",0,E15),"")</f>
-        <v/>
-      </c>
-      <c r="G15" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="n">
-        <v>46041</v>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (19/1)</t>
-        </is>
-      </c>
-      <c r="D16" s="27" t="n">
-        <v>3585</v>
-      </c>
+      <c r="A16" s="14" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="27" t="n"/>
       <c r="E16" s="28" t="n"/>
-      <c r="F16" s="15">
-        <f>IF(OR(D16&lt;&gt;"",E16&lt;&gt;""),IF(D16="",0,D16)+IF(E16="",0,E16),"")</f>
-        <v/>
-      </c>
-      <c r="G16" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="14" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
@@ -2068,32 +1973,13 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n">
-        <v>46035</v>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (13/1)</t>
-        </is>
-      </c>
-      <c r="D18" s="27" t="n">
-        <v>2940</v>
-      </c>
+      <c r="A18" s="14" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="27" t="n"/>
       <c r="E18" s="28" t="n"/>
-      <c r="F18" s="15">
-        <f>IF(OR(D18&lt;&gt;"",E18&lt;&gt;""),IF(D18="",0,D18)+IF(E18="",0,E18),"")</f>
-        <v/>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="14" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
@@ -2208,60 +2094,22 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="n">
-        <v>46030</v>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (8/1)</t>
-        </is>
-      </c>
-      <c r="D23" s="27" t="n">
-        <v>3585</v>
-      </c>
+      <c r="A23" s="14" t="n"/>
+      <c r="B23" s="17" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="27" t="n"/>
       <c r="E23" s="28" t="n"/>
-      <c r="F23" s="15">
-        <f>IF(OR(D23&lt;&gt;"",E23&lt;&gt;""),IF(D23="",0,D23)+IF(E23="",0,E23),"")</f>
-        <v/>
-      </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="14" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="n">
-        <v>46028</v>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (6/1)</t>
-        </is>
-      </c>
-      <c r="D24" s="27" t="n">
-        <v>645</v>
-      </c>
+      <c r="A24" s="14" t="n"/>
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="27" t="n"/>
       <c r="E24" s="28" t="n"/>
-      <c r="F24" s="15">
-        <f>IF(OR(D24&lt;&gt;"",E24&lt;&gt;""),IF(D24="",0,D24)+IF(E24="",0,E24),"")</f>
-        <v/>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="14" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
@@ -2713,6 +2561,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -2826,32 +2675,13 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t>Febrero</t>
-        </is>
-      </c>
-      <c r="B50" s="17" t="n">
-        <v>46077</v>
-      </c>
-      <c r="C50" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D50" s="27" t="n">
-        <v>13500</v>
-      </c>
+      <c r="A50" s="14" t="n"/>
+      <c r="B50" s="17" t="n"/>
+      <c r="C50" s="14" t="n"/>
+      <c r="D50" s="27" t="n"/>
       <c r="E50" s="28" t="n"/>
-      <c r="F50" s="15">
-        <f>IF(OR(D50&lt;&gt;"",E50&lt;&gt;""),IF(D50="",0,D50)+IF(E50="",0,E50),"")</f>
-        <v/>
-      </c>
-      <c r="G50" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F50" s="15" t="n"/>
+      <c r="G50" s="14" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
@@ -2938,32 +2768,13 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="inlineStr">
-        <is>
-          <t>Febrero</t>
-        </is>
-      </c>
-      <c r="B54" s="17" t="n">
-        <v>46071</v>
-      </c>
-      <c r="C54" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D54" s="27" t="n">
-        <v>2703</v>
-      </c>
+      <c r="A54" s="14" t="n"/>
+      <c r="B54" s="17" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="27" t="n"/>
       <c r="E54" s="28" t="n"/>
-      <c r="F54" s="15">
-        <f>IF(OR(D54&lt;&gt;"",E54&lt;&gt;""),IF(D54="",0,D54)+IF(E54="",0,E54),"")</f>
-        <v/>
-      </c>
-      <c r="G54" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="14" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
@@ -3022,60 +2833,22 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="14" t="inlineStr">
-        <is>
-          <t>Febrero</t>
-        </is>
-      </c>
-      <c r="B57" s="17" t="n">
-        <v>46063</v>
-      </c>
-      <c r="C57" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D57" s="27" t="n">
-        <v>2940</v>
-      </c>
+      <c r="A57" s="14" t="n"/>
+      <c r="B57" s="17" t="n"/>
+      <c r="C57" s="14" t="n"/>
+      <c r="D57" s="27" t="n"/>
       <c r="E57" s="28" t="n"/>
-      <c r="F57" s="15">
-        <f>IF(OR(D57&lt;&gt;"",E57&lt;&gt;""),IF(D57="",0,D57)+IF(E57="",0,E57),"")</f>
-        <v/>
-      </c>
-      <c r="G57" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F57" s="15" t="n"/>
+      <c r="G57" s="14" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="14" t="inlineStr">
-        <is>
-          <t>Febrero</t>
-        </is>
-      </c>
-      <c r="B58" s="17" t="n">
-        <v>46063</v>
-      </c>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (2)</t>
-        </is>
-      </c>
-      <c r="D58" s="27" t="n">
-        <v>1770</v>
-      </c>
+      <c r="A58" s="14" t="n"/>
+      <c r="B58" s="17" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="27" t="n"/>
       <c r="E58" s="28" t="n"/>
-      <c r="F58" s="15">
-        <f>IF(OR(D58&lt;&gt;"",E58&lt;&gt;""),IF(D58="",0,D58)+IF(E58="",0,E58),"")</f>
-        <v/>
-      </c>
-      <c r="G58" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F58" s="15" t="n"/>
+      <c r="G58" s="14" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
@@ -3190,32 +2963,13 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="14" t="inlineStr">
-        <is>
-          <t>Febrero</t>
-        </is>
-      </c>
-      <c r="B63" s="17" t="n">
-        <v>46058</v>
-      </c>
-      <c r="C63" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (5/2)</t>
-        </is>
-      </c>
-      <c r="D63" s="27" t="n">
-        <v>2940</v>
-      </c>
+      <c r="A63" s="14" t="n"/>
+      <c r="B63" s="17" t="n"/>
+      <c r="C63" s="14" t="n"/>
+      <c r="D63" s="27" t="n"/>
       <c r="E63" s="28" t="n"/>
-      <c r="F63" s="15">
-        <f>IF(OR(D63&lt;&gt;"",E63&lt;&gt;""),IF(D63="",0,D63)+IF(E63="",0,E63),"")</f>
-        <v/>
-      </c>
-      <c r="G63" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F63" s="15" t="n"/>
+      <c r="G63" s="14" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
@@ -3246,32 +3000,13 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="inlineStr">
-        <is>
-          <t>Febrero</t>
-        </is>
-      </c>
-      <c r="B65" s="17" t="n">
-        <v>46056</v>
-      </c>
-      <c r="C65" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering (3/2)</t>
-        </is>
-      </c>
-      <c r="D65" s="27" t="n">
-        <v>3585</v>
-      </c>
+      <c r="A65" s="14" t="n"/>
+      <c r="B65" s="17" t="n"/>
+      <c r="C65" s="14" t="n"/>
+      <c r="D65" s="27" t="n"/>
       <c r="E65" s="28" t="n"/>
-      <c r="F65" s="15">
-        <f>IF(OR(D65&lt;&gt;"",E65&lt;&gt;""),IF(D65="",0,D65)+IF(E65="",0,E65),"")</f>
-        <v/>
-      </c>
-      <c r="G65" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F65" s="15" t="n"/>
+      <c r="G65" s="14" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
@@ -3667,6 +3402,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -3752,32 +3488,13 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="14" t="inlineStr">
-        <is>
-          <t>Marzo</t>
-        </is>
-      </c>
-      <c r="B91" s="17" t="n">
-        <v>46112</v>
-      </c>
-      <c r="C91" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D91" s="27" t="n">
-        <v>13500</v>
-      </c>
+      <c r="A91" s="14" t="n"/>
+      <c r="B91" s="17" t="n"/>
+      <c r="C91" s="14" t="n"/>
+      <c r="D91" s="27" t="n"/>
       <c r="E91" s="28" t="n"/>
-      <c r="F91" s="15">
-        <f>IF(OR(D91&lt;&gt;"",E91&lt;&gt;""),IF(D91="",0,D91)+IF(E91="",0,E91),"")</f>
-        <v/>
-      </c>
-      <c r="G91" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F91" s="15" t="n"/>
+      <c r="G91" s="14" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
@@ -4561,6 +4278,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -4702,32 +4420,13 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="14" t="inlineStr">
-        <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="B135" s="17" t="n">
-        <v>46132</v>
-      </c>
-      <c r="C135" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D135" s="27" t="n">
-        <v>12650</v>
-      </c>
+      <c r="A135" s="14" t="n"/>
+      <c r="B135" s="17" t="n"/>
+      <c r="C135" s="14" t="n"/>
+      <c r="D135" s="27" t="n"/>
       <c r="E135" s="28" t="n"/>
-      <c r="F135" s="15">
-        <f>IF(OR(D135&lt;&gt;"",E135&lt;&gt;""),IF(D135="",0,D135)+IF(E135="",0,E135),"")</f>
-        <v/>
-      </c>
-      <c r="G135" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F135" s="15" t="n"/>
+      <c r="G135" s="14" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="14" t="inlineStr">
@@ -4870,32 +4569,13 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="14" t="inlineStr">
-        <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="B141" s="17" t="n">
-        <v>46120</v>
-      </c>
-      <c r="C141" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D141" s="27" t="n">
-        <v>17050</v>
-      </c>
+      <c r="A141" s="14" t="n"/>
+      <c r="B141" s="17" t="n"/>
+      <c r="C141" s="14" t="n"/>
+      <c r="D141" s="27" t="n"/>
       <c r="E141" s="28" t="n"/>
-      <c r="F141" s="15">
-        <f>IF(OR(D141&lt;&gt;"",E141&lt;&gt;""),IF(D141="",0,D141)+IF(E141="",0,E141),"")</f>
-        <v/>
-      </c>
-      <c r="G141" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F141" s="15" t="n"/>
+      <c r="G141" s="14" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="14" t="inlineStr">
@@ -5479,6 +5159,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -6301,6 +5982,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -6750,32 +6432,13 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="14" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="B230" s="17" t="n">
-        <v>46174</v>
-      </c>
-      <c r="C230" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D230" s="27" t="n">
-        <v>2700</v>
-      </c>
+      <c r="A230" s="14" t="n"/>
+      <c r="B230" s="17" t="n"/>
+      <c r="C230" s="14" t="n"/>
+      <c r="D230" s="27" t="n"/>
       <c r="E230" s="28" t="n"/>
-      <c r="F230" s="15">
-        <f>IF(OR(D230&lt;&gt;"",E230&lt;&gt;""),IF(D230="",0,D230)+IF(E230="",0,E230),"")</f>
-        <v/>
-      </c>
-      <c r="G230" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F230" s="15" t="n"/>
+      <c r="G230" s="14" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="14" t="inlineStr">
@@ -7219,6 +6882,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7450,32 +7114,13 @@
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="B265" s="17" t="n">
-        <v>46209</v>
-      </c>
-      <c r="C265" s="14" t="inlineStr">
-        <is>
-          <t>Copetin Catering</t>
-        </is>
-      </c>
-      <c r="D265" s="27" t="n">
-        <v>765</v>
-      </c>
+      <c r="A265" s="14" t="n"/>
+      <c r="B265" s="17" t="n"/>
+      <c r="C265" s="14" t="n"/>
+      <c r="D265" s="27" t="n"/>
       <c r="E265" s="28" t="n"/>
-      <c r="F265" s="15">
-        <f>IF(OR(D265&lt;&gt;"",E265&lt;&gt;""),IF(D265="",0,D265)+IF(E265="",0,E265),"")</f>
-        <v/>
-      </c>
-      <c r="G265" s="14" t="inlineStr">
-        <is>
-          <t>MP · catering</t>
-        </is>
-      </c>
+      <c r="F265" s="15" t="n"/>
+      <c r="G265" s="14" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="14" t="inlineStr">
@@ -8067,6 +7712,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8733,6 +8379,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9399,6 +9046,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -10065,6 +9713,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10731,6 +10380,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11397,6 +11047,99 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11408,7 +11151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13353,145 +13096,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <autoFilter ref="A3:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Move Apple purchases to personal Sol expenses.
Route Apple Mercado Pago charges onto Gasto Personal Sol instead of Extras.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1612,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G599"/>
+  <dimension ref="A1:G506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2561,7 +2561,6 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3402,7 +3401,6 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4278,7 +4276,6 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
-    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5159,7 +5156,6 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
-    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -5982,7 +5978,6 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
-    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -6882,7 +6877,6 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
-    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -7712,7 +7706,6 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
-    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8379,7 +8372,6 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
-    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9046,7 +9038,6 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
-    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9713,7 +9704,6 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
-    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10380,7 +10370,6 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
-    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11047,99 +11036,6 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20588,7 +20484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21235,108 +21131,368 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="n"/>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="14" t="n"/>
+      <c r="A38" s="17" t="n">
+        <v>46024</v>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="n">
+        <v>5621</v>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="n"/>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
+      <c r="A39" s="17" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="n">
+        <v>45711</v>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="n"/>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="14" t="n"/>
-      <c r="D40" s="15" t="n"/>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="14" t="n"/>
+      <c r="A40" s="17" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="n">
+        <v>5553</v>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="n"/>
-      <c r="B41" s="14" t="n"/>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="14" t="n"/>
-      <c r="F41" s="14" t="n"/>
+      <c r="A41" s="17" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>17631</v>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="n"/>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="15" t="n"/>
-      <c r="E42" s="14" t="n"/>
-      <c r="F42" s="14" t="n"/>
+      <c r="A42" s="17" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="n">
+        <v>5453</v>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="n"/>
-      <c r="B43" s="14" t="n"/>
-      <c r="C43" s="14" t="n"/>
-      <c r="D43" s="15" t="n"/>
-      <c r="E43" s="14" t="n"/>
-      <c r="F43" s="14" t="n"/>
+      <c r="A43" s="17" t="n">
+        <v>46103</v>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="n">
+        <v>29810</v>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="n"/>
-      <c r="B44" s="14" t="n"/>
-      <c r="C44" s="14" t="n"/>
-      <c r="D44" s="15" t="n"/>
-      <c r="E44" s="14" t="n"/>
-      <c r="F44" s="14" t="n"/>
+      <c r="A44" s="17" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="n">
+        <v>5448</v>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="n"/>
-      <c r="B45" s="14" t="n"/>
-      <c r="C45" s="14" t="n"/>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="14" t="n"/>
+      <c r="A45" s="17" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="n">
+        <v>359951</v>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="n"/>
-      <c r="B46" s="14" t="n"/>
-      <c r="C46" s="14" t="n"/>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="14" t="n"/>
-      <c r="F46" s="14" t="n"/>
+      <c r="A46" s="17" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="n">
+        <v>14520</v>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="n"/>
-      <c r="B47" s="14" t="n"/>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="15" t="n"/>
-      <c r="E47" s="14" t="n"/>
-      <c r="F47" s="14" t="n"/>
+      <c r="A47" s="17" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="n">
+        <v>18353</v>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="n"/>
-      <c r="B48" s="14" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="15" t="n"/>
-      <c r="E48" s="14" t="n"/>
-      <c r="F48" s="14" t="n"/>
+      <c r="A48" s="17" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="n">
+        <v>331291</v>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="n"/>
-      <c r="B49" s="14" t="n"/>
-      <c r="C49" s="14" t="n"/>
-      <c r="D49" s="15" t="n"/>
-      <c r="E49" s="14" t="n"/>
-      <c r="F49" s="14" t="n"/>
+      <c r="A49" s="17" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="n">
+        <v>18558</v>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="17" t="n"/>
-      <c r="B50" s="14" t="n"/>
-      <c r="C50" s="14" t="n"/>
-      <c r="D50" s="15" t="n"/>
-      <c r="E50" s="14" t="n"/>
-      <c r="F50" s="14" t="n"/>
+      <c r="A50" s="17" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="n">
+        <v>19481</v>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>Apple — gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="17" t="n"/>
@@ -22074,6 +22230,63 @@
       <c r="E142" s="14" t="n"/>
       <c r="F142" s="14" t="n"/>
     </row>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Move Ceferina purchases to personal Sol as ROPA.
Route pending Ceferina charges onto Gasto Personal Sol with clothing category.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -21495,20 +21495,60 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="n"/>
-      <c r="B51" s="14" t="n"/>
-      <c r="C51" s="14" t="n"/>
-      <c r="D51" s="15" t="n"/>
-      <c r="E51" s="14" t="n"/>
-      <c r="F51" s="14" t="n"/>
+      <c r="A51" s="17" t="n">
+        <v>46026</v>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>Ceferina</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="n">
+        <v>530000</v>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Mastercard crédito</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="n"/>
-      <c r="B52" s="14" t="n"/>
-      <c r="C52" s="14" t="n"/>
-      <c r="D52" s="15" t="n"/>
-      <c r="E52" s="14" t="n"/>
-      <c r="F52" s="14" t="n"/>
+      <c r="A52" s="17" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Ceferina</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="n">
+        <v>395000</v>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Mastercard crédito</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>ROPA</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="17" t="n"/>

</xml_diff>

<commit_message>
Fix audit findings for Almacén Sol and exclusions.
Restore the July Carrefour refund as excluded and tighten verdulería/supermarket comments.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1612,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:G599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2561,6 +2561,7 @@
       </c>
       <c r="G44" s="22" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
@@ -3401,6 +3402,7 @@
       </c>
       <c r="G86" s="22" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
@@ -4276,6 +4278,7 @@
       </c>
       <c r="G128" s="22" t="n"/>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
@@ -5156,6 +5159,7 @@
       </c>
       <c r="G170" s="22" t="n"/>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
@@ -5978,6 +5982,7 @@
       </c>
       <c r="G212" s="22" t="n"/>
     </row>
+    <row r="213"/>
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
@@ -6877,6 +6882,7 @@
       </c>
       <c r="G254" s="22" t="n"/>
     </row>
+    <row r="255"/>
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
@@ -6919,7 +6925,11 @@
         <f>IF(OR(D257&lt;&gt;"",E257&lt;&gt;""),IF(D257="",0,D257)+IF(E257="",0,E257),"")</f>
         <v/>
       </c>
-      <c r="G257" s="14" t="n"/>
+      <c r="G257" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="14" t="inlineStr">
@@ -6941,7 +6951,11 @@
         <f>IF(OR(D258&lt;&gt;"",E258&lt;&gt;""),IF(D258="",0,D258)+IF(E258="",0,E258),"")</f>
         <v/>
       </c>
-      <c r="G258" s="14" t="n"/>
+      <c r="G258" s="14" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="14" t="inlineStr">
@@ -7706,6 +7720,7 @@
       </c>
       <c r="G296" s="22" t="n"/>
     </row>
+    <row r="297"/>
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
@@ -8372,6 +8387,7 @@
       </c>
       <c r="G338" s="22" t="n"/>
     </row>
+    <row r="339"/>
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
@@ -9038,6 +9054,7 @@
       </c>
       <c r="G380" s="22" t="n"/>
     </row>
+    <row r="381"/>
     <row r="382">
       <c r="A382" s="14" t="inlineStr">
         <is>
@@ -9704,6 +9721,7 @@
       </c>
       <c r="G422" s="22" t="n"/>
     </row>
+    <row r="423"/>
     <row r="424">
       <c r="A424" s="14" t="inlineStr">
         <is>
@@ -10370,6 +10388,7 @@
       </c>
       <c r="G464" s="22" t="n"/>
     </row>
+    <row r="465"/>
     <row r="466">
       <c r="A466" s="14" t="inlineStr">
         <is>
@@ -11036,6 +11055,99 @@
       </c>
       <c r="G506" s="22" t="n"/>
     </row>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20484,7 +20596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F199"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22270,63 +22382,6 @@
       <c r="E142" s="14" t="n"/>
       <c r="F142" s="14" t="n"/>
     </row>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Fix MELI progressive tax formula
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -30,11 +30,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="[$ARS] #,##0"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -786,7 +785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1808,23 +1807,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27546,9 +27528,6 @@
           <t>DATOS EDITABLES</t>
         </is>
       </c>
-      <c r="B4" s="67" t="n"/>
-      <c r="C4" s="67" t="n"/>
-      <c r="D4" s="67" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="68" t="inlineStr">
@@ -27702,9 +27681,6 @@
           <t>PARÁMETROS LEGALES / FISCALES EDITABLES</t>
         </is>
       </c>
-      <c r="B15" s="67" t="n"/>
-      <c r="C15" s="67" t="n"/>
-      <c r="D15" s="67" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="68" t="inlineStr">
@@ -27873,9 +27849,6 @@
           <t>RECIBO MENSUAL ESTIMADO</t>
         </is>
       </c>
-      <c r="B27" s="67" t="n"/>
-      <c r="C27" s="67" t="n"/>
-      <c r="D27" s="67" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="73" t="inlineStr">
@@ -28016,9 +27989,6 @@
           <t>GANANCIAS — PROYECCIÓN ANUALIZADA</t>
         </is>
       </c>
-      <c r="B37" s="67" t="n"/>
-      <c r="C37" s="67" t="n"/>
-      <c r="D37" s="67" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="75" t="inlineStr">
@@ -28095,7 +28065,7 @@
         </is>
       </c>
       <c r="B42" s="78">
-        <f>IF(B41&lt;=2336953.69,B41*5%,IF(B41&lt;=4673907.37,116847.68+(B41-2336953.69)*9%,IF(B41&lt;=7010861.06,327173.51+(B41-4673907.37)*12%,IF(B41&lt;=10516291.59,607607.96+(B41-7010861.06)*15%,IF(B41&lt;=21032583.19,1133422.53+(B41-10516291.59)*19%,IF(B41&lt;=31548874.78,3131517.94+(B41-21032583.19)*23%,IF(B41&lt;=47323312.17,5550265.01+(B41-31548874.78)*27%,IF(B41&lt;=70984968.27,9809363.11+(B41-47323312.17)*31%,17144476.49+(B41-70984968.27)*35%)))))))))</f>
+        <f>IF(B41&lt;=2336953.69,B41*5%,IF(B41&lt;=4673907.37,116847.68+(B41-2336953.69)*9%,IF(B41&lt;=7010861.06,327173.51+(B41-4673907.37)*12%,IF(B41&lt;=10516291.59,607607.96+(B41-7010861.06)*15%,IF(B41&lt;=21032583.19,1133422.53+(B41-10516291.59)*19%,IF(B41&lt;=31548874.78,3131517.94+(B41-21032583.19)*23%,IF(B41&lt;=47323312.17,5550265.01+(B41-31548874.78)*27%,IF(B41&lt;=70984968.27,9809363.11+(B41-47323312.17)*31%,17144476.49+(B41-70984968.27)*35%))))))))</f>
         <v/>
       </c>
       <c r="C42" s="77" t="inlineStr">
@@ -28163,9 +28133,6 @@
           <t>CARGAS SOCIALES Y COSTO MELI (EMPLEADOR)</t>
         </is>
       </c>
-      <c r="B47" s="67" t="n"/>
-      <c r="C47" s="67" t="n"/>
-      <c r="D47" s="67" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="75" t="inlineStr">
@@ -28268,10 +28235,6 @@
           <t>ESCALA ART. 94 — ESTIMADA 2° SEMESTRE 2026</t>
         </is>
       </c>
-      <c r="B55" s="67" t="n"/>
-      <c r="C55" s="67" t="n"/>
-      <c r="D55" s="67" t="n"/>
-      <c r="E55" s="67" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="80" t="inlineStr">
@@ -28459,9 +28422,6 @@
           <t>ALCANCE Y FUENTES</t>
         </is>
       </c>
-      <c r="B68" s="67" t="n"/>
-      <c r="C68" s="67" t="n"/>
-      <c r="D68" s="67" t="n"/>
     </row>
     <row r="69" ht="34" customHeight="1">
       <c r="A69" s="83" t="inlineStr">
@@ -28511,9 +28471,9 @@
   <mergeCells count="15">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A70:D70"/>
+    <mergeCell ref="A27:D27"/>
     <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A70:D70"/>
     <mergeCell ref="A74:D74"/>
     <mergeCell ref="A69:D69"/>
     <mergeCell ref="A4:D4"/>

</xml_diff>

<commit_message>
Load 2026 MELI payroll receipts
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle'!$A$3:$I$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Inversión'!$A$23:$J$223</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'MELI'!$A$56:$E$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'MELI'!$A$78:$P$86</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -30,10 +30,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="[$ARS] #,##0"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="168" formatCode="[$ARS] #,##0.00"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -303,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -400,6 +402,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="13" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -785,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1796,17 +1809,34 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>• Ingresos Sol (sueldo bruto): hoja "Ingresos Sol" — ARS 11.305.702/mes desde 01/07 (cobro 01/08; +12%). No suma al total de gastos.</t>
+          <t>• Ingresos Sol: básico anterior ARS 11.305.702; +12% desde 01/07 → ARS 12.662.387 (cobro 01/08). No suma al total de gastos.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>• MELI: simulador de bruto, aportes, Ganancias y cargas patronales en hoja "MELI". Estimativo; no suma al total de gastos.</t>
-        </is>
-      </c>
-    </row>
+          <t>• MELI: simulador + detalle real de recibos 2026 (sueldos, bono y SAC). No suma al total de gastos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26820,11 +26850,11 @@
         </is>
       </c>
       <c r="B6" s="50" t="n">
-        <v>11305702</v>
+        <v>12662387</v>
       </c>
       <c r="C6" s="51" t="inlineStr">
         <is>
-          <t>ARS · a partir del 01/07/2026</t>
+          <t>ARS · vigente desde 01/07/2026 · básico anterior +12%</t>
         </is>
       </c>
     </row>
@@ -26874,9 +26904,19 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="62" t="n"/>
-      <c r="B10" s="63" t="n"/>
-      <c r="C10" s="62" t="n"/>
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>Bruto anterior confirmado</t>
+        </is>
+      </c>
+      <c r="B10" s="50" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="C10" s="51" t="inlineStr">
+        <is>
+          <t>Recibos MELI marzo–junio 2026</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
@@ -27313,7 +27353,7 @@
         <v>46235</v>
       </c>
       <c r="D30" s="61" t="n">
-        <v>11305702</v>
+        <v>12662387</v>
       </c>
       <c r="E30" s="51" t="inlineStr">
         <is>
@@ -27327,7 +27367,7 @@
       </c>
       <c r="G30" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · a partir 01/07 · incremento 12% · cobro 01/08</t>
+          <t>Ingreso bruto Sol · básico anterior ARS 11.305.702 + 12% · vigente 01/07 · cobro 01/08</t>
         </is>
       </c>
     </row>
@@ -27344,7 +27384,7 @@
         <v>46266</v>
       </c>
       <c r="D31" s="61" t="n">
-        <v>11305702</v>
+        <v>12662387</v>
       </c>
       <c r="E31" s="51" t="inlineStr">
         <is>
@@ -27358,7 +27398,7 @@
       </c>
       <c r="G31" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% · cobro mes siguiente</t>
+          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27375,7 +27415,7 @@
         <v>46296</v>
       </c>
       <c r="D32" s="61" t="n">
-        <v>11305702</v>
+        <v>12662387</v>
       </c>
       <c r="E32" s="51" t="inlineStr">
         <is>
@@ -27389,7 +27429,7 @@
       </c>
       <c r="G32" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% · cobro mes siguiente</t>
+          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27406,7 +27446,7 @@
         <v>46327</v>
       </c>
       <c r="D33" s="61" t="n">
-        <v>11305702</v>
+        <v>12662387</v>
       </c>
       <c r="E33" s="51" t="inlineStr">
         <is>
@@ -27420,7 +27460,7 @@
       </c>
       <c r="G33" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% · cobro mes siguiente</t>
+          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27437,7 +27477,7 @@
         <v>46357</v>
       </c>
       <c r="D34" s="61" t="n">
-        <v>11305702</v>
+        <v>12662387</v>
       </c>
       <c r="E34" s="51" t="inlineStr">
         <is>
@@ -27451,7 +27491,7 @@
       </c>
       <c r="G34" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% · cobro mes siguiente</t>
+          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27468,7 +27508,7 @@
         <v>46388</v>
       </c>
       <c r="D35" s="61" t="n">
-        <v>11305702</v>
+        <v>12662387</v>
       </c>
       <c r="E35" s="51" t="inlineStr">
         <is>
@@ -27482,7 +27522,7 @@
       </c>
       <c r="G35" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% · cobro mes siguiente</t>
+          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27497,7 +27537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:P151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -27505,6 +27545,17 @@
     <col width="58" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -27541,7 +27592,7 @@
       </c>
       <c r="C5" s="68" t="inlineStr">
         <is>
-          <t>Vinculado a Ingresos Sol</t>
+          <t>Vinculado a Ingresos Sol · ARS 11.305.702 + 12% desde julio</t>
         </is>
       </c>
       <c r="D5" s="68" t="n"/>
@@ -28466,19 +28517,2702 @@
       </c>
     </row>
     <row r="75" ht="20" customHeight="1"/>
+    <row r="77">
+      <c r="A77" s="84" t="inlineStr">
+        <is>
+          <t>RECIBOS MELI REALES 2026 — SUELDOS, BONO Y SAC</t>
+        </is>
+      </c>
+      <c r="B77" s="67" t="n"/>
+      <c r="C77" s="67" t="n"/>
+      <c r="D77" s="67" t="n"/>
+      <c r="E77" s="67" t="n"/>
+      <c r="F77" s="67" t="n"/>
+      <c r="G77" s="67" t="n"/>
+      <c r="H77" s="67" t="n"/>
+      <c r="I77" s="67" t="n"/>
+      <c r="J77" s="67" t="n"/>
+      <c r="K77" s="67" t="n"/>
+      <c r="L77" s="67" t="n"/>
+      <c r="M77" s="67" t="n"/>
+      <c r="N77" s="67" t="n"/>
+      <c r="O77" s="67" t="n"/>
+      <c r="P77" s="67" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="85" t="inlineStr">
+        <is>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="B78" s="85" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C78" s="85" t="inlineStr">
+        <is>
+          <t>Fecha pago</t>
+        </is>
+      </c>
+      <c r="D78" s="85" t="inlineStr">
+        <is>
+          <t>Básico</t>
+        </is>
+      </c>
+      <c r="E78" s="85" t="inlineStr">
+        <is>
+          <t>Otros haberes netos</t>
+        </is>
+      </c>
+      <c r="F78" s="85" t="inlineStr">
+        <is>
+          <t>Haberes totales</t>
+        </is>
+      </c>
+      <c r="G78" s="85" t="inlineStr">
+        <is>
+          <t>SIJP</t>
+        </is>
+      </c>
+      <c r="H78" s="85" t="inlineStr">
+        <is>
+          <t>PAMI</t>
+        </is>
+      </c>
+      <c r="I78" s="85" t="inlineStr">
+        <is>
+          <t>Obra social</t>
+        </is>
+      </c>
+      <c r="J78" s="85" t="inlineStr">
+        <is>
+          <t>Ganancias</t>
+        </is>
+      </c>
+      <c r="K78" s="85" t="inlineStr">
+        <is>
+          <t>Otros descuentos</t>
+        </is>
+      </c>
+      <c r="L78" s="85" t="inlineStr">
+        <is>
+          <t>Ajustes / devoluciones</t>
+        </is>
+      </c>
+      <c r="M78" s="85" t="inlineStr">
+        <is>
+          <t>Descuentos netos</t>
+        </is>
+      </c>
+      <c r="N78" s="85" t="inlineStr">
+        <is>
+          <t>Neto pagado</t>
+        </is>
+      </c>
+      <c r="O78" s="85" t="inlineStr">
+        <is>
+          <t>Archivo fuente</t>
+        </is>
+      </c>
+      <c r="P78" s="85" t="inlineStr">
+        <is>
+          <t>Conciliación</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B79" s="75" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C79" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D79" s="88" t="n">
+        <v>7906085</v>
+      </c>
+      <c r="E79" s="88" t="n">
+        <v>180000</v>
+      </c>
+      <c r="F79" s="88" t="n">
+        <v>8086085</v>
+      </c>
+      <c r="G79" s="88" t="n">
+        <v>420571.02</v>
+      </c>
+      <c r="H79" s="88" t="n">
+        <v>114701.19</v>
+      </c>
+      <c r="I79" s="88" t="n">
+        <v>114701.19</v>
+      </c>
+      <c r="J79" s="88" t="n">
+        <v>1221703.83</v>
+      </c>
+      <c r="K79" s="88" t="n">
+        <v>21900</v>
+      </c>
+      <c r="L79" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="88" t="n">
+        <v>1893577.23</v>
+      </c>
+      <c r="N79" s="89" t="n">
+        <v>6192507.77</v>
+      </c>
+      <c r="O79" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+      <c r="P79" s="88">
+        <f>ROUND(F79-M79-N79,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B80" s="75" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C80" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D80" s="88" t="n">
+        <v>7906085</v>
+      </c>
+      <c r="E80" s="88" t="n">
+        <v>208000</v>
+      </c>
+      <c r="F80" s="88" t="n">
+        <v>8114085</v>
+      </c>
+      <c r="G80" s="88" t="n">
+        <v>432557.3</v>
+      </c>
+      <c r="H80" s="88" t="n">
+        <v>117970.17</v>
+      </c>
+      <c r="I80" s="88" t="n">
+        <v>117970.17</v>
+      </c>
+      <c r="J80" s="88" t="n">
+        <v>1425004.25</v>
+      </c>
+      <c r="K80" s="88" t="n">
+        <v>21900</v>
+      </c>
+      <c r="L80" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="88" t="n">
+        <v>2115401.89</v>
+      </c>
+      <c r="N80" s="89" t="n">
+        <v>5998683.11</v>
+      </c>
+      <c r="O80" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+      <c r="P80" s="88">
+        <f>ROUND(F80-M80-N80,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B81" s="75" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C81" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D81" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="E81" s="88" t="n">
+        <v>7007234</v>
+      </c>
+      <c r="F81" s="88" t="n">
+        <v>18312936</v>
+      </c>
+      <c r="G81" s="88" t="n">
+        <v>445014.95</v>
+      </c>
+      <c r="H81" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="I81" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="J81" s="88" t="n">
+        <v>4658857.2</v>
+      </c>
+      <c r="K81" s="88" t="n">
+        <v>21900</v>
+      </c>
+      <c r="L81" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="88" t="n">
+        <v>5368507.57</v>
+      </c>
+      <c r="N81" s="89" t="n">
+        <v>12944428.43</v>
+      </c>
+      <c r="O81" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+      <c r="P81" s="88">
+        <f>ROUND(F81-M81-N81,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B82" s="75" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C82" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D82" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="88" t="n">
+        <v>23717162.5</v>
+      </c>
+      <c r="F82" s="88" t="n">
+        <v>23717162.5</v>
+      </c>
+      <c r="G82" s="88" t="n">
+        <v>445014.95</v>
+      </c>
+      <c r="H82" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="I82" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="J82" s="88" t="n">
+        <v>3120893.08</v>
+      </c>
+      <c r="K82" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="88" t="n">
+        <v>3808643.45</v>
+      </c>
+      <c r="N82" s="89" t="n">
+        <v>19908519.05</v>
+      </c>
+      <c r="O82" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+      <c r="P82" s="88">
+        <f>ROUND(F82-M82-N82,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B83" s="75" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C83" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D83" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="E83" s="88" t="n">
+        <v>2168752.32</v>
+      </c>
+      <c r="F83" s="88" t="n">
+        <v>13474454.32</v>
+      </c>
+      <c r="G83" s="88" t="n">
+        <v>12905.43</v>
+      </c>
+      <c r="H83" s="88" t="n">
+        <v>3519.66</v>
+      </c>
+      <c r="I83" s="88" t="n">
+        <v>3519.66</v>
+      </c>
+      <c r="J83" s="88" t="n">
+        <v>3813479.69</v>
+      </c>
+      <c r="K83" s="88" t="n">
+        <v>23400</v>
+      </c>
+      <c r="L83" s="88" t="n">
+        <v>-3564748.04</v>
+      </c>
+      <c r="M83" s="88" t="n">
+        <v>292076.4</v>
+      </c>
+      <c r="N83" s="89" t="n">
+        <v>13182377.92</v>
+      </c>
+      <c r="O83" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+      <c r="P83" s="88">
+        <f>ROUND(F83-M83-N83,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B84" s="75" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C84" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D84" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="E84" s="88" t="n">
+        <v>312000</v>
+      </c>
+      <c r="F84" s="88" t="n">
+        <v>11617702</v>
+      </c>
+      <c r="G84" s="88" t="n">
+        <v>473398.09</v>
+      </c>
+      <c r="H84" s="88" t="n">
+        <v>129108.57</v>
+      </c>
+      <c r="I84" s="88" t="n">
+        <v>129108.57</v>
+      </c>
+      <c r="J84" s="88" t="n">
+        <v>3415603.09</v>
+      </c>
+      <c r="K84" s="88" t="n">
+        <v>23400</v>
+      </c>
+      <c r="L84" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="88" t="n">
+        <v>4170618.32</v>
+      </c>
+      <c r="N84" s="89" t="n">
+        <v>7447083.68</v>
+      </c>
+      <c r="O84" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+      <c r="P84" s="88">
+        <f>ROUND(F84-M84-N84,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B85" s="75" t="inlineStr">
+        <is>
+          <t>SAC 1° semestre</t>
+        </is>
+      </c>
+      <c r="C85" s="87" t="n">
+        <v>46196</v>
+      </c>
+      <c r="D85" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="88" t="n">
+        <v>6622090.14</v>
+      </c>
+      <c r="F85" s="88" t="n">
+        <v>6622090.14</v>
+      </c>
+      <c r="G85" s="88" t="n">
+        <v>242805.88</v>
+      </c>
+      <c r="H85" s="88" t="n">
+        <v>66219.78999999999</v>
+      </c>
+      <c r="I85" s="88" t="n">
+        <v>66219.78999999999</v>
+      </c>
+      <c r="J85" s="88" t="n">
+        <v>536087.26</v>
+      </c>
+      <c r="K85" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" s="88" t="n">
+        <v>911332.72</v>
+      </c>
+      <c r="N85" s="89" t="n">
+        <v>5710757.42</v>
+      </c>
+      <c r="O85" s="86" t="inlineStr">
+        <is>
+          <t>SAC.pdf</t>
+        </is>
+      </c>
+      <c r="P85" s="88">
+        <f>ROUND(F85-M85-N85,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B86" s="75" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C86" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D86" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="E86" s="88" t="n">
+        <v>312000</v>
+      </c>
+      <c r="F86" s="88" t="n">
+        <v>11617702</v>
+      </c>
+      <c r="G86" s="88" t="n">
+        <v>485611.76</v>
+      </c>
+      <c r="H86" s="88" t="n">
+        <v>132439.57</v>
+      </c>
+      <c r="I86" s="88" t="n">
+        <v>132439.57</v>
+      </c>
+      <c r="J86" s="88" t="n">
+        <v>3408446.06</v>
+      </c>
+      <c r="K86" s="88" t="n">
+        <v>23400</v>
+      </c>
+      <c r="L86" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" s="88" t="n">
+        <v>4182336.96</v>
+      </c>
+      <c r="N86" s="89" t="n">
+        <v>7435365.04</v>
+      </c>
+      <c r="O86" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+      <c r="P86" s="88">
+        <f>ROUND(F86-M86-N86,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="90" t="inlineStr">
+        <is>
+          <t>TOTAL RECIBOS</t>
+        </is>
+      </c>
+      <c r="B87" s="68" t="n"/>
+      <c r="C87" s="68" t="n"/>
+      <c r="D87" s="91">
+        <f>SUM(D79:D86)</f>
+        <v/>
+      </c>
+      <c r="E87" s="91">
+        <f>SUM(E79:E86)</f>
+        <v/>
+      </c>
+      <c r="F87" s="91">
+        <f>SUM(F79:F86)</f>
+        <v/>
+      </c>
+      <c r="G87" s="91">
+        <f>SUM(G79:G86)</f>
+        <v/>
+      </c>
+      <c r="H87" s="91">
+        <f>SUM(H79:H86)</f>
+        <v/>
+      </c>
+      <c r="I87" s="91">
+        <f>SUM(I79:I86)</f>
+        <v/>
+      </c>
+      <c r="J87" s="91">
+        <f>SUM(J79:J86)</f>
+        <v/>
+      </c>
+      <c r="K87" s="91">
+        <f>SUM(K79:K86)</f>
+        <v/>
+      </c>
+      <c r="L87" s="91">
+        <f>SUM(L79:L86)</f>
+        <v/>
+      </c>
+      <c r="M87" s="91">
+        <f>SUM(M79:M86)</f>
+        <v/>
+      </c>
+      <c r="N87" s="91">
+        <f>SUM(N79:N86)</f>
+        <v/>
+      </c>
+      <c r="O87" s="68" t="n"/>
+      <c r="P87" s="92">
+        <f>ROUND(F87-M87-N87,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="84" t="inlineStr">
+        <is>
+          <t>DETALLE EXTRAÍDO DE CONCEPTOS</t>
+        </is>
+      </c>
+      <c r="B89" s="67" t="n"/>
+      <c r="C89" s="67" t="n"/>
+      <c r="D89" s="67" t="n"/>
+      <c r="E89" s="67" t="n"/>
+      <c r="F89" s="67" t="n"/>
+      <c r="G89" s="67" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="80" t="inlineStr">
+        <is>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="B90" s="80" t="inlineStr">
+        <is>
+          <t>Tipo recibo</t>
+        </is>
+      </c>
+      <c r="C90" s="80" t="inlineStr">
+        <is>
+          <t>Fecha pago</t>
+        </is>
+      </c>
+      <c r="D90" s="80" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="E90" s="80" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="F90" s="80" t="inlineStr">
+        <is>
+          <t>Importe</t>
+        </is>
+      </c>
+      <c r="G90" s="80" t="inlineStr">
+        <is>
+          <t>Archivo fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B91" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C91" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D91" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E91" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F91" s="88" t="n">
+        <v>7906085</v>
+      </c>
+      <c r="G91" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B92" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C92" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D92" s="86" t="inlineStr">
+        <is>
+          <t>Beneficio Auto</t>
+        </is>
+      </c>
+      <c r="E92" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F92" s="88" t="n">
+        <v>180000</v>
+      </c>
+      <c r="G92" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B93" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C93" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D93" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E93" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F93" s="88" t="n">
+        <v>420571.02</v>
+      </c>
+      <c r="G93" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B94" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C94" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D94" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E94" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F94" s="88" t="n">
+        <v>114701.19</v>
+      </c>
+      <c r="G94" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B95" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C95" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D95" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E95" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F95" s="88" t="n">
+        <v>114701.19</v>
+      </c>
+      <c r="G95" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B96" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C96" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D96" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E96" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F96" s="88" t="n">
+        <v>1221703.83</v>
+      </c>
+      <c r="G96" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="86" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B97" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C97" s="87" t="n">
+        <v>46054</v>
+      </c>
+      <c r="D97" s="86" t="inlineStr">
+        <is>
+          <t>Dto Gimnasio</t>
+        </is>
+      </c>
+      <c r="E97" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F97" s="88" t="n">
+        <v>21900</v>
+      </c>
+      <c r="G97" s="86" t="inlineStr">
+        <is>
+          <t>ENERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B98" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C98" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D98" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E98" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F98" s="88" t="n">
+        <v>7906085</v>
+      </c>
+      <c r="G98" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B99" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C99" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D99" s="86" t="inlineStr">
+        <is>
+          <t>Beneficio Auto</t>
+        </is>
+      </c>
+      <c r="E99" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F99" s="88" t="n">
+        <v>208000</v>
+      </c>
+      <c r="G99" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B100" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C100" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D100" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E100" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F100" s="88" t="n">
+        <v>432557.3</v>
+      </c>
+      <c r="G100" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B101" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C101" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D101" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E101" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F101" s="88" t="n">
+        <v>117970.17</v>
+      </c>
+      <c r="G101" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B102" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C102" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D102" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E102" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F102" s="88" t="n">
+        <v>117970.17</v>
+      </c>
+      <c r="G102" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B103" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C103" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D103" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E103" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F103" s="88" t="n">
+        <v>1425004.25</v>
+      </c>
+      <c r="G103" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="86" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B104" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C104" s="87" t="n">
+        <v>46082</v>
+      </c>
+      <c r="D104" s="86" t="inlineStr">
+        <is>
+          <t>Dto Gimnasio</t>
+        </is>
+      </c>
+      <c r="E104" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F104" s="88" t="n">
+        <v>21900</v>
+      </c>
+      <c r="G104" s="86" t="inlineStr">
+        <is>
+          <t>FEBRERO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B105" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C105" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D105" s="86" t="inlineStr">
+        <is>
+          <t>R-Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E105" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F105" s="88" t="n">
+        <v>6799234</v>
+      </c>
+      <c r="G105" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B106" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C106" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D106" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E106" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F106" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="G106" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B107" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C107" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D107" s="86" t="inlineStr">
+        <is>
+          <t>Beneficio Auto</t>
+        </is>
+      </c>
+      <c r="E107" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F107" s="88" t="n">
+        <v>208000</v>
+      </c>
+      <c r="G107" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B108" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C108" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D108" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E108" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F108" s="88" t="n">
+        <v>445014.95</v>
+      </c>
+      <c r="G108" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B109" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C109" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D109" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E109" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F109" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="G109" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B110" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C110" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D110" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E110" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F110" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="G110" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B111" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C111" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D111" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E111" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F111" s="88" t="n">
+        <v>4658857.2</v>
+      </c>
+      <c r="G111" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="86" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B112" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + retroactivo</t>
+        </is>
+      </c>
+      <c r="C112" s="87" t="n">
+        <v>46113</v>
+      </c>
+      <c r="D112" s="86" t="inlineStr">
+        <is>
+          <t>Dto Gimnasio</t>
+        </is>
+      </c>
+      <c r="E112" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F112" s="88" t="n">
+        <v>21900</v>
+      </c>
+      <c r="G112" s="86" t="inlineStr">
+        <is>
+          <t>MARZO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B113" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C113" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D113" s="86" t="inlineStr">
+        <is>
+          <t>Bono de Transición</t>
+        </is>
+      </c>
+      <c r="E113" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F113" s="88" t="n">
+        <v>7296916.15</v>
+      </c>
+      <c r="G113" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B114" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C114" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D114" s="86" t="inlineStr">
+        <is>
+          <t>Gratificación Extraordinaria Anual</t>
+        </is>
+      </c>
+      <c r="E114" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F114" s="88" t="n">
+        <v>14596298</v>
+      </c>
+      <c r="G114" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B115" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C115" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D115" s="86" t="inlineStr">
+        <is>
+          <t>SAC Gratificación Extraordinaria</t>
+        </is>
+      </c>
+      <c r="E115" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F115" s="88" t="n">
+        <v>1215872</v>
+      </c>
+      <c r="G115" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B116" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C116" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D116" s="86" t="inlineStr">
+        <is>
+          <t>SAC sobre Bono de Transición</t>
+        </is>
+      </c>
+      <c r="E116" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F116" s="88" t="n">
+        <v>608076.35</v>
+      </c>
+      <c r="G116" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B117" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C117" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D117" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E117" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F117" s="88" t="n">
+        <v>445014.95</v>
+      </c>
+      <c r="G117" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B118" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C118" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D118" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E118" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F118" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="G118" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B119" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C119" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D119" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E119" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F119" s="88" t="n">
+        <v>121367.71</v>
+      </c>
+      <c r="G119" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B120" s="86" t="inlineStr">
+        <is>
+          <t>Bono anual / transición</t>
+        </is>
+      </c>
+      <c r="C120" s="87" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D120" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E120" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F120" s="88" t="n">
+        <v>3120893.08</v>
+      </c>
+      <c r="G120" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL BONO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B121" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C121" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D121" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E121" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F121" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="G121" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B122" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C122" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D122" s="86" t="inlineStr">
+        <is>
+          <t>Beneficio Auto</t>
+        </is>
+      </c>
+      <c r="E122" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F122" s="88" t="n">
+        <v>312000</v>
+      </c>
+      <c r="G122" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B123" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C123" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D123" s="86" t="inlineStr">
+        <is>
+          <t>Pago de Vacaciones</t>
+        </is>
+      </c>
+      <c r="E123" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F123" s="88" t="n">
+        <v>9758869.68</v>
+      </c>
+      <c r="G123" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B124" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C124" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D124" s="86" t="inlineStr">
+        <is>
+          <t>Dto Días No Trabajados Vacaciones</t>
+        </is>
+      </c>
+      <c r="E124" s="73" t="inlineStr">
+        <is>
+          <t>Haber negativo</t>
+        </is>
+      </c>
+      <c r="F124" s="88" t="n">
+        <v>-8132391.4</v>
+      </c>
+      <c r="G124" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B125" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C125" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D125" s="86" t="inlineStr">
+        <is>
+          <t>R-Dto Días No Trabajados</t>
+        </is>
+      </c>
+      <c r="E125" s="73" t="inlineStr">
+        <is>
+          <t>Haber negativo</t>
+        </is>
+      </c>
+      <c r="F125" s="88" t="n">
+        <v>-1151370.2</v>
+      </c>
+      <c r="G125" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B126" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C126" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D126" s="86" t="inlineStr">
+        <is>
+          <t>R-Licencia Especial</t>
+        </is>
+      </c>
+      <c r="E126" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F126" s="88" t="n">
+        <v>1381644.24</v>
+      </c>
+      <c r="G126" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B127" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C127" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D127" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E127" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F127" s="88" t="n">
+        <v>12905.43</v>
+      </c>
+      <c r="G127" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B128" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C128" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D128" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E128" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F128" s="88" t="n">
+        <v>3519.66</v>
+      </c>
+      <c r="G128" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B129" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C129" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D129" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E129" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F129" s="88" t="n">
+        <v>3519.66</v>
+      </c>
+      <c r="G129" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B130" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C130" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D130" s="86" t="inlineStr">
+        <is>
+          <t>Diferencia impuesto año anterior</t>
+        </is>
+      </c>
+      <c r="E130" s="73" t="inlineStr">
+        <is>
+          <t>Devolución Ganancias</t>
+        </is>
+      </c>
+      <c r="F130" s="88" t="n">
+        <v>-3564748.04</v>
+      </c>
+      <c r="G130" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B131" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C131" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D131" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E131" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F131" s="88" t="n">
+        <v>3813479.69</v>
+      </c>
+      <c r="G131" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="86" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B132" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo + vacaciones</t>
+        </is>
+      </c>
+      <c r="C132" s="87" t="n">
+        <v>46143</v>
+      </c>
+      <c r="D132" s="86" t="inlineStr">
+        <is>
+          <t>Dto Gimnasio</t>
+        </is>
+      </c>
+      <c r="E132" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F132" s="88" t="n">
+        <v>23400</v>
+      </c>
+      <c r="G132" s="86" t="inlineStr">
+        <is>
+          <t>ABRIL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B133" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C133" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D133" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E133" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F133" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="G133" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B134" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C134" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D134" s="86" t="inlineStr">
+        <is>
+          <t>Beneficio Auto</t>
+        </is>
+      </c>
+      <c r="E134" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F134" s="88" t="n">
+        <v>312000</v>
+      </c>
+      <c r="G134" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B135" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C135" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D135" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E135" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F135" s="88" t="n">
+        <v>473398.09</v>
+      </c>
+      <c r="G135" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B136" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C136" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D136" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E136" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F136" s="88" t="n">
+        <v>129108.57</v>
+      </c>
+      <c r="G136" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B137" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C137" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D137" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E137" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F137" s="88" t="n">
+        <v>129108.57</v>
+      </c>
+      <c r="G137" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B138" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C138" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D138" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E138" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F138" s="88" t="n">
+        <v>3415603.09</v>
+      </c>
+      <c r="G138" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="86" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B139" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C139" s="87" t="n">
+        <v>46174</v>
+      </c>
+      <c r="D139" s="86" t="inlineStr">
+        <is>
+          <t>Dto Gimnasio</t>
+        </is>
+      </c>
+      <c r="E139" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F139" s="88" t="n">
+        <v>23400</v>
+      </c>
+      <c r="G139" s="86" t="inlineStr">
+        <is>
+          <t>MAYO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B140" s="86" t="inlineStr">
+        <is>
+          <t>SAC 1° semestre</t>
+        </is>
+      </c>
+      <c r="C140" s="87" t="n">
+        <v>46196</v>
+      </c>
+      <c r="D140" s="86" t="inlineStr">
+        <is>
+          <t>S.A.C.</t>
+        </is>
+      </c>
+      <c r="E140" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F140" s="88" t="n">
+        <v>6622090.14</v>
+      </c>
+      <c r="G140" s="86" t="inlineStr">
+        <is>
+          <t>SAC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B141" s="86" t="inlineStr">
+        <is>
+          <t>SAC 1° semestre</t>
+        </is>
+      </c>
+      <c r="C141" s="87" t="n">
+        <v>46196</v>
+      </c>
+      <c r="D141" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre SAC</t>
+        </is>
+      </c>
+      <c r="E141" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F141" s="88" t="n">
+        <v>242805.88</v>
+      </c>
+      <c r="G141" s="86" t="inlineStr">
+        <is>
+          <t>SAC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B142" s="86" t="inlineStr">
+        <is>
+          <t>SAC 1° semestre</t>
+        </is>
+      </c>
+      <c r="C142" s="87" t="n">
+        <v>46196</v>
+      </c>
+      <c r="D142" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre SAC</t>
+        </is>
+      </c>
+      <c r="E142" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F142" s="88" t="n">
+        <v>66219.78999999999</v>
+      </c>
+      <c r="G142" s="86" t="inlineStr">
+        <is>
+          <t>SAC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B143" s="86" t="inlineStr">
+        <is>
+          <t>SAC 1° semestre</t>
+        </is>
+      </c>
+      <c r="C143" s="87" t="n">
+        <v>46196</v>
+      </c>
+      <c r="D143" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre SAC</t>
+        </is>
+      </c>
+      <c r="E143" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F143" s="88" t="n">
+        <v>66219.78999999999</v>
+      </c>
+      <c r="G143" s="86" t="inlineStr">
+        <is>
+          <t>SAC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B144" s="86" t="inlineStr">
+        <is>
+          <t>SAC 1° semestre</t>
+        </is>
+      </c>
+      <c r="C144" s="87" t="n">
+        <v>46196</v>
+      </c>
+      <c r="D144" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E144" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F144" s="88" t="n">
+        <v>536087.26</v>
+      </c>
+      <c r="G144" s="86" t="inlineStr">
+        <is>
+          <t>SAC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B145" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C145" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D145" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E145" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F145" s="88" t="n">
+        <v>11305702</v>
+      </c>
+      <c r="G145" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B146" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C146" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D146" s="86" t="inlineStr">
+        <is>
+          <t>Beneficio Auto</t>
+        </is>
+      </c>
+      <c r="E146" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F146" s="88" t="n">
+        <v>312000</v>
+      </c>
+      <c r="G146" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B147" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C147" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D147" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E147" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F147" s="88" t="n">
+        <v>485611.76</v>
+      </c>
+      <c r="G147" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B148" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C148" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D148" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E148" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F148" s="88" t="n">
+        <v>132439.57</v>
+      </c>
+      <c r="G148" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B149" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C149" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D149" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E149" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F149" s="88" t="n">
+        <v>132439.57</v>
+      </c>
+      <c r="G149" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B150" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C150" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D150" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E150" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F150" s="88" t="n">
+        <v>3408446.06</v>
+      </c>
+      <c r="G150" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B151" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C151" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D151" s="86" t="inlineStr">
+        <is>
+          <t>Dto Gimnasio</t>
+        </is>
+      </c>
+      <c r="E151" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F151" s="88" t="n">
+        <v>23400</v>
+      </c>
+      <c r="G151" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A56:E65"/>
-  <mergeCells count="15">
+  <autoFilter ref="A78:P86"/>
+  <mergeCells count="17">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A70:D70"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A89:G89"/>
     <mergeCell ref="A74:D74"/>
     <mergeCell ref="A69:D69"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A72:D72"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A77:P77"/>
     <mergeCell ref="A73:D73"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A71:D71"/>

</xml_diff>

<commit_message>
Apply July increase to car allowance
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -30,12 +30,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="[$ARS] #,##0"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="168" formatCode="[$ARS] #,##0.00"/>
+    <numFmt numFmtId="167" formatCode="[$ARS] #,##0.00"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -305,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -408,11 +407,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="13" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="13" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="13" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="11" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -798,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1820,23 +1823,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27592,7 +27578,7 @@
       </c>
       <c r="C5" s="68" t="inlineStr">
         <is>
-          <t>Vinculado a Ingresos Sol · ARS 11.305.702 + 12% desde julio</t>
+          <t>Básico: ARS 11.305.702 + 12% desde julio</t>
         </is>
       </c>
       <c r="D5" s="68" t="n"/>
@@ -27600,15 +27586,15 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="68" t="inlineStr">
         <is>
-          <t>Otros conceptos remunerativos mensuales</t>
+          <t>Car allowance mensual</t>
         </is>
       </c>
       <c r="B6" s="69" t="n">
-        <v>0</v>
+        <v>349440</v>
       </c>
       <c r="C6" s="68" t="inlineStr">
         <is>
-          <t>Bonus/comisiones/otros; editar si aplica</t>
+          <t>ARS 312.000 + 12% desde 01/07/2026</t>
         </is>
       </c>
       <c r="D6" s="68" t="n"/>
@@ -28516,28 +28502,19 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1"/>
+    <row r="75" ht="34" customHeight="1">
+      <c r="A75" s="83" t="inlineStr">
+        <is>
+          <t>• Car allowance: ARS 312.000 hasta junio; +12% desde julio = ARS 349.440. Bruto mensual total proyectado: ARS 13.011.827.</t>
+        </is>
+      </c>
+    </row>
     <row r="77">
       <c r="A77" s="84" t="inlineStr">
         <is>
           <t>RECIBOS MELI REALES 2026 — SUELDOS, BONO Y SAC</t>
         </is>
       </c>
-      <c r="B77" s="67" t="n"/>
-      <c r="C77" s="67" t="n"/>
-      <c r="D77" s="67" t="n"/>
-      <c r="E77" s="67" t="n"/>
-      <c r="F77" s="67" t="n"/>
-      <c r="G77" s="67" t="n"/>
-      <c r="H77" s="67" t="n"/>
-      <c r="I77" s="67" t="n"/>
-      <c r="J77" s="67" t="n"/>
-      <c r="K77" s="67" t="n"/>
-      <c r="L77" s="67" t="n"/>
-      <c r="M77" s="67" t="n"/>
-      <c r="N77" s="67" t="n"/>
-      <c r="O77" s="67" t="n"/>
-      <c r="P77" s="67" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="85" t="inlineStr">
@@ -28635,37 +28612,37 @@
       <c r="C79" s="87" t="n">
         <v>46054</v>
       </c>
-      <c r="D79" s="88" t="n">
+      <c r="D79" s="93" t="n">
         <v>7906085</v>
       </c>
-      <c r="E79" s="88" t="n">
+      <c r="E79" s="93" t="n">
         <v>180000</v>
       </c>
-      <c r="F79" s="88" t="n">
+      <c r="F79" s="93" t="n">
         <v>8086085</v>
       </c>
-      <c r="G79" s="88" t="n">
+      <c r="G79" s="93" t="n">
         <v>420571.02</v>
       </c>
-      <c r="H79" s="88" t="n">
+      <c r="H79" s="93" t="n">
         <v>114701.19</v>
       </c>
-      <c r="I79" s="88" t="n">
+      <c r="I79" s="93" t="n">
         <v>114701.19</v>
       </c>
-      <c r="J79" s="88" t="n">
+      <c r="J79" s="93" t="n">
         <v>1221703.83</v>
       </c>
-      <c r="K79" s="88" t="n">
+      <c r="K79" s="93" t="n">
         <v>21900</v>
       </c>
-      <c r="L79" s="88" t="n">
+      <c r="L79" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="M79" s="88" t="n">
+      <c r="M79" s="93" t="n">
         <v>1893577.23</v>
       </c>
-      <c r="N79" s="89" t="n">
+      <c r="N79" s="94" t="n">
         <v>6192507.77</v>
       </c>
       <c r="O79" s="86" t="inlineStr">
@@ -28673,7 +28650,7 @@
           <t>ENERO.pdf</t>
         </is>
       </c>
-      <c r="P79" s="88">
+      <c r="P79" s="93">
         <f>ROUND(F79-M79-N79,2)</f>
         <v/>
       </c>
@@ -28692,37 +28669,37 @@
       <c r="C80" s="87" t="n">
         <v>46082</v>
       </c>
-      <c r="D80" s="88" t="n">
+      <c r="D80" s="93" t="n">
         <v>7906085</v>
       </c>
-      <c r="E80" s="88" t="n">
+      <c r="E80" s="93" t="n">
         <v>208000</v>
       </c>
-      <c r="F80" s="88" t="n">
+      <c r="F80" s="93" t="n">
         <v>8114085</v>
       </c>
-      <c r="G80" s="88" t="n">
+      <c r="G80" s="93" t="n">
         <v>432557.3</v>
       </c>
-      <c r="H80" s="88" t="n">
+      <c r="H80" s="93" t="n">
         <v>117970.17</v>
       </c>
-      <c r="I80" s="88" t="n">
+      <c r="I80" s="93" t="n">
         <v>117970.17</v>
       </c>
-      <c r="J80" s="88" t="n">
+      <c r="J80" s="93" t="n">
         <v>1425004.25</v>
       </c>
-      <c r="K80" s="88" t="n">
+      <c r="K80" s="93" t="n">
         <v>21900</v>
       </c>
-      <c r="L80" s="88" t="n">
+      <c r="L80" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="M80" s="88" t="n">
+      <c r="M80" s="93" t="n">
         <v>2115401.89</v>
       </c>
-      <c r="N80" s="89" t="n">
+      <c r="N80" s="94" t="n">
         <v>5998683.11</v>
       </c>
       <c r="O80" s="86" t="inlineStr">
@@ -28730,7 +28707,7 @@
           <t>FEBRERO.pdf</t>
         </is>
       </c>
-      <c r="P80" s="88">
+      <c r="P80" s="93">
         <f>ROUND(F80-M80-N80,2)</f>
         <v/>
       </c>
@@ -28749,37 +28726,37 @@
       <c r="C81" s="87" t="n">
         <v>46113</v>
       </c>
-      <c r="D81" s="88" t="n">
+      <c r="D81" s="93" t="n">
         <v>11305702</v>
       </c>
-      <c r="E81" s="88" t="n">
+      <c r="E81" s="93" t="n">
         <v>7007234</v>
       </c>
-      <c r="F81" s="88" t="n">
+      <c r="F81" s="93" t="n">
         <v>18312936</v>
       </c>
-      <c r="G81" s="88" t="n">
+      <c r="G81" s="93" t="n">
         <v>445014.95</v>
       </c>
-      <c r="H81" s="88" t="n">
+      <c r="H81" s="93" t="n">
         <v>121367.71</v>
       </c>
-      <c r="I81" s="88" t="n">
+      <c r="I81" s="93" t="n">
         <v>121367.71</v>
       </c>
-      <c r="J81" s="88" t="n">
+      <c r="J81" s="93" t="n">
         <v>4658857.2</v>
       </c>
-      <c r="K81" s="88" t="n">
+      <c r="K81" s="93" t="n">
         <v>21900</v>
       </c>
-      <c r="L81" s="88" t="n">
+      <c r="L81" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="M81" s="88" t="n">
+      <c r="M81" s="93" t="n">
         <v>5368507.57</v>
       </c>
-      <c r="N81" s="89" t="n">
+      <c r="N81" s="94" t="n">
         <v>12944428.43</v>
       </c>
       <c r="O81" s="86" t="inlineStr">
@@ -28787,7 +28764,7 @@
           <t>MARZO.pdf</t>
         </is>
       </c>
-      <c r="P81" s="88">
+      <c r="P81" s="93">
         <f>ROUND(F81-M81-N81,2)</f>
         <v/>
       </c>
@@ -28806,37 +28783,37 @@
       <c r="C82" s="87" t="n">
         <v>46118</v>
       </c>
-      <c r="D82" s="88" t="n">
+      <c r="D82" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="E82" s="88" t="n">
+      <c r="E82" s="93" t="n">
         <v>23717162.5</v>
       </c>
-      <c r="F82" s="88" t="n">
+      <c r="F82" s="93" t="n">
         <v>23717162.5</v>
       </c>
-      <c r="G82" s="88" t="n">
+      <c r="G82" s="93" t="n">
         <v>445014.95</v>
       </c>
-      <c r="H82" s="88" t="n">
+      <c r="H82" s="93" t="n">
         <v>121367.71</v>
       </c>
-      <c r="I82" s="88" t="n">
+      <c r="I82" s="93" t="n">
         <v>121367.71</v>
       </c>
-      <c r="J82" s="88" t="n">
+      <c r="J82" s="93" t="n">
         <v>3120893.08</v>
       </c>
-      <c r="K82" s="88" t="n">
+      <c r="K82" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="L82" s="88" t="n">
+      <c r="L82" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="M82" s="88" t="n">
+      <c r="M82" s="93" t="n">
         <v>3808643.45</v>
       </c>
-      <c r="N82" s="89" t="n">
+      <c r="N82" s="94" t="n">
         <v>19908519.05</v>
       </c>
       <c r="O82" s="86" t="inlineStr">
@@ -28844,7 +28821,7 @@
           <t>ABRIL BONO.pdf</t>
         </is>
       </c>
-      <c r="P82" s="88">
+      <c r="P82" s="93">
         <f>ROUND(F82-M82-N82,2)</f>
         <v/>
       </c>
@@ -28863,37 +28840,37 @@
       <c r="C83" s="87" t="n">
         <v>46143</v>
       </c>
-      <c r="D83" s="88" t="n">
+      <c r="D83" s="93" t="n">
         <v>11305702</v>
       </c>
-      <c r="E83" s="88" t="n">
+      <c r="E83" s="93" t="n">
         <v>2168752.32</v>
       </c>
-      <c r="F83" s="88" t="n">
+      <c r="F83" s="93" t="n">
         <v>13474454.32</v>
       </c>
-      <c r="G83" s="88" t="n">
+      <c r="G83" s="93" t="n">
         <v>12905.43</v>
       </c>
-      <c r="H83" s="88" t="n">
+      <c r="H83" s="93" t="n">
         <v>3519.66</v>
       </c>
-      <c r="I83" s="88" t="n">
+      <c r="I83" s="93" t="n">
         <v>3519.66</v>
       </c>
-      <c r="J83" s="88" t="n">
+      <c r="J83" s="93" t="n">
         <v>3813479.69</v>
       </c>
-      <c r="K83" s="88" t="n">
+      <c r="K83" s="93" t="n">
         <v>23400</v>
       </c>
-      <c r="L83" s="88" t="n">
+      <c r="L83" s="93" t="n">
         <v>-3564748.04</v>
       </c>
-      <c r="M83" s="88" t="n">
+      <c r="M83" s="93" t="n">
         <v>292076.4</v>
       </c>
-      <c r="N83" s="89" t="n">
+      <c r="N83" s="94" t="n">
         <v>13182377.92</v>
       </c>
       <c r="O83" s="86" t="inlineStr">
@@ -28901,7 +28878,7 @@
           <t>ABRIL.pdf</t>
         </is>
       </c>
-      <c r="P83" s="88">
+      <c r="P83" s="93">
         <f>ROUND(F83-M83-N83,2)</f>
         <v/>
       </c>
@@ -28920,37 +28897,37 @@
       <c r="C84" s="87" t="n">
         <v>46174</v>
       </c>
-      <c r="D84" s="88" t="n">
+      <c r="D84" s="93" t="n">
         <v>11305702</v>
       </c>
-      <c r="E84" s="88" t="n">
+      <c r="E84" s="93" t="n">
         <v>312000</v>
       </c>
-      <c r="F84" s="88" t="n">
+      <c r="F84" s="93" t="n">
         <v>11617702</v>
       </c>
-      <c r="G84" s="88" t="n">
+      <c r="G84" s="93" t="n">
         <v>473398.09</v>
       </c>
-      <c r="H84" s="88" t="n">
+      <c r="H84" s="93" t="n">
         <v>129108.57</v>
       </c>
-      <c r="I84" s="88" t="n">
+      <c r="I84" s="93" t="n">
         <v>129108.57</v>
       </c>
-      <c r="J84" s="88" t="n">
+      <c r="J84" s="93" t="n">
         <v>3415603.09</v>
       </c>
-      <c r="K84" s="88" t="n">
+      <c r="K84" s="93" t="n">
         <v>23400</v>
       </c>
-      <c r="L84" s="88" t="n">
+      <c r="L84" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="M84" s="88" t="n">
+      <c r="M84" s="93" t="n">
         <v>4170618.32</v>
       </c>
-      <c r="N84" s="89" t="n">
+      <c r="N84" s="94" t="n">
         <v>7447083.68</v>
       </c>
       <c r="O84" s="86" t="inlineStr">
@@ -28958,7 +28935,7 @@
           <t>MAYO.pdf</t>
         </is>
       </c>
-      <c r="P84" s="88">
+      <c r="P84" s="93">
         <f>ROUND(F84-M84-N84,2)</f>
         <v/>
       </c>
@@ -28977,37 +28954,37 @@
       <c r="C85" s="87" t="n">
         <v>46196</v>
       </c>
-      <c r="D85" s="88" t="n">
+      <c r="D85" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="E85" s="88" t="n">
+      <c r="E85" s="93" t="n">
         <v>6622090.14</v>
       </c>
-      <c r="F85" s="88" t="n">
+      <c r="F85" s="93" t="n">
         <v>6622090.14</v>
       </c>
-      <c r="G85" s="88" t="n">
+      <c r="G85" s="93" t="n">
         <v>242805.88</v>
       </c>
-      <c r="H85" s="88" t="n">
+      <c r="H85" s="93" t="n">
         <v>66219.78999999999</v>
       </c>
-      <c r="I85" s="88" t="n">
+      <c r="I85" s="93" t="n">
         <v>66219.78999999999</v>
       </c>
-      <c r="J85" s="88" t="n">
+      <c r="J85" s="93" t="n">
         <v>536087.26</v>
       </c>
-      <c r="K85" s="88" t="n">
+      <c r="K85" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="L85" s="88" t="n">
+      <c r="L85" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="M85" s="88" t="n">
+      <c r="M85" s="93" t="n">
         <v>911332.72</v>
       </c>
-      <c r="N85" s="89" t="n">
+      <c r="N85" s="94" t="n">
         <v>5710757.42</v>
       </c>
       <c r="O85" s="86" t="inlineStr">
@@ -29015,7 +28992,7 @@
           <t>SAC.pdf</t>
         </is>
       </c>
-      <c r="P85" s="88">
+      <c r="P85" s="93">
         <f>ROUND(F85-M85-N85,2)</f>
         <v/>
       </c>
@@ -29034,37 +29011,37 @@
       <c r="C86" s="87" t="n">
         <v>46204</v>
       </c>
-      <c r="D86" s="88" t="n">
+      <c r="D86" s="93" t="n">
         <v>11305702</v>
       </c>
-      <c r="E86" s="88" t="n">
+      <c r="E86" s="93" t="n">
         <v>312000</v>
       </c>
-      <c r="F86" s="88" t="n">
+      <c r="F86" s="93" t="n">
         <v>11617702</v>
       </c>
-      <c r="G86" s="88" t="n">
+      <c r="G86" s="93" t="n">
         <v>485611.76</v>
       </c>
-      <c r="H86" s="88" t="n">
+      <c r="H86" s="93" t="n">
         <v>132439.57</v>
       </c>
-      <c r="I86" s="88" t="n">
+      <c r="I86" s="93" t="n">
         <v>132439.57</v>
       </c>
-      <c r="J86" s="88" t="n">
+      <c r="J86" s="93" t="n">
         <v>3408446.06</v>
       </c>
-      <c r="K86" s="88" t="n">
+      <c r="K86" s="93" t="n">
         <v>23400</v>
       </c>
-      <c r="L86" s="88" t="n">
+      <c r="L86" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="M86" s="88" t="n">
+      <c r="M86" s="93" t="n">
         <v>4182336.96</v>
       </c>
-      <c r="N86" s="89" t="n">
+      <c r="N86" s="94" t="n">
         <v>7435365.04</v>
       </c>
       <c r="O86" s="86" t="inlineStr">
@@ -29072,7 +29049,7 @@
           <t>JUNIO.pdf</t>
         </is>
       </c>
-      <c r="P86" s="88">
+      <c r="P86" s="93">
         <f>ROUND(F86-M86-N86,2)</f>
         <v/>
       </c>
@@ -29085,52 +29062,52 @@
       </c>
       <c r="B87" s="68" t="n"/>
       <c r="C87" s="68" t="n"/>
-      <c r="D87" s="91">
+      <c r="D87" s="95">
         <f>SUM(D79:D86)</f>
         <v/>
       </c>
-      <c r="E87" s="91">
+      <c r="E87" s="95">
         <f>SUM(E79:E86)</f>
         <v/>
       </c>
-      <c r="F87" s="91">
+      <c r="F87" s="95">
         <f>SUM(F79:F86)</f>
         <v/>
       </c>
-      <c r="G87" s="91">
+      <c r="G87" s="95">
         <f>SUM(G79:G86)</f>
         <v/>
       </c>
-      <c r="H87" s="91">
+      <c r="H87" s="95">
         <f>SUM(H79:H86)</f>
         <v/>
       </c>
-      <c r="I87" s="91">
+      <c r="I87" s="95">
         <f>SUM(I79:I86)</f>
         <v/>
       </c>
-      <c r="J87" s="91">
+      <c r="J87" s="95">
         <f>SUM(J79:J86)</f>
         <v/>
       </c>
-      <c r="K87" s="91">
+      <c r="K87" s="95">
         <f>SUM(K79:K86)</f>
         <v/>
       </c>
-      <c r="L87" s="91">
+      <c r="L87" s="95">
         <f>SUM(L79:L86)</f>
         <v/>
       </c>
-      <c r="M87" s="91">
+      <c r="M87" s="95">
         <f>SUM(M79:M86)</f>
         <v/>
       </c>
-      <c r="N87" s="91">
+      <c r="N87" s="95">
         <f>SUM(N79:N86)</f>
         <v/>
       </c>
       <c r="O87" s="68" t="n"/>
-      <c r="P87" s="92">
+      <c r="P87" s="96">
         <f>ROUND(F87-M87-N87,2)</f>
         <v/>
       </c>
@@ -29141,12 +29118,6 @@
           <t>DETALLE EXTRAÍDO DE CONCEPTOS</t>
         </is>
       </c>
-      <c r="B89" s="67" t="n"/>
-      <c r="C89" s="67" t="n"/>
-      <c r="D89" s="67" t="n"/>
-      <c r="E89" s="67" t="n"/>
-      <c r="F89" s="67" t="n"/>
-      <c r="G89" s="67" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="80" t="inlineStr">
@@ -29209,7 +29180,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F91" s="88" t="n">
+      <c r="F91" s="93" t="n">
         <v>7906085</v>
       </c>
       <c r="G91" s="86" t="inlineStr">
@@ -29242,7 +29213,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F92" s="88" t="n">
+      <c r="F92" s="93" t="n">
         <v>180000</v>
       </c>
       <c r="G92" s="86" t="inlineStr">
@@ -29275,7 +29246,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F93" s="88" t="n">
+      <c r="F93" s="93" t="n">
         <v>420571.02</v>
       </c>
       <c r="G93" s="86" t="inlineStr">
@@ -29308,7 +29279,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F94" s="88" t="n">
+      <c r="F94" s="93" t="n">
         <v>114701.19</v>
       </c>
       <c r="G94" s="86" t="inlineStr">
@@ -29341,7 +29312,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F95" s="88" t="n">
+      <c r="F95" s="93" t="n">
         <v>114701.19</v>
       </c>
       <c r="G95" s="86" t="inlineStr">
@@ -29374,7 +29345,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F96" s="88" t="n">
+      <c r="F96" s="93" t="n">
         <v>1221703.83</v>
       </c>
       <c r="G96" s="86" t="inlineStr">
@@ -29407,7 +29378,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F97" s="88" t="n">
+      <c r="F97" s="93" t="n">
         <v>21900</v>
       </c>
       <c r="G97" s="86" t="inlineStr">
@@ -29440,7 +29411,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F98" s="88" t="n">
+      <c r="F98" s="93" t="n">
         <v>7906085</v>
       </c>
       <c r="G98" s="86" t="inlineStr">
@@ -29473,7 +29444,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F99" s="88" t="n">
+      <c r="F99" s="93" t="n">
         <v>208000</v>
       </c>
       <c r="G99" s="86" t="inlineStr">
@@ -29506,7 +29477,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F100" s="88" t="n">
+      <c r="F100" s="93" t="n">
         <v>432557.3</v>
       </c>
       <c r="G100" s="86" t="inlineStr">
@@ -29539,7 +29510,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F101" s="88" t="n">
+      <c r="F101" s="93" t="n">
         <v>117970.17</v>
       </c>
       <c r="G101" s="86" t="inlineStr">
@@ -29572,7 +29543,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F102" s="88" t="n">
+      <c r="F102" s="93" t="n">
         <v>117970.17</v>
       </c>
       <c r="G102" s="86" t="inlineStr">
@@ -29605,7 +29576,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F103" s="88" t="n">
+      <c r="F103" s="93" t="n">
         <v>1425004.25</v>
       </c>
       <c r="G103" s="86" t="inlineStr">
@@ -29638,7 +29609,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F104" s="88" t="n">
+      <c r="F104" s="93" t="n">
         <v>21900</v>
       </c>
       <c r="G104" s="86" t="inlineStr">
@@ -29671,7 +29642,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F105" s="88" t="n">
+      <c r="F105" s="93" t="n">
         <v>6799234</v>
       </c>
       <c r="G105" s="86" t="inlineStr">
@@ -29704,7 +29675,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F106" s="88" t="n">
+      <c r="F106" s="93" t="n">
         <v>11305702</v>
       </c>
       <c r="G106" s="86" t="inlineStr">
@@ -29737,7 +29708,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F107" s="88" t="n">
+      <c r="F107" s="93" t="n">
         <v>208000</v>
       </c>
       <c r="G107" s="86" t="inlineStr">
@@ -29770,7 +29741,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F108" s="88" t="n">
+      <c r="F108" s="93" t="n">
         <v>445014.95</v>
       </c>
       <c r="G108" s="86" t="inlineStr">
@@ -29803,7 +29774,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F109" s="88" t="n">
+      <c r="F109" s="93" t="n">
         <v>121367.71</v>
       </c>
       <c r="G109" s="86" t="inlineStr">
@@ -29836,7 +29807,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F110" s="88" t="n">
+      <c r="F110" s="93" t="n">
         <v>121367.71</v>
       </c>
       <c r="G110" s="86" t="inlineStr">
@@ -29869,7 +29840,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F111" s="88" t="n">
+      <c r="F111" s="93" t="n">
         <v>4658857.2</v>
       </c>
       <c r="G111" s="86" t="inlineStr">
@@ -29902,7 +29873,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F112" s="88" t="n">
+      <c r="F112" s="93" t="n">
         <v>21900</v>
       </c>
       <c r="G112" s="86" t="inlineStr">
@@ -29935,7 +29906,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F113" s="88" t="n">
+      <c r="F113" s="93" t="n">
         <v>7296916.15</v>
       </c>
       <c r="G113" s="86" t="inlineStr">
@@ -29968,7 +29939,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F114" s="88" t="n">
+      <c r="F114" s="93" t="n">
         <v>14596298</v>
       </c>
       <c r="G114" s="86" t="inlineStr">
@@ -30001,7 +29972,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F115" s="88" t="n">
+      <c r="F115" s="93" t="n">
         <v>1215872</v>
       </c>
       <c r="G115" s="86" t="inlineStr">
@@ -30034,7 +30005,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F116" s="88" t="n">
+      <c r="F116" s="93" t="n">
         <v>608076.35</v>
       </c>
       <c r="G116" s="86" t="inlineStr">
@@ -30067,7 +30038,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F117" s="88" t="n">
+      <c r="F117" s="93" t="n">
         <v>445014.95</v>
       </c>
       <c r="G117" s="86" t="inlineStr">
@@ -30100,7 +30071,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F118" s="88" t="n">
+      <c r="F118" s="93" t="n">
         <v>121367.71</v>
       </c>
       <c r="G118" s="86" t="inlineStr">
@@ -30133,7 +30104,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F119" s="88" t="n">
+      <c r="F119" s="93" t="n">
         <v>121367.71</v>
       </c>
       <c r="G119" s="86" t="inlineStr">
@@ -30166,7 +30137,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F120" s="88" t="n">
+      <c r="F120" s="93" t="n">
         <v>3120893.08</v>
       </c>
       <c r="G120" s="86" t="inlineStr">
@@ -30199,7 +30170,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F121" s="88" t="n">
+      <c r="F121" s="93" t="n">
         <v>11305702</v>
       </c>
       <c r="G121" s="86" t="inlineStr">
@@ -30232,7 +30203,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F122" s="88" t="n">
+      <c r="F122" s="93" t="n">
         <v>312000</v>
       </c>
       <c r="G122" s="86" t="inlineStr">
@@ -30265,7 +30236,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F123" s="88" t="n">
+      <c r="F123" s="93" t="n">
         <v>9758869.68</v>
       </c>
       <c r="G123" s="86" t="inlineStr">
@@ -30298,7 +30269,7 @@
           <t>Haber negativo</t>
         </is>
       </c>
-      <c r="F124" s="88" t="n">
+      <c r="F124" s="93" t="n">
         <v>-8132391.4</v>
       </c>
       <c r="G124" s="86" t="inlineStr">
@@ -30331,7 +30302,7 @@
           <t>Haber negativo</t>
         </is>
       </c>
-      <c r="F125" s="88" t="n">
+      <c r="F125" s="93" t="n">
         <v>-1151370.2</v>
       </c>
       <c r="G125" s="86" t="inlineStr">
@@ -30364,7 +30335,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F126" s="88" t="n">
+      <c r="F126" s="93" t="n">
         <v>1381644.24</v>
       </c>
       <c r="G126" s="86" t="inlineStr">
@@ -30397,7 +30368,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F127" s="88" t="n">
+      <c r="F127" s="93" t="n">
         <v>12905.43</v>
       </c>
       <c r="G127" s="86" t="inlineStr">
@@ -30430,7 +30401,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F128" s="88" t="n">
+      <c r="F128" s="93" t="n">
         <v>3519.66</v>
       </c>
       <c r="G128" s="86" t="inlineStr">
@@ -30463,7 +30434,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F129" s="88" t="n">
+      <c r="F129" s="93" t="n">
         <v>3519.66</v>
       </c>
       <c r="G129" s="86" t="inlineStr">
@@ -30496,7 +30467,7 @@
           <t>Devolución Ganancias</t>
         </is>
       </c>
-      <c r="F130" s="88" t="n">
+      <c r="F130" s="93" t="n">
         <v>-3564748.04</v>
       </c>
       <c r="G130" s="86" t="inlineStr">
@@ -30529,7 +30500,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F131" s="88" t="n">
+      <c r="F131" s="93" t="n">
         <v>3813479.69</v>
       </c>
       <c r="G131" s="86" t="inlineStr">
@@ -30562,7 +30533,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F132" s="88" t="n">
+      <c r="F132" s="93" t="n">
         <v>23400</v>
       </c>
       <c r="G132" s="86" t="inlineStr">
@@ -30595,7 +30566,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F133" s="88" t="n">
+      <c r="F133" s="93" t="n">
         <v>11305702</v>
       </c>
       <c r="G133" s="86" t="inlineStr">
@@ -30628,7 +30599,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F134" s="88" t="n">
+      <c r="F134" s="93" t="n">
         <v>312000</v>
       </c>
       <c r="G134" s="86" t="inlineStr">
@@ -30661,7 +30632,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F135" s="88" t="n">
+      <c r="F135" s="93" t="n">
         <v>473398.09</v>
       </c>
       <c r="G135" s="86" t="inlineStr">
@@ -30694,7 +30665,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F136" s="88" t="n">
+      <c r="F136" s="93" t="n">
         <v>129108.57</v>
       </c>
       <c r="G136" s="86" t="inlineStr">
@@ -30727,7 +30698,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F137" s="88" t="n">
+      <c r="F137" s="93" t="n">
         <v>129108.57</v>
       </c>
       <c r="G137" s="86" t="inlineStr">
@@ -30760,7 +30731,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F138" s="88" t="n">
+      <c r="F138" s="93" t="n">
         <v>3415603.09</v>
       </c>
       <c r="G138" s="86" t="inlineStr">
@@ -30793,7 +30764,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F139" s="88" t="n">
+      <c r="F139" s="93" t="n">
         <v>23400</v>
       </c>
       <c r="G139" s="86" t="inlineStr">
@@ -30826,7 +30797,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F140" s="88" t="n">
+      <c r="F140" s="93" t="n">
         <v>6622090.14</v>
       </c>
       <c r="G140" s="86" t="inlineStr">
@@ -30859,7 +30830,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F141" s="88" t="n">
+      <c r="F141" s="93" t="n">
         <v>242805.88</v>
       </c>
       <c r="G141" s="86" t="inlineStr">
@@ -30892,7 +30863,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F142" s="88" t="n">
+      <c r="F142" s="93" t="n">
         <v>66219.78999999999</v>
       </c>
       <c r="G142" s="86" t="inlineStr">
@@ -30925,7 +30896,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F143" s="88" t="n">
+      <c r="F143" s="93" t="n">
         <v>66219.78999999999</v>
       </c>
       <c r="G143" s="86" t="inlineStr">
@@ -30958,7 +30929,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F144" s="88" t="n">
+      <c r="F144" s="93" t="n">
         <v>536087.26</v>
       </c>
       <c r="G144" s="86" t="inlineStr">
@@ -30991,7 +30962,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F145" s="88" t="n">
+      <c r="F145" s="93" t="n">
         <v>11305702</v>
       </c>
       <c r="G145" s="86" t="inlineStr">
@@ -31024,7 +30995,7 @@
           <t>Haber</t>
         </is>
       </c>
-      <c r="F146" s="88" t="n">
+      <c r="F146" s="93" t="n">
         <v>312000</v>
       </c>
       <c r="G146" s="86" t="inlineStr">
@@ -31057,7 +31028,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F147" s="88" t="n">
+      <c r="F147" s="93" t="n">
         <v>485611.76</v>
       </c>
       <c r="G147" s="86" t="inlineStr">
@@ -31090,7 +31061,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F148" s="88" t="n">
+      <c r="F148" s="93" t="n">
         <v>132439.57</v>
       </c>
       <c r="G148" s="86" t="inlineStr">
@@ -31123,7 +31094,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F149" s="88" t="n">
+      <c r="F149" s="93" t="n">
         <v>132439.57</v>
       </c>
       <c r="G149" s="86" t="inlineStr">
@@ -31156,7 +31127,7 @@
           <t>Descuento Ganancias</t>
         </is>
       </c>
-      <c r="F150" s="88" t="n">
+      <c r="F150" s="93" t="n">
         <v>3408446.06</v>
       </c>
       <c r="G150" s="86" t="inlineStr">
@@ -31189,7 +31160,7 @@
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F151" s="88" t="n">
+      <c r="F151" s="93" t="n">
         <v>23400</v>
       </c>
       <c r="G151" s="86" t="inlineStr">
@@ -31200,13 +31171,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A78:P86"/>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A70:D70"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A55:E55"/>
     <mergeCell ref="A89:G89"/>
+    <mergeCell ref="A75:D75"/>
     <mergeCell ref="A74:D74"/>
     <mergeCell ref="A69:D69"/>
     <mergeCell ref="A4:D4"/>

</xml_diff>

<commit_message>
Classify Agustina Vissani as personal hairdressing
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1208,16 +1208,10 @@
       </c>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n">
-        <v>75000</v>
-      </c>
+      <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n">
-        <v>125000</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>135000</v>
-      </c>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="5" t="n"/>
@@ -9446,16 +9440,88 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="44" t="n"/>
-      <c r="D223" s="26" t="n"/>
+      <c r="A223" s="44" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Agustina Vissani</t>
+        </is>
+      </c>
+      <c r="D223" s="26" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Agustina Vissani · gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="224">
-      <c r="A224" s="44" t="n"/>
-      <c r="D224" s="26" t="n"/>
+      <c r="A224" s="44" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Agustina Vissani</t>
+        </is>
+      </c>
+      <c r="D224" s="26" t="n">
+        <v>125000</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Agustina Vissani · gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="225">
-      <c r="A225" s="44" t="n"/>
-      <c r="D225" s="26" t="n"/>
+      <c r="A225" s="44" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Agustina Vissani</t>
+        </is>
+      </c>
+      <c r="D225" s="26" t="n">
+        <v>135000</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Agustina Vissani · gasto personal Sol</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="44" t="n"/>

</xml_diff>

<commit_message>
Classify Saphirus as CIUDAD aromatizers
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -801,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1610,208 +1610,238 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AROMATIZANTES</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Saphirus — Aromatizantes</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="26" t="n"/>
+      <c r="G20" s="26" t="n"/>
+      <c r="H20" s="26" t="n"/>
+      <c r="I20" t="n">
+        <v>79900</v>
+      </c>
+      <c r="J20" s="26" t="n"/>
+      <c r="P20" s="26">
+        <f>SUM(D20:O20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="23" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="7">
-        <f>SUM(D5:D19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="7">
-        <f>SUM(E5:E19)</f>
-        <v/>
-      </c>
-      <c r="F20" s="7">
-        <f>SUM(F5:F19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="7">
-        <f>SUM(G5:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="7">
-        <f>SUM(H5:H19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="7">
-        <f>SUM(I5:I19)</f>
-        <v/>
-      </c>
-      <c r="J20" s="7">
-        <f>SUM(J5:J19)</f>
-        <v/>
-      </c>
-      <c r="K20" s="7">
-        <f>SUM(K5:K19)</f>
-        <v/>
-      </c>
-      <c r="L20" s="7">
-        <f>SUM(L5:L19)</f>
-        <v/>
-      </c>
-      <c r="M20" s="7">
-        <f>SUM(M5:M19)</f>
-        <v/>
-      </c>
-      <c r="N20" s="7">
-        <f>SUM(N5:N19)</f>
-        <v/>
-      </c>
-      <c r="O20" s="7">
-        <f>SUM(O5:O19)</f>
-        <v/>
-      </c>
-      <c r="P20" s="7">
-        <f>SUM(P5:P19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="B21" s="23" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="7">
+        <f>SUM(D5:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="7">
+        <f>SUM(E5:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="7">
+        <f>SUM(F5:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="7">
+        <f>SUM(G5:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="7">
+        <f>SUM(H5:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="7">
+        <f>SUM(I5:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="7">
+        <f>SUM(J5:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="7">
+        <f>SUM(K5:K20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="7">
+        <f>SUM(L5:L20)</f>
+        <v/>
+      </c>
+      <c r="M21" s="7">
+        <f>SUM(M5:M20)</f>
+        <v/>
+      </c>
+      <c r="N21" s="7">
+        <f>SUM(N5:N20)</f>
+        <v/>
+      </c>
+      <c r="O21" s="7">
+        <f>SUM(O5:O20)</f>
+        <v/>
+      </c>
+      <c r="P21" s="7">
+        <f>SUM(P5:P20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio). Julio período pendiente.</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio). Julio período pendiente.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="30" t="inlineStr">
         <is>
-          <t>• FARMACIA: Farmacity / Farmacia Selma / Farmacia Maure — nombre de farmacia en comentario</t>
+          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="30" t="inlineStr">
         <is>
-          <t>• Personal (Pago directo): va a OHIGGINS → TV CABLE-INTERNET — no CIUDAD</t>
+          <t>• FARMACIA: Farmacity / Farmacia Selma / Farmacia Maure — nombre de farmacia en comentario</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="30" t="inlineStr">
         <is>
-          <t>• Inversión: hoja "Inversión" (bonos, plazos fijos y otros; no suma al TOTAL de gastos)</t>
+          <t>• Personal (Pago directo): va a OHIGGINS → TV CABLE-INTERNET — no CIUDAD</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="30" t="inlineStr">
         <is>
-          <t>• Transferencias recibidas: hoja "Transferencias recibidas" (no suma al total de gastos)</t>
+          <t>• Inversión: hoja "Inversión" (bonos, plazos fijos y otros; no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
         <is>
-          <t>• Expensas consorcios: hoja "Expensas Consorcios" (Consorcio De Propiet = CIUDAD; no ALMACEN SOL)</t>
+          <t>• Transferencias recibidas: hoja "Transferencias recibidas" (no suma al total de gastos)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="30" t="inlineStr">
         <is>
+          <t>• Expensas consorcios: hoja "Expensas Consorcios" (Consorcio De Propiet = CIUDAD; no ALMACEN SOL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
           <t>• Gasto personal Sol (Tuenti, Apple, ropa, ML, extras, transferencias a terceros): hoja "Gasto Personal Sol" (no suma al total CIUDAD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>• Pago de tarjetas: hoja "Pago de Tarjetas" (pago de resumen TC; no es gasto nuevo de la matriz)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL: solo comida/súper/combustible en "Almacen Detalle". Resto personal → "Gasto Personal Sol"</t>
+          <t>• Pago de tarjetas: hoja "Pago de Tarjetas" (pago de resumen TC; no es gasto nuevo de la matriz)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>• ABL CIUDAD: partida AGIP 397789 (OHIGGINS = 3016365 → otra carpeta)</t>
+          <t>• ALMACEN SOL: solo comida/súper/combustible en "Almacen Detalle". Resto personal → "Gasto Personal Sol"</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>• Edesur → BONORINO. Edenor: Sanes=CIUDAD; Ivilmar/Marta Chagas=OHIGGINS. Telecentro=CIUDAD.</t>
+          <t>• ABL CIUDAD: partida AGIP 397789 (OHIGGINS = 3016365 → otra carpeta)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>• Ingresos Sol: básico anterior ARS 11.305.702; +12% desde 01/07 → ARS 12.662.387 (cobro 01/08). No suma al total de gastos.</t>
+          <t>• Edesur → BONORINO. Edenor: Sanes=CIUDAD; Ivilmar/Marta Chagas=OHIGGINS. Telecentro=CIUDAD.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
+        <is>
+          <t>• Ingresos Sol: básico anterior ARS 11.305.702; +12% desde 01/07 → ARS 12.662.387 (cobro 01/08). No suma al total de gastos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>• MELI: simulador + detalle real de recibos 2026 (sueldos, bono y SAC). No suma al total de gastos.</t>
         </is>
@@ -8404,32 +8434,8 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="44" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>Saphirus</t>
-        </is>
-      </c>
-      <c r="D186" s="26" t="n">
-        <v>79900</v>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="F186" t="inlineStr">
-        <is>
-          <t>¿hogar? · gasto personal Sol (ex-PENDIENTE)</t>
-        </is>
-      </c>
+      <c r="A186" s="44" t="n"/>
+      <c r="D186" s="26" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="44" t="n">
@@ -18989,7 +18995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20931,6 +20937,39 @@
       <c r="I60" t="inlineStr">
         <is>
           <t>Julio</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="44" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>AROMATIZANTES</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CASA — Aromatizantes Saphirus</t>
+        </is>
+      </c>
+      <c r="D61" s="26" t="n">
+        <v>79900</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>CASA · AROMATIZANTES · Saphirus · CIUDAD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Junio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classify three Mercado Libre purchases as CIUDAD repairs
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -801,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1639,208 +1639,237 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>REPARACIONES Y REPUESTOS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Reparaciones y repuestos — CIUDAD</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="26" t="n"/>
+      <c r="G21" s="26" t="n">
+        <v>150030</v>
+      </c>
+      <c r="H21" s="26" t="n"/>
+      <c r="J21" s="26" t="n"/>
+      <c r="P21" s="26">
+        <f>SUM(D21:O21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B21" s="23" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="7">
-        <f>SUM(D5:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="7">
-        <f>SUM(E5:E20)</f>
-        <v/>
-      </c>
-      <c r="F21" s="7">
-        <f>SUM(F5:F20)</f>
-        <v/>
-      </c>
-      <c r="G21" s="7">
-        <f>SUM(G5:G20)</f>
-        <v/>
-      </c>
-      <c r="H21" s="7">
-        <f>SUM(H5:H20)</f>
-        <v/>
-      </c>
-      <c r="I21" s="7">
-        <f>SUM(I5:I20)</f>
-        <v/>
-      </c>
-      <c r="J21" s="7">
-        <f>SUM(J5:J20)</f>
-        <v/>
-      </c>
-      <c r="K21" s="7">
-        <f>SUM(K5:K20)</f>
-        <v/>
-      </c>
-      <c r="L21" s="7">
-        <f>SUM(L5:L20)</f>
-        <v/>
-      </c>
-      <c r="M21" s="7">
-        <f>SUM(M5:M20)</f>
-        <v/>
-      </c>
-      <c r="N21" s="7">
-        <f>SUM(N5:N20)</f>
-        <v/>
-      </c>
-      <c r="O21" s="7">
-        <f>SUM(O5:O20)</f>
-        <v/>
-      </c>
-      <c r="P21" s="7">
-        <f>SUM(P5:P20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="7">
+        <f>SUM(D5:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="7">
+        <f>SUM(E5:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="7">
+        <f>SUM(F5:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="7">
+        <f>SUM(G5:G21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="7">
+        <f>SUM(H5:H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="7">
+        <f>SUM(I5:I21)</f>
+        <v/>
+      </c>
+      <c r="J22" s="7">
+        <f>SUM(J5:J21)</f>
+        <v/>
+      </c>
+      <c r="K22" s="7">
+        <f>SUM(K5:K21)</f>
+        <v/>
+      </c>
+      <c r="L22" s="7">
+        <f>SUM(L5:L21)</f>
+        <v/>
+      </c>
+      <c r="M22" s="7">
+        <f>SUM(M5:M21)</f>
+        <v/>
+      </c>
+      <c r="N22" s="7">
+        <f>SUM(N5:N21)</f>
+        <v/>
+      </c>
+      <c r="O22" s="7">
+        <f>SUM(O5:O21)</f>
+        <v/>
+      </c>
+      <c r="P22" s="7">
+        <f>SUM(P5:P21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio). Julio período pendiente.</t>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio). Julio período pendiente.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>• TRANSPORTE: Cabify / Uber (Ebanx) / Didi — montos enteros ceil desde Mercado Pago</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="30" t="inlineStr">
         <is>
-          <t>• FARMACIA: Farmacity / Farmacia Selma / Farmacia Maure — nombre de farmacia en comentario</t>
+          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="30" t="inlineStr">
         <is>
-          <t>• Personal (Pago directo): va a OHIGGINS → TV CABLE-INTERNET — no CIUDAD</t>
+          <t>• FARMACIA: Farmacity / Farmacia Selma / Farmacia Maure — nombre de farmacia en comentario</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="30" t="inlineStr">
         <is>
-          <t>• Inversión: hoja "Inversión" (bonos, plazos fijos y otros; no suma al TOTAL de gastos)</t>
+          <t>• Personal (Pago directo): va a OHIGGINS → TV CABLE-INTERNET — no CIUDAD</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
         <is>
-          <t>• Transferencias recibidas: hoja "Transferencias recibidas" (no suma al total de gastos)</t>
+          <t>• Inversión: hoja "Inversión" (bonos, plazos fijos y otros; no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="30" t="inlineStr">
         <is>
-          <t>• Expensas consorcios: hoja "Expensas Consorcios" (Consorcio De Propiet = CIUDAD; no ALMACEN SOL)</t>
+          <t>• Transferencias recibidas: hoja "Transferencias recibidas" (no suma al total de gastos)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="30" t="inlineStr">
         <is>
+          <t>• Expensas consorcios: hoja "Expensas Consorcios" (Consorcio De Propiet = CIUDAD; no ALMACEN SOL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
           <t>• Gasto personal Sol (Tuenti, Apple, ropa, ML, extras, transferencias a terceros): hoja "Gasto Personal Sol" (no suma al total CIUDAD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>• Pago de tarjetas: hoja "Pago de Tarjetas" (pago de resumen TC; no es gasto nuevo de la matriz)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL: solo comida/súper/combustible en "Almacen Detalle". Resto personal → "Gasto Personal Sol"</t>
+          <t>• Pago de tarjetas: hoja "Pago de Tarjetas" (pago de resumen TC; no es gasto nuevo de la matriz)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>• ABL CIUDAD: partida AGIP 397789 (OHIGGINS = 3016365 → otra carpeta)</t>
+          <t>• ALMACEN SOL: solo comida/súper/combustible en "Almacen Detalle". Resto personal → "Gasto Personal Sol"</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>• Edesur → BONORINO. Edenor: Sanes=CIUDAD; Ivilmar/Marta Chagas=OHIGGINS. Telecentro=CIUDAD.</t>
+          <t>• ABL CIUDAD: partida AGIP 397789 (OHIGGINS = 3016365 → otra carpeta)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>• Ingresos Sol: básico anterior ARS 11.305.702; +12% desde 01/07 → ARS 12.662.387 (cobro 01/08). No suma al total de gastos.</t>
+          <t>• Edesur → BONORINO. Edenor: Sanes=CIUDAD; Ivilmar/Marta Chagas=OHIGGINS. Telecentro=CIUDAD.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
+        <is>
+          <t>• Ingresos Sol: básico anterior ARS 11.305.702; +12% desde 01/07 → ARS 12.662.387 (cobro 01/08). No suma al total de gastos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>• MELI: simulador + detalle real de recibos 2026 (sueldos, bono y SAC). No suma al total de gastos.</t>
         </is>
@@ -6669,32 +6698,12 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="43" t="n">
-        <v>46122</v>
-      </c>
-      <c r="B123" s="14" t="inlineStr">
-        <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="C123" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Libre</t>
-        </is>
-      </c>
-      <c r="D123" s="15" t="n">
-        <v>17041</v>
-      </c>
-      <c r="E123" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="F123" s="14" t="inlineStr">
-        <is>
-          <t>ML · ML · gasto personal Sol (revisar)</t>
-        </is>
-      </c>
+      <c r="A123" s="43" t="n"/>
+      <c r="B123" s="14" t="n"/>
+      <c r="C123" s="14" t="n"/>
+      <c r="D123" s="15" t="n"/>
+      <c r="E123" s="14" t="n"/>
+      <c r="F123" s="14" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="43" t="n">
@@ -6809,60 +6818,20 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="43" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B128" s="14" t="inlineStr">
-        <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="C128" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Libre</t>
-        </is>
-      </c>
-      <c r="D128" s="15" t="n">
-        <v>13989</v>
-      </c>
-      <c r="E128" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="F128" s="14" t="inlineStr">
-        <is>
-          <t>ML · ML · gasto personal Sol (revisar)</t>
-        </is>
-      </c>
+      <c r="A128" s="43" t="n"/>
+      <c r="B128" s="14" t="n"/>
+      <c r="C128" s="14" t="n"/>
+      <c r="D128" s="15" t="n"/>
+      <c r="E128" s="14" t="n"/>
+      <c r="F128" s="14" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="43" t="n">
-        <v>46126</v>
-      </c>
-      <c r="B129" s="14" t="inlineStr">
-        <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="C129" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Libre</t>
-        </is>
-      </c>
-      <c r="D129" s="15" t="n">
-        <v>119000</v>
-      </c>
-      <c r="E129" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="F129" s="14" t="inlineStr">
-        <is>
-          <t>ML · ML · gasto personal Sol (revisar)</t>
-        </is>
-      </c>
+      <c r="A129" s="43" t="n"/>
+      <c r="B129" s="14" t="n"/>
+      <c r="C129" s="14" t="n"/>
+      <c r="D129" s="15" t="n"/>
+      <c r="E129" s="14" t="n"/>
+      <c r="F129" s="14" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="43" t="n">
@@ -18994,7 +18963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20969,6 +20938,105 @@
       <c r="I61" t="inlineStr">
         <is>
           <t>Junio</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="44" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>REPARACIONES Y REPUESTOS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Rollo plástico con burbujas 1 × 25 m</t>
+        </is>
+      </c>
+      <c r="D62" s="26" t="n">
+        <v>17041</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Mercado Libre · CIUDAD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="44" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>REPARACIONES Y REPUESTOS</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Control remoto Samsung con Netflix/Prime Video</t>
+        </is>
+      </c>
+      <c r="D63" s="26" t="n">
+        <v>13989</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Mercado Libre · CIUDAD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="44" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>REPARACIONES Y REPUESTOS</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Control remoto Samsung original AU7000</t>
+        </is>
+      </c>
+      <c r="D64" s="26" t="n">
+        <v>119000</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Mercado Libre · CIUDAD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Abril</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CIUDAD settlement rows and move AGUS to GPS peluquería.
Matrix 2026 now shows Cada uno / Sol / Chris net after Almacén a cuenta; Agustina Vissani is GPS PELUQUERÍA; Almacén monthly totals feed Detalle via SUMIFS.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -686,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1101,18 +1101,10 @@
       </c>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n">
-        <v>75000</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>155000</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>125000</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>135000</v>
-      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
       <c r="L11" s="5" t="n"/>
@@ -1503,168 +1495,351 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>• PedidosYa Plus / suscripciones PedidosYa → CIUDAD SUSCRIPCIONES (no Gasto Personal Sol)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Notas</t>
-        </is>
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>CADA UNO</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>Total ÷ 2 — parte de Sol y de Chris</t>
+        </is>
+      </c>
+      <c r="D22" s="7">
+        <f>D21/2</f>
+        <v/>
+      </c>
+      <c r="E22" s="7">
+        <f>E21/2</f>
+        <v/>
+      </c>
+      <c r="F22" s="7">
+        <f>F21/2</f>
+        <v/>
+      </c>
+      <c r="G22" s="7">
+        <f>G21/2</f>
+        <v/>
+      </c>
+      <c r="H22" s="7">
+        <f>H21/2</f>
+        <v/>
+      </c>
+      <c r="I22" s="7">
+        <f>I21/2</f>
+        <v/>
+      </c>
+      <c r="J22" s="7">
+        <f>J21/2</f>
+        <v/>
+      </c>
+      <c r="K22" s="7">
+        <f>K21/2</f>
+        <v/>
+      </c>
+      <c r="L22" s="7">
+        <f>L21/2</f>
+        <v/>
+      </c>
+      <c r="M22" s="7">
+        <f>M21/2</f>
+        <v/>
+      </c>
+      <c r="N22" s="7">
+        <f>N21/2</f>
+        <v/>
+      </c>
+      <c r="O22" s="7">
+        <f>O21/2</f>
+        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
-        </is>
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="n"/>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>Pendiente Sol = Cada uno − pagado por Sol (todos los servicios + ALMACEN SOL). Positivo: Sol le paga a Chris; negativo: a favor de Sol</t>
+        </is>
+      </c>
+      <c r="D24" s="7">
+        <f>D22-(D21-D14)</f>
+        <v/>
+      </c>
+      <c r="E24" s="7">
+        <f>E22-(E21-E14)</f>
+        <v/>
+      </c>
+      <c r="F24" s="7">
+        <f>F22-(F21-F14)</f>
+        <v/>
+      </c>
+      <c r="G24" s="7">
+        <f>G22-(G21-G14)</f>
+        <v/>
+      </c>
+      <c r="H24" s="7">
+        <f>H22-(H21-H14)</f>
+        <v/>
+      </c>
+      <c r="I24" s="7">
+        <f>I22-(I21-I14)</f>
+        <v/>
+      </c>
+      <c r="J24" s="7">
+        <f>J22-(J21-J14)</f>
+        <v/>
+      </c>
+      <c r="K24" s="7">
+        <f>K22-(K21-K14)</f>
+        <v/>
+      </c>
+      <c r="L24" s="7">
+        <f>L22-(L21-L14)</f>
+        <v/>
+      </c>
+      <c r="M24" s="7">
+        <f>M22-(M21-M14)</f>
+        <v/>
+      </c>
+      <c r="N24" s="7">
+        <f>N22-(N21-N14)</f>
+        <v/>
+      </c>
+      <c r="O24" s="7">
+        <f>O22-(O21-O14)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
-        </is>
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>CHRIS</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="n"/>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>Pendiente Chris = Cada uno − ALMACEN CHRIS (único pagado por Chris). Positivo: Chris le paga a Sol</t>
+        </is>
+      </c>
+      <c r="D25" s="7">
+        <f>D22-D14</f>
+        <v/>
+      </c>
+      <c r="E25" s="7">
+        <f>E22-E14</f>
+        <v/>
+      </c>
+      <c r="F25" s="7">
+        <f>F22-F14</f>
+        <v/>
+      </c>
+      <c r="G25" s="7">
+        <f>G22-G14</f>
+        <v/>
+      </c>
+      <c r="H25" s="7">
+        <f>H22-H14</f>
+        <v/>
+      </c>
+      <c r="I25" s="7">
+        <f>I22-I14</f>
+        <v/>
+      </c>
+      <c r="J25" s="7">
+        <f>J22-J14</f>
+        <v/>
+      </c>
+      <c r="K25" s="7">
+        <f>K22-K14</f>
+        <v/>
+      </c>
+      <c r="L25" s="7">
+        <f>L22-L14</f>
+        <v/>
+      </c>
+      <c r="M25" s="7">
+        <f>M22-M14</f>
+        <v/>
+      </c>
+      <c r="N25" s="7">
+        <f>N22-N14</f>
+        <v/>
+      </c>
+      <c r="O25" s="7">
+        <f>O22-O14</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+          <t>• PedidosYa Plus / suscripciones PedidosYa → CIUDAD SUSCRIPCIONES (no Gasto Personal Sol)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio). Julio período pendiente.</t>
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+          <t>• Catálogo fijo de conceptos CIUDAD 1132</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+          <t>• Telecentro: $50.000 mensuales hasta nuevo aviso</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>• Montos enteros, siempre redondeados hacia arriba</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>• Expensas: abr $235.210 (banco 7-abr → Consorcio De Propiet Patagonia); may/jun desde MP con período Gmail (pago jun=mayo, pago jul=junio). Julio período pendiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>• En Detalle: Forma de pago, N° Cliente y N° Medidor cuando existan</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>• ALMACEN SOL / ALMACEN CHRIS: totales automáticos desde hoja "Almacen Detalle"</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>• TRANSPORTE (Cabify/Uber/Didi/Emova) → solo Gasto Personal Sol; sin fila en matriz 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="30" t="inlineStr">
-        <is>
-          <t>• FARMACIA · Farmacity → Almacen Detalle. Farmacia Maure / Selma → Gasto Personal Sol · FARMACIA SALUD</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>• Personal (Pago directo): va a OHIGGINS → TV CABLE-INTERNET — no CIUDAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>• Inversión: hoja "Inversión" (bonos, plazos fijos y otros; no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
         <is>
-          <t>• Transferencias recibidas: hoja "Transferencias recibidas" (no suma al total de gastos)</t>
+          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="30" t="inlineStr">
         <is>
-          <t>• Expensas consorcios: hoja "Expensas Consorcios" (Consorcio De Propiet = CIUDAD; no ALMACEN SOL)</t>
+          <t>• FARMACIA · Farmacity → Almacen Detalle. Farmacia Maure / Selma → Gasto Personal Sol · FARMACIA SALUD</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="30" t="inlineStr">
         <is>
+          <t>• Personal (Pago directo): va a OHIGGINS → TV CABLE-INTERNET — no CIUDAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>• Inversión: hoja "Inversión" (bonos, plazos fijos y otros; no suma al TOTAL de gastos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>• Transferencias recibidas: hoja "Transferencias recibidas" (no suma al total de gastos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>• Expensas consorcios: hoja "Expensas Consorcios" (Consorcio De Propiet = CIUDAD; no ALMACEN SOL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
           <t>• Gasto personal Sol (Tuenti, Apple, ropa, ML, extras, transferencias a terceros): hoja "Gasto Personal Sol" (no suma al total CIUDAD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>• Pago de tarjetas: hoja "Pago de Tarjetas" (pago de resumen TC; no es gasto nuevo de la matriz)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>• ALMACEN SOL: solo comida/súper/combustible en "Almacen Detalle". Resto personal → "Gasto Personal Sol"</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>• ABL CIUDAD: partida AGIP 397789 (OHIGGINS = 3016365 → otra carpeta)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>• Edesur → BONORINO. Edenor: Sanes=CIUDAD; Ivilmar/Marta Chagas=OHIGGINS. Telecentro=CIUDAD.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>• STREAMING: Spotify (BBVA Visa USD) → ARS con TC MEP del mes (tabla AVA). Fila STREAMING / Streaming música — Spotify</t>
+          <t>• Pago de tarjetas: hoja "Pago de Tarjetas" (pago de resumen TC; no es gasto nuevo de la matriz)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>• GAS CIUDAD (Metrogas 30010996459): mes = fecha de cobro BBVA / pago / vencimiento factura — no período de consumo</t>
+          <t>• ALMACEN SOL: solo comida/súper/combustible en "Almacen Detalle". Resto personal → "Gasto Personal Sol"</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>• FARMACIA · Farmacity y REPUESTOS · Sodastream → hoja "Almacen Detalle" (suman en ALMACEN SOL)</t>
+          <t>• ABL CIUDAD: partida AGIP 397789 (OHIGGINS = 3016365 → otra carpeta)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
+        <is>
+          <t>• Edesur → BONORINO. Edenor: Sanes=CIUDAD; Ivilmar/Marta Chagas=OHIGGINS. Telecentro=CIUDAD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>• STREAMING: Spotify (BBVA Visa USD) → ARS con TC MEP del mes (tabla AVA). Fila STREAMING / Streaming música — Spotify</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>• GAS CIUDAD (Metrogas 30010996459): mes = fecha de cobro BBVA / pago / vencimiento factura — no período de consumo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>• FARMACIA · Farmacity y REPUESTOS · Sodastream → hoja "Almacen Detalle" (suman en ALMACEN SOL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>• TRANSPORTE personal (Cabify/Uber/Didi) → solo hoja "Gasto Personal Sol" (no fila en matriz 2026)</t>
         </is>
@@ -4012,29 +4187,49 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="53" t="n"/>
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="14" t="n"/>
-      <c r="F35" s="14" t="n"/>
+      <c r="A35" s="53" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Agustina Vissani (ex AGUS/PSA · ex CASA matriz 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="53" t="n">
-        <v>46031</v>
+        <v>46129</v>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Enero</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>Servicio - Telefonía</t>
+          <t>PELUQUERÍA</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>14700</v>
+        <v>155000</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
@@ -4043,34 +4238,54 @@
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
-          <t>Tuenti · gasto personal Sol · hoja Gasto Personal Sol</t>
+          <t>PELUQUERÍA · Agustina Vissani (ex AGUS/PSA · ex CASA matriz 2026)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="53" t="n"/>
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="14" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="14" t="n"/>
-      <c r="F37" s="14" t="n"/>
+      <c r="A37" s="53" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>125000</v>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>PELUQUERÍA · Agustina Vissani (ex AGUS/PSA · ex CASA matriz 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="53" t="n">
-        <v>46037</v>
+        <v>46185</v>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Enero</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>TRANSFERENCIAS</t>
+          <t>PELUQUERÍA</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>11000</v>
+        <v>135000</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
@@ -4079,7 +4294,7 @@
       </c>
       <c r="F38" s="14" t="inlineStr">
         <is>
-          <t>transferencia · gasto personal Sol (ex-PENDIENTE) · ex `Marcelo Alejandro Kattan`</t>
+          <t>PELUQUERÍA · Agustina Vissani (ex AGUS/PSA · ex CASA matriz 2026)</t>
         </is>
       </c>
     </row>
@@ -52987,7 +53202,7 @@
       </c>
       <c r="E6" s="28" t="n"/>
       <c r="F6" s="15">
-        <f>IF(OR(D7&lt;&gt;"",E7&lt;&gt;""),IF(D7="",0,D7)+IF(E7="",0,E7),"")</f>
+        <f>IF(OR(D6&lt;&gt;"",E6&lt;&gt;""),IF(D6="",0,D6)+IF(E6="",0,E6),"")</f>
         <v/>
       </c>
       <c r="G6" s="14" t="inlineStr">
@@ -53015,7 +53230,7 @@
       </c>
       <c r="E7" s="28" t="n"/>
       <c r="F7" s="15">
-        <f>IF(OR(D8&lt;&gt;"",E8&lt;&gt;""),IF(D8="",0,D8)+IF(E8="",0,E8),"")</f>
+        <f>IF(OR(D7&lt;&gt;"",E7&lt;&gt;""),IF(D7="",0,D7)+IF(E7="",0,E7),"")</f>
         <v/>
       </c>
       <c r="G7" s="14" t="inlineStr">
@@ -53043,7 +53258,7 @@
       </c>
       <c r="E8" s="28" t="n"/>
       <c r="F8" s="15">
-        <f>IF(OR(D9&lt;&gt;"",E9&lt;&gt;""),IF(D9="",0,D9)+IF(E9="",0,E9),"")</f>
+        <f>IF(OR(D8&lt;&gt;"",E8&lt;&gt;""),IF(D8="",0,D8)+IF(E8="",0,E8),"")</f>
         <v/>
       </c>
       <c r="G8" s="14" t="inlineStr">
@@ -53239,7 +53454,7 @@
       </c>
       <c r="E15" s="28" t="n"/>
       <c r="F15" s="15">
-        <f>IF(OR(D17&lt;&gt;"",E17&lt;&gt;""),IF(D17="",0,D17)+IF(E17="",0,E17),"")</f>
+        <f>IF(OR(D15&lt;&gt;"",E15&lt;&gt;""),IF(D15="",0,D15)+IF(E15="",0,E15),"")</f>
         <v/>
       </c>
       <c r="G15" s="14" t="inlineStr">
@@ -53295,7 +53510,7 @@
       </c>
       <c r="E17" s="28" t="n"/>
       <c r="F17" s="15">
-        <f>IF(OR(D19&lt;&gt;"",E19&lt;&gt;""),IF(D19="",0,D19)+IF(E19="",0,E19),"")</f>
+        <f>IF(OR(D17&lt;&gt;"",E17&lt;&gt;""),IF(D17="",0,D17)+IF(E17="",0,E17),"")</f>
         <v/>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -53323,7 +53538,7 @@
       </c>
       <c r="E18" s="28" t="n"/>
       <c r="F18" s="15">
-        <f>IF(OR(D20&lt;&gt;"",E20&lt;&gt;""),IF(D20="",0,D20)+IF(E20="",0,E20),"")</f>
+        <f>IF(OR(D18&lt;&gt;"",E18&lt;&gt;""),IF(D18="",0,D18)+IF(E18="",0,E18),"")</f>
         <v/>
       </c>
       <c r="G18" s="14" t="inlineStr">
@@ -53351,7 +53566,7 @@
       </c>
       <c r="E19" s="28" t="n"/>
       <c r="F19" s="15">
-        <f>IF(OR(D21&lt;&gt;"",E21&lt;&gt;""),IF(D21="",0,D21)+IF(E21="",0,E21),"")</f>
+        <f>IF(OR(D19&lt;&gt;"",E19&lt;&gt;""),IF(D19="",0,D19)+IF(E19="",0,E19),"")</f>
         <v/>
       </c>
       <c r="G19" s="14" t="inlineStr">
@@ -53379,7 +53594,7 @@
       </c>
       <c r="E20" s="28" t="n"/>
       <c r="F20" s="15">
-        <f>IF(OR(D22&lt;&gt;"",E22&lt;&gt;""),IF(D22="",0,D22)+IF(E22="",0,E22),"")</f>
+        <f>IF(OR(D20&lt;&gt;"",E20&lt;&gt;""),IF(D20="",0,D20)+IF(E20="",0,E20),"")</f>
         <v/>
       </c>
       <c r="G20" s="14" t="inlineStr">
@@ -53463,7 +53678,7 @@
       </c>
       <c r="E23" s="28" t="n"/>
       <c r="F23" s="15">
-        <f>IF(OR(D25&lt;&gt;"",E25&lt;&gt;""),IF(D25="",0,D25)+IF(E25="",0,E25),"")</f>
+        <f>IF(OR(D23&lt;&gt;"",E23&lt;&gt;""),IF(D23="",0,D23)+IF(E23="",0,E23),"")</f>
         <v/>
       </c>
       <c r="G23" s="14" t="inlineStr">
@@ -53491,7 +53706,7 @@
       </c>
       <c r="E24" s="28" t="n"/>
       <c r="F24" s="15">
-        <f>IF(OR(D26&lt;&gt;"",E26&lt;&gt;""),IF(D26="",0,D26)+IF(E26="",0,E26),"")</f>
+        <f>IF(OR(D24&lt;&gt;"",E24&lt;&gt;""),IF(D24="",0,D24)+IF(E24="",0,E24),"")</f>
         <v/>
       </c>
       <c r="G24" s="14" t="inlineStr">
@@ -53519,7 +53734,7 @@
       </c>
       <c r="E25" s="28" t="n"/>
       <c r="F25" s="15">
-        <f>IF(OR(D27&lt;&gt;"",E27&lt;&gt;""),IF(D27="",0,D27)+IF(E27="",0,E27),"")</f>
+        <f>IF(OR(D25&lt;&gt;"",E25&lt;&gt;""),IF(D25="",0,D25)+IF(E25="",0,E25),"")</f>
         <v/>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -53547,7 +53762,7 @@
       </c>
       <c r="E26" s="28" t="n"/>
       <c r="F26" s="15">
-        <f>IF(OR(D28&lt;&gt;"",E28&lt;&gt;""),IF(D28="",0,D28)+IF(E28="",0,E28),"")</f>
+        <f>IF(OR(D26&lt;&gt;"",E26&lt;&gt;""),IF(D26="",0,D26)+IF(E26="",0,E26),"")</f>
         <v/>
       </c>
       <c r="G26" s="14" t="inlineStr">
@@ -53575,7 +53790,7 @@
       </c>
       <c r="E27" s="28" t="n"/>
       <c r="F27" s="15">
-        <f>IF(OR(D29&lt;&gt;"",E29&lt;&gt;""),IF(D29="",0,D29)+IF(E29="",0,E29),"")</f>
+        <f>IF(OR(D27&lt;&gt;"",E27&lt;&gt;""),IF(D27="",0,D27)+IF(E27="",0,E27),"")</f>
         <v/>
       </c>
       <c r="G27" s="14" t="inlineStr">
@@ -53603,7 +53818,7 @@
       </c>
       <c r="E28" s="28" t="n"/>
       <c r="F28" s="15">
-        <f>IF(OR(D30&lt;&gt;"",E30&lt;&gt;""),IF(D30="",0,D30)+IF(E30="",0,E30),"")</f>
+        <f>IF(OR(D28&lt;&gt;"",E28&lt;&gt;""),IF(D28="",0,D28)+IF(E28="",0,E28),"")</f>
         <v/>
       </c>
       <c r="G28" s="14" t="inlineStr">
@@ -53631,7 +53846,7 @@
       </c>
       <c r="E29" s="28" t="n"/>
       <c r="F29" s="15">
-        <f>IF(OR(D31&lt;&gt;"",E31&lt;&gt;""),IF(D31="",0,D31)+IF(E31="",0,E31),"")</f>
+        <f>IF(OR(D29&lt;&gt;"",E29&lt;&gt;""),IF(D29="",0,D29)+IF(E29="",0,E29),"")</f>
         <v/>
       </c>
       <c r="G29" s="14" t="inlineStr">
@@ -53659,7 +53874,7 @@
       </c>
       <c r="E30" s="28" t="n"/>
       <c r="F30" s="15">
-        <f>IF(OR(D32&lt;&gt;"",E32&lt;&gt;""),IF(D32="",0,D32)+IF(E32="",0,E32),"")</f>
+        <f>IF(OR(D30&lt;&gt;"",E30&lt;&gt;""),IF(D30="",0,D30)+IF(E30="",0,E30),"")</f>
         <v/>
       </c>
       <c r="G30" s="14" t="inlineStr">
@@ -53687,7 +53902,7 @@
       </c>
       <c r="E31" s="28" t="n"/>
       <c r="F31" s="15">
-        <f>IF(OR(D33&lt;&gt;"",E33&lt;&gt;""),IF(D33="",0,D33)+IF(E33="",0,E33),"")</f>
+        <f>IF(OR(D31&lt;&gt;"",E31&lt;&gt;""),IF(D31="",0,D31)+IF(E31="",0,E31),"")</f>
         <v/>
       </c>
       <c r="G31" s="14" t="inlineStr">
@@ -53743,7 +53958,7 @@
       </c>
       <c r="E33" s="28" t="n"/>
       <c r="F33" s="15">
-        <f>IF(OR(D35&lt;&gt;"",E35&lt;&gt;""),IF(D35="",0,D35)+IF(E35="",0,E35),"")</f>
+        <f>IF(OR(D33&lt;&gt;"",E33&lt;&gt;""),IF(D33="",0,D33)+IF(E33="",0,E33),"")</f>
         <v/>
       </c>
       <c r="G33" s="14" t="inlineStr">
@@ -53771,7 +53986,7 @@
       </c>
       <c r="E34" s="28" t="n"/>
       <c r="F34" s="15">
-        <f>IF(OR(D36&lt;&gt;"",E36&lt;&gt;""),IF(D36="",0,D36)+IF(E36="",0,E36),"")</f>
+        <f>IF(OR(D34&lt;&gt;"",E34&lt;&gt;""),IF(D34="",0,D34)+IF(E34="",0,E34),"")</f>
         <v/>
       </c>
       <c r="G34" s="14" t="inlineStr">
@@ -53799,7 +54014,7 @@
       </c>
       <c r="E35" s="28" t="n"/>
       <c r="F35" s="15">
-        <f>IF(OR(D37&lt;&gt;"",E37&lt;&gt;""),IF(D37="",0,D37)+IF(E37="",0,E37),"")</f>
+        <f>IF(OR(D35&lt;&gt;"",E35&lt;&gt;""),IF(D35="",0,D35)+IF(E35="",0,E35),"")</f>
         <v/>
       </c>
       <c r="G35" s="14" t="inlineStr">
@@ -53827,7 +54042,7 @@
       </c>
       <c r="E36" s="28" t="n"/>
       <c r="F36" s="15">
-        <f>IF(OR(D38&lt;&gt;"",E38&lt;&gt;""),IF(D38="",0,D38)+IF(E38="",0,E38),"")</f>
+        <f>IF(OR(D36&lt;&gt;"",E36&lt;&gt;""),IF(D36="",0,D36)+IF(E36="",0,E36),"")</f>
         <v/>
       </c>
       <c r="G36" s="14" t="inlineStr">
@@ -53855,7 +54070,7 @@
       </c>
       <c r="E37" s="28" t="n"/>
       <c r="F37" s="15">
-        <f>IF(OR(D39&lt;&gt;"",E39&lt;&gt;""),IF(D39="",0,D39)+IF(E39="",0,E39),"")</f>
+        <f>IF(OR(D37&lt;&gt;"",E37&lt;&gt;""),IF(D37="",0,D37)+IF(E37="",0,E37),"")</f>
         <v/>
       </c>
       <c r="G37" s="14" t="inlineStr">
@@ -53883,7 +54098,7 @@
       </c>
       <c r="E38" s="28" t="n"/>
       <c r="F38" s="15">
-        <f>IF(OR(D40&lt;&gt;"",E40&lt;&gt;""),IF(D40="",0,D40)+IF(E40="",0,E40),"")</f>
+        <f>IF(OR(D38&lt;&gt;"",E38&lt;&gt;""),IF(D38="",0,D38)+IF(E38="",0,E38),"")</f>
         <v/>
       </c>
       <c r="G38" s="14" t="inlineStr">
@@ -53911,7 +54126,7 @@
       </c>
       <c r="E39" s="28" t="n"/>
       <c r="F39" s="15">
-        <f>IF(OR(D41&lt;&gt;"",E41&lt;&gt;""),IF(D41="",0,D41)+IF(E41="",0,E41),"")</f>
+        <f>IF(OR(D39&lt;&gt;"",E39&lt;&gt;""),IF(D39="",0,D39)+IF(E39="",0,E39),"")</f>
         <v/>
       </c>
       <c r="G39" s="14" t="inlineStr">
@@ -53939,7 +54154,7 @@
       </c>
       <c r="E40" s="28" t="n"/>
       <c r="F40" s="15">
-        <f>IF(OR(D42&lt;&gt;"",E42&lt;&gt;""),IF(D42="",0,D42)+IF(E42="",0,E42),"")</f>
+        <f>IF(OR(D40&lt;&gt;"",E40&lt;&gt;""),IF(D40="",0,D40)+IF(E40="",0,E40),"")</f>
         <v/>
       </c>
       <c r="G40" s="14" t="inlineStr">
@@ -53967,7 +54182,7 @@
       </c>
       <c r="E41" s="28" t="n"/>
       <c r="F41" s="15">
-        <f>IF(OR(D43&lt;&gt;"",E43&lt;&gt;""),IF(D43="",0,D43)+IF(E43="",0,E43),"")</f>
+        <f>IF(OR(D41&lt;&gt;"",E41&lt;&gt;""),IF(D41="",0,D41)+IF(E41="",0,E41),"")</f>
         <v/>
       </c>
       <c r="G41" s="14" t="inlineStr">
@@ -53994,7 +54209,10 @@
         <v>24834</v>
       </c>
       <c r="E42" s="28" t="n"/>
-      <c r="F42" s="15" t="n"/>
+      <c r="F42" s="15">
+        <f>IF(OR(D42&lt;&gt;"",E42&lt;&gt;""),IF(D42="",0,D42)+IF(E42="",0,E42),"")</f>
+        <v/>
+      </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
           <t>SUPERMERCADO · Día · SUPERDIA · BBVA MASTERCARD · ALMACEN SOL</t>
@@ -54019,7 +54237,10 @@
         <v>137929</v>
       </c>
       <c r="E43" s="28" t="n"/>
-      <c r="F43" s="15" t="n"/>
+      <c r="F43" s="15">
+        <f>IF(OR(D43&lt;&gt;"",E43&lt;&gt;""),IF(D43="",0,D43)+IF(E43="",0,E43),"")</f>
+        <v/>
+      </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
           <t>SUPERMERCADO · Día · SUPERDIA · BBVA MASTERCARD · ALMACEN SOL</t>
@@ -54044,7 +54265,10 @@
         <v>44100</v>
       </c>
       <c r="E44" s="28" t="n"/>
-      <c r="F44" s="15" t="n"/>
+      <c r="F44" s="15">
+        <f>IF(OR(D44&lt;&gt;"",E44&lt;&gt;""),IF(D44="",0,D44)+IF(E44="",0,E44),"")</f>
+        <v/>
+      </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -54069,7 +54293,10 @@
         <v>16200</v>
       </c>
       <c r="E45" s="28" t="n"/>
-      <c r="F45" s="15" t="n"/>
+      <c r="F45" s="15">
+        <f>IF(OR(D45&lt;&gt;"",E45&lt;&gt;""),IF(D45="",0,D45)+IF(E45="",0,E45),"")</f>
+        <v/>
+      </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -54094,7 +54321,10 @@
         <v>145400</v>
       </c>
       <c r="E46" s="28" t="n"/>
-      <c r="F46" s="15" t="n"/>
+      <c r="F46" s="15">
+        <f>IF(OR(D46&lt;&gt;"",E46&lt;&gt;""),IF(D46="",0,D46)+IF(E46="",0,E46),"")</f>
+        <v/>
+      </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -54114,11 +54344,11 @@
         </is>
       </c>
       <c r="D47" s="7">
-        <f>SUM(D4:D46)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Enero")</f>
         <v/>
       </c>
       <c r="E47" s="7">
-        <f>SUM(E4:E46)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Enero")</f>
         <v/>
       </c>
       <c r="F47" s="7">
@@ -54173,7 +54403,7 @@
       </c>
       <c r="E49" s="28" t="n"/>
       <c r="F49" s="15">
-        <f>IF(OR(D46&lt;&gt;"",E46&lt;&gt;""),IF(D46="",0,D46)+IF(E46="",0,E46),"")</f>
+        <f>IF(OR(D49&lt;&gt;"",E49&lt;&gt;""),IF(D49="",0,D49)+IF(E49="",0,E49),"")</f>
         <v/>
       </c>
       <c r="G49" s="14" t="inlineStr">
@@ -54201,7 +54431,7 @@
       </c>
       <c r="E50" s="28" t="n"/>
       <c r="F50" s="15">
-        <f>IF(OR(D47&lt;&gt;"",E47&lt;&gt;""),IF(D47="",0,D47)+IF(E47="",0,E47),"")</f>
+        <f>IF(OR(D50&lt;&gt;"",E50&lt;&gt;""),IF(D50="",0,D50)+IF(E50="",0,E50),"")</f>
         <v/>
       </c>
       <c r="G50" s="14" t="inlineStr">
@@ -54229,7 +54459,7 @@
       </c>
       <c r="E51" s="28" t="n"/>
       <c r="F51" s="15">
-        <f>IF(OR(D48&lt;&gt;"",E48&lt;&gt;""),IF(D48="",0,D48)+IF(E48="",0,E48),"")</f>
+        <f>IF(OR(D51&lt;&gt;"",E51&lt;&gt;""),IF(D51="",0,D51)+IF(E51="",0,E51),"")</f>
         <v/>
       </c>
       <c r="G51" s="14" t="inlineStr">
@@ -54257,7 +54487,7 @@
       </c>
       <c r="E52" s="28" t="n"/>
       <c r="F52" s="15">
-        <f>IF(OR(D49&lt;&gt;"",E49&lt;&gt;""),IF(D49="",0,D49)+IF(E49="",0,E49),"")</f>
+        <f>IF(OR(D52&lt;&gt;"",E52&lt;&gt;""),IF(D52="",0,D52)+IF(E52="",0,E52),"")</f>
         <v/>
       </c>
       <c r="G52" s="14" t="inlineStr">
@@ -54285,7 +54515,7 @@
       </c>
       <c r="E53" s="28" t="n"/>
       <c r="F53" s="15">
-        <f>IF(OR(D51&lt;&gt;"",E51&lt;&gt;""),IF(D51="",0,D51)+IF(E51="",0,E51),"")</f>
+        <f>IF(OR(D53&lt;&gt;"",E53&lt;&gt;""),IF(D53="",0,D53)+IF(E53="",0,E53),"")</f>
         <v/>
       </c>
       <c r="G53" s="14" t="inlineStr">
@@ -54313,7 +54543,7 @@
       </c>
       <c r="E54" s="28" t="n"/>
       <c r="F54" s="15">
-        <f>IF(OR(D52&lt;&gt;"",E52&lt;&gt;""),IF(D52="",0,D52)+IF(E52="",0,E52),"")</f>
+        <f>IF(OR(D54&lt;&gt;"",E54&lt;&gt;""),IF(D54="",0,D54)+IF(E54="",0,E54),"")</f>
         <v/>
       </c>
       <c r="G54" s="14" t="inlineStr">
@@ -54341,7 +54571,7 @@
       </c>
       <c r="E55" s="28" t="n"/>
       <c r="F55" s="15">
-        <f>IF(OR(D53&lt;&gt;"",E53&lt;&gt;""),IF(D53="",0,D53)+IF(E53="",0,E53),"")</f>
+        <f>IF(OR(D55&lt;&gt;"",E55&lt;&gt;""),IF(D55="",0,D55)+IF(E55="",0,E55),"")</f>
         <v/>
       </c>
       <c r="G55" s="14" t="inlineStr">
@@ -54369,7 +54599,7 @@
       </c>
       <c r="E56" s="28" t="n"/>
       <c r="F56" s="15">
-        <f>IF(OR(D55&lt;&gt;"",E55&lt;&gt;""),IF(D55="",0,D55)+IF(E55="",0,E55),"")</f>
+        <f>IF(OR(D56&lt;&gt;"",E56&lt;&gt;""),IF(D56="",0,D56)+IF(E56="",0,E56),"")</f>
         <v/>
       </c>
       <c r="G56" s="14" t="inlineStr">
@@ -54593,7 +54823,7 @@
       </c>
       <c r="E64" s="28" t="n"/>
       <c r="F64" s="15">
-        <f>IF(OR(D66&lt;&gt;"",E66&lt;&gt;""),IF(D66="",0,D66)+IF(E66="",0,E66),"")</f>
+        <f>IF(OR(D64&lt;&gt;"",E64&lt;&gt;""),IF(D64="",0,D64)+IF(E64="",0,E64),"")</f>
         <v/>
       </c>
       <c r="G64" s="14" t="inlineStr">
@@ -54621,7 +54851,7 @@
       </c>
       <c r="E65" s="28" t="n"/>
       <c r="F65" s="15">
-        <f>IF(OR(D67&lt;&gt;"",E67&lt;&gt;""),IF(D67="",0,D67)+IF(E67="",0,E67),"")</f>
+        <f>IF(OR(D65&lt;&gt;"",E65&lt;&gt;""),IF(D65="",0,D65)+IF(E65="",0,E65),"")</f>
         <v/>
       </c>
       <c r="G65" s="14" t="inlineStr">
@@ -54649,7 +54879,7 @@
       </c>
       <c r="E66" s="28" t="n"/>
       <c r="F66" s="15">
-        <f>IF(OR(D68&lt;&gt;"",E68&lt;&gt;""),IF(D68="",0,D68)+IF(E68="",0,E68),"")</f>
+        <f>IF(OR(D66&lt;&gt;"",E66&lt;&gt;""),IF(D66="",0,D66)+IF(E66="",0,E66),"")</f>
         <v/>
       </c>
       <c r="G66" s="14" t="inlineStr">
@@ -54677,7 +54907,7 @@
       </c>
       <c r="E67" s="28" t="n"/>
       <c r="F67" s="15">
-        <f>IF(OR(D69&lt;&gt;"",E69&lt;&gt;""),IF(D69="",0,D69)+IF(E69="",0,E69),"")</f>
+        <f>IF(OR(D67&lt;&gt;"",E67&lt;&gt;""),IF(D67="",0,D67)+IF(E67="",0,E67),"")</f>
         <v/>
       </c>
       <c r="G67" s="14" t="inlineStr">
@@ -54705,7 +54935,7 @@
       </c>
       <c r="E68" s="28" t="n"/>
       <c r="F68" s="15">
-        <f>IF(OR(D70&lt;&gt;"",E70&lt;&gt;""),IF(D70="",0,D70)+IF(E70="",0,E70),"")</f>
+        <f>IF(OR(D68&lt;&gt;"",E68&lt;&gt;""),IF(D68="",0,D68)+IF(E68="",0,E68),"")</f>
         <v/>
       </c>
       <c r="G68" s="14" t="inlineStr">
@@ -54733,7 +54963,7 @@
       </c>
       <c r="E69" s="28" t="n"/>
       <c r="F69" s="15">
-        <f>IF(OR(D71&lt;&gt;"",E71&lt;&gt;""),IF(D71="",0,D71)+IF(E71="",0,E71),"")</f>
+        <f>IF(OR(D69&lt;&gt;"",E69&lt;&gt;""),IF(D69="",0,D69)+IF(E69="",0,E69),"")</f>
         <v/>
       </c>
       <c r="G69" s="14" t="inlineStr">
@@ -54761,7 +54991,7 @@
       </c>
       <c r="E70" s="28" t="n"/>
       <c r="F70" s="15">
-        <f>IF(OR(D72&lt;&gt;"",E72&lt;&gt;""),IF(D72="",0,D72)+IF(E72="",0,E72),"")</f>
+        <f>IF(OR(D70&lt;&gt;"",E70&lt;&gt;""),IF(D70="",0,D70)+IF(E70="",0,E70),"")</f>
         <v/>
       </c>
       <c r="G70" s="14" t="inlineStr">
@@ -54789,7 +55019,7 @@
       </c>
       <c r="E71" s="28" t="n"/>
       <c r="F71" s="15">
-        <f>IF(OR(D73&lt;&gt;"",E73&lt;&gt;""),IF(D73="",0,D73)+IF(E73="",0,E73),"")</f>
+        <f>IF(OR(D71&lt;&gt;"",E71&lt;&gt;""),IF(D71="",0,D71)+IF(E71="",0,E71),"")</f>
         <v/>
       </c>
       <c r="G71" s="14" t="inlineStr">
@@ -54817,7 +55047,7 @@
       </c>
       <c r="E72" s="28" t="n"/>
       <c r="F72" s="15">
-        <f>IF(OR(D74&lt;&gt;"",E74&lt;&gt;""),IF(D74="",0,D74)+IF(E74="",0,E74),"")</f>
+        <f>IF(OR(D72&lt;&gt;"",E72&lt;&gt;""),IF(D72="",0,D72)+IF(E72="",0,E72),"")</f>
         <v/>
       </c>
       <c r="G72" s="14" t="inlineStr">
@@ -54845,7 +55075,7 @@
       </c>
       <c r="E73" s="28" t="n"/>
       <c r="F73" s="15">
-        <f>IF(OR(D75&lt;&gt;"",E75&lt;&gt;""),IF(D75="",0,D75)+IF(E75="",0,E75),"")</f>
+        <f>IF(OR(D73&lt;&gt;"",E73&lt;&gt;""),IF(D73="",0,D73)+IF(E73="",0,E73),"")</f>
         <v/>
       </c>
       <c r="G73" s="14" t="inlineStr">
@@ -54873,7 +55103,7 @@
       </c>
       <c r="E74" s="28" t="n"/>
       <c r="F74" s="15">
-        <f>IF(OR(D76&lt;&gt;"",E76&lt;&gt;""),IF(D76="",0,D76)+IF(E76="",0,E76),"")</f>
+        <f>IF(OR(D74&lt;&gt;"",E74&lt;&gt;""),IF(D74="",0,D74)+IF(E74="",0,E74),"")</f>
         <v/>
       </c>
       <c r="G74" s="14" t="inlineStr">
@@ -54901,7 +55131,7 @@
       </c>
       <c r="E75" s="28" t="n"/>
       <c r="F75" s="15">
-        <f>IF(OR(D77&lt;&gt;"",E77&lt;&gt;""),IF(D77="",0,D77)+IF(E77="",0,E77),"")</f>
+        <f>IF(OR(D75&lt;&gt;"",E75&lt;&gt;""),IF(D75="",0,D75)+IF(E75="",0,E75),"")</f>
         <v/>
       </c>
       <c r="G75" s="14" t="inlineStr">
@@ -54929,7 +55159,7 @@
       </c>
       <c r="E76" s="28" t="n"/>
       <c r="F76" s="15">
-        <f>IF(OR(D78&lt;&gt;"",E78&lt;&gt;""),IF(D78="",0,D78)+IF(E78="",0,E78),"")</f>
+        <f>IF(OR(D76&lt;&gt;"",E76&lt;&gt;""),IF(D76="",0,D76)+IF(E76="",0,E76),"")</f>
         <v/>
       </c>
       <c r="G76" s="14" t="inlineStr">
@@ -54957,7 +55187,7 @@
       </c>
       <c r="E77" s="28" t="n"/>
       <c r="F77" s="15">
-        <f>IF(OR(D79&lt;&gt;"",E79&lt;&gt;""),IF(D79="",0,D79)+IF(E79="",0,E79),"")</f>
+        <f>IF(OR(D77&lt;&gt;"",E77&lt;&gt;""),IF(D77="",0,D77)+IF(E77="",0,E77),"")</f>
         <v/>
       </c>
       <c r="G77" s="14" t="inlineStr">
@@ -54985,7 +55215,7 @@
       </c>
       <c r="E78" s="28" t="n"/>
       <c r="F78" s="15">
-        <f>IF(OR(D80&lt;&gt;"",E80&lt;&gt;""),IF(D80="",0,D80)+IF(E80="",0,E80),"")</f>
+        <f>IF(OR(D78&lt;&gt;"",E78&lt;&gt;""),IF(D78="",0,D78)+IF(E78="",0,E78),"")</f>
         <v/>
       </c>
       <c r="G78" s="14" t="inlineStr">
@@ -55013,7 +55243,7 @@
       </c>
       <c r="E79" s="28" t="n"/>
       <c r="F79" s="15">
-        <f>IF(OR(D81&lt;&gt;"",E81&lt;&gt;""),IF(D81="",0,D81)+IF(E81="",0,E81),"")</f>
+        <f>IF(OR(D79&lt;&gt;"",E79&lt;&gt;""),IF(D79="",0,D79)+IF(E79="",0,E79),"")</f>
         <v/>
       </c>
       <c r="G79" s="14" t="inlineStr">
@@ -55041,7 +55271,7 @@
       </c>
       <c r="E80" s="28" t="n"/>
       <c r="F80" s="15">
-        <f>IF(OR(D82&lt;&gt;"",E82&lt;&gt;""),IF(D82="",0,D82)+IF(E82="",0,E82),"")</f>
+        <f>IF(OR(D80&lt;&gt;"",E80&lt;&gt;""),IF(D80="",0,D80)+IF(E80="",0,E80),"")</f>
         <v/>
       </c>
       <c r="G80" s="14" t="inlineStr">
@@ -55069,7 +55299,7 @@
       </c>
       <c r="E81" s="28" t="n"/>
       <c r="F81" s="15">
-        <f>IF(OR(D83&lt;&gt;"",E83&lt;&gt;""),IF(D83="",0,D83)+IF(E83="",0,E83),"")</f>
+        <f>IF(OR(D81&lt;&gt;"",E81&lt;&gt;""),IF(D81="",0,D81)+IF(E81="",0,E81),"")</f>
         <v/>
       </c>
       <c r="G81" s="14" t="inlineStr">
@@ -55097,7 +55327,7 @@
       </c>
       <c r="E82" s="28" t="n"/>
       <c r="F82" s="15">
-        <f>IF(OR(D84&lt;&gt;"",E84&lt;&gt;""),IF(D84="",0,D84)+IF(E84="",0,E84),"")</f>
+        <f>IF(OR(D82&lt;&gt;"",E82&lt;&gt;""),IF(D82="",0,D82)+IF(E82="",0,E82),"")</f>
         <v/>
       </c>
       <c r="G82" s="14" t="inlineStr">
@@ -55140,7 +55370,10 @@
         <v>33100</v>
       </c>
       <c r="E84" s="28" t="n"/>
-      <c r="F84" s="15" t="n"/>
+      <c r="F84" s="15">
+        <f>IF(OR(D84&lt;&gt;"",E84&lt;&gt;""),IF(D84="",0,D84)+IF(E84="",0,E84),"")</f>
+        <v/>
+      </c>
       <c r="G84" s="14" t="inlineStr">
         <is>
           <t>COMIDA · RESTAURANTSORAYASA · MP cuenta</t>
@@ -55165,7 +55398,10 @@
         <v>72000</v>
       </c>
       <c r="E85" s="28" t="n"/>
-      <c r="F85" s="15" t="n"/>
+      <c r="F85" s="15">
+        <f>IF(OR(D85&lt;&gt;"",E85&lt;&gt;""),IF(D85="",0,D85)+IF(E85="",0,E85),"")</f>
+        <v/>
+      </c>
       <c r="G85" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -55190,7 +55426,10 @@
         <v>27200</v>
       </c>
       <c r="E86" s="28" t="n"/>
-      <c r="F86" s="15" t="n"/>
+      <c r="F86" s="15">
+        <f>IF(OR(D86&lt;&gt;"",E86&lt;&gt;""),IF(D86="",0,D86)+IF(E86="",0,E86),"")</f>
+        <v/>
+      </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
           <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
@@ -55210,11 +55449,11 @@
         </is>
       </c>
       <c r="D87" s="7">
-        <f>SUM(D49:D86)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Febrero")</f>
         <v/>
       </c>
       <c r="E87" s="7">
-        <f>SUM(E49:E86)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Febrero")</f>
         <v/>
       </c>
       <c r="F87" s="7">
@@ -55269,7 +55508,7 @@
       </c>
       <c r="E89" s="28" t="n"/>
       <c r="F89" s="15">
-        <f>IF(OR(D88&lt;&gt;"",E88&lt;&gt;""),IF(D88="",0,D88)+IF(E88="",0,E88),"")</f>
+        <f>IF(OR(D89&lt;&gt;"",E89&lt;&gt;""),IF(D89="",0,D89)+IF(E89="",0,E89),"")</f>
         <v/>
       </c>
       <c r="G89" s="14" t="inlineStr">
@@ -55297,7 +55536,7 @@
       </c>
       <c r="E90" s="28" t="n"/>
       <c r="F90" s="15">
-        <f>IF(OR(D89&lt;&gt;"",E89&lt;&gt;""),IF(D89="",0,D89)+IF(E89="",0,E89),"")</f>
+        <f>IF(OR(D90&lt;&gt;"",E90&lt;&gt;""),IF(D90="",0,D90)+IF(E90="",0,E90),"")</f>
         <v/>
       </c>
       <c r="G90" s="14" t="inlineStr">
@@ -55325,7 +55564,7 @@
       </c>
       <c r="E91" s="28" t="n"/>
       <c r="F91" s="15">
-        <f>IF(OR(D90&lt;&gt;"",E90&lt;&gt;""),IF(D90="",0,D90)+IF(E90="",0,E90),"")</f>
+        <f>IF(OR(D91&lt;&gt;"",E91&lt;&gt;""),IF(D91="",0,D91)+IF(E91="",0,E91),"")</f>
         <v/>
       </c>
       <c r="G91" s="14" t="inlineStr">
@@ -55381,7 +55620,7 @@
       </c>
       <c r="E93" s="28" t="n"/>
       <c r="F93" s="15">
-        <f>IF(OR(D92&lt;&gt;"",E92&lt;&gt;""),IF(D92="",0,D92)+IF(E92="",0,E92),"")</f>
+        <f>IF(OR(D93&lt;&gt;"",E93&lt;&gt;""),IF(D93="",0,D93)+IF(E93="",0,E93),"")</f>
         <v/>
       </c>
       <c r="G93" s="14" t="inlineStr">
@@ -55409,7 +55648,7 @@
       </c>
       <c r="E94" s="28" t="n"/>
       <c r="F94" s="15">
-        <f>IF(OR(D93&lt;&gt;"",E93&lt;&gt;""),IF(D93="",0,D93)+IF(E93="",0,E93),"")</f>
+        <f>IF(OR(D94&lt;&gt;"",E94&lt;&gt;""),IF(D94="",0,D94)+IF(E94="",0,E94),"")</f>
         <v/>
       </c>
       <c r="G94" s="14" t="inlineStr">
@@ -55437,7 +55676,7 @@
       </c>
       <c r="E95" s="28" t="n"/>
       <c r="F95" s="15">
-        <f>IF(OR(D94&lt;&gt;"",E94&lt;&gt;""),IF(D94="",0,D94)+IF(E94="",0,E94),"")</f>
+        <f>IF(OR(D95&lt;&gt;"",E95&lt;&gt;""),IF(D95="",0,D95)+IF(E95="",0,E95),"")</f>
         <v/>
       </c>
       <c r="G95" s="14" t="inlineStr">
@@ -55465,7 +55704,7 @@
       </c>
       <c r="E96" s="28" t="n"/>
       <c r="F96" s="15">
-        <f>IF(OR(D95&lt;&gt;"",E95&lt;&gt;""),IF(D95="",0,D95)+IF(E95="",0,E95),"")</f>
+        <f>IF(OR(D96&lt;&gt;"",E96&lt;&gt;""),IF(D96="",0,D96)+IF(E96="",0,E96),"")</f>
         <v/>
       </c>
       <c r="G96" s="14" t="inlineStr">
@@ -55493,7 +55732,7 @@
       </c>
       <c r="E97" s="28" t="n"/>
       <c r="F97" s="15">
-        <f>IF(OR(D96&lt;&gt;"",E96&lt;&gt;""),IF(D96="",0,D96)+IF(E96="",0,E96),"")</f>
+        <f>IF(OR(D97&lt;&gt;"",E97&lt;&gt;""),IF(D97="",0,D97)+IF(E97="",0,E97),"")</f>
         <v/>
       </c>
       <c r="G97" s="14" t="inlineStr">
@@ -56216,7 +56455,10 @@
         <v>4789</v>
       </c>
       <c r="E128" s="28" t="n"/>
-      <c r="F128" s="15" t="n"/>
+      <c r="F128" s="15">
+        <f>IF(OR(D128&lt;&gt;"",E128&lt;&gt;""),IF(D128="",0,D128)+IF(E128="",0,E128),"")</f>
+        <v/>
+      </c>
       <c r="G128" s="14" t="inlineStr">
         <is>
           <t>Combustible — Shell · MP cuenta</t>
@@ -56241,7 +56483,10 @@
         <v>9000</v>
       </c>
       <c r="E129" s="28" t="n"/>
-      <c r="F129" s="15" t="n"/>
+      <c r="F129" s="15">
+        <f>IF(OR(D129&lt;&gt;"",E129&lt;&gt;""),IF(D129="",0,D129)+IF(E129="",0,E129),"")</f>
+        <v/>
+      </c>
       <c r="G129" s="14" t="inlineStr">
         <is>
           <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
@@ -56266,7 +56511,10 @@
         <v>35700</v>
       </c>
       <c r="E130" s="28" t="n"/>
-      <c r="F130" s="15" t="n"/>
+      <c r="F130" s="15">
+        <f>IF(OR(D130&lt;&gt;"",E130&lt;&gt;""),IF(D130="",0,D130)+IF(E130="",0,E130),"")</f>
+        <v/>
+      </c>
       <c r="G130" s="14" t="inlineStr">
         <is>
           <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
@@ -56286,11 +56534,11 @@
         </is>
       </c>
       <c r="D131" s="7">
-        <f>SUM(D89:D130)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Marzo")</f>
         <v/>
       </c>
       <c r="E131" s="7">
-        <f>SUM(E89:E130)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Marzo")</f>
         <v/>
       </c>
       <c r="F131" s="7">
@@ -56345,7 +56593,7 @@
       </c>
       <c r="E133" s="28" t="n"/>
       <c r="F133" s="15">
-        <f>IF(OR(D130&lt;&gt;"",E130&lt;&gt;""),IF(D130="",0,D130)+IF(E130="",0,E130),"")</f>
+        <f>IF(OR(D133&lt;&gt;"",E133&lt;&gt;""),IF(D133="",0,D133)+IF(E133="",0,E133),"")</f>
         <v/>
       </c>
       <c r="G133" s="14" t="inlineStr">
@@ -56373,7 +56621,7 @@
       </c>
       <c r="E134" s="28" t="n"/>
       <c r="F134" s="15">
-        <f>IF(OR(D131&lt;&gt;"",E131&lt;&gt;""),IF(D131="",0,D131)+IF(E131="",0,E131),"")</f>
+        <f>IF(OR(D134&lt;&gt;"",E134&lt;&gt;""),IF(D134="",0,D134)+IF(E134="",0,E134),"")</f>
         <v/>
       </c>
       <c r="G134" s="14" t="inlineStr">
@@ -56401,7 +56649,7 @@
       </c>
       <c r="E135" s="28" t="n"/>
       <c r="F135" s="15">
-        <f>IF(OR(D132&lt;&gt;"",E132&lt;&gt;""),IF(D132="",0,D132)+IF(E132="",0,E132),"")</f>
+        <f>IF(OR(D135&lt;&gt;"",E135&lt;&gt;""),IF(D135="",0,D135)+IF(E135="",0,E135),"")</f>
         <v/>
       </c>
       <c r="G135" s="14" t="inlineStr">
@@ -56429,7 +56677,7 @@
       </c>
       <c r="E136" s="28" t="n"/>
       <c r="F136" s="15">
-        <f>IF(OR(D133&lt;&gt;"",E133&lt;&gt;""),IF(D133="",0,D133)+IF(E133="",0,E133),"")</f>
+        <f>IF(OR(D136&lt;&gt;"",E136&lt;&gt;""),IF(D136="",0,D136)+IF(E136="",0,E136),"")</f>
         <v/>
       </c>
       <c r="G136" s="14" t="inlineStr">
@@ -56457,7 +56705,7 @@
       </c>
       <c r="E137" s="28" t="n"/>
       <c r="F137" s="15">
-        <f>IF(OR(D134&lt;&gt;"",E134&lt;&gt;""),IF(D134="",0,D134)+IF(E134="",0,E134),"")</f>
+        <f>IF(OR(D137&lt;&gt;"",E137&lt;&gt;""),IF(D137="",0,D137)+IF(E137="",0,E137),"")</f>
         <v/>
       </c>
       <c r="G137" s="14" t="inlineStr">
@@ -56485,7 +56733,7 @@
       </c>
       <c r="E138" s="28" t="n"/>
       <c r="F138" s="15">
-        <f>IF(OR(D136&lt;&gt;"",E136&lt;&gt;""),IF(D136="",0,D136)+IF(E136="",0,E136),"")</f>
+        <f>IF(OR(D138&lt;&gt;"",E138&lt;&gt;""),IF(D138="",0,D138)+IF(E138="",0,E138),"")</f>
         <v/>
       </c>
       <c r="G138" s="14" t="inlineStr">
@@ -56513,7 +56761,7 @@
       </c>
       <c r="E139" s="28" t="n"/>
       <c r="F139" s="15">
-        <f>IF(OR(D137&lt;&gt;"",E137&lt;&gt;""),IF(D137="",0,D137)+IF(E137="",0,E137),"")</f>
+        <f>IF(OR(D139&lt;&gt;"",E139&lt;&gt;""),IF(D139="",0,D139)+IF(E139="",0,E139),"")</f>
         <v/>
       </c>
       <c r="G139" s="14" t="inlineStr">
@@ -56541,7 +56789,7 @@
       </c>
       <c r="E140" s="28" t="n"/>
       <c r="F140" s="15">
-        <f>IF(OR(D138&lt;&gt;"",E138&lt;&gt;""),IF(D138="",0,D138)+IF(E138="",0,E138),"")</f>
+        <f>IF(OR(D140&lt;&gt;"",E140&lt;&gt;""),IF(D140="",0,D140)+IF(E140="",0,E140),"")</f>
         <v/>
       </c>
       <c r="G140" s="14" t="inlineStr">
@@ -56569,7 +56817,7 @@
       </c>
       <c r="E141" s="28" t="n"/>
       <c r="F141" s="15">
-        <f>IF(OR(D139&lt;&gt;"",E139&lt;&gt;""),IF(D139="",0,D139)+IF(E139="",0,E139),"")</f>
+        <f>IF(OR(D141&lt;&gt;"",E141&lt;&gt;""),IF(D141="",0,D141)+IF(E141="",0,E141),"")</f>
         <v/>
       </c>
       <c r="G141" s="14" t="inlineStr">
@@ -56597,7 +56845,7 @@
       </c>
       <c r="E142" s="28" t="n"/>
       <c r="F142" s="15">
-        <f>IF(OR(D140&lt;&gt;"",E140&lt;&gt;""),IF(D140="",0,D140)+IF(E140="",0,E140),"")</f>
+        <f>IF(OR(D142&lt;&gt;"",E142&lt;&gt;""),IF(D142="",0,D142)+IF(E142="",0,E142),"")</f>
         <v/>
       </c>
       <c r="G142" s="14" t="inlineStr">
@@ -56625,7 +56873,7 @@
       </c>
       <c r="E143" s="28" t="n"/>
       <c r="F143" s="15">
-        <f>IF(OR(D142&lt;&gt;"",E142&lt;&gt;""),IF(D142="",0,D142)+IF(E142="",0,E142),"")</f>
+        <f>IF(OR(D143&lt;&gt;"",E143&lt;&gt;""),IF(D143="",0,D143)+IF(E143="",0,E143),"")</f>
         <v/>
       </c>
       <c r="G143" s="14" t="inlineStr">
@@ -56653,7 +56901,7 @@
       </c>
       <c r="E144" s="28" t="n"/>
       <c r="F144" s="15">
-        <f>IF(OR(D143&lt;&gt;"",E143&lt;&gt;""),IF(D143="",0,D143)+IF(E143="",0,E143),"")</f>
+        <f>IF(OR(D144&lt;&gt;"",E144&lt;&gt;""),IF(D144="",0,D144)+IF(E144="",0,E144),"")</f>
         <v/>
       </c>
       <c r="G144" s="14" t="inlineStr">
@@ -56681,7 +56929,7 @@
       </c>
       <c r="E145" s="28" t="n"/>
       <c r="F145" s="15">
-        <f>IF(OR(D144&lt;&gt;"",E144&lt;&gt;""),IF(D144="",0,D144)+IF(E144="",0,E144),"")</f>
+        <f>IF(OR(D145&lt;&gt;"",E145&lt;&gt;""),IF(D145="",0,D145)+IF(E145="",0,E145),"")</f>
         <v/>
       </c>
       <c r="G145" s="14" t="inlineStr">
@@ -56709,7 +56957,7 @@
       </c>
       <c r="E146" s="28" t="n"/>
       <c r="F146" s="15">
-        <f>IF(OR(D145&lt;&gt;"",E145&lt;&gt;""),IF(D145="",0,D145)+IF(E145="",0,E145),"")</f>
+        <f>IF(OR(D146&lt;&gt;"",E146&lt;&gt;""),IF(D146="",0,D146)+IF(E146="",0,E146),"")</f>
         <v/>
       </c>
       <c r="G146" s="14" t="inlineStr">
@@ -56737,7 +56985,7 @@
       </c>
       <c r="E147" s="28" t="n"/>
       <c r="F147" s="15">
-        <f>IF(OR(D146&lt;&gt;"",E146&lt;&gt;""),IF(D146="",0,D146)+IF(E146="",0,E146),"")</f>
+        <f>IF(OR(D147&lt;&gt;"",E147&lt;&gt;""),IF(D147="",0,D147)+IF(E147="",0,E147),"")</f>
         <v/>
       </c>
       <c r="G147" s="14" t="inlineStr">
@@ -56765,7 +57013,7 @@
       </c>
       <c r="E148" s="28" t="n"/>
       <c r="F148" s="15">
-        <f>IF(OR(D147&lt;&gt;"",E147&lt;&gt;""),IF(D147="",0,D147)+IF(E147="",0,E147),"")</f>
+        <f>IF(OR(D148&lt;&gt;"",E148&lt;&gt;""),IF(D148="",0,D148)+IF(E148="",0,E148),"")</f>
         <v/>
       </c>
       <c r="G148" s="14" t="inlineStr">
@@ -56793,7 +57041,7 @@
       </c>
       <c r="E149" s="28" t="n"/>
       <c r="F149" s="15">
-        <f>IF(OR(D148&lt;&gt;"",E148&lt;&gt;""),IF(D148="",0,D148)+IF(E148="",0,E148),"")</f>
+        <f>IF(OR(D149&lt;&gt;"",E149&lt;&gt;""),IF(D149="",0,D149)+IF(E149="",0,E149),"")</f>
         <v/>
       </c>
       <c r="G149" s="14" t="inlineStr">
@@ -56821,7 +57069,7 @@
       </c>
       <c r="E150" s="28" t="n"/>
       <c r="F150" s="15">
-        <f>IF(OR(D149&lt;&gt;"",E149&lt;&gt;""),IF(D149="",0,D149)+IF(E149="",0,E149),"")</f>
+        <f>IF(OR(D150&lt;&gt;"",E150&lt;&gt;""),IF(D150="",0,D150)+IF(E150="",0,E150),"")</f>
         <v/>
       </c>
       <c r="G150" s="14" t="inlineStr">
@@ -56849,7 +57097,7 @@
       </c>
       <c r="E151" s="28" t="n"/>
       <c r="F151" s="15">
-        <f>IF(OR(D150&lt;&gt;"",E150&lt;&gt;""),IF(D150="",0,D150)+IF(E150="",0,E150),"")</f>
+        <f>IF(OR(D151&lt;&gt;"",E151&lt;&gt;""),IF(D151="",0,D151)+IF(E151="",0,E151),"")</f>
         <v/>
       </c>
       <c r="G151" s="14" t="inlineStr">
@@ -56877,7 +57125,7 @@
       </c>
       <c r="E152" s="28" t="n"/>
       <c r="F152" s="15">
-        <f>IF(OR(D151&lt;&gt;"",E151&lt;&gt;""),IF(D151="",0,D151)+IF(E151="",0,E151),"")</f>
+        <f>IF(OR(D152&lt;&gt;"",E152&lt;&gt;""),IF(D152="",0,D152)+IF(E152="",0,E152),"")</f>
         <v/>
       </c>
       <c r="G152" s="14" t="inlineStr">
@@ -56905,7 +57153,7 @@
       </c>
       <c r="E153" s="28" t="n"/>
       <c r="F153" s="15">
-        <f>IF(OR(D152&lt;&gt;"",E152&lt;&gt;""),IF(D152="",0,D152)+IF(E152="",0,E152),"")</f>
+        <f>IF(OR(D153&lt;&gt;"",E153&lt;&gt;""),IF(D153="",0,D153)+IF(E153="",0,E153),"")</f>
         <v/>
       </c>
       <c r="G153" s="14" t="inlineStr">
@@ -56933,7 +57181,7 @@
       </c>
       <c r="E154" s="28" t="n"/>
       <c r="F154" s="15">
-        <f>IF(OR(D153&lt;&gt;"",E153&lt;&gt;""),IF(D153="",0,D153)+IF(E153="",0,E153),"")</f>
+        <f>IF(OR(D154&lt;&gt;"",E154&lt;&gt;""),IF(D154="",0,D154)+IF(E154="",0,E154),"")</f>
         <v/>
       </c>
       <c r="G154" s="14" t="inlineStr">
@@ -57228,7 +57476,10 @@
         <v>177300</v>
       </c>
       <c r="E171" s="28" t="n"/>
-      <c r="F171" s="15" t="n"/>
+      <c r="F171" s="15">
+        <f>IF(OR(D171&lt;&gt;"",E171&lt;&gt;""),IF(D171="",0,D171)+IF(E171="",0,E171),"")</f>
+        <v/>
+      </c>
       <c r="G171" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Cenas · Cosi Mi Piace (cena) · Mercado Pago · ALMACEN SOL</t>
@@ -57253,7 +57504,10 @@
         <v>21276</v>
       </c>
       <c r="E172" s="28" t="n"/>
-      <c r="F172" s="15" t="n"/>
+      <c r="F172" s="15">
+        <f>IF(OR(D172&lt;&gt;"",E172&lt;&gt;""),IF(D172="",0,D172)+IF(E172="",0,E172),"")</f>
+        <v/>
+      </c>
       <c r="G172" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Cenas · Cosi Mi Piace (propina) · Mercado Pago · ALMACEN SOL</t>
@@ -57278,7 +57532,10 @@
         <v>277360</v>
       </c>
       <c r="E173" s="28" t="n"/>
-      <c r="F173" s="15" t="n"/>
+      <c r="F173" s="15">
+        <f>IF(OR(D173&lt;&gt;"",E173&lt;&gt;""),IF(D173="",0,D173)+IF(E173="",0,E173),"")</f>
+        <v/>
+      </c>
       <c r="G173" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Cenas · Cosi Mi Piace (cena) · Mercado Pago · ALMACEN SOL</t>
@@ -57303,7 +57560,10 @@
         <v>33283</v>
       </c>
       <c r="E174" s="28" t="n"/>
-      <c r="F174" s="15" t="n"/>
+      <c r="F174" s="15">
+        <f>IF(OR(D174&lt;&gt;"",E174&lt;&gt;""),IF(D174="",0,D174)+IF(E174="",0,E174),"")</f>
+        <v/>
+      </c>
       <c r="G174" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Cenas · Cosi Mi Piace (propina) · Mercado Pago · ALMACEN SOL</t>
@@ -57328,7 +57588,10 @@
         <v>71400</v>
       </c>
       <c r="E175" s="28" t="n"/>
-      <c r="F175" s="15" t="n"/>
+      <c r="F175" s="15">
+        <f>IF(OR(D175&lt;&gt;"",E175&lt;&gt;""),IF(D175="",0,D175)+IF(E175="",0,E175),"")</f>
+        <v/>
+      </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
           <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
@@ -57348,11 +57611,11 @@
         </is>
       </c>
       <c r="D176" s="7">
-        <f>SUM(D133:D175)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Abril")</f>
         <v/>
       </c>
       <c r="E176" s="7">
-        <f>SUM(E133:E175)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Abril")</f>
         <v/>
       </c>
       <c r="F176" s="7">
@@ -57380,7 +57643,7 @@
       </c>
       <c r="E178" s="28" t="n"/>
       <c r="F178" s="15">
-        <f>IF(OR(D172&lt;&gt;"",E172&lt;&gt;""),IF(D172="",0,D172)+IF(E172="",0,E172),"")</f>
+        <f>IF(OR(D178&lt;&gt;"",E178&lt;&gt;""),IF(D178="",0,D178)+IF(E178="",0,E178),"")</f>
         <v/>
       </c>
       <c r="G178" s="14" t="inlineStr">
@@ -57408,7 +57671,7 @@
       </c>
       <c r="E179" s="28" t="n"/>
       <c r="F179" s="15">
-        <f>IF(OR(D173&lt;&gt;"",E173&lt;&gt;""),IF(D173="",0,D173)+IF(E173="",0,E173),"")</f>
+        <f>IF(OR(D179&lt;&gt;"",E179&lt;&gt;""),IF(D179="",0,D179)+IF(E179="",0,E179),"")</f>
         <v/>
       </c>
       <c r="G179" s="14" t="inlineStr">
@@ -57436,7 +57699,7 @@
       </c>
       <c r="E180" s="28" t="n"/>
       <c r="F180" s="15">
-        <f>IF(OR(D174&lt;&gt;"",E174&lt;&gt;""),IF(D174="",0,D174)+IF(E174="",0,E174),"")</f>
+        <f>IF(OR(D180&lt;&gt;"",E180&lt;&gt;""),IF(D180="",0,D180)+IF(E180="",0,E180),"")</f>
         <v/>
       </c>
       <c r="G180" s="14" t="inlineStr">
@@ -57464,7 +57727,7 @@
       </c>
       <c r="E181" s="28" t="n"/>
       <c r="F181" s="15">
-        <f>IF(OR(D175&lt;&gt;"",E175&lt;&gt;""),IF(D175="",0,D175)+IF(E175="",0,E175),"")</f>
+        <f>IF(OR(D181&lt;&gt;"",E181&lt;&gt;""),IF(D181="",0,D181)+IF(E181="",0,E181),"")</f>
         <v/>
       </c>
       <c r="G181" s="14" t="inlineStr">
@@ -57492,7 +57755,7 @@
       </c>
       <c r="E182" s="28" t="n"/>
       <c r="F182" s="15">
-        <f>IF(OR(D176&lt;&gt;"",E176&lt;&gt;""),IF(D176="",0,D176)+IF(E176="",0,E176),"")</f>
+        <f>IF(OR(D182&lt;&gt;"",E182&lt;&gt;""),IF(D182="",0,D182)+IF(E182="",0,E182),"")</f>
         <v/>
       </c>
       <c r="G182" s="14" t="inlineStr">
@@ -57520,7 +57783,7 @@
       </c>
       <c r="E183" s="28" t="n"/>
       <c r="F183" s="15">
-        <f>IF(OR(D177&lt;&gt;"",E177&lt;&gt;""),IF(D177="",0,D177)+IF(E177="",0,E177),"")</f>
+        <f>IF(OR(D183&lt;&gt;"",E183&lt;&gt;""),IF(D183="",0,D183)+IF(E183="",0,E183),"")</f>
         <v/>
       </c>
       <c r="G183" s="14" t="inlineStr">
@@ -57548,7 +57811,7 @@
       </c>
       <c r="E184" s="28" t="n"/>
       <c r="F184" s="15">
-        <f>IF(OR(D178&lt;&gt;"",E178&lt;&gt;""),IF(D178="",0,D178)+IF(E178="",0,E178),"")</f>
+        <f>IF(OR(D184&lt;&gt;"",E184&lt;&gt;""),IF(D184="",0,D184)+IF(E184="",0,E184),"")</f>
         <v/>
       </c>
       <c r="G184" s="14" t="inlineStr">
@@ -57576,7 +57839,7 @@
       </c>
       <c r="E185" s="28" t="n"/>
       <c r="F185" s="15">
-        <f>IF(OR(D179&lt;&gt;"",E179&lt;&gt;""),IF(D179="",0,D179)+IF(E179="",0,E179),"")</f>
+        <f>IF(OR(D185&lt;&gt;"",E185&lt;&gt;""),IF(D185="",0,D185)+IF(E185="",0,E185),"")</f>
         <v/>
       </c>
       <c r="G185" s="14" t="inlineStr">
@@ -57604,7 +57867,7 @@
       </c>
       <c r="E186" s="28" t="n"/>
       <c r="F186" s="15">
-        <f>IF(OR(D180&lt;&gt;"",E180&lt;&gt;""),IF(D180="",0,D180)+IF(E180="",0,E180),"")</f>
+        <f>IF(OR(D186&lt;&gt;"",E186&lt;&gt;""),IF(D186="",0,D186)+IF(E186="",0,E186),"")</f>
         <v/>
       </c>
       <c r="G186" s="14" t="inlineStr">
@@ -57632,7 +57895,7 @@
       </c>
       <c r="E187" s="28" t="n"/>
       <c r="F187" s="15">
-        <f>IF(OR(D181&lt;&gt;"",E181&lt;&gt;""),IF(D181="",0,D181)+IF(E181="",0,E181),"")</f>
+        <f>IF(OR(D187&lt;&gt;"",E187&lt;&gt;""),IF(D187="",0,D187)+IF(E187="",0,E187),"")</f>
         <v/>
       </c>
       <c r="G187" s="14" t="inlineStr">
@@ -57660,7 +57923,7 @@
       </c>
       <c r="E188" s="28" t="n"/>
       <c r="F188" s="15">
-        <f>IF(OR(D182&lt;&gt;"",E182&lt;&gt;""),IF(D182="",0,D182)+IF(E182="",0,E182),"")</f>
+        <f>IF(OR(D188&lt;&gt;"",E188&lt;&gt;""),IF(D188="",0,D188)+IF(E188="",0,E188),"")</f>
         <v/>
       </c>
       <c r="G188" s="14" t="inlineStr">
@@ -57688,7 +57951,7 @@
       </c>
       <c r="E189" s="28" t="n"/>
       <c r="F189" s="15">
-        <f>IF(OR(D183&lt;&gt;"",E183&lt;&gt;""),IF(D183="",0,D183)+IF(E183="",0,E183),"")</f>
+        <f>IF(OR(D189&lt;&gt;"",E189&lt;&gt;""),IF(D189="",0,D189)+IF(E189="",0,E189),"")</f>
         <v/>
       </c>
       <c r="G189" s="14" t="inlineStr">
@@ -57716,7 +57979,7 @@
       </c>
       <c r="E190" s="28" t="n"/>
       <c r="F190" s="15">
-        <f>IF(OR(D184&lt;&gt;"",E184&lt;&gt;""),IF(D184="",0,D184)+IF(E184="",0,E184),"")</f>
+        <f>IF(OR(D190&lt;&gt;"",E190&lt;&gt;""),IF(D190="",0,D190)+IF(E190="",0,E190),"")</f>
         <v/>
       </c>
       <c r="G190" s="14" t="inlineStr">
@@ -57744,7 +58007,7 @@
       </c>
       <c r="E191" s="28" t="n"/>
       <c r="F191" s="15">
-        <f>IF(OR(D185&lt;&gt;"",E185&lt;&gt;""),IF(D185="",0,D185)+IF(E185="",0,E185),"")</f>
+        <f>IF(OR(D191&lt;&gt;"",E191&lt;&gt;""),IF(D191="",0,D191)+IF(E191="",0,E191),"")</f>
         <v/>
       </c>
       <c r="G191" s="14" t="inlineStr">
@@ -57772,7 +58035,7 @@
       </c>
       <c r="E192" s="28" t="n"/>
       <c r="F192" s="15">
-        <f>IF(OR(D186&lt;&gt;"",E186&lt;&gt;""),IF(D186="",0,D186)+IF(E186="",0,E186),"")</f>
+        <f>IF(OR(D192&lt;&gt;"",E192&lt;&gt;""),IF(D192="",0,D192)+IF(E192="",0,E192),"")</f>
         <v/>
       </c>
       <c r="G192" s="14" t="inlineStr">
@@ -57800,7 +58063,7 @@
       </c>
       <c r="E193" s="28" t="n"/>
       <c r="F193" s="15">
-        <f>IF(OR(D187&lt;&gt;"",E187&lt;&gt;""),IF(D187="",0,D187)+IF(E187="",0,E187),"")</f>
+        <f>IF(OR(D193&lt;&gt;"",E193&lt;&gt;""),IF(D193="",0,D193)+IF(E193="",0,E193),"")</f>
         <v/>
       </c>
       <c r="G193" s="14" t="inlineStr">
@@ -57828,7 +58091,7 @@
       </c>
       <c r="E194" s="28" t="n"/>
       <c r="F194" s="15">
-        <f>IF(OR(D188&lt;&gt;"",E188&lt;&gt;""),IF(D188="",0,D188)+IF(E188="",0,E188),"")</f>
+        <f>IF(OR(D194&lt;&gt;"",E194&lt;&gt;""),IF(D194="",0,D194)+IF(E194="",0,E194),"")</f>
         <v/>
       </c>
       <c r="G194" s="14" t="inlineStr">
@@ -57856,7 +58119,7 @@
       </c>
       <c r="E195" s="28" t="n"/>
       <c r="F195" s="15">
-        <f>IF(OR(D189&lt;&gt;"",E189&lt;&gt;""),IF(D189="",0,D189)+IF(E189="",0,E189),"")</f>
+        <f>IF(OR(D195&lt;&gt;"",E195&lt;&gt;""),IF(D195="",0,D195)+IF(E195="",0,E195),"")</f>
         <v/>
       </c>
       <c r="G195" s="14" t="inlineStr">
@@ -57884,7 +58147,7 @@
       </c>
       <c r="E196" s="28" t="n"/>
       <c r="F196" s="15">
-        <f>IF(OR(D190&lt;&gt;"",E190&lt;&gt;""),IF(D190="",0,D190)+IF(E190="",0,E190),"")</f>
+        <f>IF(OR(D196&lt;&gt;"",E196&lt;&gt;""),IF(D196="",0,D196)+IF(E196="",0,E196),"")</f>
         <v/>
       </c>
       <c r="G196" s="14" t="inlineStr">
@@ -57912,7 +58175,7 @@
       </c>
       <c r="E197" s="28" t="n"/>
       <c r="F197" s="15">
-        <f>IF(OR(D191&lt;&gt;"",E191&lt;&gt;""),IF(D191="",0,D191)+IF(E191="",0,E191),"")</f>
+        <f>IF(OR(D197&lt;&gt;"",E197&lt;&gt;""),IF(D197="",0,D197)+IF(E197="",0,E197),"")</f>
         <v/>
       </c>
       <c r="G197" s="14" t="inlineStr">
@@ -57940,7 +58203,7 @@
       </c>
       <c r="E198" s="28" t="n"/>
       <c r="F198" s="15">
-        <f>IF(OR(D192&lt;&gt;"",E192&lt;&gt;""),IF(D192="",0,D192)+IF(E192="",0,E192),"")</f>
+        <f>IF(OR(D198&lt;&gt;"",E198&lt;&gt;""),IF(D198="",0,D198)+IF(E198="",0,E198),"")</f>
         <v/>
       </c>
       <c r="G198" s="14" t="inlineStr">
@@ -57968,7 +58231,7 @@
       </c>
       <c r="E199" s="28" t="n"/>
       <c r="F199" s="15">
-        <f>IF(OR(D193&lt;&gt;"",E193&lt;&gt;""),IF(D193="",0,D193)+IF(E193="",0,E193),"")</f>
+        <f>IF(OR(D199&lt;&gt;"",E199&lt;&gt;""),IF(D199="",0,D199)+IF(E199="",0,E199),"")</f>
         <v/>
       </c>
       <c r="G199" s="14" t="inlineStr">
@@ -58327,7 +58590,10 @@
         <v>170000</v>
       </c>
       <c r="E217" s="28" t="n"/>
-      <c r="F217" s="15" t="n"/>
+      <c r="F217" s="15">
+        <f>IF(OR(D217&lt;&gt;"",E217&lt;&gt;""),IF(D217="",0,D217)+IF(E217="",0,E217),"")</f>
+        <v/>
+      </c>
       <c r="G217" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Teatro · Plateanet · BBVA VISA · ALMACEN SOL</t>
@@ -58352,7 +58618,10 @@
         <v>20400</v>
       </c>
       <c r="E218" s="28" t="n"/>
-      <c r="F218" s="15" t="n"/>
+      <c r="F218" s="15">
+        <f>IF(OR(D218&lt;&gt;"",E218&lt;&gt;""),IF(D218="",0,D218)+IF(E218="",0,E218),"")</f>
+        <v/>
+      </c>
       <c r="G218" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Teatro · Plateanet · BBVA VISA · ALMACEN SOL</t>
@@ -58377,7 +58646,10 @@
         <v>65700</v>
       </c>
       <c r="E219" s="28" t="n"/>
-      <c r="F219" s="15" t="n"/>
+      <c r="F219" s="15">
+        <f>IF(OR(D219&lt;&gt;"",E219&lt;&gt;""),IF(D219="",0,D219)+IF(E219="",0,E219),"")</f>
+        <v/>
+      </c>
       <c r="G219" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -58402,7 +58674,10 @@
         <v>21600</v>
       </c>
       <c r="E220" s="28" t="n"/>
-      <c r="F220" s="15" t="n"/>
+      <c r="F220" s="15">
+        <f>IF(OR(D220&lt;&gt;"",E220&lt;&gt;""),IF(D220="",0,D220)+IF(E220="",0,E220),"")</f>
+        <v/>
+      </c>
       <c r="G220" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -58427,7 +58702,10 @@
         <v>90000</v>
       </c>
       <c r="E221" s="28" t="n"/>
-      <c r="F221" s="15" t="n"/>
+      <c r="F221" s="15">
+        <f>IF(OR(D221&lt;&gt;"",E221&lt;&gt;""),IF(D221="",0,D221)+IF(E221="",0,E221),"")</f>
+        <v/>
+      </c>
       <c r="G221" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -58452,7 +58730,10 @@
         <v>112500</v>
       </c>
       <c r="E222" s="28" t="n"/>
-      <c r="F222" s="15" t="n"/>
+      <c r="F222" s="15">
+        <f>IF(OR(D222&lt;&gt;"",E222&lt;&gt;""),IF(D222="",0,D222)+IF(E222="",0,E222),"")</f>
+        <v/>
+      </c>
       <c r="G222" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -58477,7 +58758,10 @@
         <v>154100</v>
       </c>
       <c r="E223" s="28" t="n"/>
-      <c r="F223" s="15" t="n"/>
+      <c r="F223" s="15">
+        <f>IF(OR(D223&lt;&gt;"",E223&lt;&gt;""),IF(D223="",0,D223)+IF(E223="",0,E223),"")</f>
+        <v/>
+      </c>
       <c r="G223" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Salidas comida · Hotel Madero (cena) · BBVA · ALMACEN SOL</t>
@@ -58502,7 +58786,10 @@
         <v>15410</v>
       </c>
       <c r="E224" s="28" t="n"/>
-      <c r="F224" s="15" t="n"/>
+      <c r="F224" s="15">
+        <f>IF(OR(D224&lt;&gt;"",E224&lt;&gt;""),IF(D224="",0,D224)+IF(E224="",0,E224),"")</f>
+        <v/>
+      </c>
       <c r="G224" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Salidas comida · Hotel Madero (propina) · BBVA · ALMACEN SOL</t>
@@ -58527,7 +58814,10 @@
         <v>30133</v>
       </c>
       <c r="E225" s="28" t="n"/>
-      <c r="F225" s="15" t="n"/>
+      <c r="F225" s="15">
+        <f>IF(OR(D225&lt;&gt;"",E225&lt;&gt;""),IF(D225="",0,D225)+IF(E225="",0,E225),"")</f>
+        <v/>
+      </c>
       <c r="G225" s="14" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Cenas · Cosi Mi Piace (cena) · Mercado Pago · ALMACEN SOL</t>
@@ -58552,7 +58842,10 @@
         <v>79924</v>
       </c>
       <c r="E226" s="28" t="n"/>
-      <c r="F226" s="15" t="n"/>
+      <c r="F226" s="15">
+        <f>IF(OR(D226&lt;&gt;"",E226&lt;&gt;""),IF(D226="",0,D226)+IF(E226="",0,E226),"")</f>
+        <v/>
+      </c>
       <c r="G226" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Leocan · Mercado Pago · ALMACEN SOL</t>
@@ -58577,7 +58870,10 @@
         <v>11100</v>
       </c>
       <c r="E227" s="28" t="n"/>
-      <c r="F227" s="15" t="n"/>
+      <c r="F227" s="15">
+        <f>IF(OR(D227&lt;&gt;"",E227&lt;&gt;""),IF(D227="",0,D227)+IF(E227="",0,E227),"")</f>
+        <v/>
+      </c>
       <c r="G227" s="14" t="inlineStr">
         <is>
           <t>RAMON · Otros · Paws Pet Market · Mercado Pago · ALMACEN SOL</t>
@@ -58597,11 +58893,11 @@
         </is>
       </c>
       <c r="D228" s="7">
-        <f>SUM(D178:D227)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Mayo")</f>
         <v/>
       </c>
       <c r="E228" s="7">
-        <f>SUM(E178:E227)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Mayo")</f>
         <v/>
       </c>
       <c r="F228" s="7">
@@ -58629,7 +58925,7 @@
       </c>
       <c r="E230" s="28" t="n"/>
       <c r="F230" s="15">
-        <f>IF(OR(D214&lt;&gt;"",E214&lt;&gt;""),IF(D214="",0,D214)+IF(E214="",0,E214),"")</f>
+        <f>IF(OR(D230&lt;&gt;"",E230&lt;&gt;""),IF(D230="",0,D230)+IF(E230="",0,E230),"")</f>
         <v/>
       </c>
       <c r="G230" s="14" t="inlineStr">
@@ -58657,7 +58953,7 @@
       </c>
       <c r="E231" s="28" t="n"/>
       <c r="F231" s="15">
-        <f>IF(OR(D215&lt;&gt;"",E215&lt;&gt;""),IF(D215="",0,D215)+IF(E215="",0,E215),"")</f>
+        <f>IF(OR(D231&lt;&gt;"",E231&lt;&gt;""),IF(D231="",0,D231)+IF(E231="",0,E231),"")</f>
         <v/>
       </c>
       <c r="G231" s="14" t="inlineStr">
@@ -58685,7 +58981,7 @@
       </c>
       <c r="E232" s="28" t="n"/>
       <c r="F232" s="15">
-        <f>IF(OR(D216&lt;&gt;"",E216&lt;&gt;""),IF(D216="",0,D216)+IF(E216="",0,E216),"")</f>
+        <f>IF(OR(D232&lt;&gt;"",E232&lt;&gt;""),IF(D232="",0,D232)+IF(E232="",0,E232),"")</f>
         <v/>
       </c>
       <c r="G232" s="14" t="inlineStr">
@@ -58713,7 +59009,7 @@
       </c>
       <c r="E233" s="28" t="n"/>
       <c r="F233" s="15">
-        <f>IF(OR(D217&lt;&gt;"",E217&lt;&gt;""),IF(D217="",0,D217)+IF(E217="",0,E217),"")</f>
+        <f>IF(OR(D233&lt;&gt;"",E233&lt;&gt;""),IF(D233="",0,D233)+IF(E233="",0,E233),"")</f>
         <v/>
       </c>
       <c r="G233" s="14" t="inlineStr">
@@ -58741,7 +59037,7 @@
       </c>
       <c r="E234" s="28" t="n"/>
       <c r="F234" s="15">
-        <f>IF(OR(D218&lt;&gt;"",E218&lt;&gt;""),IF(D218="",0,D218)+IF(E218="",0,E218),"")</f>
+        <f>IF(OR(D234&lt;&gt;"",E234&lt;&gt;""),IF(D234="",0,D234)+IF(E234="",0,E234),"")</f>
         <v/>
       </c>
       <c r="G234" s="14" t="inlineStr">
@@ -58769,7 +59065,7 @@
       </c>
       <c r="E235" s="28" t="n"/>
       <c r="F235" s="15">
-        <f>IF(OR(D219&lt;&gt;"",E219&lt;&gt;""),IF(D219="",0,D219)+IF(E219="",0,E219),"")</f>
+        <f>IF(OR(D235&lt;&gt;"",E235&lt;&gt;""),IF(D235="",0,D235)+IF(E235="",0,E235),"")</f>
         <v/>
       </c>
       <c r="G235" s="14" t="inlineStr">
@@ -58797,7 +59093,7 @@
       </c>
       <c r="E236" s="28" t="n"/>
       <c r="F236" s="15">
-        <f>IF(OR(D220&lt;&gt;"",E220&lt;&gt;""),IF(D220="",0,D220)+IF(E220="",0,E220),"")</f>
+        <f>IF(OR(D236&lt;&gt;"",E236&lt;&gt;""),IF(D236="",0,D236)+IF(E236="",0,E236),"")</f>
         <v/>
       </c>
       <c r="G236" s="14" t="inlineStr">
@@ -58825,7 +59121,7 @@
       </c>
       <c r="E237" s="28" t="n"/>
       <c r="F237" s="15">
-        <f>IF(OR(D221&lt;&gt;"",E221&lt;&gt;""),IF(D221="",0,D221)+IF(E221="",0,E221),"")</f>
+        <f>IF(OR(D237&lt;&gt;"",E237&lt;&gt;""),IF(D237="",0,D237)+IF(E237="",0,E237),"")</f>
         <v/>
       </c>
       <c r="G237" s="14" t="inlineStr">
@@ -58853,7 +59149,7 @@
       </c>
       <c r="E238" s="28" t="n"/>
       <c r="F238" s="15">
-        <f>IF(OR(D222&lt;&gt;"",E222&lt;&gt;""),IF(D222="",0,D222)+IF(E222="",0,E222),"")</f>
+        <f>IF(OR(D238&lt;&gt;"",E238&lt;&gt;""),IF(D238="",0,D238)+IF(E238="",0,E238),"")</f>
         <v/>
       </c>
       <c r="G238" s="14" t="inlineStr">
@@ -58881,7 +59177,7 @@
       </c>
       <c r="E239" s="28" t="n"/>
       <c r="F239" s="15">
-        <f>IF(OR(D223&lt;&gt;"",E223&lt;&gt;""),IF(D223="",0,D223)+IF(E223="",0,E223),"")</f>
+        <f>IF(OR(D239&lt;&gt;"",E239&lt;&gt;""),IF(D239="",0,D239)+IF(E239="",0,E239),"")</f>
         <v/>
       </c>
       <c r="G239" s="14" t="inlineStr">
@@ -58909,7 +59205,7 @@
       </c>
       <c r="E240" s="28" t="n"/>
       <c r="F240" s="15">
-        <f>IF(OR(D224&lt;&gt;"",E224&lt;&gt;""),IF(D224="",0,D224)+IF(E224="",0,E224),"")</f>
+        <f>IF(OR(D240&lt;&gt;"",E240&lt;&gt;""),IF(D240="",0,D240)+IF(E240="",0,E240),"")</f>
         <v/>
       </c>
       <c r="G240" s="14" t="inlineStr">
@@ -58937,7 +59233,7 @@
       </c>
       <c r="E241" s="28" t="n"/>
       <c r="F241" s="15">
-        <f>IF(OR(D225&lt;&gt;"",E225&lt;&gt;""),IF(D225="",0,D225)+IF(E225="",0,E225),"")</f>
+        <f>IF(OR(D241&lt;&gt;"",E241&lt;&gt;""),IF(D241="",0,D241)+IF(E241="",0,E241),"")</f>
         <v/>
       </c>
       <c r="G241" s="14" t="inlineStr">
@@ -58965,7 +59261,7 @@
       </c>
       <c r="E242" s="28" t="n"/>
       <c r="F242" s="15">
-        <f>IF(OR(D226&lt;&gt;"",E226&lt;&gt;""),IF(D226="",0,D226)+IF(E226="",0,E226),"")</f>
+        <f>IF(OR(D242&lt;&gt;"",E242&lt;&gt;""),IF(D242="",0,D242)+IF(E242="",0,E242),"")</f>
         <v/>
       </c>
       <c r="G242" s="14" t="inlineStr">
@@ -58993,7 +59289,7 @@
       </c>
       <c r="E243" s="28" t="n"/>
       <c r="F243" s="15">
-        <f>IF(OR(D227&lt;&gt;"",E227&lt;&gt;""),IF(D227="",0,D227)+IF(E227="",0,E227),"")</f>
+        <f>IF(OR(D243&lt;&gt;"",E243&lt;&gt;""),IF(D243="",0,D243)+IF(E243="",0,E243),"")</f>
         <v/>
       </c>
       <c r="G243" s="14" t="inlineStr">
@@ -59021,7 +59317,7 @@
       </c>
       <c r="E244" s="28" t="n"/>
       <c r="F244" s="15">
-        <f>IF(OR(D228&lt;&gt;"",E228&lt;&gt;""),IF(D228="",0,D228)+IF(E228="",0,E228),"")</f>
+        <f>IF(OR(D244&lt;&gt;"",E244&lt;&gt;""),IF(D244="",0,D244)+IF(E244="",0,E244),"")</f>
         <v/>
       </c>
       <c r="G244" s="14" t="inlineStr">
@@ -59049,7 +59345,7 @@
       </c>
       <c r="E245" s="28" t="n"/>
       <c r="F245" s="15">
-        <f>IF(OR(D229&lt;&gt;"",E229&lt;&gt;""),IF(D229="",0,D229)+IF(E229="",0,E229),"")</f>
+        <f>IF(OR(D245&lt;&gt;"",E245&lt;&gt;""),IF(D245="",0,D245)+IF(E245="",0,E245),"")</f>
         <v/>
       </c>
       <c r="G245" s="14" t="inlineStr">
@@ -59077,7 +59373,7 @@
       </c>
       <c r="E246" s="28" t="n"/>
       <c r="F246" s="15">
-        <f>IF(OR(D231&lt;&gt;"",E231&lt;&gt;""),IF(D231="",0,D231)+IF(E231="",0,E231),"")</f>
+        <f>IF(OR(D246&lt;&gt;"",E246&lt;&gt;""),IF(D246="",0,D246)+IF(E246="",0,E246),"")</f>
         <v/>
       </c>
       <c r="G246" s="14" t="inlineStr">
@@ -59105,7 +59401,7 @@
       </c>
       <c r="E247" s="28" t="n"/>
       <c r="F247" s="15">
-        <f>IF(OR(D232&lt;&gt;"",E232&lt;&gt;""),IF(D232="",0,D232)+IF(E232="",0,E232),"")</f>
+        <f>IF(OR(D247&lt;&gt;"",E247&lt;&gt;""),IF(D247="",0,D247)+IF(E247="",0,E247),"")</f>
         <v/>
       </c>
       <c r="G247" s="14" t="inlineStr">
@@ -59133,7 +59429,7 @@
       </c>
       <c r="E248" s="28" t="n"/>
       <c r="F248" s="15">
-        <f>IF(OR(D233&lt;&gt;"",E233&lt;&gt;""),IF(D233="",0,D233)+IF(E233="",0,E233),"")</f>
+        <f>IF(OR(D248&lt;&gt;"",E248&lt;&gt;""),IF(D248="",0,D248)+IF(E248="",0,E248),"")</f>
         <v/>
       </c>
       <c r="G248" s="14" t="inlineStr">
@@ -59161,7 +59457,7 @@
       </c>
       <c r="E249" s="28" t="n"/>
       <c r="F249" s="15">
-        <f>IF(OR(D234&lt;&gt;"",E234&lt;&gt;""),IF(D234="",0,D234)+IF(E234="",0,E234),"")</f>
+        <f>IF(OR(D249&lt;&gt;"",E249&lt;&gt;""),IF(D249="",0,D249)+IF(E249="",0,E249),"")</f>
         <v/>
       </c>
       <c r="G249" s="14" t="inlineStr">
@@ -59189,7 +59485,7 @@
       </c>
       <c r="E250" s="28" t="n"/>
       <c r="F250" s="15">
-        <f>IF(OR(D235&lt;&gt;"",E235&lt;&gt;""),IF(D235="",0,D235)+IF(E235="",0,E235),"")</f>
+        <f>IF(OR(D250&lt;&gt;"",E250&lt;&gt;""),IF(D250="",0,D250)+IF(E250="",0,E250),"")</f>
         <v/>
       </c>
       <c r="G250" s="14" t="inlineStr">
@@ -59217,7 +59513,7 @@
       </c>
       <c r="E251" s="28" t="n"/>
       <c r="F251" s="15">
-        <f>IF(OR(D236&lt;&gt;"",E236&lt;&gt;""),IF(D236="",0,D236)+IF(E236="",0,E236),"")</f>
+        <f>IF(OR(D251&lt;&gt;"",E251&lt;&gt;""),IF(D251="",0,D251)+IF(E251="",0,E251),"")</f>
         <v/>
       </c>
       <c r="G251" s="14" t="inlineStr">
@@ -59528,7 +59824,10 @@
         <v>1200</v>
       </c>
       <c r="E269" s="28" t="n"/>
-      <c r="F269" s="15" t="n"/>
+      <c r="F269" s="15">
+        <f>IF(OR(D269&lt;&gt;"",E269&lt;&gt;""),IF(D269="",0,D269)+IF(E269="",0,E269),"")</f>
+        <v/>
+      </c>
       <c r="G269" s="14" t="inlineStr">
         <is>
           <t>PEDIDOS YA · COMIDA · propina · MP cuenta</t>
@@ -59553,7 +59852,10 @@
         <v>64750</v>
       </c>
       <c r="E270" s="28" t="n"/>
-      <c r="F270" s="15" t="n"/>
+      <c r="F270" s="15">
+        <f>IF(OR(D270&lt;&gt;"",E270&lt;&gt;""),IF(D270="",0,D270)+IF(E270="",0,E270),"")</f>
+        <v/>
+      </c>
       <c r="G270" s="14" t="inlineStr">
         <is>
           <t>COMIDA · Buenos Muchachos Resto · MP cuenta</t>
@@ -59578,7 +59880,10 @@
         <v>12900</v>
       </c>
       <c r="E271" s="28" t="n"/>
-      <c r="F271" s="15" t="n"/>
+      <c r="F271" s="15">
+        <f>IF(OR(D271&lt;&gt;"",E271&lt;&gt;""),IF(D271="",0,D271)+IF(E271="",0,E271),"")</f>
+        <v/>
+      </c>
       <c r="G271" s="14" t="inlineStr">
         <is>
           <t>STREAMING TV · Directv streaming · ALMACEN SOL · resumen MP</t>
@@ -59603,7 +59908,10 @@
         <v>48600</v>
       </c>
       <c r="E272" s="28" t="n"/>
-      <c r="F272" s="15" t="n"/>
+      <c r="F272" s="15">
+        <f>IF(OR(D272&lt;&gt;"",E272&lt;&gt;""),IF(D272="",0,D272)+IF(E272="",0,E272),"")</f>
+        <v/>
+      </c>
       <c r="G272" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -59623,11 +59931,11 @@
         </is>
       </c>
       <c r="D273" s="7">
-        <f>SUM(D230:D272)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Junio")</f>
         <v/>
       </c>
       <c r="E273" s="7">
-        <f>SUM(E230:E272)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Junio")</f>
         <v/>
       </c>
       <c r="F273" s="7">
@@ -59655,7 +59963,7 @@
       </c>
       <c r="E275" s="28" t="n"/>
       <c r="F275" s="15">
-        <f>IF(OR(D256&lt;&gt;"",E256&lt;&gt;""),IF(D256="",0,D256)+IF(E256="",0,E256),"")</f>
+        <f>IF(OR(D275&lt;&gt;"",E275&lt;&gt;""),IF(D275="",0,D275)+IF(E275="",0,E275),"")</f>
         <v/>
       </c>
       <c r="G275" s="14" t="inlineStr">
@@ -59683,7 +59991,7 @@
       </c>
       <c r="E276" s="28" t="n"/>
       <c r="F276" s="15">
-        <f>IF(OR(D261&lt;&gt;"",E261&lt;&gt;""),IF(D261="",0,D261)+IF(E261="",0,E261),"")</f>
+        <f>IF(OR(D276&lt;&gt;"",E276&lt;&gt;""),IF(D276="",0,D276)+IF(E276="",0,E276),"")</f>
         <v/>
       </c>
       <c r="G276" s="14" t="inlineStr">
@@ -59711,7 +60019,7 @@
       </c>
       <c r="E277" s="28" t="n"/>
       <c r="F277" s="15">
-        <f>IF(OR(D262&lt;&gt;"",E262&lt;&gt;""),IF(D262="",0,D262)+IF(E262="",0,E262),"")</f>
+        <f>IF(OR(D277&lt;&gt;"",E277&lt;&gt;""),IF(D277="",0,D277)+IF(E277="",0,E277),"")</f>
         <v/>
       </c>
       <c r="G277" s="14" t="inlineStr">
@@ -59739,7 +60047,7 @@
       </c>
       <c r="E278" s="28" t="n"/>
       <c r="F278" s="15">
-        <f>IF(OR(D263&lt;&gt;"",E263&lt;&gt;""),IF(D263="",0,D263)+IF(E263="",0,E263),"")</f>
+        <f>IF(OR(D278&lt;&gt;"",E278&lt;&gt;""),IF(D278="",0,D278)+IF(E278="",0,E278),"")</f>
         <v/>
       </c>
       <c r="G278" s="14" t="inlineStr">
@@ -59767,7 +60075,7 @@
       </c>
       <c r="E279" s="28" t="n"/>
       <c r="F279" s="15">
-        <f>IF(OR(D264&lt;&gt;"",E264&lt;&gt;""),IF(D264="",0,D264)+IF(E264="",0,E264),"")</f>
+        <f>IF(OR(D279&lt;&gt;"",E279&lt;&gt;""),IF(D279="",0,D279)+IF(E279="",0,E279),"")</f>
         <v/>
       </c>
       <c r="G279" s="14" t="inlineStr">
@@ -59804,7 +60112,7 @@
       </c>
       <c r="E281" s="28" t="n"/>
       <c r="F281" s="15">
-        <f>IF(OR(D266&lt;&gt;"",E266&lt;&gt;""),IF(D266="",0,D266)+IF(E266="",0,E266),"")</f>
+        <f>IF(OR(D281&lt;&gt;"",E281&lt;&gt;""),IF(D281="",0,D281)+IF(E281="",0,E281),"")</f>
         <v/>
       </c>
       <c r="G281" s="14" t="inlineStr">
@@ -59832,7 +60140,7 @@
       </c>
       <c r="E282" s="28" t="n"/>
       <c r="F282" s="15">
-        <f>IF(OR(D267&lt;&gt;"",E267&lt;&gt;""),IF(D267="",0,D267)+IF(E267="",0,E267),"")</f>
+        <f>IF(OR(D282&lt;&gt;"",E282&lt;&gt;""),IF(D282="",0,D282)+IF(E282="",0,E282),"")</f>
         <v/>
       </c>
       <c r="G282" s="14" t="inlineStr">
@@ -59860,7 +60168,7 @@
       </c>
       <c r="E283" s="28" t="n"/>
       <c r="F283" s="15">
-        <f>IF(OR(D268&lt;&gt;"",E268&lt;&gt;""),IF(D268="",0,D268)+IF(E268="",0,E268),"")</f>
+        <f>IF(OR(D283&lt;&gt;"",E283&lt;&gt;""),IF(D283="",0,D283)+IF(E283="",0,E283),"")</f>
         <v/>
       </c>
       <c r="G283" s="14" t="inlineStr">
@@ -59888,7 +60196,7 @@
       </c>
       <c r="E284" s="28" t="n"/>
       <c r="F284" s="15">
-        <f>IF(OR(D269&lt;&gt;"",E269&lt;&gt;""),IF(D269="",0,D269)+IF(E269="",0,E269),"")</f>
+        <f>IF(OR(D284&lt;&gt;"",E284&lt;&gt;""),IF(D284="",0,D284)+IF(E284="",0,E284),"")</f>
         <v/>
       </c>
       <c r="G284" s="14" t="inlineStr">
@@ -59916,7 +60224,7 @@
       </c>
       <c r="E285" s="28" t="n"/>
       <c r="F285" s="15">
-        <f>IF(OR(D270&lt;&gt;"",E270&lt;&gt;""),IF(D270="",0,D270)+IF(E270="",0,E270),"")</f>
+        <f>IF(OR(D285&lt;&gt;"",E285&lt;&gt;""),IF(D285="",0,D285)+IF(E285="",0,E285),"")</f>
         <v/>
       </c>
       <c r="G285" s="14" t="inlineStr">
@@ -59944,7 +60252,7 @@
       </c>
       <c r="E286" s="28" t="n"/>
       <c r="F286" s="15">
-        <f>IF(OR(D271&lt;&gt;"",E271&lt;&gt;""),IF(D271="",0,D271)+IF(E271="",0,E271),"")</f>
+        <f>IF(OR(D286&lt;&gt;"",E286&lt;&gt;""),IF(D286="",0,D286)+IF(E286="",0,E286),"")</f>
         <v/>
       </c>
       <c r="G286" s="14" t="inlineStr">
@@ -59972,7 +60280,7 @@
       </c>
       <c r="E287" s="28" t="n"/>
       <c r="F287" s="15">
-        <f>IF(OR(D272&lt;&gt;"",E272&lt;&gt;""),IF(D272="",0,D272)+IF(E272="",0,E272),"")</f>
+        <f>IF(OR(D287&lt;&gt;"",E287&lt;&gt;""),IF(D287="",0,D287)+IF(E287="",0,E287),"")</f>
         <v/>
       </c>
       <c r="G287" s="14" t="inlineStr">
@@ -60367,7 +60675,10 @@
         <v>106650</v>
       </c>
       <c r="E311" s="28" t="n"/>
-      <c r="F311" s="15" t="n"/>
+      <c r="F311" s="15">
+        <f>IF(OR(D311&lt;&gt;"",E311&lt;&gt;""),IF(D311="",0,D311)+IF(E311="",0,E311),"")</f>
+        <v/>
+      </c>
       <c r="G311" s="14" t="inlineStr">
         <is>
           <t>RAMON · Veterinario · Valeria Mele / El Perro Verde · ALMACEN SOL</t>
@@ -60387,11 +60698,11 @@
         </is>
       </c>
       <c r="D312" s="7">
-        <f>SUM(D275:D311)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Julio")</f>
         <v/>
       </c>
       <c r="E312" s="7">
-        <f>SUM(E275:E311)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Julio")</f>
         <v/>
       </c>
       <c r="F312" s="7">
@@ -61053,11 +61364,11 @@
         </is>
       </c>
       <c r="D354" s="7">
-        <f>SUM(D314:D353)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Agosto")</f>
         <v/>
       </c>
       <c r="E354" s="7">
-        <f>SUM(E314:E353)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Agosto")</f>
         <v/>
       </c>
       <c r="F354" s="7">
@@ -61719,11 +62030,11 @@
         </is>
       </c>
       <c r="D396" s="7">
-        <f>SUM(D356:D395)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Septiembre")</f>
         <v/>
       </c>
       <c r="E396" s="7">
-        <f>SUM(E356:E395)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Septiembre")</f>
         <v/>
       </c>
       <c r="F396" s="7">
@@ -62385,11 +62696,11 @@
         </is>
       </c>
       <c r="D438" s="7">
-        <f>SUM(D398:D437)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Octubre")</f>
         <v/>
       </c>
       <c r="E438" s="7">
-        <f>SUM(E398:E437)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Octubre")</f>
         <v/>
       </c>
       <c r="F438" s="7">
@@ -63051,11 +63362,11 @@
         </is>
       </c>
       <c r="D480" s="7">
-        <f>SUM(D440:D479)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Noviembre")</f>
         <v/>
       </c>
       <c r="E480" s="7">
-        <f>SUM(E440:E479)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Noviembre")</f>
         <v/>
       </c>
       <c r="F480" s="7">
@@ -63717,11 +64028,11 @@
         </is>
       </c>
       <c r="D522" s="7">
-        <f>SUM(D482:D521)</f>
+        <f>SUMIFS($D$4:$D$600,$A$4:$A$600,"Diciembre")</f>
         <v/>
       </c>
       <c r="E522" s="7">
-        <f>SUM(E482:E521)</f>
+        <f>SUMIFS($E$4:$E$600,$A$4:$A$600,"Diciembre")</f>
         <v/>
       </c>
       <c r="F522" s="7">
@@ -63748,7 +64059,7 @@
         <v>337644</v>
       </c>
       <c r="F523">
-        <f>IF(OR(D507&lt;&gt;"",E507&lt;&gt;""),IF(D507="",0,D507)+IF(E507="",0,E507),"")</f>
+        <f>IF(OR(D523&lt;&gt;"",E523&lt;&gt;""),IF(D523="",0,D523)+IF(E523="",0,E523),"")</f>
         <v/>
       </c>
       <c r="G523" t="inlineStr">
@@ -63775,7 +64086,7 @@
         <v>-49597</v>
       </c>
       <c r="F524">
-        <f>IF(OR(D508&lt;&gt;"",E508&lt;&gt;""),IF(D508="",0,D508)+IF(E508="",0,E508),"")</f>
+        <f>IF(OR(D524&lt;&gt;"",E524&lt;&gt;""),IF(D524="",0,D524)+IF(E524="",0,E524),"")</f>
         <v/>
       </c>
       <c r="G524" t="inlineStr">
@@ -63795,7 +64106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65508,8 +65819,28 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="25" t="n"/>
-      <c r="D55" s="26" t="n"/>
+      <c r="A55" s="54" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ALMACEN</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Almacén CIUDAD — Enero 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D55" s="26">
+        <f>'Almacen Detalle'!F47</f>
+        <v/>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>FARMACIA · Farmacia Selma · cargado en Almacen Detalle</t>
@@ -65522,8 +65853,28 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="25" t="n"/>
-      <c r="D56" s="26" t="n"/>
+      <c r="A56" s="54" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ALMACEN</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Almacén CIUDAD — Febrero 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D56" s="26">
+        <f>'Almacen Detalle'!F87</f>
+        <v/>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr">
         <is>
           <t>FARMACIA · Farmacia Maure</t>
@@ -65536,8 +65887,28 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="25" t="n"/>
-      <c r="D57" s="26" t="n"/>
+      <c r="A57" s="54" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ALMACEN</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Almacén CIUDAD — Marzo 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D57" s="26">
+        <f>'Almacen Detalle'!F131</f>
+        <v/>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>FARMACIA · Farmacia Maure</t>
@@ -65550,8 +65921,28 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="25" t="n"/>
-      <c r="D58" s="26" t="n"/>
+      <c r="A58" s="54" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ALMACEN</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Almacén CIUDAD — Abril 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D58" s="26">
+        <f>'Almacen Detalle'!F176</f>
+        <v/>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>FARMACIA · Farmacia Maure</t>
@@ -65564,8 +65955,28 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="25" t="n"/>
-      <c r="D59" s="26" t="n"/>
+      <c r="A59" s="54" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ALMACEN</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Almacén CIUDAD — Mayo 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D59" s="26">
+        <f>'Almacen Detalle'!F228</f>
+        <v/>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
+      </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>FARMACIA · Farmacity</t>
@@ -65578,8 +65989,28 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="25" t="n"/>
-      <c r="D60" s="26" t="n"/>
+      <c r="A60" s="54" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ALMACEN</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Almacén CIUDAD — Junio 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D60" s="26">
+        <f>'Almacen Detalle'!F273</f>
+        <v/>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>FARMACIA · Farmacia Maure</t>
@@ -65592,69 +66023,98 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="54" t="n"/>
+      <c r="A61" s="54" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ALMACEN</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Almacén CIUDAD — Julio 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D61">
+        <f>'Almacen Detalle'!F312</f>
+        <v/>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="17" t="n">
-        <v>46204</v>
+      <c r="A62" s="53" t="n">
+        <v>46235</v>
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>LIMPIEZA CASA</t>
+          <t>ALMACEN</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
         <is>
-          <t>LIMPIEZA CASA — Julio 2026 (MP cuenta: 9.500+123.240+120.240+147.660)</t>
-        </is>
-      </c>
-      <c r="D62" s="15" t="n">
-        <v>400640</v>
+          <t>Almacén CIUDAD — Agosto 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D62" s="15">
+        <f>'Almacen Detalle'!F354</f>
+        <v/>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
+        </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="25" t="n">
-        <v>46152</v>
+      <c r="A63" s="54" t="n">
+        <v>46266</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ABL</t>
+          <t>ALMACEN</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Agip ABL GCBA · partida 397789 (5 pagos 10-may)</t>
-        </is>
-      </c>
-      <c r="D63" s="26" t="n">
-        <v>132599</v>
+          <t>Almacén CIUDAD — Septiembre 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D63" s="26">
+        <f>'Almacen Detalle'!F396</f>
+        <v/>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Mercado Pago — Dinero disponible</t>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="17" t="n">
-        <v>46031</v>
+      <c r="A64" s="53" t="n">
+        <v>46296</v>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES</t>
+          <t>ALMACEN</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>PedidosYa Plus</t>
-        </is>
-      </c>
-      <c r="D64" s="15" t="n">
-        <v>5490</v>
+          <t>Almacén CIUDAD — Octubre 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D64" s="15">
+        <f>'Almacen Detalle'!F438</f>
+        <v/>
       </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
         </is>
       </c>
       <c r="F64" s="18" t="inlineStr">
@@ -65664,25 +66124,26 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="17" t="n">
-        <v>46062</v>
+      <c r="A65" s="53" t="n">
+        <v>46327</v>
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>SUSCRIPCIONES</t>
+          <t>ALMACEN</t>
         </is>
       </c>
       <c r="C65" s="14" t="inlineStr">
         <is>
-          <t>PedidosYa Plus</t>
-        </is>
-      </c>
-      <c r="D65" s="15" t="n">
-        <v>5990</v>
+          <t>Almacén CIUDAD — Noviembre 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D65" s="15">
+        <f>'Almacen Detalle'!F480</f>
+        <v/>
       </c>
       <c r="E65" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
         </is>
       </c>
       <c r="F65" s="18" t="inlineStr">
@@ -65692,25 +66153,26 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="17" t="n">
-        <v>46129</v>
+      <c r="A66" s="53" t="n">
+        <v>46357</v>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>CASA</t>
+          <t>ALMACEN</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>AGUS/PSA — Agustina Vissani</t>
-        </is>
-      </c>
-      <c r="D66" s="15" t="n">
-        <v>155000</v>
+          <t>Almacén CIUDAD — Diciembre 2026 (total mensual Almacen Detalle)</t>
+        </is>
+      </c>
+      <c r="D66" s="15">
+        <f>'Almacen Detalle'!F522</f>
+        <v/>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>Total hoja Almacen Detalle (Sol + Chris)</t>
         </is>
       </c>
       <c r="F66" s="18" t="inlineStr">
@@ -65804,136 +66266,88 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="53" t="n">
-        <v>46157</v>
-      </c>
-      <c r="B70" s="14" t="inlineStr">
-        <is>
-          <t>CASA</t>
-        </is>
-      </c>
-      <c r="C70" s="14" t="inlineStr">
-        <is>
-          <t>AGUS/PSA — Agustina Vissani (mayo)</t>
-        </is>
-      </c>
-      <c r="D70" s="15" t="n">
-        <v>125000</v>
-      </c>
-      <c r="E70" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+      <c r="A70" s="53" t="n"/>
+      <c r="B70" s="14" t="n"/>
+      <c r="C70" s="14" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="14" t="n"/>
       <c r="F70" s="18" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="53" t="n">
-        <v>46185</v>
+        <v>46217</v>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>CASA</t>
+          <t>ABL</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
-          <t>AGUS/PSA — Agustina Vissani (junio)</t>
+          <t>Agip ABL GCBA · partida 397789</t>
         </is>
       </c>
       <c r="D71" s="15" t="n">
-        <v>135000</v>
+        <v>26175</v>
       </c>
       <c r="E71" s="14" t="inlineStr">
         <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="53" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>Telecentro</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>Telecentro CIUDAD — pago MP 17/06/2026 (junio)</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="n">
+        <v>48420</v>
+      </c>
+      <c r="E72" s="14" t="inlineStr">
+        <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="F71" s="18" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="53" t="n"/>
-      <c r="B72" s="14" t="n"/>
-      <c r="C72" s="14" t="n"/>
-      <c r="D72" s="15" t="n"/>
-      <c r="E72" s="14" t="n"/>
-      <c r="F72" s="18" t="n"/>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="53" t="n">
-        <v>46217</v>
+        <v>46203</v>
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>ABL</t>
+          <t>Telecentro</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
         <is>
-          <t>Agip ABL GCBA · partida 397789</t>
+          <t>Telecentro CIUDAD — débito BBVA 30/06/2026 (julio)</t>
         </is>
       </c>
       <c r="D73" s="15" t="n">
-        <v>26175</v>
+        <v>31999</v>
       </c>
       <c r="E73" s="14" t="inlineStr">
         <is>
-          <t>Mercado Pago — Dinero disponible</t>
-        </is>
-      </c>
-      <c r="F73" s="18" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="53" t="n">
-        <v>46190</v>
-      </c>
-      <c r="B74" s="14" t="inlineStr">
-        <is>
-          <t>Telecentro</t>
-        </is>
-      </c>
-      <c r="C74" s="14" t="inlineStr">
-        <is>
-          <t>Telecentro CIUDAD — pago MP 17/06/2026 (junio)</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="n">
-        <v>48420</v>
-      </c>
-      <c r="E74" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="F74" s="18" t="inlineStr">
-        <is>
-          <t>3491192</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="53" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B75" s="14" t="inlineStr">
-        <is>
-          <t>Telecentro</t>
-        </is>
-      </c>
-      <c r="C75" s="14" t="inlineStr">
-        <is>
-          <t>Telecentro CIUDAD — débito BBVA 30/06/2026 (julio)</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="n">
-        <v>31999</v>
-      </c>
-      <c r="E75" s="14" t="inlineStr">
-        <is>
           <t>Débito BBVA</t>
         </is>
       </c>
-      <c r="F75" s="18" t="inlineStr">
+      <c r="F73" s="18" t="inlineStr">
         <is>
           <t>3491192</t>
         </is>

</xml_diff>

<commit_message>
Add Todo Tartas $57600 to CIUDAD almacén for 21 Jul 2026.
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -60295,15 +60295,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B288" s="17" t="n"/>
-      <c r="C288" s="14" t="n"/>
-      <c r="D288" s="27" t="n"/>
+      <c r="B288" s="17" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C288" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Todo Tartas</t>
+        </is>
+      </c>
+      <c r="D288" s="27" t="n">
+        <v>57600</v>
+      </c>
       <c r="E288" s="28" t="n"/>
       <c r="F288" s="15">
-        <f>IF(OR(D273&lt;&gt;"",E273&lt;&gt;""),IF(D273="",0,D273)+IF(E273="",0,E273),"")</f>
-        <v/>
-      </c>
-      <c r="G288" s="14" t="n"/>
+        <f>IF(OR(D288&lt;&gt;"",E288&lt;&gt;""),IF(D288="",0,D288)+IF(E288="",0,E288),"")</f>
+        <v/>
+      </c>
+      <c r="G288" s="14" t="inlineStr">
+        <is>
+          <t>MP · panadería · ex `Todo Tartas`</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load Mercado Pago extract for 21–23 Jul 2026.
- Transferencia recibida Pelesson Aldo Oscar $4,900,000 (23/07)
- Uber/Ebanx net: $54 + $6,062 to GPS; exclude $5,502 refunded cycle
- Zilver SA $78,167 (ceil) to GPS COMPRAS (21/07)
- Reserva automática AVA/Susi to MP No Gasto (21/07)
- Todo Tartas $57,600 to Almacen Detalle (21/07)
- Regenerate SOL master

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3641,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F828"/>
+  <dimension ref="A1:F831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25746,6 +25746,90 @@
       <c r="F828" s="34" t="inlineStr">
         <is>
           <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · C.04/06 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="62" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B829" s="34" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C829" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D829" s="34" t="n">
+        <v>54</v>
+      </c>
+      <c r="E829" s="34" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F829" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="62" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B830" s="34" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C830" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D830" s="34" t="n">
+        <v>6062</v>
+      </c>
+      <c r="E830" s="34" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F830" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="54" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>COMPRAS</t>
+        </is>
+      </c>
+      <c r="D831" s="26" t="n">
+        <v>78167</v>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>COMPRAS · Zilver SA · ceil desde $78.166,50 · personal · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -60295,15 +60379,27 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B288" s="17" t="n"/>
-      <c r="C288" s="14" t="n"/>
-      <c r="D288" s="27" t="n"/>
+      <c r="B288" s="17" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C288" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Todo Tartas</t>
+        </is>
+      </c>
+      <c r="D288" s="27" t="n">
+        <v>57600</v>
+      </c>
       <c r="E288" s="28" t="n"/>
       <c r="F288" s="15">
-        <f>IF(OR(D273&lt;&gt;"",E273&lt;&gt;""),IF(D273="",0,D273)+IF(E273="",0,E273),"")</f>
-        <v/>
-      </c>
-      <c r="G288" s="14" t="n"/>
+        <f>IF(OR(D288&lt;&gt;"",E288&lt;&gt;""),IF(D288="",0,D288)+IF(E288="",0,E288),"")</f>
+        <v/>
+      </c>
+      <c r="G288" s="14" t="inlineStr">
+        <is>
+          <t>MP · panadería · ex `Todo Tartas`</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="14" t="inlineStr">
@@ -67766,7 +67862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69048,6 +69144,72 @@
       <c r="H51" t="inlineStr">
         <is>
           <t>Reserva automática · − · 17:15 · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="52" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Reserva automática</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="E52" s="26" t="n">
+        <v>500</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="52" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Reserva automática</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
+      <c r="E53" s="26" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
         </is>
       </c>
     </row>
@@ -72771,12 +72933,32 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="n"/>
-      <c r="B44" s="14" t="n"/>
-      <c r="C44" s="14" t="n"/>
-      <c r="D44" s="15" t="n"/>
-      <c r="E44" s="14" t="n"/>
-      <c r="F44" s="14" t="n"/>
+      <c r="A44" s="43" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Pelesson Aldo Oscar</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Transferencia recibida</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>recibida · hoja Transferencias recibidas (no gasto)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="17" t="n"/>

</xml_diff>

<commit_message>
Load Mercado Pago extract for 20 Jul 2026.
Adds Didi/Uber and ARCA AFIP to Gasto Personal Sol; Reserva automática,
Dinero reservado (Chris/Palermo), and Susi withdrawal to MP No Gasto /
Dinero Retirado. Skips 18–19 Jul items already present (Aranda, Roay, Susi).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3641,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F828"/>
+  <dimension ref="A1:F831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25746,6 +25746,90 @@
       <c r="F828" s="34" t="inlineStr">
         <is>
           <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · C.04/06 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="62" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B829" s="34" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C829" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi</t>
+        </is>
+      </c>
+      <c r="D829" s="34" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E829" s="34" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F829" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Didi · Mastercard prepaga · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="62" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B830" s="34" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C830" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber</t>
+        </is>
+      </c>
+      <c r="D830" s="34" t="n">
+        <v>5883</v>
+      </c>
+      <c r="E830" s="34" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F830" s="34" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Uber · Ebanx (=Uber) · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="54" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA</t>
+        </is>
+      </c>
+      <c r="D831" s="26" t="n">
+        <v>67246</v>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>IMPUESTOS · ARCA · ceil desde $67.245,13 · AFIP · gasto personal Sol</t>
         </is>
       </c>
     </row>
@@ -66872,12 +66956,32 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="n"/>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="14" t="n"/>
+      <c r="A33" s="17" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>171746</v>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago · ARS</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Dinero retirado · + · ceil desde $171.745,60</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="n"/>
@@ -67766,7 +67870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69048,6 +69152,196 @@
       <c r="H51" t="inlineStr">
         <is>
           <t>Reserva automática · − · 17:15 · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="52" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Reserva automática</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
+      <c r="E52" s="26" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Reserva automática · − · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="52" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Reserva automática</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="E53" s="26" t="n">
+        <v>500</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Reserva automática · − · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="52" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Dinero reservado</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Chris</t>
+        </is>
+      </c>
+      <c r="E54" s="26" t="n">
+        <v>300000</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Dinero reservado · − · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="52" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Dinero reservado</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="E55" s="26" t="n">
+        <v>593000</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Dinero reservado · − · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="52" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Dinero retirado</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
+      <c r="E56" s="26" t="n">
+        <v>171746</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Dinero retirado · + · ceil desde $171.745,60</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust 17–18 Jul MP extract: PedidosYa net and USD sale.
- PedidosYa comida 17/07: use net after partial refund ($72,042)
- Venta de dólares 18/07: update to settled ceil $1,234,694
- Drop duplicate Susi reserva automática on 17/07
- Susana $147,660 already in Julio LIMPIEZA total (not re-added)

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -59987,7 +59987,7 @@
         </is>
       </c>
       <c r="D276" s="27" t="n">
-        <v>73345</v>
+        <v>72042</v>
       </c>
       <c r="E276" s="28" t="n"/>
       <c r="F276" s="15">
@@ -59996,7 +59996,7 @@
       </c>
       <c r="G276" s="14" t="inlineStr">
         <is>
-          <t>PEDIDOS YA · COMIDA</t>
+          <t>PEDIDOS YA · COMIDA · neto tras devolución parcial $1.302,80 (bruto $73.344,30)</t>
         </is>
       </c>
     </row>
@@ -68083,7 +68083,7 @@
         </is>
       </c>
       <c r="E26" s="26" t="n">
-        <v>1261633</v>
+        <v>1234694</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -68097,7 +68097,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Venta de dólares · + · en proceso · ceil 1261632.32</t>
+          <t>Venta de dólares · + · extracto MP 18/07 · ceil 1.234.693,49 (antes provisional 1.261.632,32)</t>
         </is>
       </c>
     </row>
@@ -68591,7 +68591,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
+          <t>Reserva automática · − · 18:52 · NUNCA almacén</t>
         </is>
       </c>
     </row>
@@ -68976,42 +68976,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E50" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A50" s="52" t="n"/>
+      <c r="E50" s="26" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="52" t="n">
@@ -69513,7 +69479,7 @@
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1261633</v>
+        <v>1234694</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -69524,7 +69490,7 @@
       <c r="I24" s="37" t="n"/>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>En proceso · ceil 1.261.632,32 · también en MP No Gasto</t>
+          <t>Extracto MP 18/07 · ceil 1.234.693,49 · también en MP No Gasto</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Always drop MP dollar sales and reservas; purge existing rows.
Update CIUDAD rules and NORMA so Reserva automática, Dinero reservado,
and Venta de dólares are never loaded (not even in MP No Gasto /
Inversión). Remove matching July rows and regenerate SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -67766,7 +67766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67789,7 +67789,7 @@
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Dinero retirado · Reserva automática / Dinero reservado · Pago de resumen TC · Pago de deuda MP · Inversión (venta/compra USD, bonos, PF). NUNCA van a Almacen Detalle ni suman gastos.</t>
+          <t>Dinero retirado · Pago de resumen TC · Pago de deuda MP · Inversión (bonos/PF/fondos; NO venta/compra USD). NUNCA van a Almacen Detalle ni suman gastos. ELIMINAR siempre (no cargar): Reserva automática, Dinero reservado, Venta de dólares.</t>
         </is>
       </c>
     </row>
@@ -67835,7 +67835,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Reserva automática</t>
+          <t>Reserva automática (ELIMINAR — no cargar)</t>
         </is>
       </c>
       <c r="B7">
@@ -67850,7 +67850,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dinero reservado</t>
+          <t>Dinero reservado (ELIMINAR — no cargar)</t>
         </is>
       </c>
       <c r="B8">
@@ -67932,7 +67932,7 @@
     <row r="16">
       <c r="A16" s="50" t="inlineStr">
         <is>
-          <t>Al analizar extractos MP: si el concepto es Dinero retirado, Reserva automática, Dinero reservado, Pago de resumen / Pago de deuda MP, o Inversión (venta/compra de dólares, bonos, plazos fijos, fondos) → registrar SOLO en esta hoja (y espejo en Dinero Retirado / Inversión / Pago de Tarjetas si aplica). NUNCA en Almacen Detalle, NUNCA como gasto de la hoja 2026.</t>
+          <t>Al analizar extractos MP: Dinero retirado / Pago de resumen / Pago de deuda MP / Inversión (bonos, PF, fondos) → registrar en esta hoja (y espejo Dinero Retirado / Inversión / Pago de Tarjetas). Reserva automática, Dinero reservado y Venta de dólares → ELIMINAR / no catalogar / no cargar. NUNCA en Almacen Detalle, NUNCA como gasto de la hoja 2026.</t>
         </is>
       </c>
     </row>
@@ -68074,20 +68074,20 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Inversión</t>
+          <t>Dinero retirado</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Venta de dólares</t>
+          <t>Gastos</t>
         </is>
       </c>
       <c r="E26" s="26" t="n">
-        <v>1261633</v>
+        <v>845</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ARS</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -68097,7 +68097,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Venta de dólares · + · en proceso · ceil 1261632.32</t>
+          <t>Dinero retirado · + US$844.37 → ceil 845</t>
         </is>
       </c>
     </row>
@@ -68117,15 +68117,15 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Gastos</t>
+          <t>Susi</t>
         </is>
       </c>
       <c r="E27" s="26" t="n">
-        <v>845</v>
+        <v>120000</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>ARS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -68135,7 +68135,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Dinero retirado · + US$844.37 → ceil 845</t>
+          <t>Dinero retirado · +</t>
         </is>
       </c>
     </row>
@@ -68150,16 +68150,16 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dinero reservado</t>
+          <t>Dinero retirado</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Susi</t>
+          <t>AVA</t>
         </is>
       </c>
       <c r="E28" s="26" t="n">
-        <v>5654</v>
+        <v>36813</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -68173,7 +68173,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Dinero reservado · − · ceil 5653.97 · NUNCA almacén</t>
+          <t>Dinero retirado · + · ceil 36812.97</t>
         </is>
       </c>
     </row>
@@ -68188,16 +68188,16 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Reserva automática</t>
+          <t>Dinero retirado</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AVA</t>
+          <t>Susi</t>
         </is>
       </c>
       <c r="E29" s="26" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -68211,7 +68211,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
+          <t>Dinero retirado · +</t>
         </is>
       </c>
     </row>
@@ -68226,16 +68226,16 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Reserva automática</t>
+          <t>Pago de deuda MP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Susi</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="E30" s="26" t="n">
-        <v>3000</v>
+        <v>147660</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -68249,7 +68249,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
+          <t>Pago de deuda · − · pareado con retiro Susi 147660 · NUNCA almacén</t>
         </is>
       </c>
     </row>
@@ -68273,7 +68273,7 @@
         </is>
       </c>
       <c r="E31" s="26" t="n">
-        <v>120000</v>
+        <v>147660</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -68287,7 +68287,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Dinero retirado · +</t>
+          <t>Dinero retirado · + · pareado pago deuda / Susana</t>
         </is>
       </c>
     </row>
@@ -68302,16 +68302,16 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Dinero retirado</t>
+          <t>Pago de deuda MP</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AVA</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="E32" s="26" t="n">
-        <v>36813</v>
+        <v>60000</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -68325,7 +68325,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Dinero retirado · + · ceil 36812.97</t>
+          <t>Pago de deuda · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
@@ -68349,7 +68349,7 @@
         </is>
       </c>
       <c r="E33" s="26" t="n">
-        <v>1</v>
+        <v>60000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -68363,7 +68363,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Dinero retirado · +</t>
+          <t>Dinero retirado · + · pareado pago deuda 60k</t>
         </is>
       </c>
     </row>
@@ -68387,7 +68387,7 @@
         </is>
       </c>
       <c r="E34" s="26" t="n">
-        <v>147660</v>
+        <v>966</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -68401,13 +68401,13 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Pago de deuda · − · pareado con retiro Susi 147660 · NUNCA almacén</t>
+          <t>Pago de deuda · − · ceil 965.70 · NUNCA almacén</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="52" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -68425,7 +68425,7 @@
         </is>
       </c>
       <c r="E35" s="26" t="n">
-        <v>147660</v>
+        <v>30000</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -68439,13 +68439,13 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Dinero retirado · + · pareado pago deuda / Susana</t>
+          <t>Dinero retirado · + · 14:32</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="52" t="n">
-        <v>46221</v>
+        <v>46218</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -68454,36 +68454,36 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Pago de deuda MP</t>
+          <t>Dinero retirado</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
+          <t>Gastos</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="n">
+        <v>500</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="E36" s="26" t="n">
-        <v>60000</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Pago de deuda · − · NUNCA almacén</t>
+          <t>Dinero retirado · + US$500 · pareado transferencia propia Sanes</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="52" t="n">
-        <v>46221</v>
+        <v>46218</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -68492,16 +68492,16 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Dinero retirado</t>
+          <t>Pago de resumen TC</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Susi</t>
+          <t>Tarjeta de crédito</t>
         </is>
       </c>
       <c r="E37" s="26" t="n">
-        <v>60000</v>
+        <v>576242</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -68515,13 +68515,13 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Dinero retirado · + · pareado pago deuda 60k</t>
+          <t>Pago de resumen · − · ceil 576241.18 · NUNCA almacén / no gasto nuevo</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="52" t="n">
-        <v>46221</v>
+        <v>46218</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -68530,527 +68530,113 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Pago de deuda MP</t>
+          <t>Inversión</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
+          <t>Bonos, plazos fijos y más</t>
+        </is>
+      </c>
+      <c r="E38" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="E38" s="26" t="n">
-        <v>966</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Pago de deuda · − · ceil 965.70 · NUNCA almacén</t>
+          <t>Inversión · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E39" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A39" s="52" t="n"/>
+      <c r="E39" s="26" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E40" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A40" s="52" t="n"/>
+      <c r="E40" s="26" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E41" s="26" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · 14:32</t>
-        </is>
-      </c>
+      <c r="A41" s="52" t="n"/>
+      <c r="E41" s="26" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="52" t="n">
-        <v>46219</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Dinero reservado</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E42" s="26" t="n">
-        <v>488004</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Dinero reservado · − · ceil 488003.27 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A42" s="52" t="n"/>
+      <c r="E42" s="26" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Gastos</t>
-        </is>
-      </c>
-      <c r="E43" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + US$500 · pareado transferencia propia Sanes</t>
-        </is>
-      </c>
+      <c r="A43" s="52" t="n"/>
+      <c r="E43" s="26" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E44" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A44" s="52" t="n"/>
+      <c r="E44" s="26" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E45" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A45" s="52" t="n"/>
+      <c r="E45" s="26" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Pago de resumen TC</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Tarjeta de crédito</t>
-        </is>
-      </c>
-      <c r="E46" s="26" t="n">
-        <v>576242</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Pago de resumen · − · ceil 576241.18 · NUNCA almacén / no gasto nuevo</t>
-        </is>
-      </c>
+      <c r="A46" s="52" t="n"/>
+      <c r="E46" s="26" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Inversión</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Bonos, plazos fijos y más</t>
-        </is>
-      </c>
-      <c r="E47" s="26" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Inversión · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A47" s="52" t="n"/>
+      <c r="E47" s="26" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="52" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E48" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A48" s="52" t="n"/>
+      <c r="E48" s="26" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="52" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E49" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A49" s="52" t="n"/>
+      <c r="E49" s="26" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E50" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A50" s="52" t="n"/>
+      <c r="E50" s="26" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E51" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 17:15 · NUNCA almacén</t>
-        </is>
-      </c>
-    </row>
+      <c r="A51" s="52" t="n"/>
+      <c r="E51" s="26" t="n"/>
+    </row>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A16:H18"/>
@@ -69490,7 +69076,7 @@
     </row>
     <row r="24">
       <c r="A24" s="17" t="n">
-        <v>46221</v>
+        <v>46218</v>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
@@ -69499,21 +69085,21 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Bonos/PF</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Rescate</t>
+          <t>Inversión</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Venta de dólares</t>
+          <t>Bonos, plazos fijos y más</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1261633</v>
+        <v>1000000</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -69522,44 +69108,16 @@
       </c>
       <c r="H24" s="17" t="n"/>
       <c r="I24" s="37" t="n"/>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>En proceso · ceil 1.261.632,32 · también en MP No Gasto</t>
-        </is>
-      </c>
+      <c r="J24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>Bonos/PF</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Inversión</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Bonos, plazos fijos y más</t>
-        </is>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="14" t="n"/>
       <c r="H25" s="17" t="n"/>
       <c r="I25" s="37" t="n"/>
       <c r="J25" s="14" t="n"/>

</xml_diff>

<commit_message>
Always drop MP withdrawals; also purge reservas and USD sales.
Extend the ELIMINAR rule to Dinero retirado (deprecate Dinero Retirado
sheet), keep only deuda/resumen/bonos in MP No Gasto, and regenerate SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -721,6 +721,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1555,6 +1556,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
@@ -1743,7 +1745,7 @@
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
         <is>
-          <t>• Dinero retirado: hoja "Dinero Retirado" (no suma al TOTAL de gastos)</t>
+          <t>• Dinero retirado / reservas / venta de dólares: ELIMINAR siempre (no cargar en ninguna hoja)</t>
         </is>
       </c>
     </row>
@@ -66386,7 +66388,7 @@
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Retiros de Mercado Pago (concepto «Dinero retirado» / efectivo). No entra en el TOTAL de gastos de la hoja 2026.</t>
+          <t>HOJA DEPRECADA: «Dinero retirado» se ELIMINA siempre (no catalogar / no cargar). No entra en el TOTAL de gastos de la hoja 2026. Dejar vacía.</t>
         </is>
       </c>
     </row>
@@ -66592,284 +66594,84 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="n">
-        <v>46222</v>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · financió transferencia Matias Aranda</t>
-        </is>
-      </c>
+      <c r="A23" s="17" t="n"/>
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="n">
-        <v>593000</v>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · financió transferencia Analia Roay</t>
-        </is>
-      </c>
+      <c r="A24" s="17" t="n"/>
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>Gastos</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="n">
-        <v>845</v>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · USD</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + US$844.37 → ceil 845</t>
-        </is>
-      </c>
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="14" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="n">
-        <v>120000</v>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F26" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · +</t>
-        </is>
-      </c>
+      <c r="A26" s="17" t="n"/>
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="14" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="n">
-        <v>36813</v>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · ceil 36812.97</t>
-        </is>
-      </c>
+      <c r="A27" s="17" t="n"/>
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="14" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B28" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F28" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · +</t>
-        </is>
-      </c>
+      <c r="A28" s="17" t="n"/>
+      <c r="B28" s="14" t="n"/>
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="14" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="n">
-        <v>147660</v>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · pareado pago deuda / Susana</t>
-        </is>
-      </c>
+      <c r="A29" s="17" t="n"/>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="E30" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · pareado pago deuda 60k</t>
-        </is>
-      </c>
+      <c r="A30" s="17" t="n"/>
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · ARS</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · +</t>
-        </is>
-      </c>
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="inlineStr">
-        <is>
-          <t>Gastos</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="n">
-        <v>500</v>
-      </c>
-      <c r="E32" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago · USD</t>
-        </is>
-      </c>
-      <c r="F32" s="14" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + US$500 · pareado Sanes propia</t>
-        </is>
-      </c>
+      <c r="A32" s="17" t="n"/>
+      <c r="B32" s="14" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="17" t="n"/>
@@ -67766,7 +67568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67789,7 +67591,7 @@
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Dinero retirado · Reserva automática / Dinero reservado · Pago de resumen TC · Pago de deuda MP · Inversión (venta/compra USD, bonos, PF). NUNCA van a Almacen Detalle ni suman gastos.</t>
+          <t>Pago de resumen TC · Pago de deuda MP · Inversión (bonos/PF/fondos; NO venta/compra USD). NUNCA van a Almacen Detalle ni suman gastos. ELIMINAR siempre (no cargar): Dinero retirado, Reserva automática, Dinero reservado, Venta de dólares.</t>
         </is>
       </c>
     </row>
@@ -67820,7 +67622,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dinero retirado</t>
+          <t>Dinero retirado (ELIMINAR — no cargar)</t>
         </is>
       </c>
       <c r="B6">
@@ -67835,7 +67637,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Reserva automática</t>
+          <t>Reserva automática (ELIMINAR — no cargar)</t>
         </is>
       </c>
       <c r="B7">
@@ -67850,7 +67652,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dinero reservado</t>
+          <t>Dinero reservado (ELIMINAR — no cargar)</t>
         </is>
       </c>
       <c r="B8">
@@ -67932,7 +67734,7 @@
     <row r="16">
       <c r="A16" s="50" t="inlineStr">
         <is>
-          <t>Al analizar extractos MP: si el concepto es Dinero retirado, Reserva automática, Dinero reservado, Pago de resumen / Pago de deuda MP, o Inversión (venta/compra de dólares, bonos, plazos fijos, fondos) → registrar SOLO en esta hoja (y espejo en Dinero Retirado / Inversión / Pago de Tarjetas si aplica). NUNCA en Almacen Detalle, NUNCA como gasto de la hoja 2026.</t>
+          <t>Al analizar extractos MP: Pago de resumen / Pago de deuda MP / Inversión (bonos, PF, fondos) → registrar en esta hoja (y espejo Inversión / Pago de Tarjetas). Dinero retirado, Reserva automática, Dinero reservado y Venta de dólares → ELIMINAR / no catalogar / no cargar. NUNCA en Almacen Detalle, NUNCA como gasto de la hoja 2026.</t>
         </is>
       </c>
     </row>
@@ -67989,7 +67791,7 @@
     </row>
     <row r="24">
       <c r="A24" s="52" t="n">
-        <v>46222</v>
+        <v>46221</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -67998,16 +67800,16 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dinero retirado</t>
+          <t>Pago de deuda MP</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Susi</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="E24" s="26" t="n">
-        <v>15000</v>
+        <v>147660</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -68021,7 +67823,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Dinero retirado · + · financió transferencia Matias Aranda</t>
+          <t>Pago de deuda · − · pareado con retiro Susi 147660 · NUNCA almacén</t>
         </is>
       </c>
     </row>
@@ -68036,16 +67838,16 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dinero retirado</t>
+          <t>Pago de deuda MP</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="E25" s="26" t="n">
-        <v>593000</v>
+        <v>60000</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -68059,7 +67861,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Dinero retirado · + · financió transferencia Analia Roay</t>
+          <t>Pago de deuda · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
@@ -68074,16 +67876,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Inversión</t>
+          <t>Pago de deuda MP</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Venta de dólares</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="E26" s="26" t="n">
-        <v>1261633</v>
+        <v>966</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -68097,13 +67899,13 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Venta de dólares · + · en proceso · ceil 1261632.32</t>
+          <t>Pago de deuda · − · ceil 965.70 · NUNCA almacén</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="52" t="n">
-        <v>46221</v>
+        <v>46218</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -68112,20 +67914,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dinero retirado</t>
+          <t>Pago de resumen TC</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Gastos</t>
+          <t>Tarjeta de crédito</t>
         </is>
       </c>
       <c r="E27" s="26" t="n">
-        <v>845</v>
+        <v>576242</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>ARS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -68135,13 +67937,13 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Dinero retirado · + US$844.37 → ceil 845</t>
+          <t>Pago de resumen · − · ceil 576241.18 · NUNCA almacén / no gasto nuevo</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="52" t="n">
-        <v>46221</v>
+        <v>46218</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -68150,16 +67952,16 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dinero reservado</t>
+          <t>Inversión</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Susi</t>
+          <t>Bonos, plazos fijos y más</t>
         </is>
       </c>
       <c r="E28" s="26" t="n">
-        <v>5654</v>
+        <v>1000000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -68173,884 +67975,130 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Dinero reservado · − · ceil 5653.97 · NUNCA almacén</t>
+          <t>Inversión · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E29" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A29" s="52" t="n"/>
+      <c r="E29" s="26" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E30" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A30" s="52" t="n"/>
+      <c r="E30" s="26" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E31" s="26" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Dinero retirado · +</t>
-        </is>
-      </c>
+      <c r="A31" s="52" t="n"/>
+      <c r="E31" s="26" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E32" s="26" t="n">
-        <v>36813</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · ceil 36812.97</t>
-        </is>
-      </c>
+      <c r="A32" s="52" t="n"/>
+      <c r="E32" s="26" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E33" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Dinero retirado · +</t>
-        </is>
-      </c>
+      <c r="A33" s="52" t="n"/>
+      <c r="E33" s="26" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Pago de deuda MP</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="E34" s="26" t="n">
-        <v>147660</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Pago de deuda · − · pareado con retiro Susi 147660 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A34" s="52" t="n"/>
+      <c r="E34" s="26" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E35" s="26" t="n">
-        <v>147660</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · pareado pago deuda / Susana</t>
-        </is>
-      </c>
+      <c r="A35" s="52" t="n"/>
+      <c r="E35" s="26" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Pago de deuda MP</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="E36" s="26" t="n">
-        <v>60000</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Pago de deuda · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A36" s="52" t="n"/>
+      <c r="E36" s="26" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E37" s="26" t="n">
-        <v>60000</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · pareado pago deuda 60k</t>
-        </is>
-      </c>
+      <c r="A37" s="52" t="n"/>
+      <c r="E37" s="26" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="52" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Pago de deuda MP</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="E38" s="26" t="n">
-        <v>966</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Pago de deuda · − · ceil 965.70 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A38" s="52" t="n"/>
+      <c r="E38" s="26" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E39" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A39" s="52" t="n"/>
+      <c r="E39" s="26" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E40" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A40" s="52" t="n"/>
+      <c r="E40" s="26" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E41" s="26" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + · 14:32</t>
-        </is>
-      </c>
+      <c r="A41" s="52" t="n"/>
+      <c r="E41" s="26" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="52" t="n">
-        <v>46219</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Dinero reservado</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E42" s="26" t="n">
-        <v>488004</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Dinero reservado · − · ceil 488003.27 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A42" s="52" t="n"/>
+      <c r="E42" s="26" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Dinero retirado</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Gastos</t>
-        </is>
-      </c>
-      <c r="E43" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Dinero retirado · + US$500 · pareado transferencia propia Sanes</t>
-        </is>
-      </c>
+      <c r="A43" s="52" t="n"/>
+      <c r="E43" s="26" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E44" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A44" s="52" t="n"/>
+      <c r="E44" s="26" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E45" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A45" s="52" t="n"/>
+      <c r="E45" s="26" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Pago de resumen TC</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Tarjeta de crédito</t>
-        </is>
-      </c>
-      <c r="E46" s="26" t="n">
-        <v>576242</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Pago de resumen · − · ceil 576241.18 · NUNCA almacén / no gasto nuevo</t>
-        </is>
-      </c>
+      <c r="A46" s="52" t="n"/>
+      <c r="E46" s="26" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Inversión</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Bonos, plazos fijos y más</t>
-        </is>
-      </c>
-      <c r="E47" s="26" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Inversión · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A47" s="52" t="n"/>
+      <c r="E47" s="26" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="52" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E48" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A48" s="52" t="n"/>
+      <c r="E48" s="26" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="52" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E49" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A49" s="52" t="n"/>
+      <c r="E49" s="26" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E50" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
-        </is>
-      </c>
+      <c r="A50" s="52" t="n"/>
+      <c r="E50" s="26" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E51" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 17:15 · NUNCA almacén</t>
-        </is>
-      </c>
-    </row>
+      <c r="A51" s="52" t="n"/>
+      <c r="E51" s="26" t="n"/>
+    </row>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A16:H18"/>
@@ -69490,7 +68538,7 @@
     </row>
     <row r="24">
       <c r="A24" s="17" t="n">
-        <v>46221</v>
+        <v>46218</v>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
@@ -69499,21 +68547,21 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Bonos/PF</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Rescate</t>
+          <t>Inversión</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Venta de dólares</t>
+          <t>Bonos, plazos fijos y más</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1261633</v>
+        <v>1000000</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -69522,44 +68570,16 @@
       </c>
       <c r="H24" s="17" t="n"/>
       <c r="I24" s="37" t="n"/>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>En proceso · ceil 1.261.632,32 · también en MP No Gasto</t>
-        </is>
-      </c>
+      <c r="J24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>Bonos/PF</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Inversión</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Bonos, plazos fijos y más</t>
-        </is>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="14" t="n"/>
       <c r="H25" s="17" t="n"/>
       <c r="I25" s="37" t="n"/>
       <c r="J25" s="14" t="n"/>

</xml_diff>

<commit_message>
Add Botas CH import duty VEP to personal Vestimenta.
Registers QR VEP 1657133544 for $79,817 (ceil of $79,816.50) on
2026-07-24 under Gasto Personal Sol / VESTIMENTA and regenerates SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3641,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F828"/>
+  <dimension ref="A1:F829"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25746,6 +25746,34 @@
       <c r="F828" s="34" t="inlineStr">
         <is>
           <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · C.04/06 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="54" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>VESTIMENTA</t>
+        </is>
+      </c>
+      <c r="D829" s="26" t="n">
+        <v>79817</v>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>QR</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>VESTIMENTA · Botas CH · derecho de importación · VEP 1657133544 · CUIT 27-29039079-1 · ceil $79.816,50 · gasto personal Sol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Load Telecentro Visa *3200 charge as CIUDAD August TV.
Sets Agosto Telecentro to $31,999 from the 24/07/2026 BBVA Visa
notice (Julio already had $31,999 from the 30/06 debit).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -886,7 +886,7 @@
         <v>31999</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>50000</v>
+        <v>31999</v>
       </c>
       <c r="L6" s="9" t="n">
         <v>50000</v>
@@ -64106,7 +64106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65218,7 +65218,7 @@
     </row>
     <row r="35">
       <c r="A35" s="17" t="n">
-        <v>46235</v>
+        <v>46227</v>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
@@ -65227,18 +65227,26 @@
       </c>
       <c r="C35" s="14" t="inlineStr">
         <is>
-          <t>Telecentro CIUDAD — servicio mensual 08/2026</t>
+          <t>Telecentro CIUDAD — cobro Visa *3200 24/07/2026 (agosto)</t>
         </is>
       </c>
       <c r="D35" s="15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E35" s="14" t="inlineStr"/>
-      <c r="F35" s="18" t="inlineStr"/>
-      <c r="G35" s="18" t="inlineStr"/>
+        <v>31999</v>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>BBVA Visa *3200</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
+      <c r="G35" s="18" t="n"/>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>Recurrente $50.000/mes hasta nuevo aviso</t>
+          <t>Aviso tarjeta Visa *3200 · ARS 31.999,00 · período agosto</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
@@ -66350,6 +66358,44 @@
       <c r="F73" s="18" t="inlineStr">
         <is>
           <t>3491192</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="53" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>Telecentro</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Telecentro CIUDAD — BBVA Visa *3200 24/07/2026 (agosto)</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="n">
+        <v>31999</v>
+      </c>
+      <c r="E74" s="14" t="inlineStr">
+        <is>
+          <t>BBVA Visa *3200</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>3491192</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>TELECENTRO SA · aviso 24/07/2026</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Agosto</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Avoid duplicate Telecentro Detalle row for the August charge.
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -64106,7 +64106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66362,42 +66362,12 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="53" t="n">
-        <v>46227</v>
-      </c>
-      <c r="B74" s="14" t="inlineStr">
-        <is>
-          <t>Telecentro</t>
-        </is>
-      </c>
-      <c r="C74" s="14" t="inlineStr">
-        <is>
-          <t>Telecentro CIUDAD — BBVA Visa *3200 24/07/2026 (agosto)</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="n">
-        <v>31999</v>
-      </c>
-      <c r="E74" s="14" t="inlineStr">
-        <is>
-          <t>BBVA Visa *3200</t>
-        </is>
-      </c>
-      <c r="F74" s="18" t="inlineStr">
-        <is>
-          <t>3491192</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>TELECENTRO SA · aviso 24/07/2026</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>Agosto</t>
-        </is>
-      </c>
+      <c r="A74" s="53" t="n"/>
+      <c r="B74" s="14" t="n"/>
+      <c r="C74" s="14" t="n"/>
+      <c r="D74" s="15" t="n"/>
+      <c r="E74" s="14" t="n"/>
+      <c r="F74" s="18" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:I51"/>

</xml_diff>

<commit_message>
Add Cabify Visa *3200 ride to GPS transporte ($7,478).
Registers the 24/07/2026 BBVA Visa notice for Cabify2630LsoIZ6dR
(ceil from $7,477.77) under Gasto Personal Sol and regenerates SOL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3641,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F828"/>
+  <dimension ref="A1:F829"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25746,6 +25746,34 @@
       <c r="F828" s="34" t="inlineStr">
         <is>
           <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · C.04/06 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="54" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>TRANSPORTE · Cabify</t>
+        </is>
+      </c>
+      <c r="D829" t="n">
+        <v>7478</v>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>BBVA Visa *3200</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>Cabify · BBVA Visa *3200 · Cabify2630LsoIZ6dR · ceil $7.477,77 · gasto personal Sol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add August CIUDAD Edenor invoice
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -987,7 +987,9 @@
       <c r="J8" s="9" t="n">
         <v>128877</v>
       </c>
-      <c r="K8" s="9" t="n"/>
+      <c r="K8" s="9" t="n">
+        <v>183272</v>
+      </c>
       <c r="L8" s="9" t="n"/>
       <c r="M8" s="9" t="n"/>
       <c r="N8" s="9" t="n"/>
@@ -64106,7 +64108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66350,6 +66352,44 @@
       <c r="F73" s="18" t="inlineStr">
         <is>
           <t>3491192</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="43" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Edenor — CIUDAD DE LA PAZ 1132 · cuenta 008917502309</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="n">
+        <v>183272</v>
+      </c>
+      <c r="E74" s="14" t="inlineStr">
+        <is>
+          <t>Factura Edenor · pago pendiente</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>008917502309</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Vence 12/08/2026 · original $183.271,35 · fecha de emisión no informada</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Agosto</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update July Susana cleaning receipt
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1073,7 +1073,7 @@
         <v>876981</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>400640</v>
+        <v>517380</v>
       </c>
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
@@ -64108,7 +64108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66390,6 +66390,40 @@
       <c r="I74" t="inlineStr">
         <is>
           <t>Agosto</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="43" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>Limpieza Susana — Julio 2026</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="n">
+        <v>517380</v>
+      </c>
+      <c r="E75" s="14" t="inlineStr">
+        <is>
+          <t>Pagado · medio no informado</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="n"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Total Recibo Julio 2026</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Julio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct July Susana cleaning total
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1073,7 +1073,7 @@
         <v>876981</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>517380</v>
+        <v>629380</v>
       </c>
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
@@ -66408,7 +66408,7 @@
         </is>
       </c>
       <c r="D75" s="15" t="n">
-        <v>517380</v>
+        <v>629380</v>
       </c>
       <c r="E75" s="14" t="inlineStr">
         <is>
@@ -66418,7 +66418,7 @@
       <c r="F75" s="18" t="n"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Total Recibo Julio 2026</t>
+          <t>Total Recibo Julio 2026 · importe corregido</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">

</xml_diff>

<commit_message>
Reconcile June and July CIUDAD expenses
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -835,9 +835,11 @@
         <v>246150</v>
       </c>
       <c r="I5" s="5" t="n">
+        <v>246150</v>
+      </c>
+      <c r="J5" s="5" t="n">
         <v>273500</v>
       </c>
-      <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
@@ -1302,16 +1304,32 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="n"/>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="19" t="n"/>
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>Farmacia</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
+      <c r="I15" s="5" t="n">
+        <v>85034</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>218500</v>
+      </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="5" t="n"/>
       <c r="M15" s="5" t="n"/>
@@ -1389,12 +1407,29 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AROMATIZANTES</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Saphirus — Aromatizantes</t>
+        </is>
+      </c>
       <c r="D18" s="26" t="n"/>
       <c r="E18" s="26" t="n"/>
       <c r="F18" s="26" t="n"/>
       <c r="G18" s="26" t="n"/>
       <c r="H18" s="26" t="n"/>
-      <c r="I18" s="26" t="n"/>
+      <c r="I18" s="26" t="n">
+        <v>79900</v>
+      </c>
       <c r="J18" s="26" t="n"/>
       <c r="P18" s="26">
         <f>SUM(D18:O18)</f>
@@ -1434,6 +1469,10 @@
       <c r="E20" t="n">
         <v>5990</v>
       </c>
+      <c r="P20">
+        <f>SUM(D20:O20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -1492,7 +1531,7 @@
         <v/>
       </c>
       <c r="P21" s="7">
-        <f>SUM(P5:P19)</f>
+        <f>SUM(P5:P20)</f>
         <v/>
       </c>
     </row>
@@ -7949,32 +7988,8 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="54" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>HOGAR</t>
-        </is>
-      </c>
-      <c r="D184" s="26" t="n">
-        <v>79900</v>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>¿hogar? · gasto personal Sol (ex-PENDIENTE)</t>
-        </is>
-      </c>
+      <c r="A184" s="54" t="n"/>
+      <c r="D184" s="26" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="54" t="n">
@@ -22949,32 +22964,7 @@
       </c>
     </row>
     <row r="728">
-      <c r="A728" s="54" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B728" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C728" t="inlineStr">
-        <is>
-          <t>SUSCRIPCIONES · IA</t>
-        </is>
-      </c>
-      <c r="D728" t="n">
-        <v>16403</v>
-      </c>
-      <c r="E728" t="inlineStr">
-        <is>
-          <t>TC Mercado Pago · USD</t>
-        </is>
-      </c>
-      <c r="F728" t="inlineStr">
-        <is>
-          <t>SUSCRIPCIONES · IA · Vercel Domains · USD 11.25 × TC MEP 1458.0 · gasto personal Sol</t>
-        </is>
-      </c>
+      <c r="A728" s="54" t="n"/>
     </row>
     <row r="729">
       <c r="A729" s="54" t="n">
@@ -23932,32 +23922,7 @@
       </c>
     </row>
     <row r="764">
-      <c r="A764" s="54" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B764" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C764" t="inlineStr">
-        <is>
-          <t>FARMACIA SALUD</t>
-        </is>
-      </c>
-      <c r="D764" t="n">
-        <v>218500</v>
-      </c>
-      <c r="E764" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="F764" t="inlineStr">
-        <is>
-          <t>FARMACIA SALUD · Farmacia Maure · resumen MP cuenta</t>
-        </is>
-      </c>
+      <c r="A764" s="54" t="n"/>
     </row>
     <row r="765">
       <c r="A765" s="54" t="n">
@@ -59530,27 +59495,15 @@
           <t>Junio</t>
         </is>
       </c>
-      <c r="B252" s="53" t="n">
-        <v>46185</v>
-      </c>
-      <c r="C252" s="14" t="inlineStr">
-        <is>
-          <t>FARMACIA · Farmacity</t>
-        </is>
-      </c>
-      <c r="D252" s="27" t="n">
-        <v>85034</v>
-      </c>
+      <c r="B252" s="53" t="n"/>
+      <c r="C252" s="14" t="n"/>
+      <c r="D252" s="27" t="n"/>
       <c r="E252" s="28" t="n"/>
       <c r="F252" s="15">
         <f>IF(OR(D252&lt;&gt;"",E252&lt;&gt;""),IF(D252="",0,D252)+IF(E252="",0,E252),"")</f>
         <v/>
       </c>
-      <c r="G252" s="14" t="inlineStr">
-        <is>
-          <t>FARMACIA · Farmacity · TC Mercado Pago · compra 2026-05-29 · cobro resumen 2026-06-12 · ex CASA/FARMACIA matriz</t>
-        </is>
-      </c>
+      <c r="G252" s="14" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="14" t="inlineStr">
@@ -64108,7 +64061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66422,6 +66375,108 @@
         </is>
       </c>
       <c r="I75" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="43" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>Farmacity</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="n">
+        <v>85034</v>
+      </c>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>TC Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="n"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacity · compra 29/05 · cobro junio</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="43" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>AROMATIZANTES</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>CASA — Aromatizantes Saphirus</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="n">
+        <v>79900</v>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="n"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>CASA · AROMATIZANTES · Saphirus · CIUDAD</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="43" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>FARMACIA</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>Farmacia Maure</t>
+        </is>
+      </c>
+      <c r="D78" s="15" t="n">
+        <v>218500</v>
+      </c>
+      <c r="E78" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="n"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacia Maure · CIUDAD</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>

</xml_diff>

<commit_message>
Set MP bank investment stock to 13M @ 21% from 29 Jul.
Replace prior Bonos/PF 1M as current banco MP position with Christian 10M + Sol 3M, mirror in MP No Gasto and SOL master, and keep historical USD sale separate from stock.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -36,7 +36,7 @@
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -114,8 +114,12 @@
       <color rgb="0017365D"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -162,8 +166,18 @@
         <fgColor rgb="0017365D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -243,11 +257,17 @@
         <color rgb="00D9E1F2"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -321,6 +341,27 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="10" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="11" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="11" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="11" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="7" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -67766,7 +67807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67988,1066 +68029,1104 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="52" t="n">
+      <c r="A24" s="63" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B24" s="64" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C24" s="64" t="inlineStr">
+        <is>
+          <t>Inversión</t>
+        </is>
+      </c>
+      <c r="D24" s="64" t="inlineStr">
+        <is>
+          <t>Banco MP · Christian</t>
+        </is>
+      </c>
+      <c r="E24" s="65" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="F24" s="64" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G24" s="64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H24" s="64" t="inlineStr">
+        <is>
+          <t>Inversión · − · único stock banco MP · Christian · 21% anual · instruido Sol 2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="63" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B25" s="64" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C25" s="64" t="inlineStr">
+        <is>
+          <t>Inversión</t>
+        </is>
+      </c>
+      <c r="D25" s="64" t="inlineStr">
+        <is>
+          <t>Banco MP · Sol</t>
+        </is>
+      </c>
+      <c r="E25" s="65" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="F25" s="64" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G25" s="64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H25" s="64" t="inlineStr">
+        <is>
+          <t>Inversión · − · único stock banco MP · Sol · 21% anual · instruido Sol 2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="63" t="n">
         <v>46222</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B26" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D26" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E24" s="26" t="n">
+      <c r="E26" s="65" t="n">
         <v>15000</v>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F26" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G26" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H26" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + · financió transferencia Matias Aranda</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="52" t="n">
+    <row r="27">
+      <c r="A27" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D27" s="64" t="inlineStr">
         <is>
           <t>Palermo</t>
         </is>
       </c>
-      <c r="E25" s="26" t="n">
+      <c r="E27" s="65" t="n">
         <v>593000</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F27" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G27" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H27" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + · financió transferencia Analia Roay</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="52" t="n">
+    <row r="28">
+      <c r="A28" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C28" s="64" t="inlineStr">
         <is>
           <t>Inversión</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D28" s="64" t="inlineStr">
         <is>
           <t>Venta de dólares</t>
         </is>
       </c>
-      <c r="E26" s="26" t="n">
+      <c r="E28" s="65" t="n">
         <v>1261633</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F28" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G28" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H28" s="64" t="inlineStr">
         <is>
           <t>Venta de dólares · + · en proceso · ceil 1261632.32</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="52" t="n">
+    <row r="29">
+      <c r="A29" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C29" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D29" s="64" t="inlineStr">
         <is>
           <t>Gastos</t>
         </is>
       </c>
-      <c r="E27" s="26" t="n">
+      <c r="E29" s="65" t="n">
         <v>845</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F29" s="64" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G29" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H29" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + US$844.37 → ceil 845</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="52" t="n">
+    <row r="30">
+      <c r="A30" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" s="64" t="inlineStr">
         <is>
           <t>Dinero reservado</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D30" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E28" s="26" t="n">
+      <c r="E30" s="65" t="n">
         <v>5654</v>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F30" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G30" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H30" s="64" t="inlineStr">
         <is>
           <t>Dinero reservado · − · ceil 5653.97 · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="52" t="n">
+    <row r="31">
+      <c r="A31" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B31" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" s="64" t="inlineStr">
         <is>
           <t>Reserva automática</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D31" s="64" t="inlineStr">
         <is>
           <t>AVA</t>
         </is>
       </c>
-      <c r="E29" s="26" t="n">
+      <c r="E31" s="65" t="n">
         <v>500</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F31" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G31" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H31" s="64" t="inlineStr">
         <is>
           <t>Reserva automática · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="52" t="n">
+    <row r="32">
+      <c r="A32" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" s="64" t="inlineStr">
         <is>
           <t>Reserva automática</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D32" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E30" s="26" t="n">
+      <c r="E32" s="65" t="n">
         <v>3000</v>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F32" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G32" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H32" s="64" t="inlineStr">
         <is>
           <t>Reserva automática · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="52" t="n">
+    <row r="33">
+      <c r="A33" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B33" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D33" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E31" s="26" t="n">
+      <c r="E33" s="65" t="n">
         <v>120000</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F33" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G33" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H33" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · +</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="52" t="n">
+    <row r="34">
+      <c r="A34" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B34" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C34" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D34" s="64" t="inlineStr">
         <is>
           <t>AVA</t>
         </is>
       </c>
-      <c r="E32" s="26" t="n">
+      <c r="E34" s="65" t="n">
         <v>36813</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F34" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G34" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H34" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + · ceil 36812.97</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="52" t="n">
+    <row r="35">
+      <c r="A35" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B35" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C35" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D35" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E33" s="26" t="n">
+      <c r="E35" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F35" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G35" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H35" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · +</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="52" t="n">
+    <row r="36">
+      <c r="A36" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B36" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" s="64" t="inlineStr">
         <is>
           <t>Pago de deuda MP</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D36" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="E34" s="26" t="n">
+      <c r="E36" s="65" t="n">
         <v>147660</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F36" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G36" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H36" s="64" t="inlineStr">
         <is>
           <t>Pago de deuda · − · pareado con retiro Susi 147660 · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="52" t="n">
+    <row r="37">
+      <c r="A37" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B37" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C37" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D37" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E35" s="26" t="n">
+      <c r="E37" s="65" t="n">
         <v>147660</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F37" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G37" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H37" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + · pareado pago deuda / Susana</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="52" t="n">
+    <row r="38">
+      <c r="A38" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B38" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C38" s="64" t="inlineStr">
         <is>
           <t>Pago de deuda MP</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D38" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="E36" s="26" t="n">
+      <c r="E38" s="65" t="n">
         <v>60000</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F38" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G38" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H38" s="64" t="inlineStr">
         <is>
           <t>Pago de deuda · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="52" t="n">
+    <row r="39">
+      <c r="A39" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B39" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E37" s="26" t="n">
+      <c r="E39" s="65" t="n">
         <v>60000</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F39" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G39" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H39" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + · pareado pago deuda 60k</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="52" t="n">
+    <row r="40">
+      <c r="A40" s="63" t="n">
         <v>46221</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B40" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C40" s="64" t="inlineStr">
         <is>
           <t>Pago de deuda MP</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D40" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="E38" s="26" t="n">
+      <c r="E40" s="65" t="n">
         <v>966</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F40" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G40" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H40" s="64" t="inlineStr">
         <is>
           <t>Pago de deuda · − · ceil 965.70 · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="52" t="n">
+    <row r="41">
+      <c r="A41" s="63" t="n">
         <v>46220</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B41" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" s="64" t="inlineStr">
         <is>
           <t>Reserva automática</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D41" s="64" t="inlineStr">
         <is>
           <t>AVA</t>
         </is>
       </c>
-      <c r="E39" s="26" t="n">
+      <c r="E41" s="65" t="n">
         <v>500</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F41" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G41" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H41" s="64" t="inlineStr">
         <is>
           <t>Reserva automática · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="52" t="n">
+    <row r="42">
+      <c r="A42" s="63" t="n">
         <v>46220</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" s="64" t="inlineStr">
         <is>
           <t>Reserva automática</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D42" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E40" s="26" t="n">
+      <c r="E42" s="65" t="n">
         <v>3000</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F42" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G42" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H42" s="64" t="inlineStr">
         <is>
           <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="52" t="n">
+    <row r="43">
+      <c r="A43" s="63" t="n">
         <v>46220</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B43" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D43" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E41" s="26" t="n">
+      <c r="E43" s="65" t="n">
         <v>30000</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F43" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G43" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H43" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + · 14:32</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="52" t="n">
+    <row r="44">
+      <c r="A44" s="63" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B44" s="64" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C44" s="64" t="inlineStr">
+        <is>
+          <t>Reserva automática</t>
+        </is>
+      </c>
+      <c r="D44" s="64" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
+      <c r="E44" s="65" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F44" s="64" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G44" s="64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H44" s="64" t="inlineStr">
+        <is>
+          <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="63" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B45" s="64" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C45" s="64" t="inlineStr">
+        <is>
+          <t>Reserva automática</t>
+        </is>
+      </c>
+      <c r="D45" s="64" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="E45" s="65" t="n">
+        <v>500</v>
+      </c>
+      <c r="F45" s="64" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="G45" s="64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H45" s="64" t="inlineStr">
+        <is>
+          <t>Reserva automática · − · 17:15 · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="63" t="n">
         <v>46219</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B46" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C46" s="64" t="inlineStr">
         <is>
           <t>Dinero reservado</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D46" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E42" s="26" t="n">
+      <c r="E46" s="65" t="n">
         <v>488004</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F46" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G46" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H46" s="64" t="inlineStr">
         <is>
           <t>Dinero reservado · − · ceil 488003.27 · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="52" t="n">
+    <row r="47">
+      <c r="A47" s="63" t="n">
         <v>46218</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B47" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C47" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D47" s="64" t="inlineStr">
         <is>
           <t>Gastos</t>
         </is>
       </c>
-      <c r="E43" s="26" t="n">
+      <c r="E47" s="65" t="n">
         <v>500</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F47" s="64" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G47" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H47" s="64" t="inlineStr">
         <is>
           <t>Dinero retirado · + US$500 · pareado transferencia propia Sanes</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="52" t="n">
+    <row r="48">
+      <c r="A48" s="63" t="n">
         <v>46218</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B48" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C48" s="64" t="inlineStr">
         <is>
           <t>Reserva automática</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D48" s="64" t="inlineStr">
         <is>
           <t>AVA</t>
         </is>
       </c>
-      <c r="E44" s="26" t="n">
+      <c r="E48" s="65" t="n">
         <v>500</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F48" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G48" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H48" s="64" t="inlineStr">
         <is>
           <t>Reserva automática · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="52" t="n">
+    <row r="49">
+      <c r="A49" s="63" t="n">
         <v>46218</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B49" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C49" s="64" t="inlineStr">
         <is>
           <t>Reserva automática</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D49" s="64" t="inlineStr">
         <is>
           <t>Susi</t>
         </is>
       </c>
-      <c r="E45" s="26" t="n">
+      <c r="E49" s="65" t="n">
         <v>3000</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F49" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G49" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H49" s="64" t="inlineStr">
         <is>
           <t>Reserva automática · − · NUNCA almacén</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="52" t="n">
+    <row r="50">
+      <c r="A50" s="63" t="n">
         <v>46218</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B50" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C50" s="64" t="inlineStr">
         <is>
           <t>Pago de resumen TC</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D50" s="64" t="inlineStr">
         <is>
           <t>Tarjeta de crédito</t>
         </is>
       </c>
-      <c r="E46" s="26" t="n">
+      <c r="E50" s="65" t="n">
         <v>576242</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F50" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G50" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H50" s="64" t="inlineStr">
         <is>
           <t>Pago de resumen · − · ceil 576241.18 · NUNCA almacén / no gasto nuevo</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B47" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="63" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B51" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Inversión</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Bonos, plazos fijos y más</t>
-        </is>
-      </c>
-      <c r="E47" s="26" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="F47" t="inlineStr">
+      <c r="C51" s="64" t="inlineStr">
+        <is>
+          <t>Reserva automática</t>
+        </is>
+      </c>
+      <c r="D51" s="64" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="E51" s="65" t="n">
+        <v>500</v>
+      </c>
+      <c r="F51" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G51" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Inversión · − · NUNCA almacén</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="52" t="n">
+      <c r="H51" s="64" t="inlineStr">
+        <is>
+          <t>Reserva automática · − · NUNCA almacén</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="63" t="n">
         <v>46217</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B52" s="64" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C52" s="64" t="inlineStr">
         <is>
           <t>Reserva automática</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E48" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F48" t="inlineStr">
+      <c r="D52" s="64" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
+      <c r="E52" s="65" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F52" s="64" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G52" s="64" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H52" s="64" t="inlineStr">
         <is>
           <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="52" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E49" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · NUNCA almacén</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Susi</t>
-        </is>
-      </c>
-      <c r="E50" s="26" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 18:17 · NUNCA almacén</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="52" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Reserva automática</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>AVA</t>
-        </is>
-      </c>
-      <c r="E51" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Reserva automática · − · 17:15 · NUNCA almacén</t>
         </is>
       </c>
     </row>
@@ -69092,7 +69171,7 @@
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Bonos, plazos fijos, fondos y otros movimientos de inversión. No suma al TOTAL de gastos de la hoja 2026.</t>
+          <t>Bonos, plazos fijos, fondos y otros movimientos de inversión. No suma al TOTAL de gastos de la hoja 2026. Stock banco MP vigente = único valor instruido por Sol (no sumar inversiones previas Bonos/PF).</t>
         </is>
       </c>
     </row>
@@ -69137,15 +69216,15 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A6,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A6,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A6,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A6,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D6" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A6,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A6,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E6" s="15">
@@ -69160,15 +69239,15 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A7,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A7,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A7,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A7,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D7" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A7,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A7,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E7" s="15">
@@ -69183,15 +69262,15 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A8,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A8,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A8,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A8,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D8" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A8,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A8,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E8" s="15">
@@ -69206,15 +69285,15 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A9,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A9,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C9" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A9,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A9,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D9" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A9,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A9,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E9" s="15">
@@ -69229,15 +69308,15 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A10,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A10,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C10" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A10,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A10,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D10" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A10,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A10,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E10" s="15">
@@ -69252,15 +69331,15 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A11,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A11,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C11" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A11,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A11,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D11" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A11,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A11,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E11" s="15">
@@ -69275,15 +69354,15 @@
         </is>
       </c>
       <c r="B12" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A12,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A12,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C12" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A12,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A12,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D12" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A12,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A12,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E12" s="15">
@@ -69298,15 +69377,15 @@
         </is>
       </c>
       <c r="B13" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A13,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A13,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C13" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A13,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A13,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D13" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A13,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A13,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E13" s="15">
@@ -69321,15 +69400,15 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A14,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A14,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C14" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A14,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A14,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D14" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A14,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A14,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E14" s="15">
@@ -69344,15 +69423,15 @@
         </is>
       </c>
       <c r="B15" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A15,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A15,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C15" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A15,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A15,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D15" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A15,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A15,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E15" s="15">
@@ -69367,15 +69446,15 @@
         </is>
       </c>
       <c r="B16" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A16,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A16,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C16" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A16,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A16,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D16" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A16,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A16,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E16" s="15">
@@ -69390,15 +69469,15 @@
         </is>
       </c>
       <c r="B17" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A17,$D$24:$D$500,"Inversión")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A17,$D$27:$D$500,"Inversión")</f>
         <v/>
       </c>
       <c r="C17" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A17,$D$24:$D$500,"Rescate")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A17,$D$27:$D$500,"Rescate")</f>
         <v/>
       </c>
       <c r="D17" s="15">
-        <f>SUMIFS($F$24:$F$500,$B$24:$B$500,A17,$D$24:$D$500,"Rendimiento")</f>
+        <f>SUMIFS($F$27:$F$500,$B$27:$B$500,A17,$D$27:$D$500,"Rendimiento")</f>
         <v/>
       </c>
       <c r="E17" s="15">
@@ -69429,188 +69508,333 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="66" t="inlineStr">
+        <is>
+          <t>Posición actual — Banco MP (único stock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>Fecha stock</t>
+        </is>
+      </c>
+      <c r="B20" s="67" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="C20" s="67" t="inlineStr">
+        <is>
+          <t>Capital invertido</t>
+        </is>
+      </c>
+      <c r="D20" s="67" t="inlineStr">
+        <is>
+          <t>Tasa anual</t>
+        </is>
+      </c>
+      <c r="E20" s="67" t="inlineStr">
+        <is>
+          <t>Rendimiento anual esperado</t>
+        </is>
+      </c>
+      <c r="F20" s="67" t="inlineStr">
+        <is>
+          <t>Rendimiento mensual lineal</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="31" t="inlineStr">
-        <is>
-          <t>Detalle</t>
-        </is>
+      <c r="A21" s="68" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B21" s="69" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="C21" s="70" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="D21" s="71" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E21" s="70">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="70">
+        <f>E21/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="72" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B22" s="69" t="inlineStr">
+        <is>
+          <t>Sol</t>
+        </is>
+      </c>
+      <c r="C22" s="70" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D22" s="71" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E22" s="70">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="70">
+        <f>E22/12</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="34" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="B23" s="34" t="inlineStr">
-        <is>
-          <t>Mes</t>
-        </is>
-      </c>
-      <c r="C23" s="34" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="D23" s="34" t="inlineStr">
-        <is>
-          <t>Movimiento</t>
-        </is>
-      </c>
-      <c r="E23" s="34" t="inlineStr">
-        <is>
-          <t>Instrumento / concepto</t>
-        </is>
-      </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>Monto</t>
-        </is>
-      </c>
-      <c r="G23" s="34" t="inlineStr">
-        <is>
-          <t>Entidad / medio</t>
-        </is>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>Vencimiento</t>
-        </is>
-      </c>
-      <c r="I23" s="34" t="inlineStr">
-        <is>
-          <t>Tasa / rendimiento</t>
-        </is>
-      </c>
-      <c r="J23" s="34" t="inlineStr">
-        <is>
-          <t>Comentario</t>
-        </is>
-      </c>
+      <c r="A23" s="73" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B23" s="74" t="inlineStr">
+        <is>
+          <t>TOTAL banco MP</t>
+        </is>
+      </c>
+      <c r="C23" s="75">
+        <f>C21+C22</f>
+        <v/>
+      </c>
+      <c r="D23" s="76" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E23" s="75">
+        <f>E21+E22</f>
+        <v/>
+      </c>
+      <c r="F23" s="75">
+        <f>F21+F22</f>
+        <v/>
+      </c>
+      <c r="G23" s="34" t="n"/>
+      <c r="H23" s="34" t="n"/>
+      <c r="I23" s="34" t="n"/>
+      <c r="J23" s="34" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>Rescate</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>Venta de dólares</t>
-        </is>
-      </c>
-      <c r="F24" s="15" t="n">
-        <v>1261633</v>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+      <c r="A24" s="77" t="inlineStr">
+        <is>
+          <t>Instrucción Sol 2026-08-03: único valor invertido en banco MP = $13.000.000 (Christian $10.000.000 + Sol $3.000.000) al 21% anual desde 29/07/2026. Se deja de contar el Bonos/PF previo ($1.000.000 del 15/07) como stock.</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="14" t="n"/>
       <c r="H24" s="17" t="n"/>
       <c r="I24" s="37" t="n"/>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>En proceso · ceil 1.261.632,32 · también en MP No Gasto</t>
-        </is>
-      </c>
+      <c r="J24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>Bonos/PF</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Inversión</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Bonos, plazos fijos y más</t>
-        </is>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
+      <c r="A25" s="78" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="14" t="n"/>
       <c r="H25" s="17" t="n"/>
       <c r="I25" s="37" t="n"/>
       <c r="J25" s="14" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="n"/>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="14" t="n"/>
-      <c r="H26" s="17" t="n"/>
-      <c r="I26" s="37" t="n"/>
-      <c r="J26" s="14" t="n"/>
+      <c r="A26" s="79" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B26" s="67" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D26" s="67" t="inlineStr">
+        <is>
+          <t>Movimiento</t>
+        </is>
+      </c>
+      <c r="E26" s="67" t="inlineStr">
+        <is>
+          <t>Instrumento / concepto</t>
+        </is>
+      </c>
+      <c r="F26" s="80" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="G26" s="67" t="inlineStr">
+        <is>
+          <t>Entidad / medio</t>
+        </is>
+      </c>
+      <c r="H26" s="79" t="inlineStr">
+        <is>
+          <t>Vencimiento</t>
+        </is>
+      </c>
+      <c r="I26" s="81" t="inlineStr">
+        <is>
+          <t>Tasa / rendimiento</t>
+        </is>
+      </c>
+      <c r="J26" s="67" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="n"/>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="14" t="n"/>
-      <c r="E27" s="14" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="17" t="n"/>
-      <c r="I27" s="37" t="n"/>
-      <c r="J27" s="14" t="n"/>
+      <c r="A27" s="63" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B27" s="64" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C27" s="64" t="inlineStr">
+        <is>
+          <t>Banco MP</t>
+        </is>
+      </c>
+      <c r="D27" s="64" t="inlineStr">
+        <is>
+          <t>Inversión</t>
+        </is>
+      </c>
+      <c r="E27" s="64" t="inlineStr">
+        <is>
+          <t>Banco MP · Christian</t>
+        </is>
+      </c>
+      <c r="F27" s="65" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="G27" s="64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H27" s="82" t="n"/>
+      <c r="I27" s="83" t="inlineStr">
+        <is>
+          <t>21% anual</t>
+        </is>
+      </c>
+      <c r="J27" s="64" t="inlineStr">
+        <is>
+          <t>Único stock banco MP · titular Christian · instruido Sol 2026-08-03 · también MP No Gasto</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="n"/>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="14" t="n"/>
-      <c r="E28" s="14" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="14" t="n"/>
-      <c r="H28" s="17" t="n"/>
-      <c r="I28" s="37" t="n"/>
-      <c r="J28" s="14" t="n"/>
+      <c r="A28" s="63" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B28" s="64" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C28" s="64" t="inlineStr">
+        <is>
+          <t>Banco MP</t>
+        </is>
+      </c>
+      <c r="D28" s="64" t="inlineStr">
+        <is>
+          <t>Inversión</t>
+        </is>
+      </c>
+      <c r="E28" s="64" t="inlineStr">
+        <is>
+          <t>Banco MP · Sol</t>
+        </is>
+      </c>
+      <c r="F28" s="65" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="G28" s="64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H28" s="82" t="n"/>
+      <c r="I28" s="83" t="inlineStr">
+        <is>
+          <t>21% anual</t>
+        </is>
+      </c>
+      <c r="J28" s="64" t="inlineStr">
+        <is>
+          <t>Único stock banco MP · titular Sol · instruido Sol 2026-08-03 · también MP No Gasto</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="n"/>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="17" t="n"/>
-      <c r="I29" s="37" t="n"/>
-      <c r="J29" s="14" t="n"/>
+      <c r="A29" s="63" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B29" s="64" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C29" s="64" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D29" s="64" t="inlineStr">
+        <is>
+          <t>Rescate</t>
+        </is>
+      </c>
+      <c r="E29" s="64" t="inlineStr">
+        <is>
+          <t>Venta de dólares</t>
+        </is>
+      </c>
+      <c r="F29" s="65" t="n">
+        <v>1261633</v>
+      </c>
+      <c r="G29" s="64" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="H29" s="82" t="n"/>
+      <c r="I29" s="83" t="n"/>
+      <c r="J29" s="64" t="inlineStr">
+        <is>
+          <t>Histórico · en proceso · ceil 1.261.632,32 · NO es stock banco MP · también en MP No Gasto</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="17" t="n"/>

</xml_diff>

<commit_message>
Add August pollo $35,000 to CIUDAD Almacen Sol.
Registers COMIDA · pollo on 2026-08-03 in Almacen Detalle (Importe Sol).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -60717,15 +60717,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n"/>
-      <c r="C314" s="14" t="n"/>
-      <c r="D314" s="27" t="n"/>
+      <c r="B314" s="17" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · pollo</t>
+        </is>
+      </c>
+      <c r="D314" s="27" t="n">
+        <v>35000</v>
+      </c>
       <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
-        <f>IF(OR(D298&lt;&gt;"",E298&lt;&gt;""),IF(D298="",0,D298)+IF(E298="",0,E298),"")</f>
-        <v/>
-      </c>
-      <c r="G314" s="14" t="n"/>
+        <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
+        <v/>
+      </c>
+      <c r="G314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · pollo · ALMACEN SOL</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Load Metrogas CIUDAD July gas from Visa *3200 charge.
Registers $73,695 (ceil of $73,694.19) for July from the 05/08/2026
BBVA Visa METROGAS SA DEB AU notice (cliente 30010996459).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -939,7 +939,9 @@
       <c r="I7" s="5" t="n">
         <v>30643</v>
       </c>
-      <c r="J7" s="5" t="n"/>
+      <c r="J7" s="5" t="n">
+        <v>73695</v>
+      </c>
       <c r="K7" s="5" t="n"/>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="n"/>
@@ -64106,7 +64108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66350,6 +66352,49 @@
       <c r="F73" s="18" t="inlineStr">
         <is>
           <t>3491192</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="53" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>Metrogas</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Metrogas CIUDAD · cobro Visa *3200 05/08/2026 · mes julio (período usuario)</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="n">
+        <v>73695</v>
+      </c>
+      <c r="E74" s="14" t="inlineStr">
+        <is>
+          <t>BBVA Visa *3200 · METROGAS SA DEB AU</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>30010996459</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>40049923</t>
+        </is>
+      </c>
+      <c r="H74" s="14" t="inlineStr">
+        <is>
+          <t>ceil $73.694,19 · aviso 05/08/2026 · asignado a julio</t>
+        </is>
+      </c>
+      <c r="I74" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document CIUDAD Metrogas as BBVA Visa *3200 auto-debit.
Makes the Visa ending 3200 payment medium explicit in rules,
utilidades references, and the 2026 sheet note.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -721,6 +721,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1557,6 +1558,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
@@ -1829,7 +1831,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>• GAS CIUDAD (Metrogas 30010996459): mes = fecha de cobro BBVA / pago / vencimiento factura — no período de consumo</t>
+          <t>• GAS CIUDAD (Metrogas 30010996459): se paga con Visa BBVA *3200 (METROGAS SA DEB AU). Mes = fecha de cobro BBVA — no período de consumo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add August verdulería $13,500 to CIUDAD Almacen Sol.
Registers COMIDA · VERDULERÍA on 2026-08-05 in Almacen Detalle.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -60717,15 +60717,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n"/>
-      <c r="C314" s="14" t="n"/>
-      <c r="D314" s="27" t="n"/>
+      <c r="B314" s="17" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
+      <c r="D314" s="27" t="n">
+        <v>13500</v>
+      </c>
       <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
-        <f>IF(OR(D298&lt;&gt;"",E298&lt;&gt;""),IF(D298="",0,D298)+IF(E298="",0,E298),"")</f>
-        <v/>
-      </c>
-      <c r="G314" s="14" t="n"/>
+        <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
+        <v/>
+      </c>
+      <c r="G314" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Import actual July MELI payslip
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1727,7 +1727,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -27008,11 +27007,11 @@
         </is>
       </c>
       <c r="B6" s="50" t="n">
-        <v>12662387</v>
+        <v>12662386</v>
       </c>
       <c r="C6" s="51" t="inlineStr">
         <is>
-          <t>ARS · vigente desde 01/07/2026 · básico anterior +12%</t>
+          <t>ARS · recibo MELI julio 2026 · vigente desde 01/07/2026</t>
         </is>
       </c>
     </row>
@@ -27511,7 +27510,7 @@
         <v>46235</v>
       </c>
       <c r="D30" s="61" t="n">
-        <v>12662387</v>
+        <v>12662386</v>
       </c>
       <c r="E30" s="51" t="inlineStr">
         <is>
@@ -27525,7 +27524,7 @@
       </c>
       <c r="G30" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · básico anterior ARS 11.305.702 + 12% · vigente 01/07 · cobro 01/08</t>
+          <t>Ingreso básico MELI julio · recibo real · cobrado 01/08/2026</t>
         </is>
       </c>
     </row>
@@ -27542,7 +27541,7 @@
         <v>46266</v>
       </c>
       <c r="D31" s="61" t="n">
-        <v>12662387</v>
+        <v>12662386</v>
       </c>
       <c r="E31" s="51" t="inlineStr">
         <is>
@@ -27556,7 +27555,7 @@
       </c>
       <c r="G31" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
+          <t>Ingreso bruto básico MELI · valor real según recibo julio 2026 · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27573,7 +27572,7 @@
         <v>46296</v>
       </c>
       <c r="D32" s="61" t="n">
-        <v>12662387</v>
+        <v>12662386</v>
       </c>
       <c r="E32" s="51" t="inlineStr">
         <is>
@@ -27587,7 +27586,7 @@
       </c>
       <c r="G32" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
+          <t>Ingreso bruto básico MELI · valor real según recibo julio 2026 · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27604,7 +27603,7 @@
         <v>46327</v>
       </c>
       <c r="D33" s="61" t="n">
-        <v>12662387</v>
+        <v>12662386</v>
       </c>
       <c r="E33" s="51" t="inlineStr">
         <is>
@@ -27618,7 +27617,7 @@
       </c>
       <c r="G33" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
+          <t>Ingreso bruto básico MELI · valor real según recibo julio 2026 · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27635,7 +27634,7 @@
         <v>46357</v>
       </c>
       <c r="D34" s="61" t="n">
-        <v>12662387</v>
+        <v>12662386</v>
       </c>
       <c r="E34" s="51" t="inlineStr">
         <is>
@@ -27649,7 +27648,7 @@
       </c>
       <c r="G34" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
+          <t>Ingreso bruto básico MELI · valor real según recibo julio 2026 · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27666,7 +27665,7 @@
         <v>46388</v>
       </c>
       <c r="D35" s="61" t="n">
-        <v>12662387</v>
+        <v>12662386</v>
       </c>
       <c r="E35" s="51" t="inlineStr">
         <is>
@@ -27680,7 +27679,7 @@
       </c>
       <c r="G35" s="51" t="inlineStr">
         <is>
-          <t>Ingreso bruto Sol · incremento 12% desde julio · cobro mes siguiente</t>
+          <t>Ingreso bruto básico MELI · valor real según recibo julio 2026 · cobro mes siguiente</t>
         </is>
       </c>
     </row>
@@ -27695,7 +27694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P151"/>
+  <dimension ref="A1:P159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -27762,11 +27761,11 @@
         </is>
       </c>
       <c r="B6" s="69" t="n">
-        <v>349440</v>
+        <v>360000</v>
       </c>
       <c r="C6" s="68" t="inlineStr">
         <is>
-          <t>ARS 312.000 + 12% desde 01/07/2026</t>
+          <t>Beneficio Auto real según recibo julio 2026</t>
         </is>
       </c>
       <c r="D6" s="68" t="n"/>
@@ -28677,7 +28676,7 @@
     <row r="75" ht="34" customHeight="1">
       <c r="A75" s="83" t="inlineStr">
         <is>
-          <t>• Car allowance: ARS 312.000 hasta junio; +12% desde julio = ARS 349.440. Bruto mensual total proyectado: ARS 13.011.827.</t>
+          <t>• Recibo julio 2026: básico ARS 12.662.386 + Beneficio Auto ARS 360.000 = bruto ARS 13.022.386; neto ARS 8.784.847,44; pago 01/08/2026.</t>
         </is>
       </c>
     </row>
@@ -29227,137 +29226,162 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="90" t="inlineStr">
+      <c r="A87" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B87" s="75" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C87" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D87" s="93" t="n">
+        <v>12662386</v>
+      </c>
+      <c r="E87" s="93" t="n">
+        <v>360000</v>
+      </c>
+      <c r="F87" s="93" t="n">
+        <v>13022386</v>
+      </c>
+      <c r="G87" s="93" t="n">
+        <v>496052.42</v>
+      </c>
+      <c r="H87" s="93" t="n">
+        <v>135287.02</v>
+      </c>
+      <c r="I87" s="93" t="n">
+        <v>135287.02</v>
+      </c>
+      <c r="J87" s="93" t="n">
+        <v>3445112.1</v>
+      </c>
+      <c r="K87" s="93" t="n">
+        <v>25800</v>
+      </c>
+      <c r="L87" s="93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="93" t="n">
+        <v>4237538.56</v>
+      </c>
+      <c r="N87" s="94" t="n">
+        <v>8784847.439999999</v>
+      </c>
+      <c r="O87" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
+        </is>
+      </c>
+      <c r="P87" s="93">
+        <f>ROUND(F87-M87-N87,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="90" t="inlineStr">
         <is>
           <t>TOTAL RECIBOS</t>
         </is>
       </c>
-      <c r="B87" s="68" t="n"/>
-      <c r="C87" s="68" t="n"/>
-      <c r="D87" s="95">
-        <f>SUM(D79:D86)</f>
-        <v/>
-      </c>
-      <c r="E87" s="95">
-        <f>SUM(E79:E86)</f>
-        <v/>
-      </c>
-      <c r="F87" s="95">
-        <f>SUM(F79:F86)</f>
-        <v/>
-      </c>
-      <c r="G87" s="95">
-        <f>SUM(G79:G86)</f>
-        <v/>
-      </c>
-      <c r="H87" s="95">
-        <f>SUM(H79:H86)</f>
-        <v/>
-      </c>
-      <c r="I87" s="95">
-        <f>SUM(I79:I86)</f>
-        <v/>
-      </c>
-      <c r="J87" s="95">
-        <f>SUM(J79:J86)</f>
-        <v/>
-      </c>
-      <c r="K87" s="95">
-        <f>SUM(K79:K86)</f>
-        <v/>
-      </c>
-      <c r="L87" s="95">
-        <f>SUM(L79:L86)</f>
-        <v/>
-      </c>
-      <c r="M87" s="95">
-        <f>SUM(M79:M86)</f>
-        <v/>
-      </c>
-      <c r="N87" s="95">
-        <f>SUM(N79:N86)</f>
-        <v/>
-      </c>
-      <c r="O87" s="68" t="n"/>
-      <c r="P87" s="96">
-        <f>ROUND(F87-M87-N87,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="84" t="inlineStr">
+      <c r="B88" s="68" t="n"/>
+      <c r="C88" s="68" t="n"/>
+      <c r="D88" s="95">
+        <f>SUM(D79:D87)</f>
+        <v/>
+      </c>
+      <c r="E88" s="95">
+        <f>SUM(E79:E87)</f>
+        <v/>
+      </c>
+      <c r="F88" s="95">
+        <f>SUM(F79:F87)</f>
+        <v/>
+      </c>
+      <c r="G88" s="95">
+        <f>SUM(G79:G87)</f>
+        <v/>
+      </c>
+      <c r="H88" s="95">
+        <f>SUM(H79:H87)</f>
+        <v/>
+      </c>
+      <c r="I88" s="95">
+        <f>SUM(I79:I87)</f>
+        <v/>
+      </c>
+      <c r="J88" s="95">
+        <f>SUM(J79:J87)</f>
+        <v/>
+      </c>
+      <c r="K88" s="95">
+        <f>SUM(K79:K87)</f>
+        <v/>
+      </c>
+      <c r="L88" s="95">
+        <f>SUM(L79:L87)</f>
+        <v/>
+      </c>
+      <c r="M88" s="95">
+        <f>SUM(M79:M87)</f>
+        <v/>
+      </c>
+      <c r="N88" s="95">
+        <f>SUM(N79:N87)</f>
+        <v/>
+      </c>
+      <c r="O88" s="68" t="n"/>
+      <c r="P88" s="96">
+        <f>ROUND(F88-M88-N88,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89"/>
+    <row r="90">
+      <c r="A90" s="84" t="inlineStr">
         <is>
           <t>DETALLE EXTRAÍDO DE CONCEPTOS</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="80" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="80" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="B90" s="80" t="inlineStr">
+      <c r="B91" s="80" t="inlineStr">
         <is>
           <t>Tipo recibo</t>
         </is>
       </c>
-      <c r="C90" s="80" t="inlineStr">
+      <c r="C91" s="80" t="inlineStr">
         <is>
           <t>Fecha pago</t>
         </is>
       </c>
-      <c r="D90" s="80" t="inlineStr">
+      <c r="D91" s="80" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="E90" s="80" t="inlineStr">
+      <c r="E91" s="80" t="inlineStr">
         <is>
           <t>Clase</t>
         </is>
       </c>
-      <c r="F90" s="80" t="inlineStr">
+      <c r="F91" s="80" t="inlineStr">
         <is>
           <t>Importe</t>
         </is>
       </c>
-      <c r="G90" s="80" t="inlineStr">
+      <c r="G91" s="80" t="inlineStr">
         <is>
           <t>Archivo fuente</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="86" t="inlineStr">
-        <is>
-          <t>Enero</t>
-        </is>
-      </c>
-      <c r="B91" s="86" t="inlineStr">
-        <is>
-          <t>Sueldo</t>
-        </is>
-      </c>
-      <c r="C91" s="87" t="n">
-        <v>46054</v>
-      </c>
-      <c r="D91" s="86" t="inlineStr">
-        <is>
-          <t>Sueldo Básico</t>
-        </is>
-      </c>
-      <c r="E91" s="86" t="inlineStr">
-        <is>
-          <t>Haber</t>
-        </is>
-      </c>
-      <c r="F91" s="93" t="n">
-        <v>7906085</v>
-      </c>
-      <c r="G91" s="86" t="inlineStr">
-        <is>
-          <t>ENERO.pdf</t>
         </is>
       </c>
     </row>
@@ -29377,7 +29401,7 @@
       </c>
       <c r="D92" s="86" t="inlineStr">
         <is>
-          <t>Beneficio Auto</t>
+          <t>Sueldo Básico</t>
         </is>
       </c>
       <c r="E92" s="86" t="inlineStr">
@@ -29386,7 +29410,7 @@
         </is>
       </c>
       <c r="F92" s="93" t="n">
-        <v>180000</v>
+        <v>7906085</v>
       </c>
       <c r="G92" s="86" t="inlineStr">
         <is>
@@ -29410,16 +29434,16 @@
       </c>
       <c r="D93" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre sueldo</t>
+          <t>Beneficio Auto</t>
         </is>
       </c>
       <c r="E93" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F93" s="93" t="n">
-        <v>420571.02</v>
+        <v>180000</v>
       </c>
       <c r="G93" s="86" t="inlineStr">
         <is>
@@ -29443,7 +29467,7 @@
       </c>
       <c r="D94" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre sueldo</t>
+          <t>Aporte SIJP sobre sueldo</t>
         </is>
       </c>
       <c r="E94" s="86" t="inlineStr">
@@ -29452,7 +29476,7 @@
         </is>
       </c>
       <c r="F94" s="93" t="n">
-        <v>114701.19</v>
+        <v>420571.02</v>
       </c>
       <c r="G94" s="86" t="inlineStr">
         <is>
@@ -29476,7 +29500,7 @@
       </c>
       <c r="D95" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre sueldo</t>
+          <t>Aporte INSSJP sobre sueldo</t>
         </is>
       </c>
       <c r="E95" s="86" t="inlineStr">
@@ -29509,16 +29533,16 @@
       </c>
       <c r="D96" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
+          <t>Aporte Obra Social sobre sueldo</t>
         </is>
       </c>
       <c r="E96" s="86" t="inlineStr">
         <is>
-          <t>Descuento Ganancias</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F96" s="93" t="n">
-        <v>1221703.83</v>
+        <v>114701.19</v>
       </c>
       <c r="G96" s="86" t="inlineStr">
         <is>
@@ -29542,16 +29566,16 @@
       </c>
       <c r="D97" s="86" t="inlineStr">
         <is>
-          <t>Dto Gimnasio</t>
+          <t>Impuesto pagado/devuelto</t>
         </is>
       </c>
       <c r="E97" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Descuento Ganancias</t>
         </is>
       </c>
       <c r="F97" s="93" t="n">
-        <v>21900</v>
+        <v>1221703.83</v>
       </c>
       <c r="G97" s="86" t="inlineStr">
         <is>
@@ -29562,7 +29586,7 @@
     <row r="98">
       <c r="A98" s="86" t="inlineStr">
         <is>
-          <t>Febrero</t>
+          <t>Enero</t>
         </is>
       </c>
       <c r="B98" s="86" t="inlineStr">
@@ -29571,24 +29595,24 @@
         </is>
       </c>
       <c r="C98" s="87" t="n">
-        <v>46082</v>
+        <v>46054</v>
       </c>
       <c r="D98" s="86" t="inlineStr">
         <is>
-          <t>Sueldo Básico</t>
+          <t>Dto Gimnasio</t>
         </is>
       </c>
       <c r="E98" s="86" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F98" s="93" t="n">
-        <v>7906085</v>
+        <v>21900</v>
       </c>
       <c r="G98" s="86" t="inlineStr">
         <is>
-          <t>FEBRERO.pdf</t>
+          <t>ENERO.pdf</t>
         </is>
       </c>
     </row>
@@ -29608,7 +29632,7 @@
       </c>
       <c r="D99" s="86" t="inlineStr">
         <is>
-          <t>Beneficio Auto</t>
+          <t>Sueldo Básico</t>
         </is>
       </c>
       <c r="E99" s="86" t="inlineStr">
@@ -29617,7 +29641,7 @@
         </is>
       </c>
       <c r="F99" s="93" t="n">
-        <v>208000</v>
+        <v>7906085</v>
       </c>
       <c r="G99" s="86" t="inlineStr">
         <is>
@@ -29641,16 +29665,16 @@
       </c>
       <c r="D100" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre sueldo</t>
+          <t>Beneficio Auto</t>
         </is>
       </c>
       <c r="E100" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F100" s="93" t="n">
-        <v>432557.3</v>
+        <v>208000</v>
       </c>
       <c r="G100" s="86" t="inlineStr">
         <is>
@@ -29674,7 +29698,7 @@
       </c>
       <c r="D101" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre sueldo</t>
+          <t>Aporte SIJP sobre sueldo</t>
         </is>
       </c>
       <c r="E101" s="86" t="inlineStr">
@@ -29683,7 +29707,7 @@
         </is>
       </c>
       <c r="F101" s="93" t="n">
-        <v>117970.17</v>
+        <v>432557.3</v>
       </c>
       <c r="G101" s="86" t="inlineStr">
         <is>
@@ -29707,7 +29731,7 @@
       </c>
       <c r="D102" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre sueldo</t>
+          <t>Aporte INSSJP sobre sueldo</t>
         </is>
       </c>
       <c r="E102" s="86" t="inlineStr">
@@ -29740,16 +29764,16 @@
       </c>
       <c r="D103" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
+          <t>Aporte Obra Social sobre sueldo</t>
         </is>
       </c>
       <c r="E103" s="86" t="inlineStr">
         <is>
-          <t>Descuento Ganancias</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F103" s="93" t="n">
-        <v>1425004.25</v>
+        <v>117970.17</v>
       </c>
       <c r="G103" s="86" t="inlineStr">
         <is>
@@ -29773,16 +29797,16 @@
       </c>
       <c r="D104" s="86" t="inlineStr">
         <is>
-          <t>Dto Gimnasio</t>
+          <t>Impuesto pagado/devuelto</t>
         </is>
       </c>
       <c r="E104" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Descuento Ganancias</t>
         </is>
       </c>
       <c r="F104" s="93" t="n">
-        <v>21900</v>
+        <v>1425004.25</v>
       </c>
       <c r="G104" s="86" t="inlineStr">
         <is>
@@ -29793,33 +29817,33 @@
     <row r="105">
       <c r="A105" s="86" t="inlineStr">
         <is>
-          <t>Marzo</t>
+          <t>Febrero</t>
         </is>
       </c>
       <c r="B105" s="86" t="inlineStr">
         <is>
-          <t>Sueldo + retroactivo</t>
+          <t>Sueldo</t>
         </is>
       </c>
       <c r="C105" s="87" t="n">
-        <v>46113</v>
+        <v>46082</v>
       </c>
       <c r="D105" s="86" t="inlineStr">
         <is>
-          <t>R-Sueldo Básico</t>
+          <t>Dto Gimnasio</t>
         </is>
       </c>
       <c r="E105" s="86" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F105" s="93" t="n">
-        <v>6799234</v>
+        <v>21900</v>
       </c>
       <c r="G105" s="86" t="inlineStr">
         <is>
-          <t>MARZO.pdf</t>
+          <t>FEBRERO.pdf</t>
         </is>
       </c>
     </row>
@@ -29839,7 +29863,7 @@
       </c>
       <c r="D106" s="86" t="inlineStr">
         <is>
-          <t>Sueldo Básico</t>
+          <t>R-Sueldo Básico</t>
         </is>
       </c>
       <c r="E106" s="86" t="inlineStr">
@@ -29848,7 +29872,7 @@
         </is>
       </c>
       <c r="F106" s="93" t="n">
-        <v>11305702</v>
+        <v>6799234</v>
       </c>
       <c r="G106" s="86" t="inlineStr">
         <is>
@@ -29872,7 +29896,7 @@
       </c>
       <c r="D107" s="86" t="inlineStr">
         <is>
-          <t>Beneficio Auto</t>
+          <t>Sueldo Básico</t>
         </is>
       </c>
       <c r="E107" s="86" t="inlineStr">
@@ -29881,7 +29905,7 @@
         </is>
       </c>
       <c r="F107" s="93" t="n">
-        <v>208000</v>
+        <v>11305702</v>
       </c>
       <c r="G107" s="86" t="inlineStr">
         <is>
@@ -29905,16 +29929,16 @@
       </c>
       <c r="D108" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre sueldo</t>
+          <t>Beneficio Auto</t>
         </is>
       </c>
       <c r="E108" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F108" s="93" t="n">
-        <v>445014.95</v>
+        <v>208000</v>
       </c>
       <c r="G108" s="86" t="inlineStr">
         <is>
@@ -29938,7 +29962,7 @@
       </c>
       <c r="D109" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre sueldo</t>
+          <t>Aporte SIJP sobre sueldo</t>
         </is>
       </c>
       <c r="E109" s="86" t="inlineStr">
@@ -29947,7 +29971,7 @@
         </is>
       </c>
       <c r="F109" s="93" t="n">
-        <v>121367.71</v>
+        <v>445014.95</v>
       </c>
       <c r="G109" s="86" t="inlineStr">
         <is>
@@ -29971,7 +29995,7 @@
       </c>
       <c r="D110" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre sueldo</t>
+          <t>Aporte INSSJP sobre sueldo</t>
         </is>
       </c>
       <c r="E110" s="86" t="inlineStr">
@@ -30004,16 +30028,16 @@
       </c>
       <c r="D111" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
+          <t>Aporte Obra Social sobre sueldo</t>
         </is>
       </c>
       <c r="E111" s="86" t="inlineStr">
         <is>
-          <t>Descuento Ganancias</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F111" s="93" t="n">
-        <v>4658857.2</v>
+        <v>121367.71</v>
       </c>
       <c r="G111" s="86" t="inlineStr">
         <is>
@@ -30037,16 +30061,16 @@
       </c>
       <c r="D112" s="86" t="inlineStr">
         <is>
-          <t>Dto Gimnasio</t>
+          <t>Impuesto pagado/devuelto</t>
         </is>
       </c>
       <c r="E112" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Descuento Ganancias</t>
         </is>
       </c>
       <c r="F112" s="93" t="n">
-        <v>21900</v>
+        <v>4658857.2</v>
       </c>
       <c r="G112" s="86" t="inlineStr">
         <is>
@@ -30057,33 +30081,33 @@
     <row r="113">
       <c r="A113" s="86" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Marzo</t>
         </is>
       </c>
       <c r="B113" s="86" t="inlineStr">
         <is>
-          <t>Bono anual / transición</t>
+          <t>Sueldo + retroactivo</t>
         </is>
       </c>
       <c r="C113" s="87" t="n">
-        <v>46118</v>
+        <v>46113</v>
       </c>
       <c r="D113" s="86" t="inlineStr">
         <is>
-          <t>Bono de Transición</t>
+          <t>Dto Gimnasio</t>
         </is>
       </c>
       <c r="E113" s="86" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F113" s="93" t="n">
-        <v>7296916.15</v>
+        <v>21900</v>
       </c>
       <c r="G113" s="86" t="inlineStr">
         <is>
-          <t>ABRIL BONO.pdf</t>
+          <t>MARZO.pdf</t>
         </is>
       </c>
     </row>
@@ -30103,7 +30127,7 @@
       </c>
       <c r="D114" s="86" t="inlineStr">
         <is>
-          <t>Gratificación Extraordinaria Anual</t>
+          <t>Bono de Transición</t>
         </is>
       </c>
       <c r="E114" s="86" t="inlineStr">
@@ -30112,7 +30136,7 @@
         </is>
       </c>
       <c r="F114" s="93" t="n">
-        <v>14596298</v>
+        <v>7296916.15</v>
       </c>
       <c r="G114" s="86" t="inlineStr">
         <is>
@@ -30136,7 +30160,7 @@
       </c>
       <c r="D115" s="86" t="inlineStr">
         <is>
-          <t>SAC Gratificación Extraordinaria</t>
+          <t>Gratificación Extraordinaria Anual</t>
         </is>
       </c>
       <c r="E115" s="86" t="inlineStr">
@@ -30145,7 +30169,7 @@
         </is>
       </c>
       <c r="F115" s="93" t="n">
-        <v>1215872</v>
+        <v>14596298</v>
       </c>
       <c r="G115" s="86" t="inlineStr">
         <is>
@@ -30169,7 +30193,7 @@
       </c>
       <c r="D116" s="86" t="inlineStr">
         <is>
-          <t>SAC sobre Bono de Transición</t>
+          <t>SAC Gratificación Extraordinaria</t>
         </is>
       </c>
       <c r="E116" s="86" t="inlineStr">
@@ -30178,7 +30202,7 @@
         </is>
       </c>
       <c r="F116" s="93" t="n">
-        <v>608076.35</v>
+        <v>1215872</v>
       </c>
       <c r="G116" s="86" t="inlineStr">
         <is>
@@ -30202,16 +30226,16 @@
       </c>
       <c r="D117" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre sueldo</t>
+          <t>SAC sobre Bono de Transición</t>
         </is>
       </c>
       <c r="E117" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F117" s="93" t="n">
-        <v>445014.95</v>
+        <v>608076.35</v>
       </c>
       <c r="G117" s="86" t="inlineStr">
         <is>
@@ -30235,7 +30259,7 @@
       </c>
       <c r="D118" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre sueldo</t>
+          <t>Aporte SIJP sobre sueldo</t>
         </is>
       </c>
       <c r="E118" s="86" t="inlineStr">
@@ -30244,7 +30268,7 @@
         </is>
       </c>
       <c r="F118" s="93" t="n">
-        <v>121367.71</v>
+        <v>445014.95</v>
       </c>
       <c r="G118" s="86" t="inlineStr">
         <is>
@@ -30268,7 +30292,7 @@
       </c>
       <c r="D119" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre sueldo</t>
+          <t>Aporte INSSJP sobre sueldo</t>
         </is>
       </c>
       <c r="E119" s="86" t="inlineStr">
@@ -30301,16 +30325,16 @@
       </c>
       <c r="D120" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
+          <t>Aporte Obra Social sobre sueldo</t>
         </is>
       </c>
       <c r="E120" s="86" t="inlineStr">
         <is>
-          <t>Descuento Ganancias</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F120" s="93" t="n">
-        <v>3120893.08</v>
+        <v>121367.71</v>
       </c>
       <c r="G120" s="86" t="inlineStr">
         <is>
@@ -30326,28 +30350,28 @@
       </c>
       <c r="B121" s="86" t="inlineStr">
         <is>
-          <t>Sueldo + vacaciones</t>
+          <t>Bono anual / transición</t>
         </is>
       </c>
       <c r="C121" s="87" t="n">
-        <v>46143</v>
+        <v>46118</v>
       </c>
       <c r="D121" s="86" t="inlineStr">
         <is>
-          <t>Sueldo Básico</t>
+          <t>Impuesto pagado/devuelto</t>
         </is>
       </c>
       <c r="E121" s="86" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Descuento Ganancias</t>
         </is>
       </c>
       <c r="F121" s="93" t="n">
-        <v>11305702</v>
+        <v>3120893.08</v>
       </c>
       <c r="G121" s="86" t="inlineStr">
         <is>
-          <t>ABRIL.pdf</t>
+          <t>ABRIL BONO.pdf</t>
         </is>
       </c>
     </row>
@@ -30367,7 +30391,7 @@
       </c>
       <c r="D122" s="86" t="inlineStr">
         <is>
-          <t>Beneficio Auto</t>
+          <t>Sueldo Básico</t>
         </is>
       </c>
       <c r="E122" s="86" t="inlineStr">
@@ -30376,7 +30400,7 @@
         </is>
       </c>
       <c r="F122" s="93" t="n">
-        <v>312000</v>
+        <v>11305702</v>
       </c>
       <c r="G122" s="86" t="inlineStr">
         <is>
@@ -30400,7 +30424,7 @@
       </c>
       <c r="D123" s="86" t="inlineStr">
         <is>
-          <t>Pago de Vacaciones</t>
+          <t>Beneficio Auto</t>
         </is>
       </c>
       <c r="E123" s="86" t="inlineStr">
@@ -30409,7 +30433,7 @@
         </is>
       </c>
       <c r="F123" s="93" t="n">
-        <v>9758869.68</v>
+        <v>312000</v>
       </c>
       <c r="G123" s="86" t="inlineStr">
         <is>
@@ -30433,16 +30457,16 @@
       </c>
       <c r="D124" s="86" t="inlineStr">
         <is>
-          <t>Dto Días No Trabajados Vacaciones</t>
-        </is>
-      </c>
-      <c r="E124" s="73" t="inlineStr">
-        <is>
-          <t>Haber negativo</t>
+          <t>Pago de Vacaciones</t>
+        </is>
+      </c>
+      <c r="E124" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F124" s="93" t="n">
-        <v>-8132391.4</v>
+        <v>9758869.68</v>
       </c>
       <c r="G124" s="86" t="inlineStr">
         <is>
@@ -30466,7 +30490,7 @@
       </c>
       <c r="D125" s="86" t="inlineStr">
         <is>
-          <t>R-Dto Días No Trabajados</t>
+          <t>Dto Días No Trabajados Vacaciones</t>
         </is>
       </c>
       <c r="E125" s="73" t="inlineStr">
@@ -30475,7 +30499,7 @@
         </is>
       </c>
       <c r="F125" s="93" t="n">
-        <v>-1151370.2</v>
+        <v>-8132391.4</v>
       </c>
       <c r="G125" s="86" t="inlineStr">
         <is>
@@ -30499,16 +30523,16 @@
       </c>
       <c r="D126" s="86" t="inlineStr">
         <is>
-          <t>R-Licencia Especial</t>
-        </is>
-      </c>
-      <c r="E126" s="86" t="inlineStr">
-        <is>
-          <t>Haber</t>
+          <t>R-Dto Días No Trabajados</t>
+        </is>
+      </c>
+      <c r="E126" s="73" t="inlineStr">
+        <is>
+          <t>Haber negativo</t>
         </is>
       </c>
       <c r="F126" s="93" t="n">
-        <v>1381644.24</v>
+        <v>-1151370.2</v>
       </c>
       <c r="G126" s="86" t="inlineStr">
         <is>
@@ -30532,16 +30556,16 @@
       </c>
       <c r="D127" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre sueldo</t>
+          <t>R-Licencia Especial</t>
         </is>
       </c>
       <c r="E127" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F127" s="93" t="n">
-        <v>12905.43</v>
+        <v>1381644.24</v>
       </c>
       <c r="G127" s="86" t="inlineStr">
         <is>
@@ -30565,7 +30589,7 @@
       </c>
       <c r="D128" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre sueldo</t>
+          <t>Aporte SIJP sobre sueldo</t>
         </is>
       </c>
       <c r="E128" s="86" t="inlineStr">
@@ -30574,7 +30598,7 @@
         </is>
       </c>
       <c r="F128" s="93" t="n">
-        <v>3519.66</v>
+        <v>12905.43</v>
       </c>
       <c r="G128" s="86" t="inlineStr">
         <is>
@@ -30598,7 +30622,7 @@
       </c>
       <c r="D129" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre sueldo</t>
+          <t>Aporte INSSJP sobre sueldo</t>
         </is>
       </c>
       <c r="E129" s="86" t="inlineStr">
@@ -30631,16 +30655,16 @@
       </c>
       <c r="D130" s="86" t="inlineStr">
         <is>
-          <t>Diferencia impuesto año anterior</t>
-        </is>
-      </c>
-      <c r="E130" s="73" t="inlineStr">
-        <is>
-          <t>Devolución Ganancias</t>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E130" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F130" s="93" t="n">
-        <v>-3564748.04</v>
+        <v>3519.66</v>
       </c>
       <c r="G130" s="86" t="inlineStr">
         <is>
@@ -30664,16 +30688,16 @@
       </c>
       <c r="D131" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
-        </is>
-      </c>
-      <c r="E131" s="86" t="inlineStr">
-        <is>
-          <t>Descuento Ganancias</t>
+          <t>Diferencia impuesto año anterior</t>
+        </is>
+      </c>
+      <c r="E131" s="73" t="inlineStr">
+        <is>
+          <t>Devolución Ganancias</t>
         </is>
       </c>
       <c r="F131" s="93" t="n">
-        <v>3813479.69</v>
+        <v>-3564748.04</v>
       </c>
       <c r="G131" s="86" t="inlineStr">
         <is>
@@ -30697,16 +30721,16 @@
       </c>
       <c r="D132" s="86" t="inlineStr">
         <is>
-          <t>Dto Gimnasio</t>
+          <t>Impuesto pagado/devuelto</t>
         </is>
       </c>
       <c r="E132" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Descuento Ganancias</t>
         </is>
       </c>
       <c r="F132" s="93" t="n">
-        <v>23400</v>
+        <v>3813479.69</v>
       </c>
       <c r="G132" s="86" t="inlineStr">
         <is>
@@ -30717,33 +30741,33 @@
     <row r="133">
       <c r="A133" s="86" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="B133" s="86" t="inlineStr">
         <is>
-          <t>Sueldo</t>
+          <t>Sueldo + vacaciones</t>
         </is>
       </c>
       <c r="C133" s="87" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="D133" s="86" t="inlineStr">
         <is>
-          <t>Sueldo Básico</t>
+          <t>Dto Gimnasio</t>
         </is>
       </c>
       <c r="E133" s="86" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F133" s="93" t="n">
-        <v>11305702</v>
+        <v>23400</v>
       </c>
       <c r="G133" s="86" t="inlineStr">
         <is>
-          <t>MAYO.pdf</t>
+          <t>ABRIL.pdf</t>
         </is>
       </c>
     </row>
@@ -30763,7 +30787,7 @@
       </c>
       <c r="D134" s="86" t="inlineStr">
         <is>
-          <t>Beneficio Auto</t>
+          <t>Sueldo Básico</t>
         </is>
       </c>
       <c r="E134" s="86" t="inlineStr">
@@ -30772,7 +30796,7 @@
         </is>
       </c>
       <c r="F134" s="93" t="n">
-        <v>312000</v>
+        <v>11305702</v>
       </c>
       <c r="G134" s="86" t="inlineStr">
         <is>
@@ -30796,16 +30820,16 @@
       </c>
       <c r="D135" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre sueldo</t>
+          <t>Beneficio Auto</t>
         </is>
       </c>
       <c r="E135" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F135" s="93" t="n">
-        <v>473398.09</v>
+        <v>312000</v>
       </c>
       <c r="G135" s="86" t="inlineStr">
         <is>
@@ -30829,7 +30853,7 @@
       </c>
       <c r="D136" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre sueldo</t>
+          <t>Aporte SIJP sobre sueldo</t>
         </is>
       </c>
       <c r="E136" s="86" t="inlineStr">
@@ -30838,7 +30862,7 @@
         </is>
       </c>
       <c r="F136" s="93" t="n">
-        <v>129108.57</v>
+        <v>473398.09</v>
       </c>
       <c r="G136" s="86" t="inlineStr">
         <is>
@@ -30862,7 +30886,7 @@
       </c>
       <c r="D137" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre sueldo</t>
+          <t>Aporte INSSJP sobre sueldo</t>
         </is>
       </c>
       <c r="E137" s="86" t="inlineStr">
@@ -30895,16 +30919,16 @@
       </c>
       <c r="D138" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
+          <t>Aporte Obra Social sobre sueldo</t>
         </is>
       </c>
       <c r="E138" s="86" t="inlineStr">
         <is>
-          <t>Descuento Ganancias</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F138" s="93" t="n">
-        <v>3415603.09</v>
+        <v>129108.57</v>
       </c>
       <c r="G138" s="86" t="inlineStr">
         <is>
@@ -30928,16 +30952,16 @@
       </c>
       <c r="D139" s="86" t="inlineStr">
         <is>
-          <t>Dto Gimnasio</t>
+          <t>Impuesto pagado/devuelto</t>
         </is>
       </c>
       <c r="E139" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Descuento Ganancias</t>
         </is>
       </c>
       <c r="F139" s="93" t="n">
-        <v>23400</v>
+        <v>3415603.09</v>
       </c>
       <c r="G139" s="86" t="inlineStr">
         <is>
@@ -30948,33 +30972,33 @@
     <row r="140">
       <c r="A140" s="86" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="B140" s="86" t="inlineStr">
         <is>
-          <t>SAC 1° semestre</t>
+          <t>Sueldo</t>
         </is>
       </c>
       <c r="C140" s="87" t="n">
-        <v>46196</v>
+        <v>46174</v>
       </c>
       <c r="D140" s="86" t="inlineStr">
         <is>
-          <t>S.A.C.</t>
+          <t>Dto Gimnasio</t>
         </is>
       </c>
       <c r="E140" s="86" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F140" s="93" t="n">
-        <v>6622090.14</v>
+        <v>23400</v>
       </c>
       <c r="G140" s="86" t="inlineStr">
         <is>
-          <t>SAC.pdf</t>
+          <t>MAYO.pdf</t>
         </is>
       </c>
     </row>
@@ -30994,16 +31018,16 @@
       </c>
       <c r="D141" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre SAC</t>
+          <t>S.A.C.</t>
         </is>
       </c>
       <c r="E141" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F141" s="93" t="n">
-        <v>242805.88</v>
+        <v>6622090.14</v>
       </c>
       <c r="G141" s="86" t="inlineStr">
         <is>
@@ -31027,7 +31051,7 @@
       </c>
       <c r="D142" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre SAC</t>
+          <t>Aporte SIJP sobre SAC</t>
         </is>
       </c>
       <c r="E142" s="86" t="inlineStr">
@@ -31036,7 +31060,7 @@
         </is>
       </c>
       <c r="F142" s="93" t="n">
-        <v>66219.78999999999</v>
+        <v>242805.88</v>
       </c>
       <c r="G142" s="86" t="inlineStr">
         <is>
@@ -31060,7 +31084,7 @@
       </c>
       <c r="D143" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre SAC</t>
+          <t>Aporte INSSJP sobre SAC</t>
         </is>
       </c>
       <c r="E143" s="86" t="inlineStr">
@@ -31093,16 +31117,16 @@
       </c>
       <c r="D144" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
+          <t>Aporte Obra Social sobre SAC</t>
         </is>
       </c>
       <c r="E144" s="86" t="inlineStr">
         <is>
-          <t>Descuento Ganancias</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F144" s="93" t="n">
-        <v>536087.26</v>
+        <v>66219.78999999999</v>
       </c>
       <c r="G144" s="86" t="inlineStr">
         <is>
@@ -31118,28 +31142,28 @@
       </c>
       <c r="B145" s="86" t="inlineStr">
         <is>
-          <t>Sueldo</t>
+          <t>SAC 1° semestre</t>
         </is>
       </c>
       <c r="C145" s="87" t="n">
-        <v>46204</v>
+        <v>46196</v>
       </c>
       <c r="D145" s="86" t="inlineStr">
         <is>
-          <t>Sueldo Básico</t>
+          <t>Impuesto pagado/devuelto</t>
         </is>
       </c>
       <c r="E145" s="86" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Descuento Ganancias</t>
         </is>
       </c>
       <c r="F145" s="93" t="n">
-        <v>11305702</v>
+        <v>536087.26</v>
       </c>
       <c r="G145" s="86" t="inlineStr">
         <is>
-          <t>JUNIO.pdf</t>
+          <t>SAC.pdf</t>
         </is>
       </c>
     </row>
@@ -31159,7 +31183,7 @@
       </c>
       <c r="D146" s="86" t="inlineStr">
         <is>
-          <t>Beneficio Auto</t>
+          <t>Sueldo Básico</t>
         </is>
       </c>
       <c r="E146" s="86" t="inlineStr">
@@ -31168,7 +31192,7 @@
         </is>
       </c>
       <c r="F146" s="93" t="n">
-        <v>312000</v>
+        <v>11305702</v>
       </c>
       <c r="G146" s="86" t="inlineStr">
         <is>
@@ -31192,16 +31216,16 @@
       </c>
       <c r="D147" s="86" t="inlineStr">
         <is>
-          <t>Aporte SIJP sobre sueldo</t>
+          <t>Beneficio Auto</t>
         </is>
       </c>
       <c r="E147" s="86" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>Haber</t>
         </is>
       </c>
       <c r="F147" s="93" t="n">
-        <v>485611.76</v>
+        <v>312000</v>
       </c>
       <c r="G147" s="86" t="inlineStr">
         <is>
@@ -31225,7 +31249,7 @@
       </c>
       <c r="D148" s="86" t="inlineStr">
         <is>
-          <t>Aporte INSSJP sobre sueldo</t>
+          <t>Aporte SIJP sobre sueldo</t>
         </is>
       </c>
       <c r="E148" s="86" t="inlineStr">
@@ -31234,7 +31258,7 @@
         </is>
       </c>
       <c r="F148" s="93" t="n">
-        <v>132439.57</v>
+        <v>485611.76</v>
       </c>
       <c r="G148" s="86" t="inlineStr">
         <is>
@@ -31258,7 +31282,7 @@
       </c>
       <c r="D149" s="86" t="inlineStr">
         <is>
-          <t>Aporte Obra Social sobre sueldo</t>
+          <t>Aporte INSSJP sobre sueldo</t>
         </is>
       </c>
       <c r="E149" s="86" t="inlineStr">
@@ -31291,16 +31315,16 @@
       </c>
       <c r="D150" s="86" t="inlineStr">
         <is>
-          <t>Impuesto pagado/devuelto</t>
+          <t>Aporte Obra Social sobre sueldo</t>
         </is>
       </c>
       <c r="E150" s="86" t="inlineStr">
         <is>
-          <t>Descuento Ganancias</t>
+          <t>Descuento</t>
         </is>
       </c>
       <c r="F150" s="93" t="n">
-        <v>3408446.06</v>
+        <v>132439.57</v>
       </c>
       <c r="G150" s="86" t="inlineStr">
         <is>
@@ -31324,20 +31348,284 @@
       </c>
       <c r="D151" s="86" t="inlineStr">
         <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E151" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F151" s="93" t="n">
+        <v>3408446.06</v>
+      </c>
+      <c r="G151" s="86" t="inlineStr">
+        <is>
+          <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="86" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B152" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C152" s="87" t="n">
+        <v>46204</v>
+      </c>
+      <c r="D152" s="86" t="inlineStr">
+        <is>
           <t>Dto Gimnasio</t>
         </is>
       </c>
-      <c r="E151" s="86" t="inlineStr">
+      <c r="E152" s="86" t="inlineStr">
         <is>
           <t>Descuento</t>
         </is>
       </c>
-      <c r="F151" s="93" t="n">
+      <c r="F152" s="93" t="n">
         <v>23400</v>
       </c>
-      <c r="G151" s="86" t="inlineStr">
+      <c r="G152" s="86" t="inlineStr">
         <is>
           <t>JUNIO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B153" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C153" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D153" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo Básico</t>
+        </is>
+      </c>
+      <c r="E153" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F153" s="93" t="n">
+        <v>12662386</v>
+      </c>
+      <c r="G153" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B154" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C154" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D154" s="86" t="inlineStr">
+        <is>
+          <t>Beneficio Auto</t>
+        </is>
+      </c>
+      <c r="E154" s="86" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="F154" s="93" t="n">
+        <v>360000</v>
+      </c>
+      <c r="G154" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B155" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C155" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D155" s="86" t="inlineStr">
+        <is>
+          <t>Aporte SIJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E155" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F155" s="93" t="n">
+        <v>496052.42</v>
+      </c>
+      <c r="G155" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B156" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C156" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D156" s="86" t="inlineStr">
+        <is>
+          <t>Aporte INSSJP sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E156" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F156" s="93" t="n">
+        <v>135287.02</v>
+      </c>
+      <c r="G156" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B157" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C157" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D157" s="86" t="inlineStr">
+        <is>
+          <t>Aporte Obra Social sobre sueldo</t>
+        </is>
+      </c>
+      <c r="E157" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F157" s="93" t="n">
+        <v>135287.02</v>
+      </c>
+      <c r="G157" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B158" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C158" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D158" s="86" t="inlineStr">
+        <is>
+          <t>Impuesto pagado/devuelto</t>
+        </is>
+      </c>
+      <c r="E158" s="86" t="inlineStr">
+        <is>
+          <t>Descuento Ganancias</t>
+        </is>
+      </c>
+      <c r="F158" s="93" t="n">
+        <v>3445112.1</v>
+      </c>
+      <c r="G158" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="86" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B159" s="86" t="inlineStr">
+        <is>
+          <t>Sueldo</t>
+        </is>
+      </c>
+      <c r="C159" s="87" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D159" s="86" t="inlineStr">
+        <is>
+          <t>Dto Gimnasio</t>
+        </is>
+      </c>
+      <c r="E159" s="86" t="inlineStr">
+        <is>
+          <t>Descuento</t>
+        </is>
+      </c>
+      <c r="F159" s="93" t="n">
+        <v>25800</v>
+      </c>
+      <c r="G159" s="86" t="inlineStr">
+        <is>
+          <t>Tu Recibo.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CIUDAD Metrogas August bill (73187).
Register factura with vencimiento 18/08/2026 and débito automático; ceil from 73186.92 per GAS month rule.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -940,7 +940,9 @@
         <v>30643</v>
       </c>
       <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>73187</v>
+      </c>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
@@ -66266,12 +66268,42 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="53" t="n"/>
-      <c r="B70" s="14" t="n"/>
-      <c r="C70" s="14" t="n"/>
-      <c r="D70" s="15" t="n"/>
-      <c r="E70" s="14" t="n"/>
-      <c r="F70" s="18" t="n"/>
+      <c r="A70" s="53" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Metrogas</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>Metrogas CIUDAD · vence 18/08/2026 · emisión 05/08/2026 (débito automático; mes = vencimiento, no período consumo)</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="n">
+        <v>73187</v>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>Débito automático BBVA Visa</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>30010996459</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>40049923</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ceil desde $73.186,92 · período 06/06–07/07/2026 · 259,13 m3</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="53" t="n">

</xml_diff>

<commit_message>
Add Almacén Chris 80000 for August.
Record generic almacén spend paid by Chris in Almacen Detalle Importe Chris (2026-08-06).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -60717,15 +60717,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n"/>
-      <c r="C314" s="14" t="n"/>
+      <c r="B314" s="17" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C314" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
       <c r="D314" s="27" t="n"/>
-      <c r="E314" s="28" t="n"/>
+      <c r="E314" s="28" t="n">
+        <v>80000</v>
+      </c>
       <c r="F314" s="15">
-        <f>IF(OR(D298&lt;&gt;"",E298&lt;&gt;""),IF(D298="",0,D298)+IF(E298="",0,E298),"")</f>
-        <v/>
-      </c>
-      <c r="G314" s="14" t="n"/>
+        <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
+        <v/>
+      </c>
+      <c r="G314" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Add Almacén Chris 96932 for May.
Record May almacén spend paid by Chris in Almacen Detalle Importe Chris.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58563,14 +58564,24 @@
         </is>
       </c>
       <c r="B216" s="17" t="n"/>
-      <c r="C216" s="14" t="n"/>
+      <c r="C216" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
       <c r="D216" s="27" t="n"/>
-      <c r="E216" s="28" t="n"/>
+      <c r="E216" s="28" t="n">
+        <v>96932</v>
+      </c>
       <c r="F216" s="15">
-        <f>IF(OR(D211&lt;&gt;"",E211&lt;&gt;""),IF(D211="",0,D211)+IF(E211="",0,E211),"")</f>
-        <v/>
-      </c>
-      <c r="G216" s="14" t="n"/>
+        <f>IF(OR(D216&lt;&gt;"",E216&lt;&gt;""),IF(D216="",0,D216)+IF(E216="",0,E216),"")</f>
+        <v/>
+      </c>
+      <c r="G216" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Add Almacén Chris 101000 for June.
Record June almacén spend paid by Chris in Almacen Detalle Importe Chris.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59797,14 +59799,24 @@
         </is>
       </c>
       <c r="B268" s="17" t="n"/>
-      <c r="C268" s="14" t="n"/>
+      <c r="C268" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
       <c r="D268" s="27" t="n"/>
-      <c r="E268" s="28" t="n"/>
+      <c r="E268" s="28" t="n">
+        <v>101000</v>
+      </c>
       <c r="F268" s="15">
-        <f>IF(OR(D253&lt;&gt;"",E253&lt;&gt;""),IF(D253="",0,D253)+IF(E253="",0,E253),"")</f>
-        <v/>
-      </c>
-      <c r="G268" s="14" t="n"/>
+        <f>IF(OR(D268&lt;&gt;"",E268&lt;&gt;""),IF(D268="",0,D268)+IF(E268="",0,E268),"")</f>
+        <v/>
+      </c>
+      <c r="G268" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="14" t="inlineStr">
@@ -59944,6 +59956,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,6 +60724,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61377,6 +61391,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -62043,6 +62058,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62709,6 +62725,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63375,6 +63392,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add second May Almacén Chris entry (80000).
Correct month: both Chris almacén amounts belong to May (80000 + 96932).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -58548,14 +58548,24 @@
         </is>
       </c>
       <c r="B215" s="17" t="n"/>
-      <c r="C215" s="14" t="n"/>
+      <c r="C215" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
       <c r="D215" s="27" t="n"/>
-      <c r="E215" s="28" t="n"/>
+      <c r="E215" s="28" t="n">
+        <v>80000</v>
+      </c>
       <c r="F215" s="15">
-        <f>IF(OR(D210&lt;&gt;"",E210&lt;&gt;""),IF(D210="",0,D210)+IF(E210="",0,E210),"")</f>
-        <v/>
-      </c>
-      <c r="G215" s="14" t="n"/>
+        <f>IF(OR(D215&lt;&gt;"",E215&lt;&gt;""),IF(D215="",0,D215)+IF(E215="",0,E215),"")</f>
+        <v/>
+      </c>
+      <c r="G215" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="14" t="inlineStr">
@@ -58917,6 +58927,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59955,6 +59966,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60722,6 +60734,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61388,6 +61401,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -62054,6 +62068,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62720,6 +62735,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63386,6 +63402,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove misdated August Almacén Chris 80000.
That amount belongs to May and is recorded on the May Chris branch.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59944,6 +59946,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,33 +60714,22 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B314" s="17" t="n">
-        <v>46240</v>
-      </c>
-      <c r="C314" s="14" t="inlineStr">
-        <is>
-          <t>Almacén</t>
-        </is>
-      </c>
+      <c r="B314" s="17" t="n"/>
+      <c r="C314" s="14" t="n"/>
       <c r="D314" s="27" t="n"/>
-      <c r="E314" s="28" t="n">
-        <v>80000</v>
-      </c>
+      <c r="E314" s="28" t="n"/>
       <c r="F314" s="15">
         <f>IF(OR(D314&lt;&gt;"",E314&lt;&gt;""),IF(D314="",0,D314)+IF(E314="",0,E314),"")</f>
         <v/>
       </c>
-      <c r="G314" s="14" t="inlineStr">
-        <is>
-          <t>ALMACEN CHRIS</t>
-        </is>
-      </c>
+      <c r="G314" s="14" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="14" t="inlineStr">
@@ -61389,6 +61381,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -62055,6 +62048,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62721,6 +62715,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63387,6 +63382,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Move May Hoyts cinema from Almacén to Gasto Personal Sol.
Cine is personal Sol spend, not shared CIUDAD almacén.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3641,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F828"/>
+  <dimension ref="A1:F829"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25746,6 +25746,34 @@
       <c r="F828" s="34" t="inlineStr">
         <is>
           <t>SALUD · Vitaminas · Promarine · TC Mercado Pago · C.04/06 · gasto personal Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="52" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Cine</t>
+        </is>
+      </c>
+      <c r="D829" t="n">
+        <v>62200</v>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>BBVA MASTERCARD</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Cine · Hoyts · BBVA MASTERCARD · gasto personal Sol · ex ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -53464,32 +53492,16 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Mayo</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="n">
-        <v>46162</v>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>ENTRETENIMIENTO · Cine</t>
-        </is>
-      </c>
-      <c r="D16" s="27" t="n">
-        <v>62200</v>
-      </c>
+      <c r="A16" s="14" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="27" t="n"/>
       <c r="E16" s="28" t="n"/>
       <c r="F16" s="15">
         <f>IF(OR(D16&lt;&gt;"",E16&lt;&gt;""),IF(D16="",0,D16)+IF(E16="",0,E16),"")</f>
         <v/>
       </c>
-      <c r="G16" s="14" t="inlineStr">
-        <is>
-          <t>ENTRETENIMIENTO · Cine · Hoyts · BBVA MASTERCARD</t>
-        </is>
-      </c>
+      <c r="G16" s="14" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Move May Cosi Mi Piace dinner to Gasto Personal Sol.
Remove ENTRETENIMIENTO · Cenas from May Almacén; personal Sol spend.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -3641,7 +3641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F829"/>
+  <dimension ref="A1:F830"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25774,6 +25774,34 @@
       <c r="F829" t="inlineStr">
         <is>
           <t>ENTRETENIMIENTO · Cine · Hoyts · BBVA MASTERCARD · gasto personal Sol · ex ALMACEN SOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="52" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Cenas</t>
+        </is>
+      </c>
+      <c r="D830" t="n">
+        <v>30133</v>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>ENTRETENIMIENTO · Cenas · Cosi Mi Piace (cena) · Mercado Pago · ALMACEN SOL · gasto personal Sol · ex ALMACEN SOL</t>
         </is>
       </c>
     </row>
@@ -58814,27 +58842,15 @@
           <t>Mayo</t>
         </is>
       </c>
-      <c r="B225" s="17" t="n">
-        <v>46144</v>
-      </c>
-      <c r="C225" s="14" t="inlineStr">
-        <is>
-          <t>ENTRETENIMIENTO · Cenas</t>
-        </is>
-      </c>
-      <c r="D225" s="27" t="n">
-        <v>30133</v>
-      </c>
+      <c r="B225" s="17" t="n"/>
+      <c r="C225" s="14" t="n"/>
+      <c r="D225" s="27" t="n"/>
       <c r="E225" s="28" t="n"/>
       <c r="F225" s="15">
         <f>IF(OR(D225&lt;&gt;"",E225&lt;&gt;""),IF(D225="",0,D225)+IF(E225="",0,E225),"")</f>
         <v/>
       </c>
-      <c r="G225" s="14" t="inlineStr">
-        <is>
-          <t>ENTRETENIMIENTO · Cenas · Cosi Mi Piace (cena) · Mercado Pago · ALMACEN SOL</t>
-        </is>
-      </c>
+      <c r="G225" s="14" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Add Almacén Chris 155800 for July.
Record July almacén spend paid by Chris in Almacen Detalle Importe Chris.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59944,6 +59946,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60648,14 +60651,24 @@
         </is>
       </c>
       <c r="B310" s="17" t="n"/>
-      <c r="C310" s="14" t="n"/>
+      <c r="C310" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
       <c r="D310" s="27" t="n"/>
-      <c r="E310" s="28" t="n"/>
+      <c r="E310" s="28" t="n">
+        <v>155800</v>
+      </c>
       <c r="F310" s="15">
-        <f>IF(OR(D295&lt;&gt;"",E295&lt;&gt;""),IF(D295="",0,D295)+IF(E295="",0,E295),"")</f>
-        <v/>
-      </c>
-      <c r="G310" s="14" t="n"/>
+        <f>IF(OR(D310&lt;&gt;"",E310&lt;&gt;""),IF(D310="",0,D310)+IF(E310="",0,E310),"")</f>
+        <v/>
+      </c>
+      <c r="G310" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="14" t="inlineStr">
@@ -60711,6 +60724,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61377,6 +61391,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -62043,6 +62058,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62709,6 +62725,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63375,6 +63392,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add CIUDAD ABL August quota 08 (41344).
Register AGIP boleta with 1st due 14/08/2026; ceil from 41343.91; partida 3977389 from invoice.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>ABL — partida 397789</t>
+          <t>ABL — partida 3977389</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
@@ -1026,7 +1026,9 @@
       <c r="J9" s="5" t="n">
         <v>26175</v>
       </c>
-      <c r="K9" s="5" t="n"/>
+      <c r="K9" s="5" t="n">
+        <v>41344</v>
+      </c>
       <c r="L9" s="5" t="n"/>
       <c r="M9" s="5" t="n"/>
       <c r="N9" s="5" t="n"/>
@@ -66266,12 +66268,38 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="53" t="n"/>
-      <c r="B70" s="14" t="n"/>
-      <c r="C70" s="14" t="n"/>
-      <c r="D70" s="15" t="n"/>
-      <c r="E70" s="14" t="n"/>
+      <c r="A70" s="53" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>Agip ABL GCBA · partida 3977389 · CUOTA 08/2026</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="n">
+        <v>41344</v>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
       <c r="F70" s="18" t="n"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ceil desde $41.343,91 · 1° vto 14/08/2026 · boleta SANES · Ciudad de la Paz 1134</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="53" t="n">

</xml_diff>

<commit_message>
Record CIUDAD ABL paid by Sol via MP account balance.
Document Medio Mercado Pago — Dinero disponible and partida 3977389 in sheet notes, rules and abl_partidas.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1808,7 +1808,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>• ABL CIUDAD: partida AGIP 397789 (OHIGGINS = 3016365 → otra carpeta)</t>
+          <t>• ABL CIUDAD: partida AGIP 3977389 · paga Sol con Mercado Pago — Dinero disponible (dinero en cuenta). OHIGGINS = 3016365 → otra carpeta</t>
         </is>
       </c>
     </row>
@@ -66292,7 +66292,7 @@
       <c r="F70" s="18" t="n"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>ceil desde $41.343,91 · 1° vto 14/08/2026 · 2° vto 31/08 $49.477,73 · cuota $45.937,68 − bonif $4.593,77 · INM $19.359,65 + ABL $26.578,03 · pago electrónico 3977389 05 · Ciudad de la Paz 1134</t>
+          <t>ceil desde $41.343,91 · 1° vto 14/08/2026 · 2° vto 31/08 $49.477,73 · cuota $45.937,68 − bonif $4.593,77 · INM $19.359,65 + ABL $26.578,03 · pago electrónico 3977389 05 · Ciudad de la Paz 1134 · Sol paga MP dinero en cuenta</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">

</xml_diff>

<commit_message>
Add August verdulería 8900 to Almacén Sol.
Record COMIDA · VERDULERÍA in Almacen Detalle Importe Sol for August.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59944,6 +59946,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,6 +60714,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61341,15 +61345,27 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B353" s="17" t="n"/>
-      <c r="C353" s="14" t="n"/>
-      <c r="D353" s="27" t="n"/>
+      <c r="B353" s="17" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C353" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
+      <c r="D353" s="27" t="n">
+        <v>8900</v>
+      </c>
       <c r="E353" s="28" t="n"/>
       <c r="F353" s="15">
-        <f>IF(OR(D337&lt;&gt;"",E337&lt;&gt;""),IF(D337="",0,D337)+IF(E337="",0,E337),"")</f>
-        <v/>
-      </c>
-      <c r="G353" s="14" t="n"/>
+        <f>IF(OR(D353&lt;&gt;"",E353&lt;&gt;""),IF(D353="",0,D353)+IF(E353="",0,E353),"")</f>
+        <v/>
+      </c>
+      <c r="G353" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="10" t="inlineStr">
@@ -61377,6 +61393,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -62043,6 +62060,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62709,6 +62727,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63375,6 +63394,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Load Susana limpieza CIUDAD through 5 Sep 2026.
Update Julio (400640→653120), add Agosto 567080 and Septiembre 198800 in matriz 2026 and Detalle; leave May/Jun unchanged.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -1071,10 +1071,14 @@
         <v>876981</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>400640</v>
-      </c>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
+        <v>653120</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>567080</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>198800</v>
+      </c>
       <c r="M10" s="9" t="n"/>
       <c r="N10" s="9" t="n"/>
       <c r="O10" s="9" t="n"/>
@@ -64106,7 +64110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66350,6 +66354,111 @@
       <c r="F73" s="18" t="inlineStr">
         <is>
           <t>3491192</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="53" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA — Julio 2026</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="n">
+        <v>653120</v>
+      </c>
+      <c r="E74" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="n"/>
+      <c r="G74" s="18" t="n"/>
+      <c r="H74" s="14" t="inlineStr">
+        <is>
+          <t>Transferencia MP · Susana Carmen Ortiz consolidado (5/7 9500+123240; 12/7 120240; 18/7 147660; 25/7 126240; 31/7 126240)</t>
+        </is>
+      </c>
+      <c r="I74" s="14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="53" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA — Agosto 2026</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="n">
+        <v>567080</v>
+      </c>
+      <c r="E75" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="n"/>
+      <c r="G75" s="18" t="n"/>
+      <c r="H75" s="14" t="inlineStr">
+        <is>
+          <t>Transferencia MP · Susana Carmen Ortiz consolidado (8/8 123240; 16/8 126240; 22/8 154800+3800; 29/8 150000+9000)</t>
+        </is>
+      </c>
+      <c r="I75" s="14" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="53" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>LIMPIEZA CASA — Septiembre 2026 (al 5/9)</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="n">
+        <v>198800</v>
+      </c>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="n"/>
+      <c r="G76" s="18" t="n"/>
+      <c r="H76" s="14" t="inlineStr">
+        <is>
+          <t>Transferencia MP · Susana Carmen Ortiz · 05/09/2026 · 160000+38800</t>
+        </is>
+      </c>
+      <c r="I76" s="14" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Sodastream tube refill to September Almacén Sol.
Record $89,000 on 2026-09-08 as REPUESTOS · Sodastream (three tubes) in Almacen Detalle and refresh the SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59944,6 +59946,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,6 +60714,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61377,21 +61381,34 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B356" s="17" t="n"/>
-      <c r="C356" s="14" t="n"/>
-      <c r="D356" s="27" t="n"/>
+      <c r="B356" s="53" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C356" s="14" t="inlineStr">
+        <is>
+          <t>REPUESTOS · Sodastream</t>
+        </is>
+      </c>
+      <c r="D356" s="27" t="n">
+        <v>89000</v>
+      </c>
       <c r="E356" s="28" t="n"/>
       <c r="F356" s="15">
-        <f>IF(OR(D340&lt;&gt;"",E340&lt;&gt;""),IF(D340="",0,D340)+IF(E340="",0,E340),"")</f>
-        <v/>
-      </c>
-      <c r="G356" s="14" t="n"/>
+        <f>IF(OR(D356&lt;&gt;"",E356&lt;&gt;""),IF(D356="",0,D356)+IF(E356="",0,E356),"")</f>
+        <v/>
+      </c>
+      <c r="G356" s="14" t="inlineStr">
+        <is>
+          <t>Recambio de tres tubos de Soda Stream</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Add September Almacén cerdo purchase for $13,000.
Record COMIDA · cerdo on 2026-09-08 in Almacen Detalle and refresh the SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -61416,15 +61416,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B357" s="17" t="n"/>
-      <c r="C357" s="14" t="n"/>
-      <c r="D357" s="27" t="n"/>
+      <c r="B357" s="53" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C357" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · cerdo</t>
+        </is>
+      </c>
+      <c r="D357" s="27" t="n">
+        <v>13000</v>
+      </c>
       <c r="E357" s="28" t="n"/>
       <c r="F357" s="15">
-        <f>IF(OR(D341&lt;&gt;"",E341&lt;&gt;""),IF(D341="",0,D341)+IF(E341="",0,E341),"")</f>
-        <v/>
-      </c>
-      <c r="G357" s="14" t="n"/>
+        <f>IF(OR(D357&lt;&gt;"",E357&lt;&gt;""),IF(D357="",0,D357)+IF(E357="",0,E357),"")</f>
+        <v/>
+      </c>
+      <c r="G357" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · cerdo</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Add September Almacén verdulería purchase for $8,300.
Record COMIDA · VERDULERÍA on 2026-09-08 in Almacen Detalle and refresh the SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -61444,15 +61444,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B358" s="17" t="n"/>
-      <c r="C358" s="14" t="n"/>
-      <c r="D358" s="27" t="n"/>
+      <c r="B358" s="53" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C358" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
+      <c r="D358" s="27" t="n">
+        <v>8300</v>
+      </c>
       <c r="E358" s="28" t="n"/>
       <c r="F358" s="15">
-        <f>IF(OR(D342&lt;&gt;"",E342&lt;&gt;""),IF(D342="",0,D342)+IF(E342="",0,E342),"")</f>
-        <v/>
-      </c>
-      <c r="G358" s="14" t="n"/>
+        <f>IF(OR(D358&lt;&gt;"",E358&lt;&gt;""),IF(D358="",0,D358)+IF(E358="",0,E358),"")</f>
+        <v/>
+      </c>
+      <c r="G358" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · VERDULERÍA</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="14" t="inlineStr">
@@ -62072,6 +62084,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62738,6 +62751,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63404,6 +63418,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add September Almacén Farmacity purchase for $20,000.
Record FARMACIA · Farmacity on 2026-09-08 in Almacen Detalle and refresh the SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -61472,15 +61472,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B359" s="17" t="n"/>
-      <c r="C359" s="14" t="n"/>
-      <c r="D359" s="27" t="n"/>
+      <c r="B359" s="53" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C359" s="14" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacity</t>
+        </is>
+      </c>
+      <c r="D359" s="27" t="n">
+        <v>20000</v>
+      </c>
       <c r="E359" s="28" t="n"/>
       <c r="F359" s="15">
-        <f>IF(OR(D343&lt;&gt;"",E343&lt;&gt;""),IF(D343="",0,D343)+IF(E343="",0,E343),"")</f>
-        <v/>
-      </c>
-      <c r="G359" s="14" t="n"/>
+        <f>IF(OR(D359&lt;&gt;"",E359&lt;&gt;""),IF(D359="",0,D359)+IF(E359="",0,E359),"")</f>
+        <v/>
+      </c>
+      <c r="G359" s="14" t="inlineStr">
+        <is>
+          <t>FARMACIA · Farmacity</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="14" t="inlineStr">
@@ -62084,7 +62096,6 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
-    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62751,7 +62762,6 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
-    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63418,7 +63428,6 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
-    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Relabel September farmacia spend as FARMACIA · SMS.
Keep the $20,000 Almacén row on 2026-09-08 and refresh the SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,7 +57624,6 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58907,7 +58906,6 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
-    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59946,7 +59944,6 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
-    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60714,7 +60711,6 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
-    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61381,7 +61377,6 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
-    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -61477,7 +61472,7 @@
       </c>
       <c r="C359" s="14" t="inlineStr">
         <is>
-          <t>FARMACIA · Farmacity</t>
+          <t>FARMACIA · SMS</t>
         </is>
       </c>
       <c r="D359" s="27" t="n">
@@ -61490,7 +61485,7 @@
       </c>
       <c r="G359" s="14" t="inlineStr">
         <is>
-          <t>FARMACIA · Farmacity</t>
+          <t>FARMACIA · SMS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore Almacén Chris amounts missing from the CIUDAD workbook.
Re-add Mayo ($80.000 + $96.932), Junio ($101.000) and Julio ($155.800)
that were recorded earlier but never landed on master, then regenerate the
rendition with Sol/Chris columns.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58387,14 +58388,26 @@
         </is>
       </c>
       <c r="B205" s="17" t="n"/>
-      <c r="C205" s="14" t="n"/>
-      <c r="D205" s="27" t="n"/>
-      <c r="E205" s="28" t="n"/>
+      <c r="C205" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+      <c r="D205" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E205" s="28" t="n">
+        <v>80000</v>
+      </c>
       <c r="F205" s="15">
         <f>IF(OR(D200&lt;&gt;"",E200&lt;&gt;""),IF(D200="",0,D200)+IF(E200="",0,E200),"")</f>
         <v/>
       </c>
-      <c r="G205" s="14" t="n"/>
+      <c r="G205" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="14" t="inlineStr">
@@ -58403,14 +58416,26 @@
         </is>
       </c>
       <c r="B206" s="17" t="n"/>
-      <c r="C206" s="14" t="n"/>
-      <c r="D206" s="27" t="n"/>
-      <c r="E206" s="28" t="n"/>
+      <c r="C206" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+      <c r="D206" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E206" s="28" t="n">
+        <v>96932</v>
+      </c>
       <c r="F206" s="15">
         <f>IF(OR(D201&lt;&gt;"",E201&lt;&gt;""),IF(D201="",0,D201)+IF(E201="",0,E201),"")</f>
         <v/>
       </c>
-      <c r="G206" s="14" t="n"/>
+      <c r="G206" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="14" t="inlineStr">
@@ -58906,6 +58931,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59557,14 +59583,26 @@
         </is>
       </c>
       <c r="B253" s="17" t="n"/>
-      <c r="C253" s="14" t="n"/>
-      <c r="D253" s="27" t="n"/>
-      <c r="E253" s="28" t="n"/>
+      <c r="C253" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+      <c r="D253" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E253" s="28" t="n">
+        <v>101000</v>
+      </c>
       <c r="F253" s="15">
         <f>IF(OR(D238&lt;&gt;"",E238&lt;&gt;""),IF(D238="",0,D238)+IF(E238="",0,E238),"")</f>
         <v/>
       </c>
-      <c r="G253" s="14" t="n"/>
+      <c r="G253" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="14" t="inlineStr">
@@ -59944,6 +59982,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60296,14 +60335,26 @@
         </is>
       </c>
       <c r="B288" s="17" t="n"/>
-      <c r="C288" s="14" t="n"/>
-      <c r="D288" s="27" t="n"/>
-      <c r="E288" s="28" t="n"/>
+      <c r="C288" s="14" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+      <c r="D288" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E288" s="28" t="n">
+        <v>155800</v>
+      </c>
       <c r="F288" s="15">
         <f>IF(OR(D273&lt;&gt;"",E273&lt;&gt;""),IF(D273="",0,D273)+IF(E273="",0,E273),"")</f>
         <v/>
       </c>
-      <c r="G288" s="14" t="n"/>
+      <c r="G288" s="14" t="inlineStr">
+        <is>
+          <t>ALMACEN CHRIS</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="14" t="inlineStr">
@@ -60711,6 +60762,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61377,6 +61429,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -62043,6 +62096,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62709,6 +62763,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63375,6 +63430,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add September Almacén huevos purchase for $7,000.
Record COMIDA · Huevos Point on 2026-09-10 in Almacen Detalle and refresh the SOL master.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
+++ b/CIUDAD/Gastos_CIUDAD_1132_2026.xlsx
@@ -57624,6 +57624,7 @@
       </c>
       <c r="G176" s="22" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
@@ -58906,6 +58907,7 @@
       </c>
       <c r="G228" s="22" t="n"/>
     </row>
+    <row r="229"/>
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
@@ -59944,6 +59946,7 @@
       </c>
       <c r="G273" s="22" t="n"/>
     </row>
+    <row r="274"/>
     <row r="275">
       <c r="A275" s="14" t="inlineStr">
         <is>
@@ -60711,6 +60714,7 @@
       </c>
       <c r="G312" s="22" t="n"/>
     </row>
+    <row r="313"/>
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
@@ -61377,6 +61381,7 @@
       </c>
       <c r="G354" s="22" t="n"/>
     </row>
+    <row r="355"/>
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
@@ -61495,15 +61500,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B360" s="17" t="n"/>
-      <c r="C360" s="14" t="n"/>
-      <c r="D360" s="27" t="n"/>
+      <c r="B360" s="53" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C360" s="14" t="inlineStr">
+        <is>
+          <t>COMIDA · Huevos Point</t>
+        </is>
+      </c>
+      <c r="D360" s="27" t="n">
+        <v>7000</v>
+      </c>
       <c r="E360" s="28" t="n"/>
       <c r="F360" s="15">
-        <f>IF(OR(D344&lt;&gt;"",E344&lt;&gt;""),IF(D344="",0,D344)+IF(E344="",0,E344),"")</f>
-        <v/>
-      </c>
-      <c r="G360" s="14" t="n"/>
+        <f>IF(OR(D360&lt;&gt;"",E360&lt;&gt;""),IF(D360="",0,D360)+IF(E360="",0,E360),"")</f>
+        <v/>
+      </c>
+      <c r="G360" s="14" t="inlineStr">
+        <is>
+          <t>Compra de huevos</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="14" t="inlineStr">
@@ -62091,6 +62108,7 @@
       </c>
       <c r="G396" s="22" t="n"/>
     </row>
+    <row r="397"/>
     <row r="398">
       <c r="A398" s="14" t="inlineStr">
         <is>
@@ -62757,6 +62775,7 @@
       </c>
       <c r="G438" s="22" t="n"/>
     </row>
+    <row r="439"/>
     <row r="440">
       <c r="A440" s="14" t="inlineStr">
         <is>
@@ -63423,6 +63442,7 @@
       </c>
       <c r="G480" s="22" t="n"/>
     </row>
+    <row r="481"/>
     <row r="482">
       <c r="A482" s="14" t="inlineStr">
         <is>

</xml_diff>